<commit_message>
🤖 Daily run: 2026-09-14 17:52
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$46</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -27,7 +27,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Por_Tipo'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Por_Area'!$A$1:$B$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Por_Area'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Por_Orgao'!$A$1:$B$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Por_Orgao'!$A$1:$B$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Por_Orgao'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Perfis'!$A$1:$C$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'Perfis'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 12/09/2026 às 15:02</t>
+          <t>Gerado em 14/09/2026 às 17:46</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6">
@@ -620,7 +620,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>165288.4615384615</v>
+        <v>168816</v>
       </c>
     </row>
     <row r="20">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="24">
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25">
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O48"/>
+  <dimension ref="A1:O46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -876,16 +876,16 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>146343</v>
+        <v>146353</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
-          <t>TR 005/2026 - ASPAD - MDA - Contratação de consultoria especializada para participação social no Plano Safra da Agricultura Familiar</t>
+          <t>TR - Mobilização Territorial/2026 - Suporte técnico especializado para Avaliação de Efetividade e Metodologias para Mobilização Territorial e Acesso a Instrumentos de Desenvolvimento</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E2" s="12" t="inlineStr">
@@ -898,7 +898,7 @@
       </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H2" s="11" t="inlineStr">
@@ -908,14 +908,14 @@
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>Brasília/DF</t>
+          <t>Região Centro Oeste</t>
         </is>
       </c>
       <c r="J2" s="14" t="n">
-        <v>46268</v>
+        <v>46273</v>
       </c>
       <c r="K2" s="14" t="n">
-        <v>46277</v>
+        <v>46283</v>
       </c>
       <c r="L2" s="15" t="inlineStr"/>
       <c r="M2" s="9" t="inlineStr">
@@ -925,7 +925,7 @@
       </c>
       <c r="N2" s="12" t="inlineStr">
         <is>
-          <t>cgctf.editais@mda.gov.br</t>
+          <t>prodocbra23018@sudeco.gov.br</t>
         </is>
       </c>
       <c r="O2" s="16" t="inlineStr">
@@ -941,16 +941,16 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>146349</v>
+        <v>146368</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
-          <t>BRA/23/006 - CONSULTORIA TÉCNICA PARA O DESENVOLVIMENTO DE TECNOLOGIA APLICADA AO OBSERVATÓRIO DO NORDESTE</t>
+          <t>Edital 6/2026- UGP-PNUD/SENAD</t>
         </is>
       </c>
       <c r="D3" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E3" s="20" t="inlineStr">
@@ -963,7 +963,7 @@
       </c>
       <c r="G3" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H3" s="19" t="inlineStr">
@@ -973,14 +973,14 @@
       </c>
       <c r="I3" s="19" t="inlineStr">
         <is>
-          <t>HOME OFFICE</t>
+          <t>null</t>
         </is>
       </c>
       <c r="J3" s="22" t="n">
-        <v>46267</v>
+        <v>46275</v>
       </c>
       <c r="K3" s="22" t="n">
-        <v>46278</v>
+        <v>46280</v>
       </c>
       <c r="L3" s="23" t="inlineStr"/>
       <c r="M3" s="17" t="inlineStr">
@@ -990,7 +990,7 @@
       </c>
       <c r="N3" s="20" t="inlineStr">
         <is>
-          <t>curriculos@consorcionordeste.gov.br</t>
+          <t>cgep@mj.gov.br</t>
         </is>
       </c>
       <c r="O3" s="24" t="inlineStr">
@@ -1006,16 +1006,16 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>146353</v>
+        <v>146367</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>TR - Mobilização Territorial/2026 - Suporte técnico especializado para Avaliação de Efetividade e Metodologias para Mobilização Territorial e Acesso a Instrumentos de Desenvolvimento</t>
+          <t>EDITAL Nº 5/2026 - UGP-PNUD/SENAD</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E4" s="12" t="inlineStr">
@@ -1028,7 +1028,7 @@
       </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H4" s="11" t="inlineStr">
@@ -1038,14 +1038,14 @@
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>Região Centro Oeste</t>
+          <t>Brasília/DF</t>
         </is>
       </c>
       <c r="J4" s="14" t="n">
-        <v>46273</v>
+        <v>46275</v>
       </c>
       <c r="K4" s="14" t="n">
-        <v>46283</v>
+        <v>46280</v>
       </c>
       <c r="L4" s="15" t="inlineStr"/>
       <c r="M4" s="9" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="N4" s="12" t="inlineStr">
         <is>
-          <t>prodocbra23018@sudeco.gov.br</t>
+          <t>cgep@mj.gov.br</t>
         </is>
       </c>
       <c r="O4" s="16" t="inlineStr">
@@ -1071,11 +1071,11 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>146368</v>
+        <v>146365</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t>Edital 6/2026- UGP-PNUD/SENAD</t>
+          <t>EDITAL Nº 4/2026 - UGP-PNUD/SENAD</t>
         </is>
       </c>
       <c r="D5" s="19" t="inlineStr">
@@ -1093,7 +1093,7 @@
       </c>
       <c r="G5" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H5" s="19" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="N5" s="20" t="inlineStr">
         <is>
-          <t>cgep@mj.gov.br</t>
+          <t>dpagi@mj.gov.br</t>
         </is>
       </c>
       <c r="O5" s="24" t="inlineStr">
@@ -1136,11 +1136,11 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>146367</v>
+        <v>146364</v>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>EDITAL Nº 5/2026 - UGP-PNUD/SENAD</t>
+          <t>EDITAL Nº 3/2026 - UGP-PNUD/SENAD</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr">
@@ -1168,7 +1168,7 @@
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>Brasília/DF</t>
+          <t>null</t>
         </is>
       </c>
       <c r="J6" s="14" t="n">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="N6" s="12" t="inlineStr">
         <is>
-          <t>cgep@mj.gov.br</t>
+          <t>dpagi@mj.gov.br</t>
         </is>
       </c>
       <c r="O6" s="16" t="inlineStr">
@@ -1201,11 +1201,11 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>146365</v>
+        <v>146363</v>
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t>EDITAL Nº 4/2026 - UGP-PNUD/SENAD</t>
+          <t>EDITAL Nº 2/2026 - UGP-PNUD/SENAD</t>
         </is>
       </c>
       <c r="D7" s="19" t="inlineStr">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="G7" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H7" s="19" t="inlineStr">
@@ -1250,7 +1250,7 @@
       </c>
       <c r="N7" s="20" t="inlineStr">
         <is>
-          <t>dpagi@mj.gov.br</t>
+          <t>senad@mj.gov.br</t>
         </is>
       </c>
       <c r="O7" s="24" t="inlineStr">
@@ -1266,11 +1266,11 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>146364</v>
+        <v>146369</v>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>EDITAL Nº 3/2026 - UGP-PNUD/SENAD</t>
+          <t>Edital nº 29/2026 – Contratação de Consultoria Individual para o desenho institucional da Secretaria de Serviços Compartilhados (SSC/MGI)</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
@@ -1280,34 +1280,34 @@
       </c>
       <c r="E8" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F8" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F8" s="13" t="inlineStr"/>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H8" s="11" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>MGI</t>
         </is>
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J8" s="14" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="K8" s="14" t="n">
-        <v>46280</v>
-      </c>
-      <c r="L8" s="15" t="inlineStr"/>
+        <v>46290</v>
+      </c>
+      <c r="L8" s="15" t="n">
+        <v>120000</v>
+      </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1315,7 +1315,7 @@
       </c>
       <c r="N8" s="12" t="inlineStr">
         <is>
-          <t>dpagi@mj.gov.br</t>
+          <t>prodoc.mgi@gestao.gov.br</t>
         </is>
       </c>
       <c r="O8" s="16" t="inlineStr">
@@ -1331,11 +1331,11 @@
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>146363</v>
+        <v>146370</v>
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>EDITAL Nº 2/2026 - UGP-PNUD/SENAD</t>
+          <t xml:space="preserve">Edital nº 25/2026 – Contratação de Consultoria Individual para avaliar os efeitos de intervenções comportamentais (políticas fiscais e de arquitetura de escolha) em mercado experimental para promover escolhas alimentares mais saudáveis. </t>
         </is>
       </c>
       <c r="D9" s="19" t="inlineStr">
@@ -1345,34 +1345,34 @@
       </c>
       <c r="E9" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F9" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F9" s="21" t="inlineStr"/>
       <c r="G9" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H9" s="19" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>MGI</t>
         </is>
       </c>
       <c r="I9" s="19" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>REMOTO</t>
         </is>
       </c>
       <c r="J9" s="22" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="K9" s="22" t="n">
-        <v>46280</v>
-      </c>
-      <c r="L9" s="23" t="inlineStr"/>
+        <v>46290</v>
+      </c>
+      <c r="L9" s="23" t="n">
+        <v>126000</v>
+      </c>
       <c r="M9" s="17" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1380,7 +1380,7 @@
       </c>
       <c r="N9" s="20" t="inlineStr">
         <is>
-          <t>senad@mj.gov.br</t>
+          <t>prodoc.mgi@gestao.gov.br</t>
         </is>
       </c>
       <c r="O9" s="24" t="inlineStr">
@@ -1396,11 +1396,11 @@
         </is>
       </c>
       <c r="B10" s="10" t="n">
-        <v>146369</v>
+        <v>146360</v>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>Edital nº 29/2026 – Contratação de Consultoria Individual para o desenho institucional da Secretaria de Serviços Compartilhados (SSC/MGI)</t>
+          <t>PNUD BRA/25/024 - Edital nº 04/2026 – Contrat. de consult. - Engenharia de Dados</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
@@ -1410,33 +1410,35 @@
       </c>
       <c r="E10" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F10" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F10" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>MTE</t>
         </is>
       </c>
       <c r="I10" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J10" s="14" t="n">
-        <v>46276</v>
+        <v>46279</v>
       </c>
       <c r="K10" s="14" t="n">
-        <v>46290</v>
+        <v>46287</v>
       </c>
       <c r="L10" s="15" t="n">
-        <v>120000</v>
+        <v>130000</v>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
@@ -1445,7 +1447,7 @@
       </c>
       <c r="N10" s="12" t="inlineStr">
         <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
+          <t>estatisticastrabalho@trabalho.gov.br</t>
         </is>
       </c>
       <c r="O10" s="16" t="inlineStr">
@@ -1461,11 +1463,11 @@
         </is>
       </c>
       <c r="B11" s="18" t="n">
-        <v>146370</v>
+        <v>146361</v>
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edital nº 25/2026 – Contratação de Consultoria Individual para avaliar os efeitos de intervenções comportamentais (políticas fiscais e de arquitetura de escolha) em mercado experimental para promover escolhas alimentares mais saudáveis. </t>
+          <t>PNUD BRA/25/024 - Consultoria Especializada - Qualidade de Dados I</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
@@ -1475,33 +1477,35 @@
       </c>
       <c r="E11" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F11" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F11" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G11" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H11" s="19" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>MTE</t>
         </is>
       </c>
       <c r="I11" s="19" t="inlineStr">
         <is>
-          <t>REMOTO</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J11" s="22" t="n">
-        <v>46276</v>
+        <v>46279</v>
       </c>
       <c r="K11" s="22" t="n">
-        <v>46290</v>
+        <v>46287</v>
       </c>
       <c r="L11" s="23" t="n">
-        <v>126000</v>
+        <v>130000</v>
       </c>
       <c r="M11" s="17" t="inlineStr">
         <is>
@@ -1510,7 +1514,7 @@
       </c>
       <c r="N11" s="20" t="inlineStr">
         <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
+          <t>estatisticastrabalho@trabalho.gov.br</t>
         </is>
       </c>
       <c r="O11" s="24" t="inlineStr">
@@ -1522,17 +1526,15 @@
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B12" s="10" t="inlineStr">
-        <is>
-          <t>unesco:5c1d62c6-1efa-431c-b9e2-08df0436270c</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="n">
+        <v>146362</v>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 54/2026 - 1 vaga - Consultor Individual</t>
+          <t>PNUD BRA/25/024 - Edital nº 06/2026 - Consultoria Especializada - Qualidade de Dados II</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
@@ -1550,31 +1552,41 @@
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I12" s="11" t="inlineStr"/>
+          <t>MTE</t>
+        </is>
+      </c>
+      <c r="I12" s="11" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J12" s="14" t="n">
-        <v>46274</v>
+        <v>46279</v>
       </c>
       <c r="K12" s="14" t="n">
-        <v>46278</v>
-      </c>
-      <c r="L12" s="15" t="inlineStr"/>
+        <v>46287</v>
+      </c>
+      <c r="L12" s="15" t="n">
+        <v>130000</v>
+      </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N12" s="12" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N12" s="12" t="inlineStr">
+        <is>
+          <t>estatisticastrabalho@trabalho.gov.br</t>
+        </is>
+      </c>
       <c r="O12" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
@@ -1586,12 +1598,12 @@
       </c>
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t>unesco:1d72ac67-6c7d-4a8b-dd78-08df0757caed</t>
+          <t>unesco:8c824e7b-7b9a-4a59-7ffc-08df082d82f3</t>
         </is>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1154 - Edital 05/2026 - 01 perfil - Consultoria Individual</t>
+          <t>914BRZ1163 - Publicação -  Edital 68/2026 - 01 Vaga consultor Individual</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
@@ -1609,7 +1621,7 @@
       </c>
       <c r="G13" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H13" s="19" t="inlineStr">
@@ -1619,10 +1631,10 @@
       </c>
       <c r="I13" s="19" t="inlineStr"/>
       <c r="J13" s="22" t="n">
-        <v>46268</v>
+        <v>46276</v>
       </c>
       <c r="K13" s="22" t="n">
-        <v>46278</v>
+        <v>46281</v>
       </c>
       <c r="L13" s="23" t="inlineStr"/>
       <c r="M13" s="17" t="inlineStr">
@@ -1645,12 +1657,12 @@
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>unesco:8c824e7b-7b9a-4a59-7ffc-08df082d82f3</t>
+          <t>unesco:5907e744-d46d-4c01-2eaf-08df08e94b75</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1163 - Publicação -  Edital 68/2026 - 01 Vaga consultor Individual</t>
+          <t>914BRZ1159 - Publicação Edital 37/2026 - 2 vagas - Consultor Individual</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -1668,7 +1680,7 @@
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
@@ -1678,10 +1690,10 @@
       </c>
       <c r="I14" s="11" t="inlineStr"/>
       <c r="J14" s="14" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="K14" s="14" t="n">
-        <v>46281</v>
+        <v>46283</v>
       </c>
       <c r="L14" s="15" t="inlineStr"/>
       <c r="M14" s="9" t="inlineStr">
@@ -1704,12 +1716,12 @@
       </c>
       <c r="B15" s="18" t="inlineStr">
         <is>
-          <t>unesco:5907e744-d46d-4c01-2eaf-08df08e94b75</t>
+          <t>unesco:1011b77e-9c7a-4ea9-2632-08df0e687345</t>
         </is>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 37/2026 - 2 vagas - Consultor Individual</t>
+          <t>914BRZ1159 - Publicação Edital 39/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
@@ -1727,7 +1739,7 @@
       </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H15" s="19" t="inlineStr">
@@ -1737,7 +1749,7 @@
       </c>
       <c r="I15" s="19" t="inlineStr"/>
       <c r="J15" s="22" t="n">
-        <v>46277</v>
+        <v>46279</v>
       </c>
       <c r="K15" s="22" t="n">
         <v>46283</v>
@@ -1763,12 +1775,12 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>unesco:b0920c88-ab66-4545-2ead-08df08e94b75</t>
+          <t>unesco:030ad7b8-d33f-491a-31d9-08defb16c1ac</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ3050 - Edital N° 04/2026 - Consultor Individual PRORROGAÇÃO</t>
+          <t>Projeto 914BRZ5067 - Edital Nº 08/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -1786,7 +1798,7 @@
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
@@ -1796,10 +1808,10 @@
       </c>
       <c r="I16" s="11" t="inlineStr"/>
       <c r="J16" s="14" t="n">
-        <v>46274</v>
+        <v>46253</v>
       </c>
       <c r="K16" s="14" t="n">
-        <v>46278</v>
+        <v>46283</v>
       </c>
       <c r="L16" s="15" t="inlineStr"/>
       <c r="M16" s="9" t="inlineStr">
@@ -1822,12 +1834,12 @@
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>unesco:030ad7b8-d33f-491a-31d9-08defb16c1ac</t>
+          <t>unesco:a42aa3e1-2e33-46e6-2633-08df0e687345</t>
         </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ5067 - Edital Nº 08/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1159 - Publicação Edital 38/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1855,7 +1867,7 @@
       </c>
       <c r="I17" s="19" t="inlineStr"/>
       <c r="J17" s="22" t="n">
-        <v>46253</v>
+        <v>46279</v>
       </c>
       <c r="K17" s="22" t="n">
         <v>46283</v>
@@ -1876,57 +1888,69 @@
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>unesco:b260be61-61f9-4226-2eb0-08df08e94b75</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3061 - EDITAL Nº 13/2026 - 01 VAGA - CONSULTOR INDIVIDUAL-REPUBLICACAO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13015</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F18" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F18" s="13" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I18" s="11" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I18" s="11" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J18" s="14" t="n">
-        <v>46273</v>
+        <v>46220</v>
       </c>
       <c r="K18" s="14" t="n">
-        <v>46278</v>
-      </c>
-      <c r="L18" s="15" t="inlineStr"/>
+        <v>46225</v>
+      </c>
+      <c r="L18" s="15" t="n">
+        <v>58800</v>
+      </c>
       <c r="M18" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N18" s="12" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N18" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O18" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015/</t>
         </is>
       </c>
     </row>
@@ -1938,17 +1962,17 @@
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13078</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13098</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E19" s="20" t="inlineStr">
@@ -1957,16 +1981,16 @@
         </is>
       </c>
       <c r="F19" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I19" s="19" t="inlineStr">
@@ -1975,17 +1999,15 @@
         </is>
       </c>
       <c r="J19" s="22" t="n">
-        <v>46217</v>
+        <v>46221</v>
       </c>
       <c r="K19" s="22" t="n">
-        <v>46222</v>
-      </c>
-      <c r="L19" s="23" t="n">
-        <v>77100</v>
-      </c>
+        <v>46224</v>
+      </c>
+      <c r="L19" s="23" t="inlineStr"/>
       <c r="M19" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N19" s="20" t="inlineStr">
@@ -1995,7 +2017,7 @@
       </c>
       <c r="O19" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098/</t>
         </is>
       </c>
     </row>
@@ -2007,17 +2029,17 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/16/002 – TR13077</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
@@ -2030,7 +2052,7 @@
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
@@ -2040,17 +2062,17 @@
       </c>
       <c r="I20" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J20" s="14" t="n">
-        <v>46223</v>
+        <v>46225</v>
       </c>
       <c r="K20" s="14" t="n">
-        <v>46238</v>
+        <v>46229</v>
       </c>
       <c r="L20" s="15" t="n">
-        <v>100000</v>
+        <v>114600</v>
       </c>
       <c r="M20" s="9" t="inlineStr">
         <is>
@@ -2064,7 +2086,7 @@
       </c>
       <c r="O20" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
         </is>
       </c>
     </row>
@@ -2076,17 +2098,17 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13074</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/16/002 – TR13077</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E21" s="20" t="inlineStr">
@@ -2095,11 +2117,11 @@
         </is>
       </c>
       <c r="F21" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G21" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
@@ -2113,15 +2135,17 @@
         </is>
       </c>
       <c r="J21" s="22" t="n">
-        <v>46213</v>
+        <v>46223</v>
       </c>
       <c r="K21" s="22" t="n">
-        <v>46220</v>
-      </c>
-      <c r="L21" s="23" t="inlineStr"/>
+        <v>46238</v>
+      </c>
+      <c r="L21" s="23" t="n">
+        <v>100000</v>
+      </c>
       <c r="M21" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N21" s="20" t="inlineStr">
@@ -2131,7 +2155,7 @@
       </c>
       <c r="O21" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077/</t>
         </is>
       </c>
     </row>
@@ -2143,17 +2167,17 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13098</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E22" s="12" t="inlineStr">
@@ -2162,11 +2186,11 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
@@ -2176,19 +2200,21 @@
       </c>
       <c r="I22" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Brasília DF</t>
         </is>
       </c>
       <c r="J22" s="14" t="n">
-        <v>46221</v>
+        <v>46227</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46224</v>
-      </c>
-      <c r="L22" s="15" t="inlineStr"/>
+        <v>46231</v>
+      </c>
+      <c r="L22" s="15" t="n">
+        <v>150000</v>
+      </c>
       <c r="M22" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N22" s="12" t="inlineStr">
@@ -2198,7 +2224,7 @@
       </c>
       <c r="O22" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
         </is>
       </c>
     </row>
@@ -2210,12 +2236,12 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13015</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
@@ -2233,27 +2259,27 @@
       </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I23" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
         </is>
       </c>
       <c r="J23" s="22" t="n">
-        <v>46220</v>
+        <v>46224</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46225</v>
+        <v>46233</v>
       </c>
       <c r="L23" s="23" t="n">
-        <v>58800</v>
+        <v>288000</v>
       </c>
       <c r="M23" s="17" t="inlineStr">
         <is>
@@ -2267,7 +2293,7 @@
       </c>
       <c r="O23" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
         </is>
       </c>
     </row>
@@ -2279,17 +2305,17 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E24" s="12" t="inlineStr">
@@ -2298,35 +2324,35 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.4</v>
+        <v>0.343</v>
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I24" s="11" t="inlineStr">
         <is>
-          <t>Brasília DF</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J24" s="14" t="n">
-        <v>46227</v>
+        <v>46232</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46231</v>
+        <v>46238</v>
       </c>
       <c r="L24" s="15" t="n">
-        <v>150000</v>
+        <v>30000</v>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N24" s="12" t="inlineStr">
@@ -2336,7 +2362,7 @@
       </c>
       <c r="O24" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
         </is>
       </c>
     </row>
@@ -2348,12 +2374,12 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
@@ -2363,35 +2389,33 @@
       </c>
       <c r="E25" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F25" s="21" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F25" s="21" t="inlineStr"/>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I25" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J25" s="22" t="n">
-        <v>46225</v>
+        <v>46232</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46229</v>
+        <v>46238</v>
       </c>
       <c r="L25" s="23" t="n">
-        <v>114600</v>
+        <v>30000</v>
       </c>
       <c r="M25" s="17" t="inlineStr">
         <is>
@@ -2405,7 +2429,7 @@
       </c>
       <c r="O25" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
         </is>
       </c>
     </row>
@@ -2417,12 +2441,12 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -2445,19 +2469,19 @@
       </c>
       <c r="H26" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I26" s="11" t="inlineStr">
         <is>
-          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
+          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
         </is>
       </c>
       <c r="J26" s="14" t="n">
-        <v>46224</v>
+        <v>46232</v>
       </c>
       <c r="K26" s="14" t="n">
-        <v>46233</v>
+        <v>46237</v>
       </c>
       <c r="L26" s="15" t="n">
         <v>288000</v>
@@ -2474,7 +2498,7 @@
       </c>
       <c r="O26" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
         </is>
       </c>
     </row>
@@ -2486,12 +2510,12 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
@@ -2509,27 +2533,27 @@
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I27" s="19" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J27" s="22" t="n">
-        <v>46232</v>
+        <v>46240</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46237</v>
+        <v>46245</v>
       </c>
       <c r="L27" s="23" t="n">
-        <v>288000</v>
+        <v>204000</v>
       </c>
       <c r="M27" s="17" t="inlineStr">
         <is>
@@ -2543,7 +2567,7 @@
       </c>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
         </is>
       </c>
     </row>
@@ -2555,12 +2579,12 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
@@ -2570,13 +2594,15 @@
       </c>
       <c r="E28" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F28" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F28" s="13" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
@@ -2586,17 +2612,17 @@
       </c>
       <c r="I28" s="11" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J28" s="14" t="n">
-        <v>46232</v>
+        <v>46240</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46238</v>
+        <v>46245</v>
       </c>
       <c r="L28" s="15" t="n">
-        <v>30000</v>
+        <v>204000</v>
       </c>
       <c r="M28" s="9" t="inlineStr">
         <is>
@@ -2610,7 +2636,7 @@
       </c>
       <c r="O28" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
         </is>
       </c>
     </row>
@@ -2622,17 +2648,17 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E29" s="20" t="inlineStr">
@@ -2641,11 +2667,11 @@
         </is>
       </c>
       <c r="F29" s="21" t="n">
-        <v>0.343</v>
+        <v>0.4</v>
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
@@ -2655,17 +2681,17 @@
       </c>
       <c r="I29" s="19" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J29" s="22" t="n">
-        <v>46232</v>
+        <v>46240</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46238</v>
+        <v>46245</v>
       </c>
       <c r="L29" s="23" t="n">
-        <v>30000</v>
+        <v>80000</v>
       </c>
       <c r="M29" s="17" t="inlineStr">
         <is>
@@ -2679,7 +2705,7 @@
       </c>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
         </is>
       </c>
     </row>
@@ -2691,12 +2717,12 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
@@ -2724,7 +2750,7 @@
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Brasília - Df</t>
         </is>
       </c>
       <c r="J30" s="14" t="n">
@@ -2734,7 +2760,7 @@
         <v>46245</v>
       </c>
       <c r="L30" s="15" t="n">
-        <v>204000</v>
+        <v>80000</v>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
@@ -2748,7 +2774,7 @@
       </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
         </is>
       </c>
     </row>
@@ -2760,12 +2786,12 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
@@ -2775,35 +2801,33 @@
       </c>
       <c r="E31" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F31" s="21" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F31" s="21" t="inlineStr"/>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I31" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
         </is>
       </c>
       <c r="J31" s="22" t="n">
-        <v>46240</v>
+        <v>46227</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46245</v>
+        <v>46252</v>
       </c>
       <c r="L31" s="23" t="n">
-        <v>204000</v>
+        <v>286000</v>
       </c>
       <c r="M31" s="17" t="inlineStr">
         <is>
@@ -2817,7 +2841,7 @@
       </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
@@ -2829,12 +2853,12 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
@@ -2872,7 +2896,7 @@
         <v>46245</v>
       </c>
       <c r="L32" s="15" t="n">
-        <v>80000</v>
+        <v>100000</v>
       </c>
       <c r="M32" s="9" t="inlineStr">
         <is>
@@ -2886,7 +2910,7 @@
       </c>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
         </is>
       </c>
     </row>
@@ -2898,12 +2922,12 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
@@ -2917,11 +2941,11 @@
         </is>
       </c>
       <c r="F33" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
@@ -2931,21 +2955,19 @@
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>Brasília - Df</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J33" s="22" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46245</v>
-      </c>
-      <c r="L33" s="23" t="n">
-        <v>80000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L33" s="23" t="inlineStr"/>
       <c r="M33" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N33" s="20" t="inlineStr">
@@ -2955,7 +2977,7 @@
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -2967,12 +2989,12 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -2990,27 +3012,27 @@
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J34" s="14" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46245</v>
+        <v>46257</v>
       </c>
       <c r="L34" s="15" t="n">
-        <v>100000</v>
+        <v>54000</v>
       </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
@@ -3024,7 +3046,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -3105,12 +3127,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -3120,13 +3142,15 @@
       </c>
       <c r="E36" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F36" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F36" s="13" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
@@ -3136,17 +3160,17 @@
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46227</v>
+        <v>46246</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46252</v>
+        <v>46257</v>
       </c>
       <c r="L36" s="15" t="n">
-        <v>286000</v>
+        <v>54000</v>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
@@ -3160,7 +3184,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -3172,17 +3196,17 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E37" s="20" t="inlineStr">
@@ -3191,33 +3215,35 @@
         </is>
       </c>
       <c r="F37" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46246</v>
+        <v>46251</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L37" s="23" t="inlineStr"/>
+        <v>46256</v>
+      </c>
+      <c r="L37" s="23" t="n">
+        <v>50000</v>
+      </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N37" s="20" t="inlineStr">
@@ -3227,7 +3253,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -3239,12 +3265,12 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
@@ -3262,7 +3288,7 @@
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
@@ -3272,17 +3298,17 @@
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46246</v>
+        <v>46252</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46257</v>
+        <v>46259</v>
       </c>
       <c r="L38" s="15" t="n">
-        <v>54000</v>
+        <v>60000</v>
       </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
@@ -3296,7 +3322,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -3308,17 +3334,17 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E39" s="20" t="inlineStr">
@@ -3331,41 +3357,41 @@
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46246</v>
+        <v>46208</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46257</v>
+        <v>46259</v>
       </c>
       <c r="L39" s="23" t="n">
-        <v>54000</v>
+        <v>500000</v>
       </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N39" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -3377,17 +3403,17 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E40" s="12" t="inlineStr">
@@ -3400,7 +3426,7 @@
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
@@ -3410,21 +3436,21 @@
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46251</v>
+        <v>46246</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46256</v>
+        <v>46272</v>
       </c>
       <c r="L40" s="15" t="n">
-        <v>50000</v>
+        <v>54000</v>
       </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N40" s="12" t="inlineStr">
@@ -3434,7 +3460,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -3446,22 +3472,22 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E41" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F41" s="21" t="n">
@@ -3469,27 +3495,27 @@
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46252</v>
+        <v>46265</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46259</v>
+        <v>46270</v>
       </c>
       <c r="L41" s="23" t="n">
-        <v>60000</v>
+        <v>30000</v>
       </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
@@ -3503,7 +3529,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -3515,12 +3541,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3538,31 +3564,31 @@
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46246</v>
+        <v>46275</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46272</v>
+        <v>46280</v>
       </c>
       <c r="L42" s="15" t="n">
-        <v>54000</v>
+        <v>50000</v>
       </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N42" s="12" t="inlineStr">
@@ -3572,7 +3598,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
@@ -3584,17 +3610,17 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E43" s="20" t="inlineStr">
@@ -3607,41 +3633,41 @@
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46208</v>
+        <v>46266</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46259</v>
+        <v>46283</v>
       </c>
       <c r="L43" s="23" t="n">
-        <v>500000</v>
+        <v>70000</v>
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N43" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
@@ -3653,22 +3679,22 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E44" s="12" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F44" s="13" t="n">
@@ -3676,41 +3702,41 @@
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46265</v>
+        <v>46244</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46270</v>
+        <v>46300</v>
       </c>
       <c r="L44" s="15" t="n">
-        <v>30000</v>
+        <v>350000</v>
       </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N44" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -3722,17 +3748,17 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E45" s="20" t="inlineStr">
@@ -3741,45 +3767,45 @@
         </is>
       </c>
       <c r="F45" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46244</v>
+        <v>46278</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46300</v>
+        <v>46283</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>350000</v>
+        <v>17000000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N45" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>ugp@educacao.sp.gov.br</t>
         </is>
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
         </is>
       </c>
     </row>
@@ -3791,12 +3817,12 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -3810,11 +3836,11 @@
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
@@ -3824,18 +3850,16 @@
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J46" s="14" t="n">
         <v>46275</v>
       </c>
       <c r="K46" s="14" t="n">
-        <v>46280</v>
-      </c>
-      <c r="L46" s="15" t="n">
-        <v>50000</v>
-      </c>
+        <v>46281</v>
+      </c>
+      <c r="L46" s="15" t="inlineStr"/>
       <c r="M46" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3848,148 +3872,12 @@
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="17" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B47" s="18" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
-        </is>
-      </c>
-      <c r="C47" s="19" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
-        </is>
-      </c>
-      <c r="D47" s="19" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E47" s="20" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F47" s="21" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G47" s="19" t="inlineStr">
-        <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
-        </is>
-      </c>
-      <c r="H47" s="19" t="inlineStr">
-        <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I47" s="19" t="inlineStr">
-        <is>
-          <t>São Paulo - SP</t>
-        </is>
-      </c>
-      <c r="J47" s="22" t="n">
-        <v>46266</v>
-      </c>
-      <c r="K47" s="22" t="n">
-        <v>46283</v>
-      </c>
-      <c r="L47" s="23" t="n">
-        <v>70000</v>
-      </c>
-      <c r="M47" s="17" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N47" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O47" s="24" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="9" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B48" s="10" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
-        </is>
-      </c>
-      <c r="C48" s="11" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13238</t>
-        </is>
-      </c>
-      <c r="D48" s="11" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E48" s="12" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F48" s="13" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="G48" s="11" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
-        </is>
-      </c>
-      <c r="H48" s="11" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I48" s="11" t="inlineStr">
-        <is>
-          <t>Porto Alegre - RS</t>
-        </is>
-      </c>
-      <c r="J48" s="14" t="n">
-        <v>46275</v>
-      </c>
-      <c r="K48" s="14" t="n">
-        <v>46281</v>
-      </c>
-      <c r="L48" s="15" t="inlineStr"/>
-      <c r="M48" s="9" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N48" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O48" s="16" t="inlineStr">
-        <is>
           <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O48"/>
+  <autoFilter ref="A1:O46"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -4036,8 +3924,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId47"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -4076,7 +3962,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3">
@@ -4086,7 +3972,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4">
@@ -4096,7 +3982,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -4138,7 +4024,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3">
@@ -4148,7 +4034,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -4200,7 +4086,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3">
@@ -4210,27 +4096,27 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -4282,7 +4168,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4">
@@ -4292,7 +4178,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5">
@@ -4312,7 +4198,7 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -4348,7 +4234,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4384,7 +4270,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4">
@@ -4394,7 +4280,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5">
@@ -4404,13 +4290,13 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>MTE</t>
         </is>
       </c>
       <c r="B6" s="10" t="n">
@@ -4420,15 +4306,25 @@
     <row r="7">
       <c r="A7" s="19" t="inlineStr">
         <is>
+          <t>OEI/MDHC</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
           <t>MGI</t>
         </is>
       </c>
-      <c r="B7" s="18" t="n">
+      <c r="B8" s="10" t="n">
         <v>2</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B7"/>
+  <autoFilter ref="A1:B8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -4472,7 +4368,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -4487,7 +4383,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -4502,7 +4398,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
@@ -4517,7 +4413,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-09-15 16:27
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$49</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 14/09/2026 às 17:46</t>
+          <t>Gerado em 15/09/2026 às 16:20</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="24">
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O46"/>
+  <dimension ref="A1:O49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1396,11 +1396,11 @@
         </is>
       </c>
       <c r="B10" s="10" t="n">
-        <v>146360</v>
+        <v>146373</v>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>PNUD BRA/25/024 - Edital nº 04/2026 – Contrat. de consult. - Engenharia de Dados</t>
+          <t xml:space="preserve">Edital nº 26/2026 – Contratação de Consultoria Individual para aprimoramento de soluções analíticas e computacionais aplicadas ao Modelo de Mensuração de Custos da Digitalização de Serviços Públicos </t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
@@ -1418,27 +1418,27 @@
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
         <is>
-          <t>MTE</t>
+          <t>MGI</t>
         </is>
       </c>
       <c r="I10" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J10" s="14" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="K10" s="14" t="n">
-        <v>46287</v>
+        <v>46295</v>
       </c>
       <c r="L10" s="15" t="n">
-        <v>130000</v>
+        <v>108000</v>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
@@ -1447,7 +1447,7 @@
       </c>
       <c r="N10" s="12" t="inlineStr">
         <is>
-          <t>estatisticastrabalho@trabalho.gov.br</t>
+          <t>prodoc.mgi@gestao.gov.br</t>
         </is>
       </c>
       <c r="O10" s="16" t="inlineStr">
@@ -1463,11 +1463,11 @@
         </is>
       </c>
       <c r="B11" s="18" t="n">
-        <v>146361</v>
+        <v>146360</v>
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>PNUD BRA/25/024 - Consultoria Especializada - Qualidade de Dados I</t>
+          <t>PNUD BRA/25/024 - Edital nº 04/2026 – Contrat. de consult. - Engenharia de Dados</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
@@ -1530,11 +1530,11 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>146362</v>
+        <v>146361</v>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>PNUD BRA/25/024 - Edital nº 06/2026 - Consultoria Especializada - Qualidade de Dados II</t>
+          <t>PNUD BRA/25/024 - Consultoria Especializada - Qualidade de Dados I</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
@@ -1593,17 +1593,15 @@
     <row r="13">
       <c r="A13" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B13" s="18" t="inlineStr">
-        <is>
-          <t>unesco:8c824e7b-7b9a-4a59-7ffc-08df082d82f3</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B13" s="18" t="n">
+        <v>146362</v>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1163 - Publicação -  Edital 68/2026 - 01 Vaga consultor Individual</t>
+          <t>PNUD BRA/25/024 - Edital nº 06/2026 - Consultoria Especializada - Qualidade de Dados II</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
@@ -1621,48 +1619,56 @@
       </c>
       <c r="G13" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H13" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I13" s="19" t="inlineStr"/>
+          <t>MTE</t>
+        </is>
+      </c>
+      <c r="I13" s="19" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J13" s="22" t="n">
-        <v>46276</v>
+        <v>46279</v>
       </c>
       <c r="K13" s="22" t="n">
-        <v>46281</v>
-      </c>
-      <c r="L13" s="23" t="inlineStr"/>
+        <v>46287</v>
+      </c>
+      <c r="L13" s="23" t="n">
+        <v>130000</v>
+      </c>
       <c r="M13" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N13" s="20" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N13" s="20" t="inlineStr">
+        <is>
+          <t>estatisticastrabalho@trabalho.gov.br</t>
+        </is>
+      </c>
       <c r="O13" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>unesco:5907e744-d46d-4c01-2eaf-08df08e94b75</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="n">
+        <v>146374</v>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 37/2026 - 2 vagas - Consultor Individual</t>
+          <t>Edital nº 27/2026 – Contratação de Consultoria Individual II - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Servidões de Passagem para Orlas e Praias</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -1680,48 +1686,56 @@
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I14" s="11" t="inlineStr"/>
+          <t>MGI</t>
+        </is>
+      </c>
+      <c r="I14" s="11" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
       <c r="J14" s="14" t="n">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="K14" s="14" t="n">
-        <v>46283</v>
-      </c>
-      <c r="L14" s="15" t="inlineStr"/>
+        <v>46295</v>
+      </c>
+      <c r="L14" s="15" t="n">
+        <v>120000</v>
+      </c>
       <c r="M14" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N14" s="12" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N14" s="12" t="inlineStr">
+        <is>
+          <t>prodoc.mgi@gestao.gov.br</t>
+        </is>
+      </c>
       <c r="O14" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B15" s="18" t="inlineStr">
-        <is>
-          <t>unesco:1011b77e-9c7a-4ea9-2632-08df0e687345</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="n">
+        <v>146375</v>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 39/2026 - 1 vaga - Consultor Individual</t>
+          <t>Edital nº 28/2026 - Contratação de Consultoria Individual I - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Acessibilidade em Orlas e Praias</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
@@ -1739,31 +1753,41 @@
       </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H15" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I15" s="19" t="inlineStr"/>
+          <t>MGI</t>
+        </is>
+      </c>
+      <c r="I15" s="19" t="inlineStr">
+        <is>
+          <t>REMOTO</t>
+        </is>
+      </c>
       <c r="J15" s="22" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="K15" s="22" t="n">
-        <v>46283</v>
-      </c>
-      <c r="L15" s="23" t="inlineStr"/>
+        <v>46295</v>
+      </c>
+      <c r="L15" s="23" t="n">
+        <v>120000</v>
+      </c>
       <c r="M15" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N15" s="20" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N15" s="20" t="inlineStr">
+        <is>
+          <t>prodoc.mgi@gestao.gov.br</t>
+        </is>
+      </c>
       <c r="O15" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
@@ -1775,12 +1799,12 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>unesco:030ad7b8-d33f-491a-31d9-08defb16c1ac</t>
+          <t>unesco:8c824e7b-7b9a-4a59-7ffc-08df082d82f3</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ5067 - Edital Nº 08/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1163 - Publicação -  Edital 68/2026 - 04 Vagas consultor Individual</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -1798,7 +1822,7 @@
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
@@ -1808,10 +1832,10 @@
       </c>
       <c r="I16" s="11" t="inlineStr"/>
       <c r="J16" s="14" t="n">
-        <v>46253</v>
+        <v>46276</v>
       </c>
       <c r="K16" s="14" t="n">
-        <v>46283</v>
+        <v>46281</v>
       </c>
       <c r="L16" s="15" t="inlineStr"/>
       <c r="M16" s="9" t="inlineStr">
@@ -1834,12 +1858,12 @@
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>unesco:a42aa3e1-2e33-46e6-2633-08df0e687345</t>
+          <t>unesco:5907e744-d46d-4c01-2eaf-08df08e94b75</t>
         </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 38/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1159 - Publicação Edital 37/2026 - 2 vagas - Consultor Individual</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1867,7 +1891,7 @@
       </c>
       <c r="I17" s="19" t="inlineStr"/>
       <c r="J17" s="22" t="n">
-        <v>46279</v>
+        <v>46277</v>
       </c>
       <c r="K17" s="22" t="n">
         <v>46283</v>
@@ -1888,22 +1912,22 @@
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015</t>
+          <t>unesco:1011b77e-9c7a-4ea9-2632-08df0e687345</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13015</t>
+          <t>914BRZ1159 - Publicação Edital 39/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
@@ -1912,67 +1936,57 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I18" s="11" t="inlineStr">
-        <is>
-          <t>Brasília - DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I18" s="11" t="inlineStr"/>
       <c r="J18" s="14" t="n">
-        <v>46220</v>
+        <v>46279</v>
       </c>
       <c r="K18" s="14" t="n">
-        <v>46225</v>
-      </c>
-      <c r="L18" s="15" t="n">
-        <v>58800</v>
-      </c>
+        <v>46283</v>
+      </c>
+      <c r="L18" s="15" t="inlineStr"/>
       <c r="M18" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N18" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N18" s="12" t="inlineStr"/>
       <c r="O18" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="17" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098</t>
+          <t>unesco:030ad7b8-d33f-491a-31d9-08defb16c1ac</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13098</t>
+          <t>Projeto 914BRZ5067 - Edital Nº 08/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E19" s="20" t="inlineStr">
@@ -1985,61 +1999,53 @@
       </c>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I19" s="19" t="inlineStr">
-        <is>
-          <t>Brasília - DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I19" s="19" t="inlineStr"/>
       <c r="J19" s="22" t="n">
-        <v>46221</v>
+        <v>46253</v>
       </c>
       <c r="K19" s="22" t="n">
-        <v>46224</v>
+        <v>46283</v>
       </c>
       <c r="L19" s="23" t="inlineStr"/>
       <c r="M19" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
-        </is>
-      </c>
-      <c r="N19" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N19" s="20" t="inlineStr"/>
       <c r="O19" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
+          <t>unesco:a42aa3e1-2e33-46e6-2633-08df0e687345</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
+          <t>914BRZ1159 - Publicação Edital 38/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
@@ -2048,45 +2054,35 @@
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I20" s="11" t="inlineStr">
-        <is>
-          <t>Recife - PE</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="inlineStr"/>
       <c r="J20" s="14" t="n">
-        <v>46225</v>
+        <v>46279</v>
       </c>
       <c r="K20" s="14" t="n">
-        <v>46229</v>
-      </c>
-      <c r="L20" s="15" t="n">
-        <v>114600</v>
-      </c>
+        <v>46283</v>
+      </c>
+      <c r="L20" s="15" t="inlineStr"/>
       <c r="M20" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N20" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N20" s="12" t="inlineStr"/>
       <c r="O20" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
@@ -2098,17 +2094,17 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/16/002 – TR13077</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13098</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E21" s="20" t="inlineStr">
@@ -2117,11 +2113,11 @@
         </is>
       </c>
       <c r="F21" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G21" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
@@ -2135,17 +2131,15 @@
         </is>
       </c>
       <c r="J21" s="22" t="n">
-        <v>46223</v>
+        <v>46221</v>
       </c>
       <c r="K21" s="22" t="n">
-        <v>46238</v>
-      </c>
-      <c r="L21" s="23" t="n">
-        <v>100000</v>
-      </c>
+        <v>46224</v>
+      </c>
+      <c r="L21" s="23" t="inlineStr"/>
       <c r="M21" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N21" s="20" t="inlineStr">
@@ -2155,7 +2149,7 @@
       </c>
       <c r="O21" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098/</t>
         </is>
       </c>
     </row>
@@ -2167,12 +2161,12 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13015</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -2190,7 +2184,7 @@
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
@@ -2200,21 +2194,21 @@
       </c>
       <c r="I22" s="11" t="inlineStr">
         <is>
-          <t>Brasília DF</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J22" s="14" t="n">
-        <v>46227</v>
+        <v>46220</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46231</v>
+        <v>46225</v>
       </c>
       <c r="L22" s="15" t="n">
-        <v>150000</v>
+        <v>58800</v>
       </c>
       <c r="M22" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N22" s="12" t="inlineStr">
@@ -2224,7 +2218,7 @@
       </c>
       <c r="O22" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015/</t>
         </is>
       </c>
     </row>
@@ -2236,12 +2230,12 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
@@ -2259,27 +2253,27 @@
       </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I23" s="19" t="inlineStr">
         <is>
-          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J23" s="22" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46233</v>
+        <v>46229</v>
       </c>
       <c r="L23" s="23" t="n">
-        <v>288000</v>
+        <v>114600</v>
       </c>
       <c r="M23" s="17" t="inlineStr">
         <is>
@@ -2293,7 +2287,7 @@
       </c>
       <c r="O23" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
         </is>
       </c>
     </row>
@@ -2305,12 +2299,12 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/16/002 – TR13077</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -2324,31 +2318,31 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.343</v>
+        <v>0.4</v>
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I24" s="11" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J24" s="14" t="n">
-        <v>46232</v>
+        <v>46223</v>
       </c>
       <c r="K24" s="14" t="n">
         <v>46238</v>
       </c>
       <c r="L24" s="15" t="n">
-        <v>30000</v>
+        <v>100000</v>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
@@ -2362,7 +2356,7 @@
       </c>
       <c r="O24" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077/</t>
         </is>
       </c>
     </row>
@@ -2374,12 +2368,12 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
@@ -2389,37 +2383,39 @@
       </c>
       <c r="E25" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F25" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F25" s="21" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I25" s="19" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Brasília DF</t>
         </is>
       </c>
       <c r="J25" s="22" t="n">
-        <v>46232</v>
+        <v>46227</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46238</v>
+        <v>46231</v>
       </c>
       <c r="L25" s="23" t="n">
-        <v>30000</v>
+        <v>150000</v>
       </c>
       <c r="M25" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N25" s="20" t="inlineStr">
@@ -2429,7 +2425,7 @@
       </c>
       <c r="O25" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
         </is>
       </c>
     </row>
@@ -2441,12 +2437,12 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -2469,19 +2465,19 @@
       </c>
       <c r="H26" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I26" s="11" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
+          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
         </is>
       </c>
       <c r="J26" s="14" t="n">
-        <v>46232</v>
+        <v>46224</v>
       </c>
       <c r="K26" s="14" t="n">
-        <v>46237</v>
+        <v>46233</v>
       </c>
       <c r="L26" s="15" t="n">
         <v>288000</v>
@@ -2498,7 +2494,7 @@
       </c>
       <c r="O26" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
         </is>
       </c>
     </row>
@@ -2510,17 +2506,17 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E27" s="20" t="inlineStr">
@@ -2529,11 +2525,11 @@
         </is>
       </c>
       <c r="F27" s="21" t="n">
-        <v>0.4</v>
+        <v>0.343</v>
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
@@ -2543,17 +2539,17 @@
       </c>
       <c r="I27" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J27" s="22" t="n">
-        <v>46240</v>
+        <v>46232</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46245</v>
+        <v>46238</v>
       </c>
       <c r="L27" s="23" t="n">
-        <v>204000</v>
+        <v>30000</v>
       </c>
       <c r="M27" s="17" t="inlineStr">
         <is>
@@ -2567,7 +2563,7 @@
       </c>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
         </is>
       </c>
     </row>
@@ -2579,12 +2575,12 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
@@ -2594,15 +2590,13 @@
       </c>
       <c r="E28" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F28" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F28" s="13" t="inlineStr"/>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
@@ -2612,17 +2606,17 @@
       </c>
       <c r="I28" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J28" s="14" t="n">
-        <v>46240</v>
+        <v>46232</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46245</v>
+        <v>46238</v>
       </c>
       <c r="L28" s="15" t="n">
-        <v>204000</v>
+        <v>30000</v>
       </c>
       <c r="M28" s="9" t="inlineStr">
         <is>
@@ -2636,7 +2630,7 @@
       </c>
       <c r="O28" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
         </is>
       </c>
     </row>
@@ -2648,12 +2642,12 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
@@ -2671,27 +2665,27 @@
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I29" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
         </is>
       </c>
       <c r="J29" s="22" t="n">
-        <v>46240</v>
+        <v>46232</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46245</v>
+        <v>46237</v>
       </c>
       <c r="L29" s="23" t="n">
-        <v>80000</v>
+        <v>288000</v>
       </c>
       <c r="M29" s="17" t="inlineStr">
         <is>
@@ -2705,7 +2699,7 @@
       </c>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
         </is>
       </c>
     </row>
@@ -2717,12 +2711,12 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
@@ -2740,7 +2734,7 @@
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
@@ -2750,7 +2744,7 @@
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>Brasília - Df</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J30" s="14" t="n">
@@ -2760,7 +2754,7 @@
         <v>46245</v>
       </c>
       <c r="L30" s="15" t="n">
-        <v>80000</v>
+        <v>204000</v>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
@@ -2774,7 +2768,7 @@
       </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
         </is>
       </c>
     </row>
@@ -2786,12 +2780,12 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
@@ -2801,33 +2795,35 @@
       </c>
       <c r="E31" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F31" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F31" s="21" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I31" s="19" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J31" s="22" t="n">
-        <v>46227</v>
+        <v>46240</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46252</v>
+        <v>46245</v>
       </c>
       <c r="L31" s="23" t="n">
-        <v>286000</v>
+        <v>204000</v>
       </c>
       <c r="M31" s="17" t="inlineStr">
         <is>
@@ -2841,7 +2837,7 @@
       </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
         </is>
       </c>
     </row>
@@ -2853,12 +2849,12 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
@@ -2896,7 +2892,7 @@
         <v>46245</v>
       </c>
       <c r="L32" s="15" t="n">
-        <v>100000</v>
+        <v>80000</v>
       </c>
       <c r="M32" s="9" t="inlineStr">
         <is>
@@ -2910,7 +2906,7 @@
       </c>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
         </is>
       </c>
     </row>
@@ -2922,12 +2918,12 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
@@ -2941,11 +2937,11 @@
         </is>
       </c>
       <c r="F33" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
@@ -2955,19 +2951,21 @@
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>Brasília - Df</t>
         </is>
       </c>
       <c r="J33" s="22" t="n">
-        <v>46246</v>
+        <v>46240</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L33" s="23" t="inlineStr"/>
+        <v>46245</v>
+      </c>
+      <c r="L33" s="23" t="n">
+        <v>80000</v>
+      </c>
       <c r="M33" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N33" s="20" t="inlineStr">
@@ -2977,7 +2975,7 @@
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
         </is>
       </c>
     </row>
@@ -2989,12 +2987,12 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -3012,27 +3010,27 @@
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J34" s="14" t="n">
-        <v>46246</v>
+        <v>46240</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46257</v>
+        <v>46245</v>
       </c>
       <c r="L34" s="15" t="n">
-        <v>54000</v>
+        <v>100000</v>
       </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
@@ -3046,7 +3044,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
         </is>
       </c>
     </row>
@@ -3058,64 +3056,62 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E35" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F35" s="21" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F35" s="21" t="inlineStr"/>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46244</v>
+        <v>46227</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46296</v>
+        <v>46252</v>
       </c>
       <c r="L35" s="23" t="n">
-        <v>935000</v>
+        <v>286000</v>
       </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N35" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
@@ -3127,12 +3123,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -3146,35 +3142,33 @@
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
         <v>46246</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46257</v>
-      </c>
-      <c r="L36" s="15" t="n">
-        <v>54000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L36" s="15" t="inlineStr"/>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N36" s="12" t="inlineStr">
@@ -3184,7 +3178,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -3196,17 +3190,17 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E37" s="20" t="inlineStr">
@@ -3219,7 +3213,7 @@
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
@@ -3229,17 +3223,17 @@
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46251</v>
+        <v>46246</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="L37" s="23" t="n">
-        <v>50000</v>
+        <v>54000</v>
       </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
@@ -3253,7 +3247,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -3265,17 +3259,17 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E38" s="12" t="inlineStr">
@@ -3288,7 +3282,7 @@
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
@@ -3298,17 +3292,17 @@
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46252</v>
+        <v>46251</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46259</v>
+        <v>46256</v>
       </c>
       <c r="L38" s="15" t="n">
-        <v>60000</v>
+        <v>50000</v>
       </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
@@ -3322,7 +3316,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -3334,17 +3328,17 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E39" s="20" t="inlineStr">
@@ -3357,41 +3351,41 @@
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46208</v>
+        <v>46246</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46259</v>
+        <v>46257</v>
       </c>
       <c r="L39" s="23" t="n">
-        <v>500000</v>
+        <v>54000</v>
       </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N39" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -3403,12 +3397,12 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
@@ -3426,7 +3420,7 @@
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
@@ -3436,21 +3430,21 @@
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46246</v>
+        <v>46252</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46272</v>
+        <v>46259</v>
       </c>
       <c r="L40" s="15" t="n">
-        <v>54000</v>
+        <v>60000</v>
       </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N40" s="12" t="inlineStr">
@@ -3460,7 +3454,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -3472,22 +3466,22 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E41" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F41" s="21" t="n">
@@ -3495,41 +3489,41 @@
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46265</v>
+        <v>46208</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46270</v>
+        <v>46259</v>
       </c>
       <c r="L41" s="23" t="n">
-        <v>30000</v>
+        <v>500000</v>
       </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N41" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -3541,12 +3535,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3564,31 +3558,31 @@
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46275</v>
+        <v>46246</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46280</v>
+        <v>46272</v>
       </c>
       <c r="L42" s="15" t="n">
-        <v>50000</v>
+        <v>54000</v>
       </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N42" s="12" t="inlineStr">
@@ -3598,7 +3592,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -3610,22 +3604,22 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E43" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F43" s="21" t="n">
@@ -3633,27 +3627,27 @@
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46283</v>
+        <v>46270</v>
       </c>
       <c r="L43" s="23" t="n">
-        <v>70000</v>
+        <v>30000</v>
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
@@ -3667,7 +3661,7 @@
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -3679,17 +3673,17 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E44" s="12" t="inlineStr">
@@ -3702,41 +3696,41 @@
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46244</v>
+        <v>46275</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46300</v>
+        <v>46280</v>
       </c>
       <c r="L44" s="15" t="n">
-        <v>350000</v>
+        <v>50000</v>
       </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N44" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
@@ -3748,12 +3742,12 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
@@ -3767,7 +3761,7 @@
         </is>
       </c>
       <c r="F45" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
@@ -3785,27 +3779,27 @@
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46278</v>
+        <v>46266</v>
       </c>
       <c r="K45" s="22" t="n">
         <v>46283</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>17000000</v>
+        <v>70000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N45" s="20" t="inlineStr">
         <is>
-          <t>ugp@educacao.sp.gov.br</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
@@ -3817,67 +3811,272 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+        </is>
+      </c>
+      <c r="C46" s="11" t="inlineStr">
+        <is>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+        </is>
+      </c>
+      <c r="D46" s="11" t="inlineStr">
+        <is>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+        </is>
+      </c>
+      <c r="E46" s="12" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F46" s="13" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G46" s="11" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+        </is>
+      </c>
+      <c r="H46" s="11" t="inlineStr">
+        <is>
+          <t>OEI/MDHC</t>
+        </is>
+      </c>
+      <c r="I46" s="11" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="J46" s="14" t="n">
+        <v>46244</v>
+      </c>
+      <c r="K46" s="14" t="n">
+        <v>46300</v>
+      </c>
+      <c r="L46" s="15" t="n">
+        <v>350000</v>
+      </c>
+      <c r="M46" s="9" t="inlineStr">
+        <is>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N46" s="12" t="inlineStr">
+        <is>
+          <t>compras.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O46" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B47" s="18" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+        </is>
+      </c>
+      <c r="C47" s="19" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+        </is>
+      </c>
+      <c r="D47" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E47" s="20" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F47" s="21" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G47" s="19" t="inlineStr">
+        <is>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+        </is>
+      </c>
+      <c r="H47" s="19" t="inlineStr">
+        <is>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I47" s="19" t="inlineStr">
+        <is>
+          <t>São Paulo - SP</t>
+        </is>
+      </c>
+      <c r="J47" s="22" t="n">
+        <v>46278</v>
+      </c>
+      <c r="K47" s="22" t="n">
+        <v>46283</v>
+      </c>
+      <c r="L47" s="23" t="inlineStr"/>
+      <c r="M47" s="17" t="inlineStr">
+        <is>
+          <t>En presentación</t>
+        </is>
+      </c>
+      <c r="N47" s="20" t="inlineStr">
+        <is>
+          <t>ugp@educacao.sp.gov.br</t>
+        </is>
+      </c>
+      <c r="O47" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="9" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B48" s="10" t="inlineStr">
+        <is>
           <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
         </is>
       </c>
-      <c r="C46" s="11" t="inlineStr">
+      <c r="C48" s="11" t="inlineStr">
         <is>
           <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
         </is>
       </c>
-      <c r="D46" s="11" t="inlineStr">
+      <c r="D48" s="11" t="inlineStr">
         <is>
           <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
-      <c r="E46" s="12" t="inlineStr">
+      <c r="E48" s="12" t="inlineStr">
         <is>
           <t>Analista Powerbi</t>
         </is>
       </c>
-      <c r="F46" s="13" t="n">
+      <c r="F48" s="13" t="n">
         <v>0.3</v>
       </c>
-      <c r="G46" s="11" t="inlineStr">
+      <c r="G48" s="11" t="inlineStr">
         <is>
           <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
-      <c r="H46" s="11" t="inlineStr">
+      <c r="H48" s="11" t="inlineStr">
         <is>
           <t>OEI</t>
         </is>
       </c>
-      <c r="I46" s="11" t="inlineStr">
+      <c r="I48" s="11" t="inlineStr">
         <is>
           <t>Porto Alegre - RS</t>
         </is>
       </c>
-      <c r="J46" s="14" t="n">
+      <c r="J48" s="14" t="n">
         <v>46275</v>
       </c>
-      <c r="K46" s="14" t="n">
+      <c r="K48" s="14" t="n">
         <v>46281</v>
       </c>
-      <c r="L46" s="15" t="inlineStr"/>
-      <c r="M46" s="9" t="inlineStr">
+      <c r="L48" s="15" t="inlineStr"/>
+      <c r="M48" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
         </is>
       </c>
-      <c r="N46" s="12" t="inlineStr">
+      <c r="N48" s="12" t="inlineStr">
         <is>
           <t>selecao.bra@oei.int</t>
         </is>
       </c>
-      <c r="O46" s="16" t="inlineStr">
+      <c r="O48" s="16" t="inlineStr">
         <is>
           <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B49" s="18" t="inlineStr">
+        <is>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+        </is>
+      </c>
+      <c r="C49" s="19" t="inlineStr">
+        <is>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+        </is>
+      </c>
+      <c r="D49" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+        </is>
+      </c>
+      <c r="E49" s="20" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F49" s="21" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G49" s="19" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+        </is>
+      </c>
+      <c r="H49" s="19" t="inlineStr">
+        <is>
+          <t>OEI/MDHC</t>
+        </is>
+      </c>
+      <c r="I49" s="19" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="J49" s="22" t="n">
+        <v>46244</v>
+      </c>
+      <c r="K49" s="22" t="n">
+        <v>46296</v>
+      </c>
+      <c r="L49" s="23" t="n">
+        <v>935000</v>
+      </c>
+      <c r="M49" s="17" t="inlineStr">
+        <is>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N49" s="20" t="inlineStr">
+        <is>
+          <t>compras.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O49" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O46"/>
+  <autoFilter ref="A1:O49"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -3924,6 +4123,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId48"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -3972,7 +4174,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4">
@@ -4024,7 +4226,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3">
@@ -4096,7 +4298,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
@@ -4158,7 +4360,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3">
@@ -4286,7 +4488,7 @@
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>MGI</t>
         </is>
       </c>
       <c r="B5" s="18" t="n">
@@ -4296,17 +4498,17 @@
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>MTE</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>MTE</t>
         </is>
       </c>
       <c r="B7" s="18" t="n">
@@ -4316,11 +4518,11 @@
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -4368,7 +4570,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -4383,7 +4585,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -4413,7 +4615,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-09-16 16:18
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$45</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 15/09/2026 às 16:20</t>
+          <t>Gerado em 16/09/2026 às 16:12</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>48</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>168816</v>
+        <v>170864</v>
       </c>
     </row>
     <row r="20">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>80000</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>43</v>
+        <v>39</v>
       </c>
     </row>
     <row r="24">
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O49"/>
+  <dimension ref="A1:O45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -941,11 +941,11 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>146368</v>
+        <v>146369</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
-          <t>Edital 6/2026- UGP-PNUD/SENAD</t>
+          <t>Edital nº 29/2026 – Contratação de Consultoria Individual para o desenho institucional da Secretaria de Serviços Compartilhados (SSC/MGI)</t>
         </is>
       </c>
       <c r="D3" s="19" t="inlineStr">
@@ -955,34 +955,34 @@
       </c>
       <c r="E3" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F3" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F3" s="21" t="inlineStr"/>
       <c r="G3" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H3" s="19" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>MGI</t>
         </is>
       </c>
       <c r="I3" s="19" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J3" s="22" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="K3" s="22" t="n">
-        <v>46280</v>
-      </c>
-      <c r="L3" s="23" t="inlineStr"/>
+        <v>46290</v>
+      </c>
+      <c r="L3" s="23" t="n">
+        <v>120000</v>
+      </c>
       <c r="M3" s="17" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -990,7 +990,7 @@
       </c>
       <c r="N3" s="20" t="inlineStr">
         <is>
-          <t>cgep@mj.gov.br</t>
+          <t>prodoc.mgi@gestao.gov.br</t>
         </is>
       </c>
       <c r="O3" s="24" t="inlineStr">
@@ -1006,11 +1006,11 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>146367</v>
+        <v>146370</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>EDITAL Nº 5/2026 - UGP-PNUD/SENAD</t>
+          <t xml:space="preserve">Edital nº 25/2026 – Contratação de Consultoria Individual para avaliar os efeitos de intervenções comportamentais (políticas fiscais e de arquitetura de escolha) em mercado experimental para promover escolhas alimentares mais saudáveis. </t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
@@ -1020,34 +1020,34 @@
       </c>
       <c r="E4" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F4" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F4" s="13" t="inlineStr"/>
       <c r="G4" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H4" s="11" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>MGI</t>
         </is>
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>Brasília/DF</t>
+          <t>REMOTO</t>
         </is>
       </c>
       <c r="J4" s="14" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="K4" s="14" t="n">
-        <v>46280</v>
-      </c>
-      <c r="L4" s="15" t="inlineStr"/>
+        <v>46290</v>
+      </c>
+      <c r="L4" s="15" t="n">
+        <v>126000</v>
+      </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1055,7 +1055,7 @@
       </c>
       <c r="N4" s="12" t="inlineStr">
         <is>
-          <t>cgep@mj.gov.br</t>
+          <t>prodoc.mgi@gestao.gov.br</t>
         </is>
       </c>
       <c r="O4" s="16" t="inlineStr">
@@ -1071,11 +1071,11 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>146365</v>
+        <v>146373</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t>EDITAL Nº 4/2026 - UGP-PNUD/SENAD</t>
+          <t xml:space="preserve">Edital nº 26/2026 – Contratação de Consultoria Individual para aprimoramento de soluções analíticas e computacionais aplicadas ao Modelo de Mensuração de Custos da Digitalização de Serviços Públicos </t>
         </is>
       </c>
       <c r="D5" s="19" t="inlineStr">
@@ -1093,26 +1093,28 @@
       </c>
       <c r="G5" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H5" s="19" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>MGI</t>
         </is>
       </c>
       <c r="I5" s="19" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J5" s="22" t="n">
-        <v>46275</v>
+        <v>46280</v>
       </c>
       <c r="K5" s="22" t="n">
-        <v>46280</v>
-      </c>
-      <c r="L5" s="23" t="inlineStr"/>
+        <v>46295</v>
+      </c>
+      <c r="L5" s="23" t="n">
+        <v>108000</v>
+      </c>
       <c r="M5" s="17" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1120,7 +1122,7 @@
       </c>
       <c r="N5" s="20" t="inlineStr">
         <is>
-          <t>dpagi@mj.gov.br</t>
+          <t>prodoc.mgi@gestao.gov.br</t>
         </is>
       </c>
       <c r="O5" s="24" t="inlineStr">
@@ -1136,11 +1138,11 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>146364</v>
+        <v>146360</v>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>EDITAL Nº 3/2026 - UGP-PNUD/SENAD</t>
+          <t>PNUD BRA/25/024 - Edital nº 04/2026 – Contrat. de consult. - Engenharia de Dados</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
@@ -1163,21 +1165,23 @@
       </c>
       <c r="H6" s="11" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>MTE</t>
         </is>
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J6" s="14" t="n">
-        <v>46275</v>
+        <v>46279</v>
       </c>
       <c r="K6" s="14" t="n">
-        <v>46280</v>
-      </c>
-      <c r="L6" s="15" t="inlineStr"/>
+        <v>46287</v>
+      </c>
+      <c r="L6" s="15" t="n">
+        <v>130000</v>
+      </c>
       <c r="M6" s="9" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1185,7 +1189,7 @@
       </c>
       <c r="N6" s="12" t="inlineStr">
         <is>
-          <t>dpagi@mj.gov.br</t>
+          <t>estatisticastrabalho@trabalho.gov.br</t>
         </is>
       </c>
       <c r="O6" s="16" t="inlineStr">
@@ -1201,11 +1205,11 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>146363</v>
+        <v>146361</v>
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t>EDITAL Nº 2/2026 - UGP-PNUD/SENAD</t>
+          <t>PNUD BRA/25/024 - Consultoria Especializada - Qualidade de Dados I</t>
         </is>
       </c>
       <c r="D7" s="19" t="inlineStr">
@@ -1223,26 +1227,28 @@
       </c>
       <c r="G7" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H7" s="19" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>MTE</t>
         </is>
       </c>
       <c r="I7" s="19" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J7" s="22" t="n">
-        <v>46275</v>
+        <v>46279</v>
       </c>
       <c r="K7" s="22" t="n">
-        <v>46280</v>
-      </c>
-      <c r="L7" s="23" t="inlineStr"/>
+        <v>46287</v>
+      </c>
+      <c r="L7" s="23" t="n">
+        <v>130000</v>
+      </c>
       <c r="M7" s="17" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1250,7 +1256,7 @@
       </c>
       <c r="N7" s="20" t="inlineStr">
         <is>
-          <t>senad@mj.gov.br</t>
+          <t>estatisticastrabalho@trabalho.gov.br</t>
         </is>
       </c>
       <c r="O7" s="24" t="inlineStr">
@@ -1266,11 +1272,11 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>146369</v>
+        <v>146362</v>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>Edital nº 29/2026 – Contratação de Consultoria Individual para o desenho institucional da Secretaria de Serviços Compartilhados (SSC/MGI)</t>
+          <t>PNUD BRA/25/024 - Edital nº 06/2026 - Consultoria Especializada - Qualidade de Dados II</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
@@ -1280,33 +1286,35 @@
       </c>
       <c r="E8" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F8" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F8" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H8" s="11" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>MTE</t>
         </is>
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J8" s="14" t="n">
-        <v>46276</v>
+        <v>46279</v>
       </c>
       <c r="K8" s="14" t="n">
-        <v>46290</v>
+        <v>46287</v>
       </c>
       <c r="L8" s="15" t="n">
-        <v>120000</v>
+        <v>130000</v>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
@@ -1315,7 +1323,7 @@
       </c>
       <c r="N8" s="12" t="inlineStr">
         <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
+          <t>estatisticastrabalho@trabalho.gov.br</t>
         </is>
       </c>
       <c r="O8" s="16" t="inlineStr">
@@ -1331,11 +1339,11 @@
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>146370</v>
+        <v>146374</v>
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edital nº 25/2026 – Contratação de Consultoria Individual para avaliar os efeitos de intervenções comportamentais (políticas fiscais e de arquitetura de escolha) em mercado experimental para promover escolhas alimentares mais saudáveis. </t>
+          <t>Edital nº 27/2026 – Contratação de Consultoria Individual II - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Servidões de Passagem para Orlas e Praias</t>
         </is>
       </c>
       <c r="D9" s="19" t="inlineStr">
@@ -1345,13 +1353,15 @@
       </c>
       <c r="E9" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F9" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F9" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G9" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H9" s="19" t="inlineStr">
@@ -1361,17 +1371,17 @@
       </c>
       <c r="I9" s="19" t="inlineStr">
         <is>
-          <t>REMOTO</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J9" s="22" t="n">
-        <v>46276</v>
+        <v>46280</v>
       </c>
       <c r="K9" s="22" t="n">
-        <v>46290</v>
+        <v>46295</v>
       </c>
       <c r="L9" s="23" t="n">
-        <v>126000</v>
+        <v>120000</v>
       </c>
       <c r="M9" s="17" t="inlineStr">
         <is>
@@ -1396,11 +1406,11 @@
         </is>
       </c>
       <c r="B10" s="10" t="n">
-        <v>146373</v>
+        <v>146375</v>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edital nº 26/2026 – Contratação de Consultoria Individual para aprimoramento de soluções analíticas e computacionais aplicadas ao Modelo de Mensuração de Custos da Digitalização de Serviços Públicos </t>
+          <t>Edital nº 28/2026 - Contratação de Consultoria Individual I - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Acessibilidade em Orlas e Praias</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
@@ -1428,7 +1438,7 @@
       </c>
       <c r="I10" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>REMOTO</t>
         </is>
       </c>
       <c r="J10" s="14" t="n">
@@ -1438,7 +1448,7 @@
         <v>46295</v>
       </c>
       <c r="L10" s="15" t="n">
-        <v>108000</v>
+        <v>120000</v>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
@@ -1459,15 +1469,17 @@
     <row r="11">
       <c r="A11" s="17" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B11" s="18" t="n">
-        <v>146360</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>unesco:7863ef0f-6e11-4770-df18-08df01dbdf45</t>
+        </is>
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>PNUD BRA/25/024 - Edital nº 04/2026 – Contrat. de consult. - Engenharia de Dados</t>
+          <t>914BRZ1155 - EDITAL Nº 51/2026 - 3 vagas - Consultor Individual - REPUBLICAÇÃO</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
@@ -1485,56 +1497,48 @@
       </c>
       <c r="G11" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H11" s="19" t="inlineStr">
         <is>
-          <t>MTE</t>
-        </is>
-      </c>
-      <c r="I11" s="19" t="inlineStr">
-        <is>
-          <t>Brasília - DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I11" s="19" t="inlineStr"/>
       <c r="J11" s="22" t="n">
-        <v>46279</v>
+        <v>46281</v>
       </c>
       <c r="K11" s="22" t="n">
-        <v>46287</v>
-      </c>
-      <c r="L11" s="23" t="n">
-        <v>130000</v>
-      </c>
+        <v>46286</v>
+      </c>
+      <c r="L11" s="23" t="inlineStr"/>
       <c r="M11" s="17" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N11" s="20" t="inlineStr">
-        <is>
-          <t>estatisticastrabalho@trabalho.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N11" s="20" t="inlineStr"/>
       <c r="O11" s="24" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B12" s="10" t="n">
-        <v>146361</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>unesco:8c824e7b-7b9a-4a59-7ffc-08df082d82f3</t>
+        </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>PNUD BRA/25/024 - Consultoria Especializada - Qualidade de Dados I</t>
+          <t>914BRZ1163 - Publicação -  Edital 68/2026 - 04 Vagas consultor Individual</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
@@ -1552,56 +1556,48 @@
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>MTE</t>
-        </is>
-      </c>
-      <c r="I12" s="11" t="inlineStr">
-        <is>
-          <t>Brasília - DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I12" s="11" t="inlineStr"/>
       <c r="J12" s="14" t="n">
-        <v>46279</v>
+        <v>46276</v>
       </c>
       <c r="K12" s="14" t="n">
-        <v>46287</v>
-      </c>
-      <c r="L12" s="15" t="n">
-        <v>130000</v>
-      </c>
+        <v>46281</v>
+      </c>
+      <c r="L12" s="15" t="inlineStr"/>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N12" s="12" t="inlineStr">
-        <is>
-          <t>estatisticastrabalho@trabalho.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N12" s="12" t="inlineStr"/>
       <c r="O12" s="16" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="17" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B13" s="18" t="n">
-        <v>146362</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>unesco:5907e744-d46d-4c01-2eaf-08df08e94b75</t>
+        </is>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>PNUD BRA/25/024 - Edital nº 06/2026 - Consultoria Especializada - Qualidade de Dados II</t>
+          <t>914BRZ1159 - Publicação Edital 37/2026 - 2 vagas - Consultor Individual</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
@@ -1619,56 +1615,48 @@
       </c>
       <c r="G13" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H13" s="19" t="inlineStr">
         <is>
-          <t>MTE</t>
-        </is>
-      </c>
-      <c r="I13" s="19" t="inlineStr">
-        <is>
-          <t>Brasília - DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I13" s="19" t="inlineStr"/>
       <c r="J13" s="22" t="n">
-        <v>46279</v>
+        <v>46277</v>
       </c>
       <c r="K13" s="22" t="n">
-        <v>46287</v>
-      </c>
-      <c r="L13" s="23" t="n">
-        <v>130000</v>
-      </c>
+        <v>46283</v>
+      </c>
+      <c r="L13" s="23" t="inlineStr"/>
       <c r="M13" s="17" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N13" s="20" t="inlineStr">
-        <is>
-          <t>estatisticastrabalho@trabalho.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N13" s="20" t="inlineStr"/>
       <c r="O13" s="24" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="n">
-        <v>146374</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>unesco:1011b77e-9c7a-4ea9-2632-08df0e687345</t>
+        </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>Edital nº 27/2026 – Contratação de Consultoria Individual II - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Servidões de Passagem para Orlas e Praias</t>
+          <t>914BRZ1159 - Publicação Edital 39/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -1686,56 +1674,48 @@
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
         <is>
-          <t>MGI</t>
-        </is>
-      </c>
-      <c r="I14" s="11" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I14" s="11" t="inlineStr"/>
       <c r="J14" s="14" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="K14" s="14" t="n">
-        <v>46295</v>
-      </c>
-      <c r="L14" s="15" t="n">
-        <v>120000</v>
-      </c>
+        <v>46283</v>
+      </c>
+      <c r="L14" s="15" t="inlineStr"/>
       <c r="M14" s="9" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N14" s="12" t="inlineStr">
-        <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N14" s="12" t="inlineStr"/>
       <c r="O14" s="16" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="17" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B15" s="18" t="n">
-        <v>146375</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>unesco:030ad7b8-d33f-491a-31d9-08defb16c1ac</t>
+        </is>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>Edital nº 28/2026 - Contratação de Consultoria Individual I - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Acessibilidade em Orlas e Praias</t>
+          <t>Projeto 914BRZ5067 - Edital Nº 08/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
@@ -1753,41 +1733,31 @@
       </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H15" s="19" t="inlineStr">
         <is>
-          <t>MGI</t>
-        </is>
-      </c>
-      <c r="I15" s="19" t="inlineStr">
-        <is>
-          <t>REMOTO</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I15" s="19" t="inlineStr"/>
       <c r="J15" s="22" t="n">
-        <v>46280</v>
+        <v>46253</v>
       </c>
       <c r="K15" s="22" t="n">
-        <v>46295</v>
-      </c>
-      <c r="L15" s="23" t="n">
-        <v>120000</v>
-      </c>
+        <v>46283</v>
+      </c>
+      <c r="L15" s="23" t="inlineStr"/>
       <c r="M15" s="17" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N15" s="20" t="inlineStr">
-        <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N15" s="20" t="inlineStr"/>
       <c r="O15" s="24" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
@@ -1799,12 +1769,12 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>unesco:8c824e7b-7b9a-4a59-7ffc-08df082d82f3</t>
+          <t>unesco:a42aa3e1-2e33-46e6-2633-08df0e687345</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1163 - Publicação -  Edital 68/2026 - 04 Vagas consultor Individual</t>
+          <t>914BRZ1159 - Publicação Edital 38/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -1822,7 +1792,7 @@
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
@@ -1832,10 +1802,10 @@
       </c>
       <c r="I16" s="11" t="inlineStr"/>
       <c r="J16" s="14" t="n">
-        <v>46276</v>
+        <v>46279</v>
       </c>
       <c r="K16" s="14" t="n">
-        <v>46281</v>
+        <v>46283</v>
       </c>
       <c r="L16" s="15" t="inlineStr"/>
       <c r="M16" s="9" t="inlineStr">
@@ -1853,17 +1823,17 @@
     <row r="17">
       <c r="A17" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>unesco:5907e744-d46d-4c01-2eaf-08df08e94b75</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077</t>
         </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 37/2026 - 2 vagas - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/16/002 – TR13077</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1877,57 +1847,67 @@
         </is>
       </c>
       <c r="F17" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I17" s="19" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I17" s="19" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J17" s="22" t="n">
-        <v>46277</v>
+        <v>46223</v>
       </c>
       <c r="K17" s="22" t="n">
-        <v>46283</v>
-      </c>
-      <c r="L17" s="23" t="inlineStr"/>
+        <v>46238</v>
+      </c>
+      <c r="L17" s="23" t="n">
+        <v>100000</v>
+      </c>
       <c r="M17" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N17" s="20" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N17" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O17" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077/</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>unesco:1011b77e-9c7a-4ea9-2632-08df0e687345</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 39/2026 - 1 vaga - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13098</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
@@ -1940,53 +1920,61 @@
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I18" s="11" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I18" s="11" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J18" s="14" t="n">
-        <v>46279</v>
+        <v>46221</v>
       </c>
       <c r="K18" s="14" t="n">
-        <v>46283</v>
+        <v>46224</v>
       </c>
       <c r="L18" s="15" t="inlineStr"/>
       <c r="M18" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N18" s="12" t="inlineStr"/>
+          <t>En presentación</t>
+        </is>
+      </c>
+      <c r="N18" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O18" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098/</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>unesco:030ad7b8-d33f-491a-31d9-08defb16c1ac</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ5067 - Edital Nº 08/2026 - 1 vaga - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E19" s="20" t="inlineStr">
@@ -1995,57 +1983,67 @@
         </is>
       </c>
       <c r="F19" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I19" s="19" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I19" s="19" t="inlineStr">
+        <is>
+          <t>Brasília DF</t>
+        </is>
+      </c>
       <c r="J19" s="22" t="n">
-        <v>46253</v>
+        <v>46227</v>
       </c>
       <c r="K19" s="22" t="n">
-        <v>46283</v>
-      </c>
-      <c r="L19" s="23" t="inlineStr"/>
+        <v>46231</v>
+      </c>
+      <c r="L19" s="23" t="n">
+        <v>150000</v>
+      </c>
       <c r="M19" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N19" s="20" t="inlineStr"/>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N19" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O19" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>unesco:a42aa3e1-2e33-46e6-2633-08df0e687345</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 38/2026 - 1 vaga - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
@@ -2054,35 +2052,45 @@
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I20" s="11" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="inlineStr">
+        <is>
+          <t>Recife - PE</t>
+        </is>
+      </c>
       <c r="J20" s="14" t="n">
-        <v>46279</v>
+        <v>46225</v>
       </c>
       <c r="K20" s="14" t="n">
-        <v>46283</v>
-      </c>
-      <c r="L20" s="15" t="inlineStr"/>
+        <v>46229</v>
+      </c>
+      <c r="L20" s="15" t="n">
+        <v>114600</v>
+      </c>
       <c r="M20" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N20" s="12" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N20" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O20" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
         </is>
       </c>
     </row>
@@ -2094,17 +2102,17 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13098</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E21" s="20" t="inlineStr">
@@ -2113,33 +2121,35 @@
         </is>
       </c>
       <c r="F21" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G21" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I21" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
         </is>
       </c>
       <c r="J21" s="22" t="n">
-        <v>46221</v>
+        <v>46224</v>
       </c>
       <c r="K21" s="22" t="n">
-        <v>46224</v>
-      </c>
-      <c r="L21" s="23" t="inlineStr"/>
+        <v>46233</v>
+      </c>
+      <c r="L21" s="23" t="n">
+        <v>288000</v>
+      </c>
       <c r="M21" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N21" s="20" t="inlineStr">
@@ -2149,7 +2159,7 @@
       </c>
       <c r="O21" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
         </is>
       </c>
     </row>
@@ -2161,17 +2171,17 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13015</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E22" s="12" t="inlineStr">
@@ -2180,31 +2190,31 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.4</v>
+        <v>0.343</v>
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I22" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J22" s="14" t="n">
-        <v>46220</v>
+        <v>46232</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46225</v>
+        <v>46238</v>
       </c>
       <c r="L22" s="15" t="n">
-        <v>58800</v>
+        <v>30000</v>
       </c>
       <c r="M22" s="9" t="inlineStr">
         <is>
@@ -2218,7 +2228,7 @@
       </c>
       <c r="O22" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
         </is>
       </c>
     </row>
@@ -2230,12 +2240,12 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
@@ -2245,35 +2255,33 @@
       </c>
       <c r="E23" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F23" s="21" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F23" s="21" t="inlineStr"/>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I23" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J23" s="22" t="n">
-        <v>46225</v>
+        <v>46232</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46229</v>
+        <v>46238</v>
       </c>
       <c r="L23" s="23" t="n">
-        <v>114600</v>
+        <v>30000</v>
       </c>
       <c r="M23" s="17" t="inlineStr">
         <is>
@@ -2287,7 +2295,7 @@
       </c>
       <c r="O23" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
         </is>
       </c>
     </row>
@@ -2299,17 +2307,17 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/16/002 – TR13077</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E24" s="12" t="inlineStr">
@@ -2322,7 +2330,7 @@
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
@@ -2332,17 +2340,17 @@
       </c>
       <c r="I24" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
         </is>
       </c>
       <c r="J24" s="14" t="n">
-        <v>46223</v>
+        <v>46232</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46238</v>
+        <v>46237</v>
       </c>
       <c r="L24" s="15" t="n">
-        <v>100000</v>
+        <v>288000</v>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
@@ -2356,7 +2364,7 @@
       </c>
       <c r="O24" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
         </is>
       </c>
     </row>
@@ -2368,12 +2376,12 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
@@ -2391,31 +2399,31 @@
       </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I25" s="19" t="inlineStr">
         <is>
-          <t>Brasília DF</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J25" s="22" t="n">
-        <v>46227</v>
+        <v>46240</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46231</v>
+        <v>46245</v>
       </c>
       <c r="L25" s="23" t="n">
-        <v>150000</v>
+        <v>204000</v>
       </c>
       <c r="M25" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N25" s="20" t="inlineStr">
@@ -2425,7 +2433,7 @@
       </c>
       <c r="O25" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
         </is>
       </c>
     </row>
@@ -2437,12 +2445,12 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -2460,7 +2468,7 @@
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
@@ -2470,17 +2478,17 @@
       </c>
       <c r="I26" s="11" t="inlineStr">
         <is>
-          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J26" s="14" t="n">
-        <v>46224</v>
+        <v>46240</v>
       </c>
       <c r="K26" s="14" t="n">
-        <v>46233</v>
+        <v>46245</v>
       </c>
       <c r="L26" s="15" t="n">
-        <v>288000</v>
+        <v>204000</v>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
@@ -2494,7 +2502,7 @@
       </c>
       <c r="O26" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
         </is>
       </c>
     </row>
@@ -2506,17 +2514,17 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E27" s="20" t="inlineStr">
@@ -2525,11 +2533,11 @@
         </is>
       </c>
       <c r="F27" s="21" t="n">
-        <v>0.343</v>
+        <v>0.4</v>
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
@@ -2539,17 +2547,17 @@
       </c>
       <c r="I27" s="19" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Brasília - Df</t>
         </is>
       </c>
       <c r="J27" s="22" t="n">
-        <v>46232</v>
+        <v>46240</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46238</v>
+        <v>46245</v>
       </c>
       <c r="L27" s="23" t="n">
-        <v>30000</v>
+        <v>80000</v>
       </c>
       <c r="M27" s="17" t="inlineStr">
         <is>
@@ -2563,7 +2571,7 @@
       </c>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
         </is>
       </c>
     </row>
@@ -2575,12 +2583,12 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
@@ -2590,13 +2598,15 @@
       </c>
       <c r="E28" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F28" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F28" s="13" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
@@ -2606,17 +2616,17 @@
       </c>
       <c r="I28" s="11" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J28" s="14" t="n">
-        <v>46232</v>
+        <v>46240</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46238</v>
+        <v>46245</v>
       </c>
       <c r="L28" s="15" t="n">
-        <v>30000</v>
+        <v>80000</v>
       </c>
       <c r="M28" s="9" t="inlineStr">
         <is>
@@ -2630,7 +2640,7 @@
       </c>
       <c r="O28" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
         </is>
       </c>
     </row>
@@ -2642,12 +2652,12 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
@@ -2665,27 +2675,27 @@
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I29" s="19" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J29" s="22" t="n">
-        <v>46232</v>
+        <v>46240</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46237</v>
+        <v>46245</v>
       </c>
       <c r="L29" s="23" t="n">
-        <v>288000</v>
+        <v>100000</v>
       </c>
       <c r="M29" s="17" t="inlineStr">
         <is>
@@ -2699,7 +2709,7 @@
       </c>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
         </is>
       </c>
     </row>
@@ -2711,12 +2721,12 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
@@ -2726,35 +2736,33 @@
       </c>
       <c r="E30" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F30" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F30" s="13" t="inlineStr"/>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
         </is>
       </c>
       <c r="J30" s="14" t="n">
-        <v>46240</v>
+        <v>46227</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>46245</v>
+        <v>46252</v>
       </c>
       <c r="L30" s="15" t="n">
-        <v>204000</v>
+        <v>286000</v>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
@@ -2768,7 +2776,7 @@
       </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
@@ -2780,12 +2788,12 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
@@ -2803,27 +2811,27 @@
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I31" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J31" s="22" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46245</v>
+        <v>46257</v>
       </c>
       <c r="L31" s="23" t="n">
-        <v>204000</v>
+        <v>54000</v>
       </c>
       <c r="M31" s="17" t="inlineStr">
         <is>
@@ -2837,7 +2845,7 @@
       </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -2849,12 +2857,12 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
@@ -2872,27 +2880,27 @@
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I32" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J32" s="14" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K32" s="14" t="n">
-        <v>46245</v>
+        <v>46257</v>
       </c>
       <c r="L32" s="15" t="n">
-        <v>80000</v>
+        <v>54000</v>
       </c>
       <c r="M32" s="9" t="inlineStr">
         <is>
@@ -2906,7 +2914,7 @@
       </c>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -2918,12 +2926,12 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
@@ -2937,11 +2945,11 @@
         </is>
       </c>
       <c r="F33" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
@@ -2951,21 +2959,19 @@
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>Brasília - Df</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J33" s="22" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46245</v>
-      </c>
-      <c r="L33" s="23" t="n">
-        <v>80000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L33" s="23" t="inlineStr"/>
       <c r="M33" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N33" s="20" t="inlineStr">
@@ -2975,7 +2981,7 @@
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -2987,17 +2993,17 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E34" s="12" t="inlineStr">
@@ -3010,27 +3016,27 @@
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J34" s="14" t="n">
-        <v>46240</v>
+        <v>46251</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46245</v>
+        <v>46256</v>
       </c>
       <c r="L34" s="15" t="n">
-        <v>100000</v>
+        <v>50000</v>
       </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
@@ -3044,7 +3050,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -3056,12 +3062,12 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
@@ -3071,13 +3077,15 @@
       </c>
       <c r="E35" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F35" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F35" s="21" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
@@ -3087,17 +3095,17 @@
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46227</v>
+        <v>46252</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46252</v>
+        <v>46259</v>
       </c>
       <c r="L35" s="23" t="n">
-        <v>286000</v>
+        <v>60000</v>
       </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
@@ -3111,7 +3119,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -3123,12 +3131,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -3142,30 +3150,32 @@
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
         <v>46246</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L36" s="15" t="inlineStr"/>
+        <v>46272</v>
+      </c>
+      <c r="L36" s="15" t="n">
+        <v>54000</v>
+      </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
           <t>En fase de apresentação</t>
@@ -3178,7 +3188,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -3190,22 +3200,22 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E37" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F37" s="21" t="n">
@@ -3213,27 +3223,27 @@
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46246</v>
+        <v>46265</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46257</v>
+        <v>46270</v>
       </c>
       <c r="L37" s="23" t="n">
-        <v>54000</v>
+        <v>30000</v>
       </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
@@ -3247,7 +3257,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -3259,17 +3269,17 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E38" s="12" t="inlineStr">
@@ -3282,41 +3292,41 @@
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46251</v>
+        <v>46208</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46256</v>
+        <v>46259</v>
       </c>
       <c r="L38" s="15" t="n">
-        <v>50000</v>
+        <v>500000</v>
       </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N38" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -3328,12 +3338,12 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
@@ -3347,11 +3357,11 @@
         </is>
       </c>
       <c r="F39" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
@@ -3361,31 +3371,29 @@
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46246</v>
+        <v>46278</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46257</v>
-      </c>
-      <c r="L39" s="23" t="n">
-        <v>54000</v>
-      </c>
+        <v>46283</v>
+      </c>
+      <c r="L39" s="23" t="inlineStr"/>
       <c r="M39" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N39" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>ugp@educacao.sp.gov.br</t>
         </is>
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
         </is>
       </c>
     </row>
@@ -3397,12 +3405,12 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
@@ -3420,7 +3428,7 @@
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
@@ -3434,13 +3442,13 @@
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46252</v>
+        <v>46266</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46259</v>
+        <v>46283</v>
       </c>
       <c r="L40" s="15" t="n">
-        <v>60000</v>
+        <v>70000</v>
       </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
@@ -3454,7 +3462,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
@@ -3466,17 +3474,17 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E41" s="20" t="inlineStr">
@@ -3489,41 +3497,41 @@
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46208</v>
+        <v>46275</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46259</v>
+        <v>46280</v>
       </c>
       <c r="L41" s="23" t="n">
-        <v>500000</v>
+        <v>50000</v>
       </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N41" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
@@ -3535,12 +3543,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3554,35 +3562,33 @@
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46246</v>
+        <v>46275</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46272</v>
-      </c>
-      <c r="L42" s="15" t="n">
-        <v>54000</v>
-      </c>
+        <v>46281</v>
+      </c>
+      <c r="L42" s="15" t="inlineStr"/>
       <c r="M42" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N42" s="12" t="inlineStr">
@@ -3592,7 +3598,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
         </is>
       </c>
     </row>
@@ -3604,22 +3610,22 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E43" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F43" s="21" t="n">
@@ -3627,41 +3633,41 @@
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46265</v>
+        <v>46244</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46270</v>
+        <v>46296</v>
       </c>
       <c r="L43" s="23" t="n">
-        <v>30000</v>
+        <v>935000</v>
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N43" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -3673,17 +3679,17 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E44" s="12" t="inlineStr">
@@ -3696,41 +3702,41 @@
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46275</v>
+        <v>46244</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46280</v>
+        <v>46300</v>
       </c>
       <c r="L44" s="15" t="n">
-        <v>50000</v>
+        <v>350000</v>
       </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N44" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -3742,17 +3748,17 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E45" s="20" t="inlineStr">
@@ -3765,27 +3771,27 @@
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Dados Remoto</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46266</v>
+        <v>46281</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46283</v>
+        <v>46286</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>70000</v>
+        <v>110000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
@@ -3799,284 +3805,12 @@
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="9" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B46" s="10" t="inlineStr">
-        <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
-        </is>
-      </c>
-      <c r="C46" s="11" t="inlineStr">
-        <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
-        </is>
-      </c>
-      <c r="D46" s="11" t="inlineStr">
-        <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
-        </is>
-      </c>
-      <c r="E46" s="12" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F46" s="13" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G46" s="11" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
-        </is>
-      </c>
-      <c r="H46" s="11" t="inlineStr">
-        <is>
-          <t>OEI/MDHC</t>
-        </is>
-      </c>
-      <c r="I46" s="11" t="inlineStr">
-        <is>
-          <t>Nacional</t>
-        </is>
-      </c>
-      <c r="J46" s="14" t="n">
-        <v>46244</v>
-      </c>
-      <c r="K46" s="14" t="n">
-        <v>46300</v>
-      </c>
-      <c r="L46" s="15" t="n">
-        <v>350000</v>
-      </c>
-      <c r="M46" s="9" t="inlineStr">
-        <is>
-          <t>En fase de apresentação</t>
-        </is>
-      </c>
-      <c r="N46" s="12" t="inlineStr">
-        <is>
-          <t>compras.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O46" s="16" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="17" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B47" s="18" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
-        </is>
-      </c>
-      <c r="C47" s="19" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
-        </is>
-      </c>
-      <c r="D47" s="19" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E47" s="20" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F47" s="21" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="G47" s="19" t="inlineStr">
-        <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
-        </is>
-      </c>
-      <c r="H47" s="19" t="inlineStr">
-        <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I47" s="19" t="inlineStr">
-        <is>
-          <t>São Paulo - SP</t>
-        </is>
-      </c>
-      <c r="J47" s="22" t="n">
-        <v>46278</v>
-      </c>
-      <c r="K47" s="22" t="n">
-        <v>46283</v>
-      </c>
-      <c r="L47" s="23" t="inlineStr"/>
-      <c r="M47" s="17" t="inlineStr">
-        <is>
-          <t>En presentación</t>
-        </is>
-      </c>
-      <c r="N47" s="20" t="inlineStr">
-        <is>
-          <t>ugp@educacao.sp.gov.br</t>
-        </is>
-      </c>
-      <c r="O47" s="24" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="9" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B48" s="10" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
-        </is>
-      </c>
-      <c r="C48" s="11" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
-        </is>
-      </c>
-      <c r="D48" s="11" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E48" s="12" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F48" s="13" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="G48" s="11" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
-        </is>
-      </c>
-      <c r="H48" s="11" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I48" s="11" t="inlineStr">
-        <is>
-          <t>Porto Alegre - RS</t>
-        </is>
-      </c>
-      <c r="J48" s="14" t="n">
-        <v>46275</v>
-      </c>
-      <c r="K48" s="14" t="n">
-        <v>46281</v>
-      </c>
-      <c r="L48" s="15" t="inlineStr"/>
-      <c r="M48" s="9" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N48" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O48" s="16" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="17" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B49" s="18" t="inlineStr">
-        <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
-        </is>
-      </c>
-      <c r="C49" s="19" t="inlineStr">
-        <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
-        </is>
-      </c>
-      <c r="D49" s="19" t="inlineStr">
-        <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
-        </is>
-      </c>
-      <c r="E49" s="20" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F49" s="21" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G49" s="19" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
-        </is>
-      </c>
-      <c r="H49" s="19" t="inlineStr">
-        <is>
-          <t>OEI/MDHC</t>
-        </is>
-      </c>
-      <c r="I49" s="19" t="inlineStr">
-        <is>
-          <t>Nacional</t>
-        </is>
-      </c>
-      <c r="J49" s="22" t="n">
-        <v>46244</v>
-      </c>
-      <c r="K49" s="22" t="n">
-        <v>46296</v>
-      </c>
-      <c r="L49" s="23" t="n">
-        <v>935000</v>
-      </c>
-      <c r="M49" s="17" t="inlineStr">
-        <is>
-          <t>En fase de apresentação</t>
-        </is>
-      </c>
-      <c r="N49" s="20" t="inlineStr">
-        <is>
-          <t>compras.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O49" s="24" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O49"/>
+  <autoFilter ref="A1:O45"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -4122,10 +3856,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId48"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -4174,7 +3904,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4">
@@ -4184,7 +3914,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -4226,7 +3956,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>43</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3">
@@ -4288,7 +4018,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3">
@@ -4298,7 +4028,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4">
@@ -4360,7 +4090,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>39</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3">
@@ -4370,7 +4100,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>32</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4">
@@ -4380,7 +4110,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5">
@@ -4462,7 +4192,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3">
@@ -4472,13 +4202,13 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B4" s="10" t="n">
@@ -4498,17 +4228,17 @@
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>MTE</t>
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>MTE</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="B7" s="18" t="n">
@@ -4518,11 +4248,11 @@
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -4570,7 +4300,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -4585,7 +4315,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -4600,7 +4330,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
@@ -4615,7 +4345,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-09-17 16:24
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$49</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -25,7 +25,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Por_Perfil'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Por_Tipo'!$A$1:$B$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Por_Tipo'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Por_Area'!$A$1:$B$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Por_Area'!$A$1:$B$9</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Por_Area'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Por_Orgao'!$A$1:$B$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Por_Orgao'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 16/09/2026 às 16:12</t>
+          <t>Gerado em 17/09/2026 às 16:18</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="17">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>170864</v>
+        <v>165446.1538461538</v>
       </c>
     </row>
     <row r="20">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="24">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O45"/>
+  <dimension ref="A1:O49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1469,17 +1469,15 @@
     <row r="11">
       <c r="A11" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B11" s="18" t="inlineStr">
-        <is>
-          <t>unesco:7863ef0f-6e11-4770-df18-08df01dbdf45</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B11" s="18" t="n">
+        <v>146386</v>
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 51/2026 - 3 vagas - Consultor Individual - REPUBLICAÇÃO</t>
+          <t>BRA/25/024 - Edital nº 08/2026 – Contratação de 6 (seis) consultorias especializadas (pessoa física) para revisão, consolidação, simplificação e otimização de atos normativos trabalhistas infralegais no Brasil</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
@@ -1497,53 +1495,61 @@
       </c>
       <c r="G11" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Saúde, Direito / Jurídico</t>
         </is>
       </c>
       <c r="H11" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I11" s="19" t="inlineStr"/>
+          <t>MTE</t>
+        </is>
+      </c>
+      <c r="I11" s="19" t="inlineStr">
+        <is>
+          <t>Híbrido, com eventuais reuniões presenciais em Brasília/DF</t>
+        </is>
+      </c>
       <c r="J11" s="22" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="K11" s="22" t="n">
-        <v>46286</v>
-      </c>
-      <c r="L11" s="23" t="inlineStr"/>
+        <v>46292</v>
+      </c>
+      <c r="L11" s="23" t="n">
+        <v>92520</v>
+      </c>
       <c r="M11" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N11" s="20" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N11" s="20" t="inlineStr">
+        <is>
+          <t>processoseletivo.sat@trabalho.gov.br</t>
+        </is>
+      </c>
       <c r="O11" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B12" s="10" t="inlineStr">
-        <is>
-          <t>unesco:8c824e7b-7b9a-4a59-7ffc-08df082d82f3</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="n">
+        <v>146390</v>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1163 - Publicação -  Edital 68/2026 - 04 Vagas consultor Individual</t>
+          <t>BRA/24/018 - CONTRATAÇÃO DE CONSULTOR ESPECIALIZADO EM POLÍTICA DE INOVAÇÃO E DE TRANSFORMAÇÃO DIGITAL</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E12" s="12" t="inlineStr">
@@ -1561,26 +1567,36 @@
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I12" s="11" t="inlineStr"/>
+          <t>Não identificado</t>
+        </is>
+      </c>
+      <c r="I12" s="11" t="inlineStr">
+        <is>
+          <t>Salvador/BA</t>
+        </is>
+      </c>
       <c r="J12" s="14" t="n">
-        <v>46276</v>
+        <v>46282</v>
       </c>
       <c r="K12" s="14" t="n">
-        <v>46281</v>
-      </c>
-      <c r="L12" s="15" t="inlineStr"/>
+        <v>46296</v>
+      </c>
+      <c r="L12" s="15" t="n">
+        <v>49580</v>
+      </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N12" s="12" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N12" s="12" t="inlineStr">
+        <is>
+          <t>selecaopnud0326@pge.ba.gov.br</t>
+        </is>
+      </c>
       <c r="O12" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
@@ -1592,12 +1608,12 @@
       </c>
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t>unesco:5907e744-d46d-4c01-2eaf-08df08e94b75</t>
+          <t>unesco:7863ef0f-6e11-4770-df18-08df01dbdf45</t>
         </is>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 37/2026 - 2 vagas - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 51/2026 - 3 vagas - Consultor Individual - REPUBLICAÇÃO</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
@@ -1615,7 +1631,7 @@
       </c>
       <c r="G13" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H13" s="19" t="inlineStr">
@@ -1625,10 +1641,10 @@
       </c>
       <c r="I13" s="19" t="inlineStr"/>
       <c r="J13" s="22" t="n">
-        <v>46277</v>
+        <v>46281</v>
       </c>
       <c r="K13" s="22" t="n">
-        <v>46283</v>
+        <v>46286</v>
       </c>
       <c r="L13" s="23" t="inlineStr"/>
       <c r="M13" s="17" t="inlineStr">
@@ -1651,12 +1667,12 @@
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>unesco:1011b77e-9c7a-4ea9-2632-08df0e687345</t>
+          <t>unesco:c9020343-9d28-49e3-b9e3-08df0436270c</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 39/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 52/2026 - 1 vaga - Consultor Individual - REPUBLICAÇÃO</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -1674,7 +1690,7 @@
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
@@ -1684,10 +1700,10 @@
       </c>
       <c r="I14" s="11" t="inlineStr"/>
       <c r="J14" s="14" t="n">
-        <v>46279</v>
+        <v>46282</v>
       </c>
       <c r="K14" s="14" t="n">
-        <v>46283</v>
+        <v>46286</v>
       </c>
       <c r="L14" s="15" t="inlineStr"/>
       <c r="M14" s="9" t="inlineStr">
@@ -1710,12 +1726,12 @@
       </c>
       <c r="B15" s="18" t="inlineStr">
         <is>
-          <t>unesco:030ad7b8-d33f-491a-31d9-08defb16c1ac</t>
+          <t>unesco:6f0bebf7-7be2-4b29-17c5-08df04786cdd</t>
         </is>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ5067 - Edital Nº 08/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 53/2026 - 1 vaga - Consultor Individual - REPUBLICAÇÃO</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
@@ -1733,7 +1749,7 @@
       </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H15" s="19" t="inlineStr">
@@ -1743,10 +1759,10 @@
       </c>
       <c r="I15" s="19" t="inlineStr"/>
       <c r="J15" s="22" t="n">
-        <v>46253</v>
+        <v>46282</v>
       </c>
       <c r="K15" s="22" t="n">
-        <v>46283</v>
+        <v>46286</v>
       </c>
       <c r="L15" s="23" t="inlineStr"/>
       <c r="M15" s="17" t="inlineStr">
@@ -1769,12 +1785,12 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>unesco:a42aa3e1-2e33-46e6-2633-08df0e687345</t>
+          <t>unesco:34a61630-55f8-4262-9489-08df0f3a2d32</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 38/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1156 - edital 08/2026 - Consultor Individual</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -1792,7 +1808,7 @@
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
@@ -1802,10 +1818,10 @@
       </c>
       <c r="I16" s="11" t="inlineStr"/>
       <c r="J16" s="14" t="n">
-        <v>46279</v>
+        <v>46282</v>
       </c>
       <c r="K16" s="14" t="n">
-        <v>46283</v>
+        <v>46289</v>
       </c>
       <c r="L16" s="15" t="inlineStr"/>
       <c r="M16" s="9" t="inlineStr">
@@ -1823,17 +1839,17 @@
     <row r="17">
       <c r="A17" s="17" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077</t>
+          <t>unesco:5907e744-d46d-4c01-2eaf-08df08e94b75</t>
         </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/16/002 – TR13077</t>
+          <t>914BRZ1159 - Publicação Edital 37/2026 - 2 vagas - Consultor Individual</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1847,67 +1863,57 @@
         </is>
       </c>
       <c r="F17" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I17" s="19" t="inlineStr">
-        <is>
-          <t>Brasília - DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I17" s="19" t="inlineStr"/>
       <c r="J17" s="22" t="n">
-        <v>46223</v>
+        <v>46277</v>
       </c>
       <c r="K17" s="22" t="n">
-        <v>46238</v>
-      </c>
-      <c r="L17" s="23" t="n">
-        <v>100000</v>
-      </c>
+        <v>46283</v>
+      </c>
+      <c r="L17" s="23" t="inlineStr"/>
       <c r="M17" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N17" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N17" s="20" t="inlineStr"/>
       <c r="O17" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098</t>
+          <t>unesco:1011b77e-9c7a-4ea9-2632-08df0e687345</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13098</t>
+          <t>914BRZ1159 - Publicação Edital 39/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
@@ -1920,61 +1926,53 @@
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I18" s="11" t="inlineStr">
-        <is>
-          <t>Brasília - DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I18" s="11" t="inlineStr"/>
       <c r="J18" s="14" t="n">
-        <v>46221</v>
+        <v>46279</v>
       </c>
       <c r="K18" s="14" t="n">
-        <v>46224</v>
+        <v>46283</v>
       </c>
       <c r="L18" s="15" t="inlineStr"/>
       <c r="M18" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
-        </is>
-      </c>
-      <c r="N18" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N18" s="12" t="inlineStr"/>
       <c r="O18" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="17" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
+          <t>unesco:030ad7b8-d33f-491a-31d9-08defb16c1ac</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
+          <t>Projeto 914BRZ5067 - Edital Nº 08/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E19" s="20" t="inlineStr">
@@ -1983,67 +1981,57 @@
         </is>
       </c>
       <c r="F19" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I19" s="19" t="inlineStr">
-        <is>
-          <t>Brasília DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I19" s="19" t="inlineStr"/>
       <c r="J19" s="22" t="n">
-        <v>46227</v>
+        <v>46253</v>
       </c>
       <c r="K19" s="22" t="n">
-        <v>46231</v>
-      </c>
-      <c r="L19" s="23" t="n">
-        <v>150000</v>
-      </c>
+        <v>46283</v>
+      </c>
+      <c r="L19" s="23" t="inlineStr"/>
       <c r="M19" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
-        </is>
-      </c>
-      <c r="N19" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N19" s="20" t="inlineStr"/>
       <c r="O19" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
+          <t>unesco:a42aa3e1-2e33-46e6-2633-08df0e687345</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
+          <t>914BRZ1159 - Publicação Edital 38/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
@@ -2052,45 +2040,35 @@
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I20" s="11" t="inlineStr">
-        <is>
-          <t>Recife - PE</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="inlineStr"/>
       <c r="J20" s="14" t="n">
-        <v>46225</v>
+        <v>46279</v>
       </c>
       <c r="K20" s="14" t="n">
-        <v>46229</v>
-      </c>
-      <c r="L20" s="15" t="n">
-        <v>114600</v>
-      </c>
+        <v>46283</v>
+      </c>
+      <c r="L20" s="15" t="inlineStr"/>
       <c r="M20" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N20" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N20" s="12" t="inlineStr"/>
       <c r="O20" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
@@ -2102,17 +2080,17 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/16/002 – TR13077</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E21" s="20" t="inlineStr">
@@ -2125,27 +2103,27 @@
       </c>
       <c r="G21" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I21" s="19" t="inlineStr">
         <is>
-          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J21" s="22" t="n">
-        <v>46224</v>
+        <v>46223</v>
       </c>
       <c r="K21" s="22" t="n">
-        <v>46233</v>
+        <v>46238</v>
       </c>
       <c r="L21" s="23" t="n">
-        <v>288000</v>
+        <v>100000</v>
       </c>
       <c r="M21" s="17" t="inlineStr">
         <is>
@@ -2159,7 +2137,7 @@
       </c>
       <c r="O21" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077/</t>
         </is>
       </c>
     </row>
@@ -2171,17 +2149,17 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E22" s="12" t="inlineStr">
@@ -2190,31 +2168,31 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.343</v>
+        <v>0.4</v>
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I22" s="11" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J22" s="14" t="n">
-        <v>46232</v>
+        <v>46225</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46238</v>
+        <v>46229</v>
       </c>
       <c r="L22" s="15" t="n">
-        <v>30000</v>
+        <v>114600</v>
       </c>
       <c r="M22" s="9" t="inlineStr">
         <is>
@@ -2228,7 +2206,7 @@
       </c>
       <c r="O22" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
         </is>
       </c>
     </row>
@@ -2240,12 +2218,12 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
@@ -2255,13 +2233,15 @@
       </c>
       <c r="E23" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F23" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F23" s="21" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
@@ -2271,17 +2251,17 @@
       </c>
       <c r="I23" s="19" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
         </is>
       </c>
       <c r="J23" s="22" t="n">
-        <v>46232</v>
+        <v>46224</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46238</v>
+        <v>46233</v>
       </c>
       <c r="L23" s="23" t="n">
-        <v>30000</v>
+        <v>288000</v>
       </c>
       <c r="M23" s="17" t="inlineStr">
         <is>
@@ -2295,7 +2275,7 @@
       </c>
       <c r="O23" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
         </is>
       </c>
     </row>
@@ -2307,12 +2287,12 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -2330,7 +2310,7 @@
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
@@ -2340,21 +2320,21 @@
       </c>
       <c r="I24" s="11" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
+          <t>Brasília DF</t>
         </is>
       </c>
       <c r="J24" s="14" t="n">
-        <v>46232</v>
+        <v>46227</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46237</v>
+        <v>46231</v>
       </c>
       <c r="L24" s="15" t="n">
-        <v>288000</v>
+        <v>150000</v>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N24" s="12" t="inlineStr">
@@ -2364,7 +2344,7 @@
       </c>
       <c r="O24" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
         </is>
       </c>
     </row>
@@ -2376,17 +2356,17 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E25" s="20" t="inlineStr">
@@ -2395,11 +2375,11 @@
         </is>
       </c>
       <c r="F25" s="21" t="n">
-        <v>0.4</v>
+        <v>0.343</v>
       </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
@@ -2409,17 +2389,17 @@
       </c>
       <c r="I25" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J25" s="22" t="n">
-        <v>46240</v>
+        <v>46232</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46245</v>
+        <v>46238</v>
       </c>
       <c r="L25" s="23" t="n">
-        <v>204000</v>
+        <v>30000</v>
       </c>
       <c r="M25" s="17" t="inlineStr">
         <is>
@@ -2433,7 +2413,7 @@
       </c>
       <c r="O25" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
         </is>
       </c>
     </row>
@@ -2445,12 +2425,12 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -2460,15 +2440,13 @@
       </c>
       <c r="E26" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F26" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F26" s="13" t="inlineStr"/>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
@@ -2478,17 +2456,17 @@
       </c>
       <c r="I26" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J26" s="14" t="n">
-        <v>46240</v>
+        <v>46232</v>
       </c>
       <c r="K26" s="14" t="n">
-        <v>46245</v>
+        <v>46238</v>
       </c>
       <c r="L26" s="15" t="n">
-        <v>204000</v>
+        <v>30000</v>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
@@ -2502,7 +2480,7 @@
       </c>
       <c r="O26" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
         </is>
       </c>
     </row>
@@ -2514,12 +2492,12 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
@@ -2547,7 +2525,7 @@
       </c>
       <c r="I27" s="19" t="inlineStr">
         <is>
-          <t>Brasília - Df</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J27" s="22" t="n">
@@ -2557,7 +2535,7 @@
         <v>46245</v>
       </c>
       <c r="L27" s="23" t="n">
-        <v>80000</v>
+        <v>204000</v>
       </c>
       <c r="M27" s="17" t="inlineStr">
         <is>
@@ -2571,7 +2549,7 @@
       </c>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
         </is>
       </c>
     </row>
@@ -2583,12 +2561,12 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
@@ -2606,27 +2584,27 @@
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I28" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
         </is>
       </c>
       <c r="J28" s="14" t="n">
-        <v>46240</v>
+        <v>46232</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46245</v>
+        <v>46237</v>
       </c>
       <c r="L28" s="15" t="n">
-        <v>80000</v>
+        <v>288000</v>
       </c>
       <c r="M28" s="9" t="inlineStr">
         <is>
@@ -2640,7 +2618,7 @@
       </c>
       <c r="O28" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
         </is>
       </c>
     </row>
@@ -2652,12 +2630,12 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
@@ -2675,7 +2653,7 @@
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
@@ -2695,7 +2673,7 @@
         <v>46245</v>
       </c>
       <c r="L29" s="23" t="n">
-        <v>100000</v>
+        <v>204000</v>
       </c>
       <c r="M29" s="17" t="inlineStr">
         <is>
@@ -2709,7 +2687,7 @@
       </c>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
         </is>
       </c>
     </row>
@@ -2721,12 +2699,12 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
@@ -2736,33 +2714,35 @@
       </c>
       <c r="E30" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F30" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F30" s="13" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>Brasília - Df</t>
         </is>
       </c>
       <c r="J30" s="14" t="n">
-        <v>46227</v>
+        <v>46240</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>46252</v>
+        <v>46245</v>
       </c>
       <c r="L30" s="15" t="n">
-        <v>286000</v>
+        <v>80000</v>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
@@ -2776,7 +2756,7 @@
       </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
         </is>
       </c>
     </row>
@@ -2788,12 +2768,12 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
@@ -2811,27 +2791,27 @@
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I31" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J31" s="22" t="n">
-        <v>46246</v>
+        <v>46240</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46257</v>
+        <v>46245</v>
       </c>
       <c r="L31" s="23" t="n">
-        <v>54000</v>
+        <v>80000</v>
       </c>
       <c r="M31" s="17" t="inlineStr">
         <is>
@@ -2845,7 +2825,7 @@
       </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
         </is>
       </c>
     </row>
@@ -2857,12 +2837,12 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
@@ -2880,27 +2860,27 @@
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I32" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J32" s="14" t="n">
-        <v>46246</v>
+        <v>46240</v>
       </c>
       <c r="K32" s="14" t="n">
-        <v>46257</v>
+        <v>46245</v>
       </c>
       <c r="L32" s="15" t="n">
-        <v>54000</v>
+        <v>100000</v>
       </c>
       <c r="M32" s="9" t="inlineStr">
         <is>
@@ -2914,7 +2894,7 @@
       </c>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
         </is>
       </c>
     </row>
@@ -2926,12 +2906,12 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
@@ -2941,37 +2921,37 @@
       </c>
       <c r="E33" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F33" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F33" s="21" t="inlineStr"/>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
         </is>
       </c>
       <c r="J33" s="22" t="n">
-        <v>46246</v>
+        <v>46227</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L33" s="23" t="inlineStr"/>
+        <v>46252</v>
+      </c>
+      <c r="L33" s="23" t="n">
+        <v>286000</v>
+      </c>
       <c r="M33" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N33" s="20" t="inlineStr">
@@ -2981,7 +2961,7 @@
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
@@ -2993,17 +2973,17 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E34" s="12" t="inlineStr">
@@ -3012,35 +2992,33 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J34" s="14" t="n">
-        <v>46251</v>
+        <v>46246</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46256</v>
-      </c>
-      <c r="L34" s="15" t="n">
-        <v>50000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L34" s="15" t="inlineStr"/>
       <c r="M34" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N34" s="12" t="inlineStr">
@@ -3050,7 +3028,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -3062,12 +3040,12 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
@@ -3085,7 +3063,7 @@
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
@@ -3095,17 +3073,17 @@
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46252</v>
+        <v>46246</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46259</v>
+        <v>46257</v>
       </c>
       <c r="L35" s="23" t="n">
-        <v>60000</v>
+        <v>54000</v>
       </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
@@ -3119,7 +3097,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -3131,12 +3109,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -3154,7 +3132,7 @@
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
@@ -3171,14 +3149,14 @@
         <v>46246</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46272</v>
+        <v>46257</v>
       </c>
       <c r="L36" s="15" t="n">
         <v>54000</v>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N36" s="12" t="inlineStr">
@@ -3188,7 +3166,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -3200,22 +3178,22 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E37" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F37" s="21" t="n">
@@ -3223,27 +3201,27 @@
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46265</v>
+        <v>46252</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46270</v>
+        <v>46259</v>
       </c>
       <c r="L37" s="23" t="n">
-        <v>30000</v>
+        <v>60000</v>
       </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
@@ -3257,7 +3235,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -3269,17 +3247,17 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E38" s="12" t="inlineStr">
@@ -3292,41 +3270,41 @@
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46208</v>
+        <v>46251</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46259</v>
+        <v>46256</v>
       </c>
       <c r="L38" s="15" t="n">
-        <v>500000</v>
+        <v>50000</v>
       </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N38" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -3338,12 +3316,12 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
@@ -3357,11 +3335,11 @@
         </is>
       </c>
       <c r="F39" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
@@ -3371,29 +3349,31 @@
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46278</v>
+        <v>46246</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46283</v>
-      </c>
-      <c r="L39" s="23" t="inlineStr"/>
+        <v>46272</v>
+      </c>
+      <c r="L39" s="23" t="n">
+        <v>54000</v>
+      </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N39" s="20" t="inlineStr">
         <is>
-          <t>ugp@educacao.sp.gov.br</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -3405,17 +3385,17 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E40" s="12" t="inlineStr">
@@ -3428,41 +3408,41 @@
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46266</v>
+        <v>46208</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46283</v>
+        <v>46259</v>
       </c>
       <c r="L40" s="15" t="n">
-        <v>70000</v>
+        <v>500000</v>
       </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N40" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -3474,22 +3454,22 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E41" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F41" s="21" t="n">
@@ -3497,7 +3477,7 @@
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
@@ -3507,17 +3487,17 @@
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46275</v>
+        <v>46265</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46280</v>
+        <v>46270</v>
       </c>
       <c r="L41" s="23" t="n">
-        <v>50000</v>
+        <v>30000</v>
       </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
@@ -3531,7 +3511,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -3543,12 +3523,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3562,11 +3542,11 @@
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
@@ -3576,16 +3556,18 @@
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
         <v>46275</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46281</v>
-      </c>
-      <c r="L42" s="15" t="inlineStr"/>
+        <v>46280</v>
+      </c>
+      <c r="L42" s="15" t="n">
+        <v>50000</v>
+      </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3598,7 +3580,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
@@ -3610,17 +3592,17 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E43" s="20" t="inlineStr">
@@ -3633,41 +3615,41 @@
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46244</v>
+        <v>46266</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46296</v>
+        <v>46283</v>
       </c>
       <c r="L43" s="23" t="n">
-        <v>935000</v>
+        <v>70000</v>
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N43" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
@@ -3679,17 +3661,17 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E44" s="12" t="inlineStr">
@@ -3698,45 +3680,43 @@
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46244</v>
+        <v>46278</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46300</v>
-      </c>
-      <c r="L44" s="15" t="n">
-        <v>350000</v>
-      </c>
+        <v>46283</v>
+      </c>
+      <c r="L44" s="15" t="inlineStr"/>
       <c r="M44" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N44" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>ugp@educacao.sp.gov.br</t>
         </is>
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
         </is>
       </c>
     </row>
@@ -3748,69 +3728,343 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
+        </is>
+      </c>
+      <c r="C45" s="19" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
+        </is>
+      </c>
+      <c r="D45" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E45" s="20" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F45" s="21" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G45" s="19" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+        </is>
+      </c>
+      <c r="H45" s="19" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I45" s="19" t="inlineStr">
+        <is>
+          <t>Porto Alegre - RS</t>
+        </is>
+      </c>
+      <c r="J45" s="22" t="n">
+        <v>46275</v>
+      </c>
+      <c r="K45" s="22" t="n">
+        <v>46281</v>
+      </c>
+      <c r="L45" s="23" t="inlineStr"/>
+      <c r="M45" s="17" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N45" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O45" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="9" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B46" s="10" t="inlineStr">
+        <is>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+        </is>
+      </c>
+      <c r="C46" s="11" t="inlineStr">
+        <is>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+        </is>
+      </c>
+      <c r="D46" s="11" t="inlineStr">
+        <is>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+        </is>
+      </c>
+      <c r="E46" s="12" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F46" s="13" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G46" s="11" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+        </is>
+      </c>
+      <c r="H46" s="11" t="inlineStr">
+        <is>
+          <t>OEI/MDHC</t>
+        </is>
+      </c>
+      <c r="I46" s="11" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="J46" s="14" t="n">
+        <v>46244</v>
+      </c>
+      <c r="K46" s="14" t="n">
+        <v>46296</v>
+      </c>
+      <c r="L46" s="15" t="n">
+        <v>935000</v>
+      </c>
+      <c r="M46" s="9" t="inlineStr">
+        <is>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N46" s="12" t="inlineStr">
+        <is>
+          <t>compras.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O46" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B47" s="18" t="inlineStr">
+        <is>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+        </is>
+      </c>
+      <c r="C47" s="19" t="inlineStr">
+        <is>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+        </is>
+      </c>
+      <c r="D47" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+        </is>
+      </c>
+      <c r="E47" s="20" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F47" s="21" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G47" s="19" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+        </is>
+      </c>
+      <c r="H47" s="19" t="inlineStr">
+        <is>
+          <t>OEI/MDHC</t>
+        </is>
+      </c>
+      <c r="I47" s="19" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="J47" s="22" t="n">
+        <v>46244</v>
+      </c>
+      <c r="K47" s="22" t="n">
+        <v>46300</v>
+      </c>
+      <c r="L47" s="23" t="n">
+        <v>350000</v>
+      </c>
+      <c r="M47" s="17" t="inlineStr">
+        <is>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N47" s="20" t="inlineStr">
+        <is>
+          <t>compras.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O47" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="9" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B48" s="10" t="inlineStr">
+        <is>
           <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
         </is>
       </c>
-      <c r="C45" s="19" t="inlineStr">
+      <c r="C48" s="11" t="inlineStr">
         <is>
           <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
         </is>
       </c>
-      <c r="D45" s="19" t="inlineStr">
+      <c r="D48" s="11" t="inlineStr">
         <is>
           <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
-      <c r="E45" s="20" t="inlineStr">
+      <c r="E48" s="12" t="inlineStr">
         <is>
           <t>Analista Powerbi</t>
         </is>
       </c>
-      <c r="F45" s="21" t="n">
+      <c r="F48" s="13" t="n">
         <v>0.4</v>
       </c>
-      <c r="G45" s="19" t="inlineStr">
+      <c r="G48" s="11" t="inlineStr">
         <is>
           <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
-      <c r="H45" s="19" t="inlineStr">
+      <c r="H48" s="11" t="inlineStr">
         <is>
           <t>OEI</t>
         </is>
       </c>
-      <c r="I45" s="19" t="inlineStr">
+      <c r="I48" s="11" t="inlineStr">
         <is>
           <t>Dados Remoto</t>
         </is>
       </c>
-      <c r="J45" s="22" t="n">
+      <c r="J48" s="14" t="n">
         <v>46281</v>
       </c>
-      <c r="K45" s="22" t="n">
+      <c r="K48" s="14" t="n">
         <v>46286</v>
       </c>
-      <c r="L45" s="23" t="n">
+      <c r="L48" s="15" t="n">
         <v>110000</v>
       </c>
-      <c r="M45" s="17" t="inlineStr">
+      <c r="M48" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
         </is>
       </c>
-      <c r="N45" s="20" t="inlineStr">
+      <c r="N48" s="12" t="inlineStr">
         <is>
           <t>selecao.bra@oei.int</t>
         </is>
       </c>
-      <c r="O45" s="24" t="inlineStr">
+      <c r="O48" s="16" t="inlineStr">
         <is>
           <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B49" s="18" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
+        </is>
+      </c>
+      <c r="C49" s="19" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
+        </is>
+      </c>
+      <c r="D49" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E49" s="20" t="inlineStr">
+        <is>
+          <t>Economista</t>
+        </is>
+      </c>
+      <c r="F49" s="21" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G49" s="19" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+        </is>
+      </c>
+      <c r="H49" s="19" t="inlineStr">
+        <is>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I49" s="19" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="J49" s="22" t="n">
+        <v>46282</v>
+      </c>
+      <c r="K49" s="22" t="n">
+        <v>46286</v>
+      </c>
+      <c r="L49" s="23" t="n">
+        <v>30000</v>
+      </c>
+      <c r="M49" s="17" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N49" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O49" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O45"/>
+  <autoFilter ref="A1:O49"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -3856,6 +4110,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId48"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -3904,7 +4162,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4">
@@ -3914,7 +4172,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -3956,7 +4214,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3">
@@ -3976,7 +4234,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -4018,7 +4276,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3">
@@ -4028,7 +4286,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
@@ -4064,7 +4322,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4090,7 +4348,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3">
@@ -4100,7 +4358,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4">
@@ -4110,7 +4368,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5">
@@ -4120,7 +4378,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6">
@@ -4150,11 +4408,21 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>Saúde</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B8"/>
+  <autoFilter ref="A1:B9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -4212,7 +4480,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
@@ -4232,7 +4500,7 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -4252,7 +4520,7 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -4300,7 +4568,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -4315,7 +4583,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -4330,7 +4598,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
@@ -4345,7 +4613,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-09-18 16:00
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$51</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 17/09/2026 às 16:18</t>
+          <t>Gerado em 18/09/2026 às 15:54</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="24">
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="25">
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O49"/>
+  <dimension ref="A1:O51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1473,11 +1473,11 @@
         </is>
       </c>
       <c r="B11" s="18" t="n">
-        <v>146386</v>
+        <v>146384</v>
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>BRA/25/024 - Edital nº 08/2026 – Contratação de 6 (seis) consultorias especializadas (pessoa física) para revisão, consolidação, simplificação e otimização de atos normativos trabalhistas infralegais no Brasil</t>
+          <t>Edital 05/2026 - Estudos e análises para o fortalecimento da perspectiva de gênero nas políticas públicas de direitos humanos</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
@@ -1495,27 +1495,27 @@
       </c>
       <c r="G11" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Saúde, Direito / Jurídico</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H11" s="19" t="inlineStr">
         <is>
-          <t>MTE</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I11" s="19" t="inlineStr">
         <is>
-          <t>Híbrido, com eventuais reuniões presenciais em Brasília/DF</t>
+          <t>Território Nacional</t>
         </is>
       </c>
       <c r="J11" s="22" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="K11" s="22" t="n">
-        <v>46292</v>
+        <v>46296</v>
       </c>
       <c r="L11" s="23" t="n">
-        <v>92520</v>
+        <v>120000</v>
       </c>
       <c r="M11" s="17" t="inlineStr">
         <is>
@@ -1524,7 +1524,7 @@
       </c>
       <c r="N11" s="20" t="inlineStr">
         <is>
-          <t>processoseletivo.sat@trabalho.gov.br</t>
+          <t>dirp@mdh.gov.br</t>
         </is>
       </c>
       <c r="O11" s="24" t="inlineStr">
@@ -1540,16 +1540,16 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>146390</v>
+        <v>146386</v>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>BRA/24/018 - CONTRATAÇÃO DE CONSULTOR ESPECIALIZADO EM POLÍTICA DE INOVAÇÃO E DE TRANSFORMAÇÃO DIGITAL</t>
+          <t>BRA/25/024 - Edital nº 08/2026 – Contratação de 6 (seis) consultorias especializadas (pessoa física) para revisão, consolidação, simplificação e otimização de atos normativos trabalhistas infralegais no Brasil</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E12" s="12" t="inlineStr">
@@ -1562,27 +1562,27 @@
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Saúde, Direito / Jurídico</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>MTE</t>
         </is>
       </c>
       <c r="I12" s="11" t="inlineStr">
         <is>
-          <t>Salvador/BA</t>
+          <t>Híbrido, com eventuais reuniões presenciais em Brasília/DF</t>
         </is>
       </c>
       <c r="J12" s="14" t="n">
         <v>46282</v>
       </c>
       <c r="K12" s="14" t="n">
-        <v>46296</v>
+        <v>46292</v>
       </c>
       <c r="L12" s="15" t="n">
-        <v>49580</v>
+        <v>92520</v>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
@@ -1591,7 +1591,7 @@
       </c>
       <c r="N12" s="12" t="inlineStr">
         <is>
-          <t>selecaopnud0326@pge.ba.gov.br</t>
+          <t>processoseletivo.sat@trabalho.gov.br</t>
         </is>
       </c>
       <c r="O12" s="16" t="inlineStr">
@@ -1603,22 +1603,20 @@
     <row r="13">
       <c r="A13" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B13" s="18" t="inlineStr">
-        <is>
-          <t>unesco:7863ef0f-6e11-4770-df18-08df01dbdf45</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B13" s="18" t="n">
+        <v>146390</v>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 51/2026 - 3 vagas - Consultor Individual - REPUBLICAÇÃO</t>
+          <t>BRA/24/018 - CONTRATAÇÃO DE CONSULTOR ESPECIALIZADO EM POLÍTICA DE INOVAÇÃO E DE TRANSFORMAÇÃO DIGITAL</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E13" s="20" t="inlineStr">
@@ -1631,31 +1629,41 @@
       </c>
       <c r="G13" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H13" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I13" s="19" t="inlineStr"/>
+          <t>Não identificado</t>
+        </is>
+      </c>
+      <c r="I13" s="19" t="inlineStr">
+        <is>
+          <t>Salvador/BA</t>
+        </is>
+      </c>
       <c r="J13" s="22" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="K13" s="22" t="n">
-        <v>46286</v>
-      </c>
-      <c r="L13" s="23" t="inlineStr"/>
+        <v>46296</v>
+      </c>
+      <c r="L13" s="23" t="n">
+        <v>49580</v>
+      </c>
       <c r="M13" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N13" s="20" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N13" s="20" t="inlineStr">
+        <is>
+          <t>selecaopnud0326@pge.ba.gov.br</t>
+        </is>
+      </c>
       <c r="O13" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
@@ -1667,12 +1675,12 @@
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>unesco:c9020343-9d28-49e3-b9e3-08df0436270c</t>
+          <t>unesco:7863ef0f-6e11-4770-df18-08df01dbdf45</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 52/2026 - 1 vaga - Consultor Individual - REPUBLICAÇÃO</t>
+          <t>914BRZ1155 - EDITAL Nº 51/2026 - 3 vagas - Consultor Individual - REPUBLICAÇÃO</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -1690,7 +1698,7 @@
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
@@ -1700,7 +1708,7 @@
       </c>
       <c r="I14" s="11" t="inlineStr"/>
       <c r="J14" s="14" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="K14" s="14" t="n">
         <v>46286</v>
@@ -1726,12 +1734,12 @@
       </c>
       <c r="B15" s="18" t="inlineStr">
         <is>
-          <t>unesco:6f0bebf7-7be2-4b29-17c5-08df04786cdd</t>
+          <t>unesco:c9020343-9d28-49e3-b9e3-08df0436270c</t>
         </is>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 53/2026 - 1 vaga - Consultor Individual - REPUBLICAÇÃO</t>
+          <t>914BRZ1155 - EDITAL Nº 52/2026 - 1 vaga - Consultor Individual - REPUBLICAÇÃO</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
@@ -1749,7 +1757,7 @@
       </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H15" s="19" t="inlineStr">
@@ -1785,12 +1793,12 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>unesco:34a61630-55f8-4262-9489-08df0f3a2d32</t>
+          <t>unesco:6f0bebf7-7be2-4b29-17c5-08df04786cdd</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1156 - edital 08/2026 - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 53/2026 - 1 vaga - Consultor Individual - REPUBLICAÇÃO</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -1808,7 +1816,7 @@
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
@@ -1821,7 +1829,7 @@
         <v>46282</v>
       </c>
       <c r="K16" s="14" t="n">
-        <v>46289</v>
+        <v>46286</v>
       </c>
       <c r="L16" s="15" t="inlineStr"/>
       <c r="M16" s="9" t="inlineStr">
@@ -1844,12 +1852,12 @@
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>unesco:5907e744-d46d-4c01-2eaf-08df08e94b75</t>
+          <t>unesco:3622350f-775c-4cc9-9b64-08df0ff5ff21</t>
         </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 37/2026 - 2 vagas - Consultor Individual</t>
+          <t xml:space="preserve"> 914BRZ1166 - Edital nº 01.2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1859,15 +1867,13 @@
       </c>
       <c r="E17" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F17" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F17" s="21" t="inlineStr"/>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
@@ -1877,10 +1883,10 @@
       </c>
       <c r="I17" s="19" t="inlineStr"/>
       <c r="J17" s="22" t="n">
-        <v>46277</v>
+        <v>46283</v>
       </c>
       <c r="K17" s="22" t="n">
-        <v>46283</v>
+        <v>46288</v>
       </c>
       <c r="L17" s="23" t="inlineStr"/>
       <c r="M17" s="17" t="inlineStr">
@@ -1903,12 +1909,12 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>unesco:1011b77e-9c7a-4ea9-2632-08df0e687345</t>
+          <t>unesco:34a61630-55f8-4262-9489-08df0f3a2d32</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 39/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1156 - edital 08/2026 - Consultor Individual</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -1926,7 +1932,7 @@
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -1936,10 +1942,10 @@
       </c>
       <c r="I18" s="11" t="inlineStr"/>
       <c r="J18" s="14" t="n">
-        <v>46279</v>
+        <v>46282</v>
       </c>
       <c r="K18" s="14" t="n">
-        <v>46283</v>
+        <v>46289</v>
       </c>
       <c r="L18" s="15" t="inlineStr"/>
       <c r="M18" s="9" t="inlineStr">
@@ -1962,12 +1968,12 @@
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>unesco:030ad7b8-d33f-491a-31d9-08defb16c1ac</t>
+          <t>unesco:5907e744-d46d-4c01-2eaf-08df08e94b75</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ5067 - Edital Nº 08/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1159 - Publicação Edital 37/2026 - 2 vagas - Consultor Individual</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
@@ -1995,7 +2001,7 @@
       </c>
       <c r="I19" s="19" t="inlineStr"/>
       <c r="J19" s="22" t="n">
-        <v>46253</v>
+        <v>46277</v>
       </c>
       <c r="K19" s="22" t="n">
         <v>46283</v>
@@ -2021,12 +2027,12 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>unesco:a42aa3e1-2e33-46e6-2633-08df0e687345</t>
+          <t>unesco:1011b77e-9c7a-4ea9-2632-08df0e687345</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 38/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1159 - Publicação Edital 39/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -2044,7 +2050,7 @@
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
@@ -2075,17 +2081,17 @@
     <row r="21">
       <c r="A21" s="17" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077</t>
+          <t>unesco:030ad7b8-d33f-491a-31d9-08defb16c1ac</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/16/002 – TR13077</t>
+          <t>Projeto 914BRZ5067 - Edital Nº 08/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
@@ -2099,67 +2105,57 @@
         </is>
       </c>
       <c r="F21" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G21" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I21" s="19" t="inlineStr">
-        <is>
-          <t>Brasília - DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I21" s="19" t="inlineStr"/>
       <c r="J21" s="22" t="n">
-        <v>46223</v>
+        <v>46253</v>
       </c>
       <c r="K21" s="22" t="n">
-        <v>46238</v>
-      </c>
-      <c r="L21" s="23" t="n">
-        <v>100000</v>
-      </c>
+        <v>46283</v>
+      </c>
+      <c r="L21" s="23" t="inlineStr"/>
       <c r="M21" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N21" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N21" s="20" t="inlineStr"/>
       <c r="O21" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
+          <t>unesco:a42aa3e1-2e33-46e6-2633-08df0e687345</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
+          <t>914BRZ1159 - Publicação Edital 38/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E22" s="12" t="inlineStr">
@@ -2168,45 +2164,35 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I22" s="11" t="inlineStr">
-        <is>
-          <t>Recife - PE</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I22" s="11" t="inlineStr"/>
       <c r="J22" s="14" t="n">
-        <v>46225</v>
+        <v>46279</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46229</v>
-      </c>
-      <c r="L22" s="15" t="n">
-        <v>114600</v>
-      </c>
+        <v>46283</v>
+      </c>
+      <c r="L22" s="15" t="inlineStr"/>
       <c r="M22" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N22" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N22" s="12" t="inlineStr"/>
       <c r="O22" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
@@ -2218,17 +2204,17 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/16/002 – TR13077</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E23" s="20" t="inlineStr">
@@ -2241,27 +2227,27 @@
       </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I23" s="19" t="inlineStr">
         <is>
-          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J23" s="22" t="n">
-        <v>46224</v>
+        <v>46223</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46233</v>
+        <v>46238</v>
       </c>
       <c r="L23" s="23" t="n">
-        <v>288000</v>
+        <v>100000</v>
       </c>
       <c r="M23" s="17" t="inlineStr">
         <is>
@@ -2275,7 +2261,7 @@
       </c>
       <c r="O23" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077/</t>
         </is>
       </c>
     </row>
@@ -2287,12 +2273,12 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -2310,7 +2296,7 @@
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
@@ -2320,21 +2306,21 @@
       </c>
       <c r="I24" s="11" t="inlineStr">
         <is>
-          <t>Brasília DF</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J24" s="14" t="n">
-        <v>46227</v>
+        <v>46225</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46231</v>
+        <v>46229</v>
       </c>
       <c r="L24" s="15" t="n">
-        <v>150000</v>
+        <v>114600</v>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N24" s="12" t="inlineStr">
@@ -2344,7 +2330,7 @@
       </c>
       <c r="O24" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
         </is>
       </c>
     </row>
@@ -2356,17 +2342,17 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E25" s="20" t="inlineStr">
@@ -2375,35 +2361,35 @@
         </is>
       </c>
       <c r="F25" s="21" t="n">
-        <v>0.343</v>
+        <v>0.4</v>
       </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I25" s="19" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Brasília DF</t>
         </is>
       </c>
       <c r="J25" s="22" t="n">
-        <v>46232</v>
+        <v>46227</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46238</v>
+        <v>46231</v>
       </c>
       <c r="L25" s="23" t="n">
-        <v>30000</v>
+        <v>150000</v>
       </c>
       <c r="M25" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N25" s="20" t="inlineStr">
@@ -2413,7 +2399,7 @@
       </c>
       <c r="O25" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
         </is>
       </c>
     </row>
@@ -2425,12 +2411,12 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -2440,13 +2426,15 @@
       </c>
       <c r="E26" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F26" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F26" s="13" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
@@ -2456,17 +2444,17 @@
       </c>
       <c r="I26" s="11" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
         </is>
       </c>
       <c r="J26" s="14" t="n">
-        <v>46232</v>
+        <v>46224</v>
       </c>
       <c r="K26" s="14" t="n">
-        <v>46238</v>
+        <v>46233</v>
       </c>
       <c r="L26" s="15" t="n">
-        <v>30000</v>
+        <v>288000</v>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
@@ -2480,7 +2468,7 @@
       </c>
       <c r="O26" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
         </is>
       </c>
     </row>
@@ -2492,17 +2480,17 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E27" s="20" t="inlineStr">
@@ -2511,11 +2499,11 @@
         </is>
       </c>
       <c r="F27" s="21" t="n">
-        <v>0.4</v>
+        <v>0.343</v>
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
@@ -2525,17 +2513,17 @@
       </c>
       <c r="I27" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J27" s="22" t="n">
-        <v>46240</v>
+        <v>46232</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46245</v>
+        <v>46238</v>
       </c>
       <c r="L27" s="23" t="n">
-        <v>204000</v>
+        <v>30000</v>
       </c>
       <c r="M27" s="17" t="inlineStr">
         <is>
@@ -2549,7 +2537,7 @@
       </c>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
         </is>
       </c>
     </row>
@@ -2630,12 +2618,12 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
@@ -2653,7 +2641,7 @@
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
@@ -2687,7 +2675,7 @@
       </c>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
         </is>
       </c>
     </row>
@@ -2699,12 +2687,12 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
@@ -2722,7 +2710,7 @@
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
@@ -2732,7 +2720,7 @@
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>Brasília - Df</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J30" s="14" t="n">
@@ -2756,7 +2744,7 @@
       </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
         </is>
       </c>
     </row>
@@ -2768,12 +2756,12 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
@@ -2783,15 +2771,13 @@
       </c>
       <c r="E31" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F31" s="21" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F31" s="21" t="inlineStr"/>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
@@ -2801,17 +2787,17 @@
       </c>
       <c r="I31" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J31" s="22" t="n">
-        <v>46240</v>
+        <v>46232</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46245</v>
+        <v>46238</v>
       </c>
       <c r="L31" s="23" t="n">
-        <v>80000</v>
+        <v>30000</v>
       </c>
       <c r="M31" s="17" t="inlineStr">
         <is>
@@ -2825,7 +2811,7 @@
       </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
         </is>
       </c>
     </row>
@@ -2837,12 +2823,12 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
@@ -2860,7 +2846,7 @@
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
@@ -2880,7 +2866,7 @@
         <v>46245</v>
       </c>
       <c r="L32" s="15" t="n">
-        <v>100000</v>
+        <v>204000</v>
       </c>
       <c r="M32" s="9" t="inlineStr">
         <is>
@@ -2894,7 +2880,7 @@
       </c>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
         </is>
       </c>
     </row>
@@ -2906,12 +2892,12 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
@@ -2921,33 +2907,35 @@
       </c>
       <c r="E33" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F33" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F33" s="21" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>Brasília - Df</t>
         </is>
       </c>
       <c r="J33" s="22" t="n">
-        <v>46227</v>
+        <v>46240</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46252</v>
+        <v>46245</v>
       </c>
       <c r="L33" s="23" t="n">
-        <v>286000</v>
+        <v>80000</v>
       </c>
       <c r="M33" s="17" t="inlineStr">
         <is>
@@ -2961,7 +2949,7 @@
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
         </is>
       </c>
     </row>
@@ -3040,12 +3028,12 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
@@ -3063,27 +3051,27 @@
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46246</v>
+        <v>46240</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46257</v>
+        <v>46245</v>
       </c>
       <c r="L35" s="23" t="n">
-        <v>54000</v>
+        <v>100000</v>
       </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
@@ -3097,7 +3085,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
         </is>
       </c>
     </row>
@@ -3109,12 +3097,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -3124,15 +3112,13 @@
       </c>
       <c r="E36" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F36" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F36" s="13" t="inlineStr"/>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
@@ -3142,17 +3128,17 @@
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46246</v>
+        <v>46227</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46257</v>
+        <v>46252</v>
       </c>
       <c r="L36" s="15" t="n">
-        <v>54000</v>
+        <v>286000</v>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
@@ -3166,7 +3152,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
@@ -3178,12 +3164,12 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
@@ -3201,7 +3187,7 @@
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
@@ -3211,17 +3197,17 @@
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46252</v>
+        <v>46246</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46259</v>
+        <v>46257</v>
       </c>
       <c r="L37" s="23" t="n">
-        <v>60000</v>
+        <v>54000</v>
       </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
@@ -3235,7 +3221,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -3247,17 +3233,17 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E38" s="12" t="inlineStr">
@@ -3270,7 +3256,7 @@
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
@@ -3280,17 +3266,17 @@
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46251</v>
+        <v>46246</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="L38" s="15" t="n">
-        <v>50000</v>
+        <v>54000</v>
       </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
@@ -3304,7 +3290,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -3316,17 +3302,17 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E39" s="20" t="inlineStr">
@@ -3339,7 +3325,7 @@
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
@@ -3349,21 +3335,21 @@
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46246</v>
+        <v>46251</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46272</v>
+        <v>46256</v>
       </c>
       <c r="L39" s="23" t="n">
-        <v>54000</v>
+        <v>50000</v>
       </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N39" s="20" t="inlineStr">
@@ -3373,7 +3359,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -3385,17 +3371,17 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E40" s="12" t="inlineStr">
@@ -3413,36 +3399,36 @@
       </c>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46208</v>
+        <v>46252</v>
       </c>
       <c r="K40" s="14" t="n">
         <v>46259</v>
       </c>
       <c r="L40" s="15" t="n">
-        <v>500000</v>
+        <v>60000</v>
       </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N40" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -3454,22 +3440,22 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E41" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F41" s="21" t="n">
@@ -3477,41 +3463,41 @@
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46265</v>
+        <v>46208</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46270</v>
+        <v>46259</v>
       </c>
       <c r="L41" s="23" t="n">
-        <v>30000</v>
+        <v>500000</v>
       </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N41" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -3523,12 +3509,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3546,31 +3532,31 @@
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46275</v>
+        <v>46246</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46280</v>
+        <v>46272</v>
       </c>
       <c r="L42" s="15" t="n">
-        <v>50000</v>
+        <v>54000</v>
       </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N42" s="12" t="inlineStr">
@@ -3580,7 +3566,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -3592,22 +3578,22 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E43" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F43" s="21" t="n">
@@ -3615,27 +3601,27 @@
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46283</v>
+        <v>46270</v>
       </c>
       <c r="L43" s="23" t="n">
-        <v>70000</v>
+        <v>30000</v>
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
@@ -3649,7 +3635,7 @@
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -3661,12 +3647,12 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
@@ -3680,43 +3666,45 @@
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46278</v>
+        <v>46275</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46283</v>
-      </c>
-      <c r="L44" s="15" t="inlineStr"/>
+        <v>46280</v>
+      </c>
+      <c r="L44" s="15" t="n">
+        <v>50000</v>
+      </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N44" s="12" t="inlineStr">
         <is>
-          <t>ugp@educacao.sp.gov.br</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
@@ -3728,12 +3716,12 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
@@ -3747,30 +3735,32 @@
         </is>
       </c>
       <c r="F45" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46275</v>
+        <v>46266</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46281</v>
-      </c>
-      <c r="L45" s="23" t="inlineStr"/>
+        <v>46283</v>
+      </c>
+      <c r="L45" s="23" t="n">
+        <v>70000</v>
+      </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3783,7 +3773,7 @@
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
@@ -3795,17 +3785,17 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E46" s="12" t="inlineStr">
@@ -3814,45 +3804,43 @@
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J46" s="14" t="n">
-        <v>46244</v>
+        <v>46278</v>
       </c>
       <c r="K46" s="14" t="n">
-        <v>46296</v>
-      </c>
-      <c r="L46" s="15" t="n">
-        <v>935000</v>
-      </c>
+        <v>46283</v>
+      </c>
+      <c r="L46" s="15" t="inlineStr"/>
       <c r="M46" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N46" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>ugp@educacao.sp.gov.br</t>
         </is>
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
         </is>
       </c>
     </row>
@@ -3864,12 +3852,12 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
@@ -3904,10 +3892,10 @@
         <v>46244</v>
       </c>
       <c r="K47" s="22" t="n">
-        <v>46300</v>
+        <v>46296</v>
       </c>
       <c r="L47" s="23" t="n">
-        <v>350000</v>
+        <v>935000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
@@ -3921,7 +3909,7 @@
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -3933,17 +3921,17 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E48" s="12" t="inlineStr">
@@ -3952,11 +3940,11 @@
         </is>
       </c>
       <c r="F48" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
@@ -3966,18 +3954,16 @@
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>Dados Remoto</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J48" s="14" t="n">
+        <v>46275</v>
+      </c>
+      <c r="K48" s="14" t="n">
         <v>46281</v>
       </c>
-      <c r="K48" s="14" t="n">
-        <v>46286</v>
-      </c>
-      <c r="L48" s="15" t="n">
-        <v>110000</v>
-      </c>
+      <c r="L48" s="15" t="inlineStr"/>
       <c r="M48" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3990,7 +3976,7 @@
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
         </is>
       </c>
     </row>
@@ -4002,22 +3988,22 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E49" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F49" s="21" t="n">
@@ -4025,46 +4011,184 @@
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Dados Remoto</t>
         </is>
       </c>
       <c r="J49" s="22" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="K49" s="22" t="n">
         <v>46286</v>
       </c>
       <c r="L49" s="23" t="n">
+        <v>110000</v>
+      </c>
+      <c r="M49" s="17" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N49" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O49" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="9" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B50" s="10" t="inlineStr">
+        <is>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+        </is>
+      </c>
+      <c r="C50" s="11" t="inlineStr">
+        <is>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+        </is>
+      </c>
+      <c r="D50" s="11" t="inlineStr">
+        <is>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+        </is>
+      </c>
+      <c r="E50" s="12" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F50" s="13" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G50" s="11" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+        </is>
+      </c>
+      <c r="H50" s="11" t="inlineStr">
+        <is>
+          <t>OEI/MDHC</t>
+        </is>
+      </c>
+      <c r="I50" s="11" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="J50" s="14" t="n">
+        <v>46244</v>
+      </c>
+      <c r="K50" s="14" t="n">
+        <v>46300</v>
+      </c>
+      <c r="L50" s="15" t="n">
+        <v>350000</v>
+      </c>
+      <c r="M50" s="9" t="inlineStr">
+        <is>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N50" s="12" t="inlineStr">
+        <is>
+          <t>compras.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O50" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B51" s="18" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
+        </is>
+      </c>
+      <c r="C51" s="19" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
+        </is>
+      </c>
+      <c r="D51" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E51" s="20" t="inlineStr">
+        <is>
+          <t>Economista</t>
+        </is>
+      </c>
+      <c r="F51" s="21" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G51" s="19" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+        </is>
+      </c>
+      <c r="H51" s="19" t="inlineStr">
+        <is>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I51" s="19" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="J51" s="22" t="n">
+        <v>46282</v>
+      </c>
+      <c r="K51" s="22" t="n">
+        <v>46286</v>
+      </c>
+      <c r="L51" s="23" t="n">
         <v>30000</v>
       </c>
-      <c r="M49" s="17" t="inlineStr">
+      <c r="M51" s="17" t="inlineStr">
         <is>
           <t>En evaluación</t>
         </is>
       </c>
-      <c r="N49" s="20" t="inlineStr">
+      <c r="N51" s="20" t="inlineStr">
         <is>
           <t>selecao.bra@oei.int</t>
         </is>
       </c>
-      <c r="O49" s="24" t="inlineStr">
+      <c r="O51" s="24" t="inlineStr">
         <is>
           <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O49"/>
+  <autoFilter ref="A1:O51"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -4114,6 +4238,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId47"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId50"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -4162,7 +4288,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4">
@@ -4172,7 +4298,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -4214,7 +4340,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3">
@@ -4224,7 +4350,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -4272,21 +4398,21 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4">
@@ -4348,7 +4474,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3">
@@ -4358,7 +4484,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4">
@@ -4368,7 +4494,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5">
@@ -4388,7 +4514,7 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
@@ -4480,7 +4606,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
@@ -4506,7 +4632,7 @@
     <row r="7">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="B7" s="18" t="n">
@@ -4516,11 +4642,11 @@
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -4568,7 +4694,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -4583,7 +4709,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -4598,7 +4724,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
@@ -4613,7 +4739,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-09-20 15:37
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$47</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 18/09/2026 às 15:54</t>
+          <t>Gerado em 20/09/2026 às 15:31</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6">
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>165446.1538461538</v>
+        <v>168064</v>
       </c>
     </row>
     <row r="20">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>100000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>43</v>
+        <v>38</v>
       </c>
     </row>
     <row r="24">
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25">
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O51"/>
+  <dimension ref="A1:O47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -876,48 +876,48 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>146353</v>
+        <v>146369</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
-          <t>TR - Mobilização Territorial/2026 - Suporte técnico especializado para Avaliação de Efetividade e Metodologias para Mobilização Territorial e Acesso a Instrumentos de Desenvolvimento</t>
+          <t>Edital nº 29/2026 – Contratação de Consultoria Individual para o desenho institucional da Secretaria de Serviços Compartilhados (SSC/MGI)</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E2" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F2" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F2" s="13" t="inlineStr"/>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H2" s="11" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>MGI</t>
         </is>
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>Região Centro Oeste</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J2" s="14" t="n">
-        <v>46273</v>
+        <v>46276</v>
       </c>
       <c r="K2" s="14" t="n">
-        <v>46283</v>
-      </c>
-      <c r="L2" s="15" t="inlineStr"/>
+        <v>46290</v>
+      </c>
+      <c r="L2" s="15" t="n">
+        <v>120000</v>
+      </c>
       <c r="M2" s="9" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -925,7 +925,7 @@
       </c>
       <c r="N2" s="12" t="inlineStr">
         <is>
-          <t>prodocbra23018@sudeco.gov.br</t>
+          <t>prodoc.mgi@gestao.gov.br</t>
         </is>
       </c>
       <c r="O2" s="16" t="inlineStr">
@@ -941,11 +941,11 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>146369</v>
+        <v>146370</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
-          <t>Edital nº 29/2026 – Contratação de Consultoria Individual para o desenho institucional da Secretaria de Serviços Compartilhados (SSC/MGI)</t>
+          <t xml:space="preserve">Edital nº 25/2026 – Contratação de Consultoria Individual para avaliar os efeitos de intervenções comportamentais (políticas fiscais e de arquitetura de escolha) em mercado experimental para promover escolhas alimentares mais saudáveis. </t>
         </is>
       </c>
       <c r="D3" s="19" t="inlineStr">
@@ -971,7 +971,7 @@
       </c>
       <c r="I3" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>REMOTO</t>
         </is>
       </c>
       <c r="J3" s="22" t="n">
@@ -981,7 +981,7 @@
         <v>46290</v>
       </c>
       <c r="L3" s="23" t="n">
-        <v>120000</v>
+        <v>126000</v>
       </c>
       <c r="M3" s="17" t="inlineStr">
         <is>
@@ -1006,11 +1006,11 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>146370</v>
+        <v>146373</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edital nº 25/2026 – Contratação de Consultoria Individual para avaliar os efeitos de intervenções comportamentais (políticas fiscais e de arquitetura de escolha) em mercado experimental para promover escolhas alimentares mais saudáveis. </t>
+          <t xml:space="preserve">Edital nº 26/2026 – Contratação de Consultoria Individual para aprimoramento de soluções analíticas e computacionais aplicadas ao Modelo de Mensuração de Custos da Digitalização de Serviços Públicos </t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
@@ -1020,13 +1020,15 @@
       </c>
       <c r="E4" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F4" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F4" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H4" s="11" t="inlineStr">
@@ -1036,17 +1038,17 @@
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>REMOTO</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J4" s="14" t="n">
-        <v>46276</v>
+        <v>46280</v>
       </c>
       <c r="K4" s="14" t="n">
-        <v>46290</v>
+        <v>46295</v>
       </c>
       <c r="L4" s="15" t="n">
-        <v>126000</v>
+        <v>108000</v>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
@@ -1071,11 +1073,11 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>146373</v>
+        <v>146360</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edital nº 26/2026 – Contratação de Consultoria Individual para aprimoramento de soluções analíticas e computacionais aplicadas ao Modelo de Mensuração de Custos da Digitalização de Serviços Públicos </t>
+          <t>PNUD BRA/25/024 - Edital nº 04/2026 – Contrat. de consult. - Engenharia de Dados</t>
         </is>
       </c>
       <c r="D5" s="19" t="inlineStr">
@@ -1093,27 +1095,27 @@
       </c>
       <c r="G5" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H5" s="19" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>MTE</t>
         </is>
       </c>
       <c r="I5" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J5" s="22" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="K5" s="22" t="n">
-        <v>46295</v>
+        <v>46287</v>
       </c>
       <c r="L5" s="23" t="n">
-        <v>108000</v>
+        <v>130000</v>
       </c>
       <c r="M5" s="17" t="inlineStr">
         <is>
@@ -1122,7 +1124,7 @@
       </c>
       <c r="N5" s="20" t="inlineStr">
         <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
+          <t>estatisticastrabalho@trabalho.gov.br</t>
         </is>
       </c>
       <c r="O5" s="24" t="inlineStr">
@@ -1138,11 +1140,11 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>146360</v>
+        <v>146361</v>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>PNUD BRA/25/024 - Edital nº 04/2026 – Contrat. de consult. - Engenharia de Dados</t>
+          <t>PNUD BRA/25/024 - Consultoria Especializada - Qualidade de Dados I</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
@@ -1205,11 +1207,11 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>146361</v>
+        <v>146362</v>
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t>PNUD BRA/25/024 - Consultoria Especializada - Qualidade de Dados I</t>
+          <t>PNUD BRA/25/024 - Edital nº 06/2026 - Consultoria Especializada - Qualidade de Dados II</t>
         </is>
       </c>
       <c r="D7" s="19" t="inlineStr">
@@ -1272,11 +1274,11 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>146362</v>
+        <v>146374</v>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>PNUD BRA/25/024 - Edital nº 06/2026 - Consultoria Especializada - Qualidade de Dados II</t>
+          <t>Edital nº 27/2026 – Contratação de Consultoria Individual II - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Servidões de Passagem para Orlas e Praias</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
@@ -1294,27 +1296,27 @@
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H8" s="11" t="inlineStr">
         <is>
-          <t>MTE</t>
+          <t>MGI</t>
         </is>
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J8" s="14" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="K8" s="14" t="n">
-        <v>46287</v>
+        <v>46295</v>
       </c>
       <c r="L8" s="15" t="n">
-        <v>130000</v>
+        <v>120000</v>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
@@ -1323,7 +1325,7 @@
       </c>
       <c r="N8" s="12" t="inlineStr">
         <is>
-          <t>estatisticastrabalho@trabalho.gov.br</t>
+          <t>prodoc.mgi@gestao.gov.br</t>
         </is>
       </c>
       <c r="O8" s="16" t="inlineStr">
@@ -1339,11 +1341,11 @@
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>146374</v>
+        <v>146375</v>
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>Edital nº 27/2026 – Contratação de Consultoria Individual II - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Servidões de Passagem para Orlas e Praias</t>
+          <t>Edital nº 28/2026 - Contratação de Consultoria Individual I - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Acessibilidade em Orlas e Praias</t>
         </is>
       </c>
       <c r="D9" s="19" t="inlineStr">
@@ -1371,7 +1373,7 @@
       </c>
       <c r="I9" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>REMOTO</t>
         </is>
       </c>
       <c r="J9" s="22" t="n">
@@ -1406,11 +1408,11 @@
         </is>
       </c>
       <c r="B10" s="10" t="n">
-        <v>146375</v>
+        <v>146384</v>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>Edital nº 28/2026 - Contratação de Consultoria Individual I - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Acessibilidade em Orlas e Praias</t>
+          <t>Edital 05/2026 - Estudos e análises para o fortalecimento da perspectiva de gênero nas políticas públicas de direitos humanos</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
@@ -1428,24 +1430,24 @@
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I10" s="11" t="inlineStr">
         <is>
-          <t>REMOTO</t>
+          <t>Território Nacional</t>
         </is>
       </c>
       <c r="J10" s="14" t="n">
-        <v>46280</v>
+        <v>46283</v>
       </c>
       <c r="K10" s="14" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="L10" s="15" t="n">
         <v>120000</v>
@@ -1457,7 +1459,7 @@
       </c>
       <c r="N10" s="12" t="inlineStr">
         <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
+          <t>dirp@mdh.gov.br</t>
         </is>
       </c>
       <c r="O10" s="16" t="inlineStr">
@@ -1473,11 +1475,11 @@
         </is>
       </c>
       <c r="B11" s="18" t="n">
-        <v>146384</v>
+        <v>146386</v>
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>Edital 05/2026 - Estudos e análises para o fortalecimento da perspectiva de gênero nas políticas públicas de direitos humanos</t>
+          <t>BRA/25/024 - Edital nº 08/2026 – Contratação de 6 (seis) consultorias especializadas (pessoa física) para revisão, consolidação, simplificação e otimização de atos normativos trabalhistas infralegais no Brasil</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
@@ -1495,27 +1497,27 @@
       </c>
       <c r="G11" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Saúde, Direito / Jurídico</t>
         </is>
       </c>
       <c r="H11" s="19" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>MTE</t>
         </is>
       </c>
       <c r="I11" s="19" t="inlineStr">
         <is>
-          <t>Território Nacional</t>
+          <t>Híbrido, com eventuais reuniões presenciais em Brasília/DF</t>
         </is>
       </c>
       <c r="J11" s="22" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="K11" s="22" t="n">
-        <v>46296</v>
+        <v>46292</v>
       </c>
       <c r="L11" s="23" t="n">
-        <v>120000</v>
+        <v>92520</v>
       </c>
       <c r="M11" s="17" t="inlineStr">
         <is>
@@ -1524,7 +1526,7 @@
       </c>
       <c r="N11" s="20" t="inlineStr">
         <is>
-          <t>dirp@mdh.gov.br</t>
+          <t>processoseletivo.sat@trabalho.gov.br</t>
         </is>
       </c>
       <c r="O11" s="24" t="inlineStr">
@@ -1540,16 +1542,16 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>146386</v>
+        <v>146390</v>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>BRA/25/024 - Edital nº 08/2026 – Contratação de 6 (seis) consultorias especializadas (pessoa física) para revisão, consolidação, simplificação e otimização de atos normativos trabalhistas infralegais no Brasil</t>
+          <t>BRA/24/018 - CONTRATAÇÃO DE CONSULTOR ESPECIALIZADO EM POLÍTICA DE INOVAÇÃO E DE TRANSFORMAÇÃO DIGITAL</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E12" s="12" t="inlineStr">
@@ -1562,27 +1564,27 @@
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Saúde, Direito / Jurídico</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>MTE</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I12" s="11" t="inlineStr">
         <is>
-          <t>Híbrido, com eventuais reuniões presenciais em Brasília/DF</t>
+          <t>Salvador/BA</t>
         </is>
       </c>
       <c r="J12" s="14" t="n">
         <v>46282</v>
       </c>
       <c r="K12" s="14" t="n">
-        <v>46292</v>
+        <v>46296</v>
       </c>
       <c r="L12" s="15" t="n">
-        <v>92520</v>
+        <v>49580</v>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
@@ -1591,7 +1593,7 @@
       </c>
       <c r="N12" s="12" t="inlineStr">
         <is>
-          <t>processoseletivo.sat@trabalho.gov.br</t>
+          <t>selecaopnud0326@pge.ba.gov.br</t>
         </is>
       </c>
       <c r="O12" s="16" t="inlineStr">
@@ -1603,20 +1605,22 @@
     <row r="13">
       <c r="A13" s="17" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B13" s="18" t="n">
-        <v>146390</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>unesco:7863ef0f-6e11-4770-df18-08df01dbdf45</t>
+        </is>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>BRA/24/018 - CONTRATAÇÃO DE CONSULTOR ESPECIALIZADO EM POLÍTICA DE INOVAÇÃO E DE TRANSFORMAÇÃO DIGITAL</t>
+          <t>914BRZ1155 - EDITAL Nº 51/2026 - 3 vagas - Consultor Individual - REPUBLICAÇÃO</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E13" s="20" t="inlineStr">
@@ -1629,41 +1633,31 @@
       </c>
       <c r="G13" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H13" s="19" t="inlineStr">
         <is>
-          <t>Não identificado</t>
-        </is>
-      </c>
-      <c r="I13" s="19" t="inlineStr">
-        <is>
-          <t>Salvador/BA</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I13" s="19" t="inlineStr"/>
       <c r="J13" s="22" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="K13" s="22" t="n">
-        <v>46296</v>
-      </c>
-      <c r="L13" s="23" t="n">
-        <v>49580</v>
-      </c>
+        <v>46286</v>
+      </c>
+      <c r="L13" s="23" t="inlineStr"/>
       <c r="M13" s="17" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N13" s="20" t="inlineStr">
-        <is>
-          <t>selecaopnud0326@pge.ba.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N13" s="20" t="inlineStr"/>
       <c r="O13" s="24" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
@@ -1675,12 +1669,12 @@
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>unesco:7863ef0f-6e11-4770-df18-08df01dbdf45</t>
+          <t>unesco:c9020343-9d28-49e3-b9e3-08df0436270c</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 51/2026 - 3 vagas - Consultor Individual - REPUBLICAÇÃO</t>
+          <t>914BRZ1155 - EDITAL Nº 52/2026 - 1 vaga - Consultor Individual - REPUBLICAÇÃO</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -1698,7 +1692,7 @@
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
@@ -1708,7 +1702,7 @@
       </c>
       <c r="I14" s="11" t="inlineStr"/>
       <c r="J14" s="14" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="K14" s="14" t="n">
         <v>46286</v>
@@ -1734,12 +1728,12 @@
       </c>
       <c r="B15" s="18" t="inlineStr">
         <is>
-          <t>unesco:c9020343-9d28-49e3-b9e3-08df0436270c</t>
+          <t>unesco:6f0bebf7-7be2-4b29-17c5-08df04786cdd</t>
         </is>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 52/2026 - 1 vaga - Consultor Individual - REPUBLICAÇÃO</t>
+          <t>914BRZ1155 - EDITAL Nº 53/2026 - 1 vaga - Consultor Individual - REPUBLICAÇÃO</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
@@ -1757,7 +1751,7 @@
       </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H15" s="19" t="inlineStr">
@@ -1793,12 +1787,12 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>unesco:6f0bebf7-7be2-4b29-17c5-08df04786cdd</t>
+          <t>unesco:3622350f-775c-4cc9-9b64-08df0ff5ff21</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 53/2026 - 1 vaga - Consultor Individual - REPUBLICAÇÃO</t>
+          <t xml:space="preserve"> 914BRZ1166 - Edital nº 01.2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -1808,15 +1802,13 @@
       </c>
       <c r="E16" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F16" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F16" s="13" t="inlineStr"/>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
@@ -1826,10 +1818,10 @@
       </c>
       <c r="I16" s="11" t="inlineStr"/>
       <c r="J16" s="14" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="K16" s="14" t="n">
-        <v>46286</v>
+        <v>46288</v>
       </c>
       <c r="L16" s="15" t="inlineStr"/>
       <c r="M16" s="9" t="inlineStr">
@@ -1852,12 +1844,12 @@
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>unesco:3622350f-775c-4cc9-9b64-08df0ff5ff21</t>
+          <t>unesco:34a61630-55f8-4262-9489-08df0f3a2d32</t>
         </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 914BRZ1166 - Edital nº 01.2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ1156 - edital 08/2026 - Consultor Individual</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1867,13 +1859,15 @@
       </c>
       <c r="E17" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F17" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F17" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
@@ -1883,10 +1877,10 @@
       </c>
       <c r="I17" s="19" t="inlineStr"/>
       <c r="J17" s="22" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="K17" s="22" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="L17" s="23" t="inlineStr"/>
       <c r="M17" s="17" t="inlineStr">
@@ -1909,30 +1903,28 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>unesco:34a61630-55f8-4262-9489-08df0f3a2d32</t>
+          <t>unesco:a4685014-44a0-4ec8-9b63-08df0ff5ff21</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1156 - edital 08/2026 - Consultor Individual</t>
+          <t>Projeto 914BRZ3051 - EDITAL 11/2026 (REPUBLICAÇÃO)</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F18" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F18" s="13" t="inlineStr"/>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -1942,10 +1934,10 @@
       </c>
       <c r="I18" s="11" t="inlineStr"/>
       <c r="J18" s="14" t="n">
-        <v>46282</v>
+        <v>46285</v>
       </c>
       <c r="K18" s="14" t="n">
-        <v>46289</v>
+        <v>46292</v>
       </c>
       <c r="L18" s="15" t="inlineStr"/>
       <c r="M18" s="9" t="inlineStr">
@@ -1968,17 +1960,17 @@
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>unesco:5907e744-d46d-4c01-2eaf-08df08e94b75</t>
+          <t>unesco:f0e2f0e3-b50c-4695-6d11-08df126138f3</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 37/2026 - 2 vagas - Consultor Individual</t>
+          <t>Projeto 914BRZ3051 - EDITAL 17/2026 (REPUBLICAÇÃO)</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E19" s="20" t="inlineStr">
@@ -1991,7 +1983,7 @@
       </c>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
@@ -2001,10 +1993,10 @@
       </c>
       <c r="I19" s="19" t="inlineStr"/>
       <c r="J19" s="22" t="n">
-        <v>46277</v>
+        <v>46285</v>
       </c>
       <c r="K19" s="22" t="n">
-        <v>46283</v>
+        <v>46292</v>
       </c>
       <c r="L19" s="23" t="inlineStr"/>
       <c r="M19" s="17" t="inlineStr">
@@ -2022,22 +2014,22 @@
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>unesco:1011b77e-9c7a-4ea9-2632-08df0e687345</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 39/2026 - 1 vaga - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
@@ -2046,57 +2038,67 @@
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I20" s="11" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="inlineStr">
+        <is>
+          <t>Recife - PE</t>
+        </is>
+      </c>
       <c r="J20" s="14" t="n">
-        <v>46279</v>
+        <v>46225</v>
       </c>
       <c r="K20" s="14" t="n">
-        <v>46283</v>
-      </c>
-      <c r="L20" s="15" t="inlineStr"/>
+        <v>46229</v>
+      </c>
+      <c r="L20" s="15" t="n">
+        <v>114600</v>
+      </c>
       <c r="M20" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N20" s="12" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N20" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O20" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>unesco:030ad7b8-d33f-491a-31d9-08defb16c1ac</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ5067 - Edital Nº 08/2026 - 1 vaga - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E21" s="20" t="inlineStr">
@@ -2105,57 +2107,67 @@
         </is>
       </c>
       <c r="F21" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G21" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I21" s="19" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I21" s="19" t="inlineStr">
+        <is>
+          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
+        </is>
+      </c>
       <c r="J21" s="22" t="n">
-        <v>46253</v>
+        <v>46224</v>
       </c>
       <c r="K21" s="22" t="n">
-        <v>46283</v>
-      </c>
-      <c r="L21" s="23" t="inlineStr"/>
+        <v>46233</v>
+      </c>
+      <c r="L21" s="23" t="n">
+        <v>288000</v>
+      </c>
       <c r="M21" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N21" s="20" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N21" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O21" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>unesco:a42aa3e1-2e33-46e6-2633-08df0e687345</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 38/2026 - 1 vaga - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E22" s="12" t="inlineStr">
@@ -2164,35 +2176,45 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I22" s="11" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I22" s="11" t="inlineStr">
+        <is>
+          <t>Brasília DF</t>
+        </is>
+      </c>
       <c r="J22" s="14" t="n">
-        <v>46279</v>
+        <v>46227</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46283</v>
-      </c>
-      <c r="L22" s="15" t="inlineStr"/>
+        <v>46231</v>
+      </c>
+      <c r="L22" s="15" t="n">
+        <v>150000</v>
+      </c>
       <c r="M22" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N22" s="12" t="inlineStr"/>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N22" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O22" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
         </is>
       </c>
     </row>
@@ -2204,12 +2226,12 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/16/002 – TR13077</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
@@ -2223,31 +2245,31 @@
         </is>
       </c>
       <c r="F23" s="21" t="n">
-        <v>0.4</v>
+        <v>0.343</v>
       </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I23" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J23" s="22" t="n">
-        <v>46223</v>
+        <v>46232</v>
       </c>
       <c r="K23" s="22" t="n">
         <v>46238</v>
       </c>
       <c r="L23" s="23" t="n">
-        <v>100000</v>
+        <v>30000</v>
       </c>
       <c r="M23" s="17" t="inlineStr">
         <is>
@@ -2261,7 +2283,7 @@
       </c>
       <c r="O23" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
         </is>
       </c>
     </row>
@@ -2273,12 +2295,12 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -2288,35 +2310,33 @@
       </c>
       <c r="E24" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F24" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F24" s="13" t="inlineStr"/>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I24" s="11" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J24" s="14" t="n">
-        <v>46225</v>
+        <v>46232</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46229</v>
+        <v>46238</v>
       </c>
       <c r="L24" s="15" t="n">
-        <v>114600</v>
+        <v>30000</v>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
@@ -2330,7 +2350,7 @@
       </c>
       <c r="O24" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
         </is>
       </c>
     </row>
@@ -2342,12 +2362,12 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
@@ -2365,7 +2385,7 @@
       </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
@@ -2375,21 +2395,21 @@
       </c>
       <c r="I25" s="19" t="inlineStr">
         <is>
-          <t>Brasília DF</t>
+          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
         </is>
       </c>
       <c r="J25" s="22" t="n">
-        <v>46227</v>
+        <v>46232</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46231</v>
+        <v>46237</v>
       </c>
       <c r="L25" s="23" t="n">
-        <v>150000</v>
+        <v>288000</v>
       </c>
       <c r="M25" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N25" s="20" t="inlineStr">
@@ -2399,7 +2419,7 @@
       </c>
       <c r="O25" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
         </is>
       </c>
     </row>
@@ -2411,12 +2431,12 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -2434,7 +2454,7 @@
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
@@ -2444,17 +2464,17 @@
       </c>
       <c r="I26" s="11" t="inlineStr">
         <is>
-          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J26" s="14" t="n">
-        <v>46224</v>
+        <v>46240</v>
       </c>
       <c r="K26" s="14" t="n">
-        <v>46233</v>
+        <v>46245</v>
       </c>
       <c r="L26" s="15" t="n">
-        <v>288000</v>
+        <v>204000</v>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
@@ -2468,7 +2488,7 @@
       </c>
       <c r="O26" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
         </is>
       </c>
     </row>
@@ -2480,17 +2500,17 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E27" s="20" t="inlineStr">
@@ -2499,11 +2519,11 @@
         </is>
       </c>
       <c r="F27" s="21" t="n">
-        <v>0.343</v>
+        <v>0.4</v>
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
@@ -2513,17 +2533,17 @@
       </c>
       <c r="I27" s="19" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J27" s="22" t="n">
-        <v>46232</v>
+        <v>46240</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46238</v>
+        <v>46245</v>
       </c>
       <c r="L27" s="23" t="n">
-        <v>30000</v>
+        <v>204000</v>
       </c>
       <c r="M27" s="17" t="inlineStr">
         <is>
@@ -2537,7 +2557,7 @@
       </c>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
         </is>
       </c>
     </row>
@@ -2549,12 +2569,12 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
@@ -2572,27 +2592,27 @@
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I28" s="11" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J28" s="14" t="n">
-        <v>46232</v>
+        <v>46240</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46237</v>
+        <v>46245</v>
       </c>
       <c r="L28" s="15" t="n">
-        <v>288000</v>
+        <v>80000</v>
       </c>
       <c r="M28" s="9" t="inlineStr">
         <is>
@@ -2606,7 +2626,7 @@
       </c>
       <c r="O28" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
         </is>
       </c>
     </row>
@@ -2618,12 +2638,12 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
@@ -2651,7 +2671,7 @@
       </c>
       <c r="I29" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Brasília - Df</t>
         </is>
       </c>
       <c r="J29" s="22" t="n">
@@ -2661,7 +2681,7 @@
         <v>46245</v>
       </c>
       <c r="L29" s="23" t="n">
-        <v>204000</v>
+        <v>80000</v>
       </c>
       <c r="M29" s="17" t="inlineStr">
         <is>
@@ -2675,7 +2695,7 @@
       </c>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
         </is>
       </c>
     </row>
@@ -2687,12 +2707,12 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
@@ -2702,35 +2722,33 @@
       </c>
       <c r="E30" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F30" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F30" s="13" t="inlineStr"/>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
         </is>
       </c>
       <c r="J30" s="14" t="n">
-        <v>46240</v>
+        <v>46227</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>46245</v>
+        <v>46252</v>
       </c>
       <c r="L30" s="15" t="n">
-        <v>80000</v>
+        <v>286000</v>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
@@ -2744,7 +2762,7 @@
       </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
@@ -2756,12 +2774,12 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
@@ -2771,13 +2789,15 @@
       </c>
       <c r="E31" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F31" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F31" s="21" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
@@ -2787,17 +2807,17 @@
       </c>
       <c r="I31" s="19" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J31" s="22" t="n">
-        <v>46232</v>
+        <v>46240</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46238</v>
+        <v>46245</v>
       </c>
       <c r="L31" s="23" t="n">
-        <v>30000</v>
+        <v>100000</v>
       </c>
       <c r="M31" s="17" t="inlineStr">
         <is>
@@ -2811,7 +2831,7 @@
       </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
         </is>
       </c>
     </row>
@@ -2823,12 +2843,12 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
@@ -2846,27 +2866,27 @@
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I32" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J32" s="14" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K32" s="14" t="n">
-        <v>46245</v>
+        <v>46257</v>
       </c>
       <c r="L32" s="15" t="n">
-        <v>204000</v>
+        <v>54000</v>
       </c>
       <c r="M32" s="9" t="inlineStr">
         <is>
@@ -2880,7 +2900,7 @@
       </c>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -2892,12 +2912,12 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
@@ -2915,27 +2935,27 @@
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>Brasília - Df</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J33" s="22" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46245</v>
+        <v>46257</v>
       </c>
       <c r="L33" s="23" t="n">
-        <v>80000</v>
+        <v>54000</v>
       </c>
       <c r="M33" s="17" t="inlineStr">
         <is>
@@ -2949,7 +2969,7 @@
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -3028,17 +3048,17 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E35" s="20" t="inlineStr">
@@ -3051,27 +3071,27 @@
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46240</v>
+        <v>46251</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46245</v>
+        <v>46256</v>
       </c>
       <c r="L35" s="23" t="n">
-        <v>100000</v>
+        <v>50000</v>
       </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
@@ -3085,7 +3105,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -3097,12 +3117,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -3112,13 +3132,15 @@
       </c>
       <c r="E36" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F36" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F36" s="13" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
@@ -3128,17 +3150,17 @@
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46227</v>
+        <v>46252</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46252</v>
+        <v>46259</v>
       </c>
       <c r="L36" s="15" t="n">
-        <v>286000</v>
+        <v>60000</v>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
@@ -3152,7 +3174,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -3164,17 +3186,17 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E37" s="20" t="inlineStr">
@@ -3187,41 +3209,41 @@
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46246</v>
+        <v>46208</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46257</v>
+        <v>46259</v>
       </c>
       <c r="L37" s="23" t="n">
-        <v>54000</v>
+        <v>500000</v>
       </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N37" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -3233,22 +3255,22 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E38" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F38" s="13" t="n">
@@ -3256,27 +3278,27 @@
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46246</v>
+        <v>46265</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46257</v>
+        <v>46270</v>
       </c>
       <c r="L38" s="15" t="n">
-        <v>54000</v>
+        <v>30000</v>
       </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
@@ -3290,7 +3312,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -3302,17 +3324,17 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E39" s="20" t="inlineStr">
@@ -3325,7 +3347,7 @@
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
@@ -3335,21 +3357,21 @@
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46251</v>
+        <v>46246</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46256</v>
+        <v>46272</v>
       </c>
       <c r="L39" s="23" t="n">
-        <v>50000</v>
+        <v>54000</v>
       </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N39" s="20" t="inlineStr">
@@ -3359,7 +3381,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -3371,12 +3393,12 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
@@ -3394,27 +3416,27 @@
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46252</v>
+        <v>46275</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46259</v>
+        <v>46280</v>
       </c>
       <c r="L40" s="15" t="n">
-        <v>60000</v>
+        <v>50000</v>
       </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
@@ -3428,7 +3450,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
@@ -3440,17 +3462,17 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E41" s="20" t="inlineStr">
@@ -3463,41 +3485,41 @@
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Dados Remoto</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46208</v>
+        <v>46281</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46259</v>
+        <v>46286</v>
       </c>
       <c r="L41" s="23" t="n">
-        <v>500000</v>
+        <v>110000</v>
       </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N41" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
         </is>
       </c>
     </row>
@@ -3509,12 +3531,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3528,35 +3550,33 @@
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46246</v>
+        <v>46275</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46272</v>
-      </c>
-      <c r="L42" s="15" t="n">
-        <v>54000</v>
-      </c>
+        <v>46281</v>
+      </c>
+      <c r="L42" s="15" t="inlineStr"/>
       <c r="M42" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N42" s="12" t="inlineStr">
@@ -3566,7 +3586,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
         </is>
       </c>
     </row>
@@ -3578,64 +3598,62 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E43" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F43" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46265</v>
+        <v>46278</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46270</v>
-      </c>
-      <c r="L43" s="23" t="n">
-        <v>30000</v>
-      </c>
+        <v>46283</v>
+      </c>
+      <c r="L43" s="23" t="inlineStr"/>
       <c r="M43" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N43" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>ugp@educacao.sp.gov.br</t>
         </is>
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
         </is>
       </c>
     </row>
@@ -3647,17 +3665,17 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E44" s="12" t="inlineStr">
@@ -3670,41 +3688,41 @@
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46275</v>
+        <v>46244</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46280</v>
+        <v>46296</v>
       </c>
       <c r="L44" s="15" t="n">
-        <v>50000</v>
+        <v>935000</v>
       </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N44" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -3716,17 +3734,17 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E45" s="20" t="inlineStr">
@@ -3739,41 +3757,41 @@
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46266</v>
+        <v>46244</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46283</v>
+        <v>46300</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>70000</v>
+        <v>350000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N45" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -3785,12 +3803,12 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -3800,15 +3818,15 @@
       </c>
       <c r="E46" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
@@ -3818,29 +3836,31 @@
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J46" s="14" t="n">
-        <v>46278</v>
+        <v>46282</v>
       </c>
       <c r="K46" s="14" t="n">
-        <v>46283</v>
-      </c>
-      <c r="L46" s="15" t="inlineStr"/>
+        <v>46286</v>
+      </c>
+      <c r="L46" s="15" t="n">
+        <v>30000</v>
+      </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N46" s="12" t="inlineStr">
         <is>
-          <t>ugp@educacao.sp.gov.br</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
         </is>
       </c>
     </row>
@@ -3852,17 +3872,17 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E47" s="20" t="inlineStr">
@@ -3875,320 +3895,46 @@
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J47" s="22" t="n">
-        <v>46244</v>
+        <v>46266</v>
       </c>
       <c r="K47" s="22" t="n">
-        <v>46296</v>
+        <v>46289</v>
       </c>
       <c r="L47" s="23" t="n">
-        <v>935000</v>
+        <v>70000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N47" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="9" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B48" s="10" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
-        </is>
-      </c>
-      <c r="C48" s="11" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
-        </is>
-      </c>
-      <c r="D48" s="11" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E48" s="12" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F48" s="13" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="G48" s="11" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
-        </is>
-      </c>
-      <c r="H48" s="11" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I48" s="11" t="inlineStr">
-        <is>
-          <t>Porto Alegre - RS</t>
-        </is>
-      </c>
-      <c r="J48" s="14" t="n">
-        <v>46275</v>
-      </c>
-      <c r="K48" s="14" t="n">
-        <v>46281</v>
-      </c>
-      <c r="L48" s="15" t="inlineStr"/>
-      <c r="M48" s="9" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N48" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O48" s="16" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="17" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B49" s="18" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
-        </is>
-      </c>
-      <c r="C49" s="19" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
-        </is>
-      </c>
-      <c r="D49" s="19" t="inlineStr">
-        <is>
-          <t>Consultoria Pessoa Física (PF)</t>
-        </is>
-      </c>
-      <c r="E49" s="20" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F49" s="21" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G49" s="19" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
-        </is>
-      </c>
-      <c r="H49" s="19" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I49" s="19" t="inlineStr">
-        <is>
-          <t>Dados Remoto</t>
-        </is>
-      </c>
-      <c r="J49" s="22" t="n">
-        <v>46281</v>
-      </c>
-      <c r="K49" s="22" t="n">
-        <v>46286</v>
-      </c>
-      <c r="L49" s="23" t="n">
-        <v>110000</v>
-      </c>
-      <c r="M49" s="17" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N49" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O49" s="24" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="9" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B50" s="10" t="inlineStr">
-        <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
-        </is>
-      </c>
-      <c r="C50" s="11" t="inlineStr">
-        <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
-        </is>
-      </c>
-      <c r="D50" s="11" t="inlineStr">
-        <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
-        </is>
-      </c>
-      <c r="E50" s="12" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F50" s="13" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G50" s="11" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
-        </is>
-      </c>
-      <c r="H50" s="11" t="inlineStr">
-        <is>
-          <t>OEI/MDHC</t>
-        </is>
-      </c>
-      <c r="I50" s="11" t="inlineStr">
-        <is>
-          <t>Nacional</t>
-        </is>
-      </c>
-      <c r="J50" s="14" t="n">
-        <v>46244</v>
-      </c>
-      <c r="K50" s="14" t="n">
-        <v>46300</v>
-      </c>
-      <c r="L50" s="15" t="n">
-        <v>350000</v>
-      </c>
-      <c r="M50" s="9" t="inlineStr">
-        <is>
-          <t>En fase de apresentação</t>
-        </is>
-      </c>
-      <c r="N50" s="12" t="inlineStr">
-        <is>
-          <t>compras.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O50" s="16" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="17" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B51" s="18" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
-        </is>
-      </c>
-      <c r="C51" s="19" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
-        </is>
-      </c>
-      <c r="D51" s="19" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E51" s="20" t="inlineStr">
-        <is>
-          <t>Economista</t>
-        </is>
-      </c>
-      <c r="F51" s="21" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G51" s="19" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
-        </is>
-      </c>
-      <c r="H51" s="19" t="inlineStr">
-        <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I51" s="19" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="J51" s="22" t="n">
-        <v>46282</v>
-      </c>
-      <c r="K51" s="22" t="n">
-        <v>46286</v>
-      </c>
-      <c r="L51" s="23" t="n">
-        <v>30000</v>
-      </c>
-      <c r="M51" s="17" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N51" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O51" s="24" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O51"/>
+  <autoFilter ref="A1:O47"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -4236,10 +3982,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId50"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -4278,7 +4020,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3">
@@ -4288,7 +4030,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4">
@@ -4298,7 +4040,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -4340,7 +4082,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>43</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3">
@@ -4350,7 +4092,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -4398,27 +4140,27 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="B4" s="10" t="n">
@@ -4428,11 +4170,11 @@
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -4474,7 +4216,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>39</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3">
@@ -4484,7 +4226,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4">
@@ -4494,7 +4236,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5">
@@ -4504,7 +4246,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
@@ -4514,7 +4256,7 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -4582,7 +4324,7 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
@@ -4592,11 +4334,11 @@
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4">
@@ -4606,7 +4348,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5">
@@ -4632,7 +4374,7 @@
     <row r="7">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="B7" s="18" t="n">
@@ -4642,11 +4384,11 @@
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -4694,7 +4436,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -4709,7 +4451,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -4724,7 +4466,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
@@ -4739,7 +4481,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-09-21 18:00
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$52</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 20/09/2026 às 15:31</t>
+          <t>Gerado em 21/09/2026 às 17:55</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>46</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6">
@@ -638,27 +638,27 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>PNUD</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>PNUD</t>
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="17">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>168064</v>
+        <v>170291.6666666667</v>
       </c>
     </row>
     <row r="20">
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="25">
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O47"/>
+  <dimension ref="A1:O52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1787,12 +1787,12 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>unesco:3622350f-775c-4cc9-9b64-08df0ff5ff21</t>
+          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 914BRZ1166 - Edital nº 01.2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -1818,10 +1818,10 @@
       </c>
       <c r="I16" s="11" t="inlineStr"/>
       <c r="J16" s="14" t="n">
-        <v>46283</v>
+        <v>46286</v>
       </c>
       <c r="K16" s="14" t="n">
-        <v>46288</v>
+        <v>46316</v>
       </c>
       <c r="L16" s="15" t="inlineStr"/>
       <c r="M16" s="9" t="inlineStr">
@@ -1844,12 +1844,12 @@
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>unesco:34a61630-55f8-4262-9489-08df0f3a2d32</t>
+          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
         </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1156 - edital 08/2026 - Consultor Individual</t>
+          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1877,10 +1877,10 @@
       </c>
       <c r="I17" s="19" t="inlineStr"/>
       <c r="J17" s="22" t="n">
-        <v>46282</v>
+        <v>46286</v>
       </c>
       <c r="K17" s="22" t="n">
-        <v>46289</v>
+        <v>46316</v>
       </c>
       <c r="L17" s="23" t="inlineStr"/>
       <c r="M17" s="17" t="inlineStr">
@@ -1903,17 +1903,17 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>unesco:a4685014-44a0-4ec8-9b63-08df0ff5ff21</t>
+          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ3051 - EDITAL 11/2026 (REPUBLICAÇÃO)</t>
+          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
@@ -1924,7 +1924,7 @@
       <c r="F18" s="13" t="inlineStr"/>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -1934,10 +1934,10 @@
       </c>
       <c r="I18" s="11" t="inlineStr"/>
       <c r="J18" s="14" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="K18" s="14" t="n">
-        <v>46292</v>
+        <v>46316</v>
       </c>
       <c r="L18" s="15" t="inlineStr"/>
       <c r="M18" s="9" t="inlineStr">
@@ -1960,30 +1960,28 @@
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>unesco:f0e2f0e3-b50c-4695-6d11-08df126138f3</t>
+          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ3051 - EDITAL 17/2026 (REPUBLICAÇÃO)</t>
+          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E19" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F19" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F19" s="21" t="inlineStr"/>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
@@ -1993,10 +1991,10 @@
       </c>
       <c r="I19" s="19" t="inlineStr"/>
       <c r="J19" s="22" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="K19" s="22" t="n">
-        <v>46292</v>
+        <v>46316</v>
       </c>
       <c r="L19" s="23" t="inlineStr"/>
       <c r="M19" s="17" t="inlineStr">
@@ -2014,224 +2012,188 @@
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
+          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
+          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F20" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F20" s="13" t="inlineStr"/>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I20" s="11" t="inlineStr">
-        <is>
-          <t>Recife - PE</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="inlineStr"/>
       <c r="J20" s="14" t="n">
-        <v>46225</v>
+        <v>46286</v>
       </c>
       <c r="K20" s="14" t="n">
-        <v>46229</v>
-      </c>
-      <c r="L20" s="15" t="n">
-        <v>114600</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L20" s="15" t="inlineStr"/>
       <c r="M20" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N20" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N20" s="12" t="inlineStr"/>
       <c r="O20" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="17" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
+          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
+          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E21" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F21" s="21" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F21" s="21" t="inlineStr"/>
       <c r="G21" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I21" s="19" t="inlineStr">
-        <is>
-          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I21" s="19" t="inlineStr"/>
       <c r="J21" s="22" t="n">
-        <v>46224</v>
+        <v>46286</v>
       </c>
       <c r="K21" s="22" t="n">
-        <v>46233</v>
-      </c>
-      <c r="L21" s="23" t="n">
-        <v>288000</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L21" s="23" t="inlineStr"/>
       <c r="M21" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N21" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N21" s="20" t="inlineStr"/>
       <c r="O21" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
+          <t>unesco:3622350f-775c-4cc9-9b64-08df0ff5ff21</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
+          <t xml:space="preserve"> 914BRZ1166 - Edital nº 01.2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F22" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F22" s="13" t="inlineStr"/>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I22" s="11" t="inlineStr">
-        <is>
-          <t>Brasília DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I22" s="11" t="inlineStr"/>
       <c r="J22" s="14" t="n">
-        <v>46227</v>
+        <v>46283</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46231</v>
-      </c>
-      <c r="L22" s="15" t="n">
-        <v>150000</v>
-      </c>
+        <v>46288</v>
+      </c>
+      <c r="L22" s="15" t="inlineStr"/>
       <c r="M22" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
-        </is>
-      </c>
-      <c r="N22" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N22" s="12" t="inlineStr"/>
       <c r="O22" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="17" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
+          <t>unesco:34a61630-55f8-4262-9489-08df0f3a2d32</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
+          <t>914BRZ1156 - edital 08/2026 - Consultor Individual</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
@@ -2245,62 +2207,52 @@
         </is>
       </c>
       <c r="F23" s="21" t="n">
-        <v>0.343</v>
+        <v>0.3</v>
       </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I23" s="19" t="inlineStr">
-        <is>
-          <t>Remoto, Brasília - DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I23" s="19" t="inlineStr"/>
       <c r="J23" s="22" t="n">
-        <v>46232</v>
+        <v>46282</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46238</v>
-      </c>
-      <c r="L23" s="23" t="n">
-        <v>30000</v>
-      </c>
+        <v>46289</v>
+      </c>
+      <c r="L23" s="23" t="inlineStr"/>
       <c r="M23" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N23" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N23" s="20" t="inlineStr"/>
       <c r="O23" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
+          <t>unesco:a4685014-44a0-4ec8-9b63-08df0ff5ff21</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
+          <t>Projeto 914BRZ3051 - EDITAL 11/2026 (REPUBLICAÇÃO)</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -2321,58 +2273,48 @@
       </c>
       <c r="H24" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I24" s="11" t="inlineStr">
-        <is>
-          <t>Remoto, Brasília - DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I24" s="11" t="inlineStr"/>
       <c r="J24" s="14" t="n">
-        <v>46232</v>
+        <v>46285</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46238</v>
-      </c>
-      <c r="L24" s="15" t="n">
-        <v>30000</v>
-      </c>
+        <v>46292</v>
+      </c>
+      <c r="L24" s="15" t="inlineStr"/>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N24" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N24" s="12" t="inlineStr"/>
       <c r="O24" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="17" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
+          <t>unesco:f0e2f0e3-b50c-4695-6d11-08df126138f3</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
+          <t>Projeto 914BRZ3051 - EDITAL 17/2026 (REPUBLICAÇÃO)</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E25" s="20" t="inlineStr">
@@ -2381,45 +2323,35 @@
         </is>
       </c>
       <c r="F25" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I25" s="19" t="inlineStr">
-        <is>
-          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I25" s="19" t="inlineStr"/>
       <c r="J25" s="22" t="n">
-        <v>46232</v>
+        <v>46285</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46237</v>
-      </c>
-      <c r="L25" s="23" t="n">
-        <v>288000</v>
-      </c>
+        <v>46292</v>
+      </c>
+      <c r="L25" s="23" t="inlineStr"/>
       <c r="M25" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N25" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N25" s="20" t="inlineStr"/>
       <c r="O25" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
@@ -2431,12 +2363,12 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -2459,26 +2391,26 @@
       </c>
       <c r="H26" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I26" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Brasília DF</t>
         </is>
       </c>
       <c r="J26" s="14" t="n">
-        <v>46240</v>
+        <v>46227</v>
       </c>
       <c r="K26" s="14" t="n">
-        <v>46245</v>
+        <v>46231</v>
       </c>
       <c r="L26" s="15" t="n">
-        <v>204000</v>
+        <v>150000</v>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N26" s="12" t="inlineStr">
@@ -2488,7 +2420,7 @@
       </c>
       <c r="O26" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
         </is>
       </c>
     </row>
@@ -2500,12 +2432,12 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
@@ -2523,7 +2455,7 @@
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
@@ -2533,17 +2465,17 @@
       </c>
       <c r="I27" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
         </is>
       </c>
       <c r="J27" s="22" t="n">
-        <v>46240</v>
+        <v>46224</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46245</v>
+        <v>46233</v>
       </c>
       <c r="L27" s="23" t="n">
-        <v>204000</v>
+        <v>288000</v>
       </c>
       <c r="M27" s="17" t="inlineStr">
         <is>
@@ -2557,7 +2489,7 @@
       </c>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
         </is>
       </c>
     </row>
@@ -2569,12 +2501,12 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
@@ -2592,27 +2524,27 @@
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I28" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
         </is>
       </c>
       <c r="J28" s="14" t="n">
-        <v>46240</v>
+        <v>46232</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46245</v>
+        <v>46237</v>
       </c>
       <c r="L28" s="15" t="n">
-        <v>80000</v>
+        <v>288000</v>
       </c>
       <c r="M28" s="9" t="inlineStr">
         <is>
@@ -2626,7 +2558,7 @@
       </c>
       <c r="O28" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
         </is>
       </c>
     </row>
@@ -2638,12 +2570,12 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
@@ -2653,15 +2585,13 @@
       </c>
       <c r="E29" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F29" s="21" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F29" s="21" t="inlineStr"/>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
@@ -2671,17 +2601,17 @@
       </c>
       <c r="I29" s="19" t="inlineStr">
         <is>
-          <t>Brasília - Df</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J29" s="22" t="n">
-        <v>46240</v>
+        <v>46232</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46245</v>
+        <v>46238</v>
       </c>
       <c r="L29" s="23" t="n">
-        <v>80000</v>
+        <v>30000</v>
       </c>
       <c r="M29" s="17" t="inlineStr">
         <is>
@@ -2695,7 +2625,7 @@
       </c>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
         </is>
       </c>
     </row>
@@ -2707,12 +2637,12 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
@@ -2722,33 +2652,35 @@
       </c>
       <c r="E30" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F30" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F30" s="13" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J30" s="14" t="n">
-        <v>46227</v>
+        <v>46240</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>46252</v>
+        <v>46245</v>
       </c>
       <c r="L30" s="15" t="n">
-        <v>286000</v>
+        <v>204000</v>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
@@ -2762,7 +2694,7 @@
       </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
         </is>
       </c>
     </row>
@@ -2774,12 +2706,12 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
@@ -2797,7 +2729,7 @@
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
@@ -2817,7 +2749,7 @@
         <v>46245</v>
       </c>
       <c r="L31" s="23" t="n">
-        <v>100000</v>
+        <v>204000</v>
       </c>
       <c r="M31" s="17" t="inlineStr">
         <is>
@@ -2831,7 +2763,7 @@
       </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
         </is>
       </c>
     </row>
@@ -2843,17 +2775,17 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E32" s="12" t="inlineStr">
@@ -2862,31 +2794,31 @@
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.4</v>
+        <v>0.343</v>
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I32" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J32" s="14" t="n">
-        <v>46246</v>
+        <v>46232</v>
       </c>
       <c r="K32" s="14" t="n">
-        <v>46257</v>
+        <v>46238</v>
       </c>
       <c r="L32" s="15" t="n">
-        <v>54000</v>
+        <v>30000</v>
       </c>
       <c r="M32" s="9" t="inlineStr">
         <is>
@@ -2900,7 +2832,7 @@
       </c>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
         </is>
       </c>
     </row>
@@ -2912,12 +2844,12 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
@@ -2935,27 +2867,27 @@
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Brasília - Df</t>
         </is>
       </c>
       <c r="J33" s="22" t="n">
-        <v>46246</v>
+        <v>46240</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46257</v>
+        <v>46245</v>
       </c>
       <c r="L33" s="23" t="n">
-        <v>54000</v>
+        <v>80000</v>
       </c>
       <c r="M33" s="17" t="inlineStr">
         <is>
@@ -2969,7 +2901,7 @@
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
         </is>
       </c>
     </row>
@@ -2981,12 +2913,12 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -3000,7 +2932,7 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
@@ -3014,19 +2946,21 @@
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J34" s="14" t="n">
-        <v>46246</v>
+        <v>46240</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L34" s="15" t="inlineStr"/>
+        <v>46245</v>
+      </c>
+      <c r="L34" s="15" t="n">
+        <v>80000</v>
+      </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N34" s="12" t="inlineStr">
@@ -3036,7 +2970,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
         </is>
       </c>
     </row>
@@ -3048,17 +2982,17 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E35" s="20" t="inlineStr">
@@ -3071,7 +3005,7 @@
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
@@ -3081,17 +3015,17 @@
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46251</v>
+        <v>46246</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="L35" s="23" t="n">
-        <v>50000</v>
+        <v>54000</v>
       </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
@@ -3105,7 +3039,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -3117,12 +3051,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -3132,15 +3066,13 @@
       </c>
       <c r="E36" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F36" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F36" s="13" t="inlineStr"/>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
@@ -3150,17 +3082,17 @@
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
+        <v>46227</v>
+      </c>
+      <c r="K36" s="14" t="n">
         <v>46252</v>
       </c>
-      <c r="K36" s="14" t="n">
-        <v>46259</v>
-      </c>
       <c r="L36" s="15" t="n">
-        <v>60000</v>
+        <v>286000</v>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
@@ -3174,7 +3106,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
@@ -3186,17 +3118,17 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E37" s="20" t="inlineStr">
@@ -3205,45 +3137,43 @@
         </is>
       </c>
       <c r="F37" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46208</v>
+        <v>46246</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46259</v>
-      </c>
-      <c r="L37" s="23" t="n">
-        <v>500000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L37" s="23" t="inlineStr"/>
       <c r="M37" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N37" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -3255,22 +3185,22 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E38" s="12" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F38" s="13" t="n">
@@ -3278,7 +3208,7 @@
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
@@ -3288,17 +3218,17 @@
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46265</v>
+        <v>46240</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46270</v>
+        <v>46245</v>
       </c>
       <c r="L38" s="15" t="n">
-        <v>30000</v>
+        <v>100000</v>
       </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
@@ -3312,7 +3242,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
         </is>
       </c>
     </row>
@@ -3324,12 +3254,12 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
@@ -3347,7 +3277,7 @@
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
@@ -3364,14 +3294,14 @@
         <v>46246</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46272</v>
+        <v>46257</v>
       </c>
       <c r="L39" s="23" t="n">
         <v>54000</v>
       </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N39" s="20" t="inlineStr">
@@ -3381,7 +3311,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -3393,17 +3323,17 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E40" s="12" t="inlineStr">
@@ -3416,24 +3346,24 @@
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46275</v>
+        <v>46251</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46280</v>
+        <v>46256</v>
       </c>
       <c r="L40" s="15" t="n">
         <v>50000</v>
@@ -3450,7 +3380,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -3462,17 +3392,17 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E41" s="20" t="inlineStr">
@@ -3485,27 +3415,27 @@
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Dados Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46281</v>
+        <v>46252</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46286</v>
+        <v>46259</v>
       </c>
       <c r="L41" s="23" t="n">
-        <v>110000</v>
+        <v>60000</v>
       </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
@@ -3519,7 +3449,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -3531,17 +3461,17 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
+          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
+          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E42" s="12" t="inlineStr">
@@ -3550,43 +3480,45 @@
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46275</v>
+        <v>46208</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46281</v>
-      </c>
-      <c r="L42" s="15" t="inlineStr"/>
+        <v>46259</v>
+      </c>
+      <c r="L42" s="15" t="n">
+        <v>500000</v>
+      </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N42" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -3598,12 +3530,12 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
@@ -3617,11 +3549,11 @@
         </is>
       </c>
       <c r="F43" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
@@ -3631,29 +3563,31 @@
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46278</v>
+        <v>46246</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46283</v>
-      </c>
-      <c r="L43" s="23" t="inlineStr"/>
+        <v>46272</v>
+      </c>
+      <c r="L43" s="23" t="n">
+        <v>54000</v>
+      </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N43" s="20" t="inlineStr">
         <is>
-          <t>ugp@educacao.sp.gov.br</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -3665,17 +3599,17 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E44" s="12" t="inlineStr">
@@ -3688,41 +3622,41 @@
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46244</v>
+        <v>46275</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46296</v>
+        <v>46280</v>
       </c>
       <c r="L44" s="15" t="n">
-        <v>935000</v>
+        <v>50000</v>
       </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N44" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
@@ -3734,22 +3668,22 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E45" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F45" s="21" t="n">
@@ -3757,41 +3691,41 @@
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46244</v>
+        <v>46265</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46300</v>
+        <v>46270</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>350000</v>
+        <v>30000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N45" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -3803,12 +3737,12 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -3818,15 +3752,15 @@
       </c>
       <c r="E46" s="12" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
@@ -3836,31 +3770,29 @@
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J46" s="14" t="n">
-        <v>46282</v>
+        <v>46278</v>
       </c>
       <c r="K46" s="14" t="n">
-        <v>46286</v>
-      </c>
-      <c r="L46" s="15" t="n">
-        <v>30000</v>
-      </c>
+        <v>46283</v>
+      </c>
+      <c r="L46" s="15" t="inlineStr"/>
       <c r="M46" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N46" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>ugp@educacao.sp.gov.br</t>
         </is>
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
         </is>
       </c>
     </row>
@@ -3872,69 +3804,412 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
+        </is>
+      </c>
+      <c r="C47" s="19" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
+        </is>
+      </c>
+      <c r="D47" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E47" s="20" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F47" s="21" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G47" s="19" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+        </is>
+      </c>
+      <c r="H47" s="19" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I47" s="19" t="inlineStr">
+        <is>
+          <t>Porto Alegre - RS</t>
+        </is>
+      </c>
+      <c r="J47" s="22" t="n">
+        <v>46275</v>
+      </c>
+      <c r="K47" s="22" t="n">
+        <v>46281</v>
+      </c>
+      <c r="L47" s="23" t="inlineStr"/>
+      <c r="M47" s="17" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N47" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O47" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="9" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B48" s="10" t="inlineStr">
+        <is>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+        </is>
+      </c>
+      <c r="C48" s="11" t="inlineStr">
+        <is>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+        </is>
+      </c>
+      <c r="D48" s="11" t="inlineStr">
+        <is>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+        </is>
+      </c>
+      <c r="E48" s="12" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F48" s="13" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G48" s="11" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+        </is>
+      </c>
+      <c r="H48" s="11" t="inlineStr">
+        <is>
+          <t>OEI/MDHC</t>
+        </is>
+      </c>
+      <c r="I48" s="11" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="J48" s="14" t="n">
+        <v>46244</v>
+      </c>
+      <c r="K48" s="14" t="n">
+        <v>46296</v>
+      </c>
+      <c r="L48" s="15" t="n">
+        <v>935000</v>
+      </c>
+      <c r="M48" s="9" t="inlineStr">
+        <is>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N48" s="12" t="inlineStr">
+        <is>
+          <t>compras.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O48" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B49" s="18" t="inlineStr">
+        <is>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+        </is>
+      </c>
+      <c r="C49" s="19" t="inlineStr">
+        <is>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+        </is>
+      </c>
+      <c r="D49" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+        </is>
+      </c>
+      <c r="E49" s="20" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F49" s="21" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G49" s="19" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+        </is>
+      </c>
+      <c r="H49" s="19" t="inlineStr">
+        <is>
+          <t>OEI/MDHC</t>
+        </is>
+      </c>
+      <c r="I49" s="19" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="J49" s="22" t="n">
+        <v>46244</v>
+      </c>
+      <c r="K49" s="22" t="n">
+        <v>46300</v>
+      </c>
+      <c r="L49" s="23" t="n">
+        <v>350000</v>
+      </c>
+      <c r="M49" s="17" t="inlineStr">
+        <is>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N49" s="20" t="inlineStr">
+        <is>
+          <t>compras.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O49" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="9" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B50" s="10" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
+        </is>
+      </c>
+      <c r="C50" s="11" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
+        </is>
+      </c>
+      <c r="D50" s="11" t="inlineStr">
+        <is>
+          <t>Consultoria Pessoa Física (PF)</t>
+        </is>
+      </c>
+      <c r="E50" s="12" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F50" s="13" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G50" s="11" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+        </is>
+      </c>
+      <c r="H50" s="11" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I50" s="11" t="inlineStr">
+        <is>
+          <t>Dados Remoto</t>
+        </is>
+      </c>
+      <c r="J50" s="14" t="n">
+        <v>46281</v>
+      </c>
+      <c r="K50" s="14" t="n">
+        <v>46286</v>
+      </c>
+      <c r="L50" s="15" t="n">
+        <v>110000</v>
+      </c>
+      <c r="M50" s="9" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N50" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O50" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B51" s="18" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
+        </is>
+      </c>
+      <c r="C51" s="19" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
+        </is>
+      </c>
+      <c r="D51" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E51" s="20" t="inlineStr">
+        <is>
+          <t>Economista</t>
+        </is>
+      </c>
+      <c r="F51" s="21" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G51" s="19" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+        </is>
+      </c>
+      <c r="H51" s="19" t="inlineStr">
+        <is>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I51" s="19" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="J51" s="22" t="n">
+        <v>46282</v>
+      </c>
+      <c r="K51" s="22" t="n">
+        <v>46286</v>
+      </c>
+      <c r="L51" s="23" t="n">
+        <v>30000</v>
+      </c>
+      <c r="M51" s="17" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N51" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O51" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="9" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B52" s="10" t="inlineStr">
+        <is>
           <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
-      <c r="C47" s="19" t="inlineStr">
+      <c r="C52" s="11" t="inlineStr">
         <is>
           <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
-      <c r="D47" s="19" t="inlineStr">
+      <c r="D52" s="11" t="inlineStr">
         <is>
           <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
-      <c r="E47" s="20" t="inlineStr">
+      <c r="E52" s="12" t="inlineStr">
         <is>
           <t>Analista Powerbi</t>
         </is>
       </c>
-      <c r="F47" s="21" t="n">
+      <c r="F52" s="13" t="n">
         <v>0.4</v>
       </c>
-      <c r="G47" s="19" t="inlineStr">
+      <c r="G52" s="11" t="inlineStr">
         <is>
           <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
-      <c r="H47" s="19" t="inlineStr">
+      <c r="H52" s="11" t="inlineStr">
         <is>
           <t>OEI/BRA</t>
         </is>
       </c>
-      <c r="I47" s="19" t="inlineStr">
+      <c r="I52" s="11" t="inlineStr">
         <is>
           <t>São Paulo - SP</t>
         </is>
       </c>
-      <c r="J47" s="22" t="n">
+      <c r="J52" s="14" t="n">
         <v>46266</v>
       </c>
-      <c r="K47" s="22" t="n">
+      <c r="K52" s="14" t="n">
         <v>46289</v>
       </c>
-      <c r="L47" s="23" t="n">
+      <c r="L52" s="15" t="n">
         <v>70000</v>
       </c>
-      <c r="M47" s="17" t="inlineStr">
+      <c r="M52" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
         </is>
       </c>
-      <c r="N47" s="20" t="inlineStr">
+      <c r="N52" s="12" t="inlineStr">
         <is>
           <t>selecao.bra@oei.int</t>
         </is>
       </c>
-      <c r="O47" s="24" t="inlineStr">
+      <c r="O52" s="16" t="inlineStr">
         <is>
           <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O47"/>
+  <autoFilter ref="A1:O52"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -3982,6 +4257,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId51"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -4020,27 +4300,27 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Pnud</t>
+          <t>Unesco</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Unesco</t>
+          <t>Pnud</t>
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -4092,7 +4372,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4">
@@ -4140,21 +4420,21 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
@@ -4242,21 +4522,21 @@
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
-          <t>Meio Ambiente / Clima / Geografia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7">
@@ -4286,7 +4566,7 @@
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -4324,7 +4604,7 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
@@ -4334,21 +4614,21 @@
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
🤖 Daily run: 2026-09-22 16:28
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$55</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -27,7 +27,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Por_Tipo'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Por_Area'!$A$1:$B$9</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Por_Area'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Por_Orgao'!$A$1:$B$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Por_Orgao'!$A$1:$B$9</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Por_Orgao'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Perfis'!$A$1:$C$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'Perfis'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 21/09/2026 às 17:55</t>
+          <t>Gerado em 22/09/2026 às 16:21</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6">
@@ -620,7 +620,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
@@ -644,17 +644,17 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>PNUD</t>
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>PNUD</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B13" s="6" t="n">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row r="17">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>170291.6666666667</v>
+        <v>161372.4137931034</v>
       </c>
     </row>
     <row r="20">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>80000</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="24">
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O52"/>
+  <dimension ref="A1:O55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1542,16 +1542,16 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>146390</v>
+        <v>146380</v>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>BRA/24/018 - CONTRATAÇÃO DE CONSULTOR ESPECIALIZADO EM POLÍTICA DE INOVAÇÃO E DE TRANSFORMAÇÃO DIGITAL</t>
+          <t>PROJETO BRA 23/023 - TR 138/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A PROPOSIÇÃO DE PLATAFORMAS E DASHBOARDS DE VISUALIZAÇÃO DE DADOS PARA A AGENDA DE DESENVOLVIMENTO HUMANO</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E12" s="12" t="inlineStr">
@@ -1560,31 +1560,31 @@
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>IBGE</t>
         </is>
       </c>
       <c r="I12" s="11" t="inlineStr">
         <is>
-          <t>Salvador/BA</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J12" s="14" t="n">
-        <v>46282</v>
+        <v>46287</v>
       </c>
       <c r="K12" s="14" t="n">
         <v>46296</v>
       </c>
       <c r="L12" s="15" t="n">
-        <v>49580</v>
+        <v>126500</v>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
@@ -1593,7 +1593,7 @@
       </c>
       <c r="N12" s="12" t="inlineStr">
         <is>
-          <t>selecaopnud0326@pge.ba.gov.br</t>
+          <t>projetos.especiais@ibge.gov.br</t>
         </is>
       </c>
       <c r="O12" s="16" t="inlineStr">
@@ -1605,17 +1605,15 @@
     <row r="13">
       <c r="A13" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B13" s="18" t="inlineStr">
-        <is>
-          <t>unesco:7863ef0f-6e11-4770-df18-08df01dbdf45</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B13" s="18" t="n">
+        <v>146381</v>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 51/2026 - 3 vagas - Consultor Individual - REPUBLICAÇÃO</t>
+          <t>PROJETO BRA 23/023 - TR 139/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A SISTEMATIZAÇÃO E ELABORAÇÃO DO DOSSIÊ INSTITUCIONAL DA SÉRIE DIÁLOGOS NACIONAIS PARA O DESENVOLVIMENTO.</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
@@ -1629,52 +1627,60 @@
         </is>
       </c>
       <c r="F13" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G13" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H13" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I13" s="19" t="inlineStr"/>
+          <t>IBGE</t>
+        </is>
+      </c>
+      <c r="I13" s="19" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
       <c r="J13" s="22" t="n">
-        <v>46281</v>
+        <v>46287</v>
       </c>
       <c r="K13" s="22" t="n">
-        <v>46286</v>
-      </c>
-      <c r="L13" s="23" t="inlineStr"/>
+        <v>46296</v>
+      </c>
+      <c r="L13" s="23" t="n">
+        <v>126500</v>
+      </c>
       <c r="M13" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N13" s="20" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N13" s="20" t="inlineStr">
+        <is>
+          <t>projetos.especiais@ibge.gov.br</t>
+        </is>
+      </c>
       <c r="O13" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>unesco:c9020343-9d28-49e3-b9e3-08df0436270c</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="n">
+        <v>146383</v>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 52/2026 - 1 vaga - Consultor Individual - REPUBLICAÇÃO</t>
+          <t>PROJETO BRA 23/023 - TR 145/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA DESENVOLVIMENTO DE PROPOSTA DE ALGORITMO DE GEOCODIFICAÇÃO DE ENDEREÇOS BRASILEIROS.</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -1688,57 +1694,65 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I14" s="11" t="inlineStr"/>
+          <t>IBGE</t>
+        </is>
+      </c>
+      <c r="I14" s="11" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
       <c r="J14" s="14" t="n">
-        <v>46282</v>
+        <v>46287</v>
       </c>
       <c r="K14" s="14" t="n">
-        <v>46286</v>
-      </c>
-      <c r="L14" s="15" t="inlineStr"/>
+        <v>46296</v>
+      </c>
+      <c r="L14" s="15" t="n">
+        <v>86800</v>
+      </c>
       <c r="M14" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N14" s="12" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N14" s="12" t="inlineStr">
+        <is>
+          <t>projetos.especiais@ibge.gov.br</t>
+        </is>
+      </c>
       <c r="O14" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B15" s="18" t="inlineStr">
-        <is>
-          <t>unesco:6f0bebf7-7be2-4b29-17c5-08df04786cdd</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="n">
+        <v>146357</v>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 53/2026 - 1 vaga - Consultor Individual - REPUBLICAÇÃO</t>
+          <t>PROJETO BRA 23/023 - TR 141/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE METODOLOGIA DE MODELAGEM PREDITIVA PARA ANÁLISE TERRITORIAL DO DESENVOLVIMENTO HUMANO.</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E15" s="20" t="inlineStr">
@@ -1747,114 +1761,132 @@
         </is>
       </c>
       <c r="F15" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H15" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I15" s="19" t="inlineStr"/>
+          <t>IBGE</t>
+        </is>
+      </c>
+      <c r="I15" s="19" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
       <c r="J15" s="22" t="n">
-        <v>46282</v>
+        <v>46287</v>
       </c>
       <c r="K15" s="22" t="n">
-        <v>46286</v>
-      </c>
-      <c r="L15" s="23" t="inlineStr"/>
+        <v>46296</v>
+      </c>
+      <c r="L15" s="23" t="n">
+        <v>126500</v>
+      </c>
       <c r="M15" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N15" s="20" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N15" s="20" t="inlineStr">
+        <is>
+          <t>projetos.especiais@ibge.gov.br</t>
+        </is>
+      </c>
       <c r="O15" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B16" s="10" t="inlineStr">
-        <is>
-          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="n">
+        <v>146358</v>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
+          <t>PROJETO BRA 23/023 - TR 142/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE METODOLOGIA DE MODELAGEM PREDITIVA COM FOCO NO PROCESSAMENTO E INTEGRAÇÃO DE DADOS GEOESPACIAIS.</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E16" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F16" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F16" s="13" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I16" s="11" t="inlineStr"/>
+          <t>IBGE</t>
+        </is>
+      </c>
+      <c r="I16" s="11" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
       <c r="J16" s="14" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="K16" s="14" t="n">
-        <v>46316</v>
-      </c>
-      <c r="L16" s="15" t="inlineStr"/>
+        <v>46296</v>
+      </c>
+      <c r="L16" s="15" t="n">
+        <v>126500</v>
+      </c>
       <c r="M16" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N16" s="12" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N16" s="12" t="inlineStr">
+        <is>
+          <t>projetos.especiais@ibge.gov.br</t>
+        </is>
+      </c>
       <c r="O16" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B17" s="18" t="inlineStr">
-        <is>
-          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="n">
+        <v>146390</v>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
+          <t>BRA/24/018 - CONTRATAÇÃO DE CONSULTOR ESPECIALIZADO EM POLÍTICA DE INOVAÇÃO E DE TRANSFORMAÇÃO DIGITAL</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E17" s="20" t="inlineStr">
@@ -1872,26 +1904,36 @@
       </c>
       <c r="H17" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I17" s="19" t="inlineStr"/>
+          <t>Não identificado</t>
+        </is>
+      </c>
+      <c r="I17" s="19" t="inlineStr">
+        <is>
+          <t>Salvador/BA</t>
+        </is>
+      </c>
       <c r="J17" s="22" t="n">
-        <v>46286</v>
+        <v>46282</v>
       </c>
       <c r="K17" s="22" t="n">
-        <v>46316</v>
-      </c>
-      <c r="L17" s="23" t="inlineStr"/>
+        <v>46296</v>
+      </c>
+      <c r="L17" s="23" t="n">
+        <v>49580</v>
+      </c>
       <c r="M17" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N17" s="20" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N17" s="20" t="inlineStr">
+        <is>
+          <t>selecaopnud0326@pge.ba.gov.br</t>
+        </is>
+      </c>
       <c r="O17" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
@@ -1903,12 +1945,12 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
+          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
+          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -1924,7 +1966,7 @@
       <c r="F18" s="13" t="inlineStr"/>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -1960,12 +2002,12 @@
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
+          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
+          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
@@ -1975,13 +2017,15 @@
       </c>
       <c r="E19" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F19" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F19" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
@@ -2017,12 +2061,12 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
+          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
+          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -2038,7 +2082,7 @@
       <c r="F20" s="13" t="inlineStr"/>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
@@ -2074,12 +2118,12 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
+          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
+          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
@@ -2131,12 +2175,12 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>unesco:3622350f-775c-4cc9-9b64-08df0ff5ff21</t>
+          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 914BRZ1166 - Edital nº 01.2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -2162,10 +2206,10 @@
       </c>
       <c r="I22" s="11" t="inlineStr"/>
       <c r="J22" s="14" t="n">
-        <v>46283</v>
+        <v>46286</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46288</v>
+        <v>46316</v>
       </c>
       <c r="L22" s="15" t="inlineStr"/>
       <c r="M22" s="9" t="inlineStr">
@@ -2188,12 +2232,12 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>unesco:34a61630-55f8-4262-9489-08df0f3a2d32</t>
+          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1156 - edital 08/2026 - Consultor Individual</t>
+          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
@@ -2203,15 +2247,13 @@
       </c>
       <c r="E23" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F23" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F23" s="21" t="inlineStr"/>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
@@ -2221,10 +2263,10 @@
       </c>
       <c r="I23" s="19" t="inlineStr"/>
       <c r="J23" s="22" t="n">
-        <v>46282</v>
+        <v>46286</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46289</v>
+        <v>46316</v>
       </c>
       <c r="L23" s="23" t="inlineStr"/>
       <c r="M23" s="17" t="inlineStr">
@@ -2247,17 +2289,17 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>unesco:a4685014-44a0-4ec8-9b63-08df0ff5ff21</t>
+          <t>unesco:3622350f-775c-4cc9-9b64-08df0ff5ff21</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ3051 - EDITAL 11/2026 (REPUBLICAÇÃO)</t>
+          <t xml:space="preserve"> 914BRZ1166 - Edital nº 01.2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E24" s="12" t="inlineStr">
@@ -2278,10 +2320,10 @@
       </c>
       <c r="I24" s="11" t="inlineStr"/>
       <c r="J24" s="14" t="n">
-        <v>46285</v>
+        <v>46283</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46292</v>
+        <v>46288</v>
       </c>
       <c r="L24" s="15" t="inlineStr"/>
       <c r="M24" s="9" t="inlineStr">
@@ -2304,17 +2346,17 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>unesco:f0e2f0e3-b50c-4695-6d11-08df126138f3</t>
+          <t>unesco:34a61630-55f8-4262-9489-08df0f3a2d32</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ3051 - EDITAL 17/2026 (REPUBLICAÇÃO)</t>
+          <t>914BRZ1156 - edital 08/2026 - Consultor Individual</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E25" s="20" t="inlineStr">
@@ -2327,7 +2369,7 @@
       </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
@@ -2337,10 +2379,10 @@
       </c>
       <c r="I25" s="19" t="inlineStr"/>
       <c r="J25" s="22" t="n">
-        <v>46285</v>
+        <v>46282</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46292</v>
+        <v>46289</v>
       </c>
       <c r="L25" s="23" t="inlineStr"/>
       <c r="M25" s="17" t="inlineStr">
@@ -2358,17 +2400,17 @@
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
+          <t>unesco:a4685014-44a0-4ec8-9b63-08df0ff5ff21</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
+          <t>Projeto 914BRZ3051 - EDITAL 11/2026 (REPUBLICAÇÃO)</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -2378,71 +2420,59 @@
       </c>
       <c r="E26" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F26" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F26" s="13" t="inlineStr"/>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I26" s="11" t="inlineStr">
-        <is>
-          <t>Brasília DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I26" s="11" t="inlineStr"/>
       <c r="J26" s="14" t="n">
-        <v>46227</v>
+        <v>46285</v>
       </c>
       <c r="K26" s="14" t="n">
-        <v>46231</v>
-      </c>
-      <c r="L26" s="15" t="n">
-        <v>150000</v>
-      </c>
+        <v>46292</v>
+      </c>
+      <c r="L26" s="15" t="inlineStr"/>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
-        </is>
-      </c>
-      <c r="N26" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N26" s="12" t="inlineStr"/>
       <c r="O26" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="17" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
+          <t>unesco:49fa6512-497b-43c7-9b65-08df0ff5ff21</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
+          <t>Projeto 914BRZ1085 - Edital nº 04/2026 - 4 vagas - Consultores Individuais</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E27" s="20" t="inlineStr">
@@ -2451,67 +2481,57 @@
         </is>
       </c>
       <c r="F27" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Saúde</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I27" s="19" t="inlineStr">
-        <is>
-          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I27" s="19" t="inlineStr"/>
       <c r="J27" s="22" t="n">
-        <v>46224</v>
+        <v>46287</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46233</v>
-      </c>
-      <c r="L27" s="23" t="n">
-        <v>288000</v>
-      </c>
+        <v>46292</v>
+      </c>
+      <c r="L27" s="23" t="inlineStr"/>
       <c r="M27" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N27" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N27" s="20" t="inlineStr"/>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
+          <t>unesco:f0e2f0e3-b50c-4695-6d11-08df126138f3</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
+          <t>Projeto 914BRZ3051 - EDITAL 17/2026 (REPUBLICAÇÃO)</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr">
@@ -2520,45 +2540,35 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I28" s="11" t="inlineStr">
-        <is>
-          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I28" s="11" t="inlineStr"/>
       <c r="J28" s="14" t="n">
-        <v>46232</v>
+        <v>46285</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46237</v>
-      </c>
-      <c r="L28" s="15" t="n">
-        <v>288000</v>
-      </c>
+        <v>46292</v>
+      </c>
+      <c r="L28" s="15" t="inlineStr"/>
       <c r="M28" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N28" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N28" s="12" t="inlineStr"/>
       <c r="O28" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
@@ -2570,12 +2580,12 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
@@ -2585,13 +2595,15 @@
       </c>
       <c r="E29" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F29" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F29" s="21" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
@@ -2601,17 +2613,17 @@
       </c>
       <c r="I29" s="19" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
         </is>
       </c>
       <c r="J29" s="22" t="n">
-        <v>46232</v>
+        <v>46224</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46238</v>
+        <v>46233</v>
       </c>
       <c r="L29" s="23" t="n">
-        <v>30000</v>
+        <v>288000</v>
       </c>
       <c r="M29" s="17" t="inlineStr">
         <is>
@@ -2625,7 +2637,7 @@
       </c>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
         </is>
       </c>
     </row>
@@ -2637,12 +2649,12 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
@@ -2660,31 +2672,31 @@
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Brasília DF</t>
         </is>
       </c>
       <c r="J30" s="14" t="n">
-        <v>46240</v>
+        <v>46227</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>46245</v>
+        <v>46231</v>
       </c>
       <c r="L30" s="15" t="n">
-        <v>204000</v>
+        <v>150000</v>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N30" s="12" t="inlineStr">
@@ -2694,7 +2706,7 @@
       </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
         </is>
       </c>
     </row>
@@ -2706,12 +2718,12 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
@@ -2721,15 +2733,13 @@
       </c>
       <c r="E31" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F31" s="21" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F31" s="21" t="inlineStr"/>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
@@ -2739,17 +2749,17 @@
       </c>
       <c r="I31" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J31" s="22" t="n">
-        <v>46240</v>
+        <v>46232</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46245</v>
+        <v>46238</v>
       </c>
       <c r="L31" s="23" t="n">
-        <v>204000</v>
+        <v>30000</v>
       </c>
       <c r="M31" s="17" t="inlineStr">
         <is>
@@ -2763,7 +2773,7 @@
       </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
         </is>
       </c>
     </row>
@@ -2844,12 +2854,12 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
@@ -2877,7 +2887,7 @@
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>Brasília - Df</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J33" s="22" t="n">
@@ -2887,7 +2897,7 @@
         <v>46245</v>
       </c>
       <c r="L33" s="23" t="n">
-        <v>80000</v>
+        <v>204000</v>
       </c>
       <c r="M33" s="17" t="inlineStr">
         <is>
@@ -2901,7 +2911,7 @@
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
         </is>
       </c>
     </row>
@@ -2913,12 +2923,12 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -2936,27 +2946,27 @@
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
         </is>
       </c>
       <c r="J34" s="14" t="n">
-        <v>46240</v>
+        <v>46232</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46245</v>
+        <v>46237</v>
       </c>
       <c r="L34" s="15" t="n">
-        <v>80000</v>
+        <v>288000</v>
       </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
@@ -2970,7 +2980,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
         </is>
       </c>
     </row>
@@ -2982,12 +2992,12 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
@@ -3005,27 +3015,27 @@
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46246</v>
+        <v>46240</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46257</v>
+        <v>46245</v>
       </c>
       <c r="L35" s="23" t="n">
-        <v>54000</v>
+        <v>204000</v>
       </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
@@ -3039,7 +3049,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
         </is>
       </c>
     </row>
@@ -3051,12 +3061,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -3066,33 +3076,35 @@
       </c>
       <c r="E36" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F36" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F36" s="13" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46227</v>
+        <v>46240</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46252</v>
+        <v>46245</v>
       </c>
       <c r="L36" s="15" t="n">
-        <v>286000</v>
+        <v>80000</v>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
@@ -3106,7 +3118,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
         </is>
       </c>
     </row>
@@ -3118,12 +3130,12 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
@@ -3137,11 +3149,11 @@
         </is>
       </c>
       <c r="F37" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
@@ -3151,19 +3163,21 @@
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>Brasília - Df</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46246</v>
+        <v>46240</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L37" s="23" t="inlineStr"/>
+        <v>46245</v>
+      </c>
+      <c r="L37" s="23" t="n">
+        <v>80000</v>
+      </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N37" s="20" t="inlineStr">
@@ -3173,7 +3187,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
         </is>
       </c>
     </row>
@@ -3254,12 +3268,12 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
@@ -3273,35 +3287,33 @@
         </is>
       </c>
       <c r="F39" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
         <v>46246</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46257</v>
-      </c>
-      <c r="L39" s="23" t="n">
-        <v>54000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L39" s="23" t="inlineStr"/>
       <c r="M39" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N39" s="20" t="inlineStr">
@@ -3311,7 +3323,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -3323,30 +3335,28 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E40" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F40" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F40" s="13" t="inlineStr"/>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
@@ -3356,17 +3366,17 @@
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46251</v>
+        <v>46227</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46256</v>
+        <v>46252</v>
       </c>
       <c r="L40" s="15" t="n">
-        <v>50000</v>
+        <v>286000</v>
       </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
@@ -3380,7 +3390,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
@@ -3392,12 +3402,12 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
@@ -3415,7 +3425,7 @@
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
@@ -3425,17 +3435,17 @@
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46252</v>
+        <v>46246</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46259</v>
+        <v>46257</v>
       </c>
       <c r="L41" s="23" t="n">
-        <v>60000</v>
+        <v>54000</v>
       </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
@@ -3449,7 +3459,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -3461,17 +3471,17 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E42" s="12" t="inlineStr">
@@ -3484,41 +3494,41 @@
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46208</v>
+        <v>46246</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46259</v>
+        <v>46257</v>
       </c>
       <c r="L42" s="15" t="n">
-        <v>500000</v>
+        <v>54000</v>
       </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N42" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -3530,17 +3540,17 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E43" s="20" t="inlineStr">
@@ -3553,7 +3563,7 @@
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
@@ -3563,21 +3573,21 @@
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46246</v>
+        <v>46251</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46272</v>
+        <v>46256</v>
       </c>
       <c r="L43" s="23" t="n">
-        <v>54000</v>
+        <v>50000</v>
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N43" s="20" t="inlineStr">
@@ -3587,7 +3597,7 @@
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -3599,12 +3609,12 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
@@ -3622,27 +3632,27 @@
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46275</v>
+        <v>46252</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46280</v>
+        <v>46259</v>
       </c>
       <c r="L44" s="15" t="n">
-        <v>50000</v>
+        <v>60000</v>
       </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
@@ -3656,7 +3666,7 @@
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -3668,22 +3678,22 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E45" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F45" s="21" t="n">
@@ -3691,31 +3701,31 @@
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46265</v>
+        <v>46246</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46270</v>
+        <v>46272</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>30000</v>
+        <v>54000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N45" s="20" t="inlineStr">
@@ -3725,7 +3735,7 @@
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -3737,17 +3747,17 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E46" s="12" t="inlineStr">
@@ -3756,30 +3766,32 @@
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J46" s="14" t="n">
-        <v>46278</v>
+        <v>46208</v>
       </c>
       <c r="K46" s="14" t="n">
-        <v>46283</v>
-      </c>
-      <c r="L46" s="15" t="inlineStr"/>
+        <v>46259</v>
+      </c>
+      <c r="L46" s="15" t="n">
+        <v>500000</v>
+      </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
           <t>En presentación</t>
@@ -3787,12 +3799,12 @@
       </c>
       <c r="N46" s="12" t="inlineStr">
         <is>
-          <t>ugp@educacao.sp.gov.br</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -3804,30 +3816,30 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E47" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F47" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
@@ -3837,16 +3849,18 @@
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J47" s="22" t="n">
-        <v>46275</v>
+        <v>46265</v>
       </c>
       <c r="K47" s="22" t="n">
-        <v>46281</v>
-      </c>
-      <c r="L47" s="23" t="inlineStr"/>
+        <v>46270</v>
+      </c>
+      <c r="L47" s="23" t="n">
+        <v>30000</v>
+      </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3859,7 +3873,7 @@
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -3871,17 +3885,17 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E48" s="12" t="inlineStr">
@@ -3894,41 +3908,41 @@
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J48" s="14" t="n">
-        <v>46244</v>
+        <v>46266</v>
       </c>
       <c r="K48" s="14" t="n">
-        <v>46296</v>
+        <v>46288</v>
       </c>
       <c r="L48" s="15" t="n">
-        <v>935000</v>
+        <v>70000</v>
       </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N48" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
@@ -3940,17 +3954,17 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E49" s="20" t="inlineStr">
@@ -3963,41 +3977,41 @@
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J49" s="22" t="n">
-        <v>46244</v>
+        <v>46275</v>
       </c>
       <c r="K49" s="22" t="n">
-        <v>46300</v>
+        <v>46280</v>
       </c>
       <c r="L49" s="23" t="n">
-        <v>350000</v>
+        <v>50000</v>
       </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N49" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
@@ -4009,17 +4023,17 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E50" s="12" t="inlineStr">
@@ -4028,11 +4042,11 @@
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
@@ -4042,18 +4056,16 @@
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>Dados Remoto</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J50" s="14" t="n">
+        <v>46275</v>
+      </c>
+      <c r="K50" s="14" t="n">
         <v>46281</v>
       </c>
-      <c r="K50" s="14" t="n">
-        <v>46286</v>
-      </c>
-      <c r="L50" s="15" t="n">
-        <v>110000</v>
-      </c>
+      <c r="L50" s="15" t="inlineStr"/>
       <c r="M50" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -4066,7 +4078,7 @@
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
         </is>
       </c>
     </row>
@@ -4078,22 +4090,22 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E51" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F51" s="21" t="n">
@@ -4101,41 +4113,41 @@
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
-        <v>46282</v>
+        <v>46244</v>
       </c>
       <c r="K51" s="22" t="n">
-        <v>46286</v>
+        <v>46296</v>
       </c>
       <c r="L51" s="23" t="n">
-        <v>30000</v>
+        <v>935000</v>
       </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N51" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -4147,17 +4159,17 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E52" s="12" t="inlineStr">
@@ -4170,46 +4182,251 @@
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+        </is>
+      </c>
+      <c r="H52" s="11" t="inlineStr">
+        <is>
+          <t>OEI/MDHC</t>
+        </is>
+      </c>
+      <c r="I52" s="11" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="J52" s="14" t="n">
+        <v>46244</v>
+      </c>
+      <c r="K52" s="14" t="n">
+        <v>46300</v>
+      </c>
+      <c r="L52" s="15" t="n">
+        <v>350000</v>
+      </c>
+      <c r="M52" s="9" t="inlineStr">
+        <is>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N52" s="12" t="inlineStr">
+        <is>
+          <t>compras.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O52" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B53" s="18" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
+        </is>
+      </c>
+      <c r="C53" s="19" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
+        </is>
+      </c>
+      <c r="D53" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria Pessoa Física (PF)</t>
+        </is>
+      </c>
+      <c r="E53" s="20" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F53" s="21" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G53" s="19" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+        </is>
+      </c>
+      <c r="H53" s="19" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I53" s="19" t="inlineStr">
+        <is>
+          <t>Dados Remoto</t>
+        </is>
+      </c>
+      <c r="J53" s="22" t="n">
+        <v>46281</v>
+      </c>
+      <c r="K53" s="22" t="n">
+        <v>46286</v>
+      </c>
+      <c r="L53" s="23" t="n">
+        <v>110000</v>
+      </c>
+      <c r="M53" s="17" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N53" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O53" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="9" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B54" s="10" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
+        </is>
+      </c>
+      <c r="C54" s="11" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
+        </is>
+      </c>
+      <c r="D54" s="11" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E54" s="12" t="inlineStr">
+        <is>
+          <t>Economista</t>
+        </is>
+      </c>
+      <c r="F54" s="13" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G54" s="11" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+        </is>
+      </c>
+      <c r="H54" s="11" t="inlineStr">
+        <is>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I54" s="11" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="J54" s="14" t="n">
+        <v>46282</v>
+      </c>
+      <c r="K54" s="14" t="n">
+        <v>46286</v>
+      </c>
+      <c r="L54" s="15" t="n">
+        <v>30000</v>
+      </c>
+      <c r="M54" s="9" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N54" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O54" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B55" s="18" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+        </is>
+      </c>
+      <c r="C55" s="19" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+        </is>
+      </c>
+      <c r="D55" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E55" s="20" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F55" s="21" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G55" s="19" t="inlineStr">
+        <is>
           <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
-      <c r="H52" s="11" t="inlineStr">
+      <c r="H55" s="19" t="inlineStr">
         <is>
           <t>OEI/BRA</t>
         </is>
       </c>
-      <c r="I52" s="11" t="inlineStr">
+      <c r="I55" s="19" t="inlineStr">
         <is>
           <t>São Paulo - SP</t>
         </is>
       </c>
-      <c r="J52" s="14" t="n">
-        <v>46266</v>
-      </c>
-      <c r="K52" s="14" t="n">
+      <c r="J55" s="22" t="n">
+        <v>46278</v>
+      </c>
+      <c r="K55" s="22" t="n">
         <v>46289</v>
       </c>
-      <c r="L52" s="15" t="n">
-        <v>70000</v>
-      </c>
-      <c r="M52" s="9" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N52" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O52" s="16" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+      <c r="L55" s="23" t="inlineStr"/>
+      <c r="M55" s="17" t="inlineStr">
+        <is>
+          <t>En presentación</t>
+        </is>
+      </c>
+      <c r="N55" s="20" t="inlineStr">
+        <is>
+          <t>ugp@educacao.sp.gov.br</t>
+        </is>
+      </c>
+      <c r="O55" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O52"/>
+  <autoFilter ref="A1:O55"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -4262,6 +4479,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId49"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId50"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId54"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -4306,17 +4526,17 @@
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Unesco</t>
+          <t>Pnud</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Pnud</t>
+          <t>Unesco</t>
         </is>
       </c>
       <c r="B4" s="10" t="n">
@@ -4362,7 +4582,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3">
@@ -4444,7 +4664,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5">
@@ -4496,7 +4716,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>34</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3">
@@ -4506,7 +4726,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4">
@@ -4516,7 +4736,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5">
@@ -4536,7 +4756,7 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
@@ -4552,7 +4772,7 @@
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>Direito / Jurídico</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="B8" s="10" t="n">
@@ -4562,7 +4782,7 @@
     <row r="9">
       <c r="A9" s="19" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Direito / Jurídico</t>
         </is>
       </c>
       <c r="B9" s="18" t="n">
@@ -4582,7 +4802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4604,7 +4824,7 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
@@ -4614,11 +4834,11 @@
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4">
@@ -4644,35 +4864,45 @@
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>MTE</t>
+          <t>IBGE</t>
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>MTE</t>
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
+          <t>OEI/MDHC</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
           <t>Não identificado</t>
         </is>
       </c>
-      <c r="B8" s="10" t="n">
+      <c r="B9" s="18" t="n">
         <v>2</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B8"/>
+  <autoFilter ref="A1:B9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -4716,7 +4946,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -4731,7 +4961,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -4746,7 +4976,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
@@ -4761,7 +4991,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-09-25 17:02
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -16,7 +16,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Por_Orgao" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$59</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -566,7 +566,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 24/09/2026 às 16:43</t>
+          <t>Gerado em 25/09/2026 às 17:02</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6">
@@ -641,21 +641,21 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>PNUD</t>
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>PNUD</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -731,7 +731,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -749,7 +749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O56"/>
+  <dimension ref="A1:O59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1759,17 +1759,15 @@
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B16" s="10" t="inlineStr">
-        <is>
-          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="n">
+        <v>146394</v>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
+          <t>Edital nº 30/2026 – Contratação de Consultoria Individual para realizar estudo de caso sobre a Secretaria de Serviços Compartilhados</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -1785,48 +1783,56 @@
       <c r="F16" s="13" t="inlineStr"/>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I16" s="11" t="inlineStr"/>
+          <t>MGI</t>
+        </is>
+      </c>
+      <c r="I16" s="11" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
       <c r="J16" s="14" t="n">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="K16" s="14" t="n">
-        <v>46316</v>
-      </c>
-      <c r="L16" s="15" t="inlineStr"/>
+        <v>46304</v>
+      </c>
+      <c r="L16" s="15" t="n">
+        <v>90000</v>
+      </c>
       <c r="M16" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N16" s="12" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N16" s="12" t="inlineStr">
+        <is>
+          <t>prodoc.mgi@gestao.gov.br</t>
+        </is>
+      </c>
       <c r="O16" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B17" s="18" t="inlineStr">
-        <is>
-          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="n">
+        <v>146396</v>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
+          <t>BRA/25/024 - Edital nº 013/2026 – Contratação de consultoria especializada (pessoa física) para desenvolvimento de estudo e análise sobre os efeitos econômicos e sociais dos recursos mobilizados pelo FAT e pelo FGTS</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1842,31 +1848,41 @@
       <c r="F17" s="21" t="inlineStr"/>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I17" s="19" t="inlineStr"/>
+          <t>MTE</t>
+        </is>
+      </c>
+      <c r="I17" s="19" t="inlineStr">
+        <is>
+          <t>Brasília, com disponibilidade para viagens</t>
+        </is>
+      </c>
       <c r="J17" s="22" t="n">
-        <v>46286</v>
+        <v>46290</v>
       </c>
       <c r="K17" s="22" t="n">
-        <v>46316</v>
-      </c>
-      <c r="L17" s="23" t="inlineStr"/>
+        <v>46303</v>
+      </c>
+      <c r="L17" s="23" t="n">
+        <v>208966.53</v>
+      </c>
       <c r="M17" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N17" s="20" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N17" s="20" t="inlineStr">
+        <is>
+          <t>selecao.spt@trabalho.gov.br</t>
+        </is>
+      </c>
       <c r="O17" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
@@ -1878,12 +1894,12 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
+          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
+          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -1899,7 +1915,7 @@
       <c r="F18" s="13" t="inlineStr"/>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -1935,12 +1951,12 @@
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
+          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
+          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
@@ -1956,7 +1972,7 @@
       <c r="F19" s="21" t="inlineStr"/>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
@@ -1992,12 +2008,12 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
+          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
+          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -2013,7 +2029,7 @@
       <c r="F20" s="13" t="inlineStr"/>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
@@ -2049,12 +2065,12 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
+          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
+          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
@@ -2106,12 +2122,12 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>unesco:6277cc83-3d55-4575-091b-08df172a76c5</t>
+          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>14BRZ1163 - Publicação -  Edital 69/2026 - 01 Vaga consultor Individual</t>
+          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -2127,7 +2143,7 @@
       <c r="F22" s="13" t="inlineStr"/>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
@@ -2137,10 +2153,10 @@
       </c>
       <c r="I22" s="11" t="inlineStr"/>
       <c r="J22" s="14" t="n">
-        <v>46289</v>
+        <v>46286</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46294</v>
+        <v>46316</v>
       </c>
       <c r="L22" s="15" t="inlineStr"/>
       <c r="M22" s="9" t="inlineStr">
@@ -2163,12 +2179,12 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>unesco:6c8e0acd-2d12-4dc7-e28e-08df14acbbca</t>
+          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1102- Edital nº 36/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
@@ -2194,10 +2210,10 @@
       </c>
       <c r="I23" s="19" t="inlineStr"/>
       <c r="J23" s="22" t="n">
-        <v>46289</v>
+        <v>46286</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46293</v>
+        <v>46316</v>
       </c>
       <c r="L23" s="23" t="inlineStr"/>
       <c r="M23" s="17" t="inlineStr">
@@ -2220,12 +2236,12 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>unesco:5f5ec6eb-c0e8-4e67-e28f-08df14acbbca</t>
+          <t>unesco:5028b251-6c79-4f6d-f98d-08df189e5e5f</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1102- Edital nº 37/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ1102- Edital nº 39/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -2241,7 +2257,7 @@
       <c r="F24" s="13" t="inlineStr"/>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
@@ -2251,10 +2267,10 @@
       </c>
       <c r="I24" s="11" t="inlineStr"/>
       <c r="J24" s="14" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="L24" s="15" t="inlineStr"/>
       <c r="M24" s="9" t="inlineStr">
@@ -2277,12 +2293,12 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>unesco:dceb9c82-2a2c-4ba9-e290-08df14acbbca</t>
+          <t>unesco:31acdc9f-bf0b-43fe-5017-08df1966cd05</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1102- Edital nº 38/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ1161.2 - Edital nº 01/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
@@ -2298,7 +2314,7 @@
       <c r="F25" s="21" t="inlineStr"/>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
@@ -2308,10 +2324,10 @@
       </c>
       <c r="I25" s="19" t="inlineStr"/>
       <c r="J25" s="22" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46293</v>
+        <v>46295</v>
       </c>
       <c r="L25" s="23" t="inlineStr"/>
       <c r="M25" s="17" t="inlineStr">
@@ -2334,12 +2350,12 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>unesco:7f118a1a-eb71-48a2-e28d-08df14acbbca</t>
+          <t>unesco:6277cc83-3d55-4575-091b-08df172a76c5</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 40/2026 - 1 vaga - Consultor Individual</t>
+          <t>14BRZ1163 - Publicação -  Edital 69/2026 - 01 Vaga consultor Individual</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -2355,7 +2371,7 @@
       <c r="F26" s="13" t="inlineStr"/>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
@@ -2368,7 +2384,7 @@
         <v>46289</v>
       </c>
       <c r="K26" s="14" t="n">
-        <v>46295</v>
+        <v>46294</v>
       </c>
       <c r="L26" s="15" t="inlineStr"/>
       <c r="M26" s="9" t="inlineStr">
@@ -2391,12 +2407,12 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>unesco:34a61630-55f8-4262-9489-08df0f3a2d32</t>
+          <t>unesco:6c8e0acd-2d12-4dc7-e28e-08df14acbbca</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1156 - edital 08/2026 - Consultor Individual</t>
+          <t>914BRZ1102- Edital nº 36/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
@@ -2412,7 +2428,7 @@
       <c r="F27" s="21" t="inlineStr"/>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
@@ -2422,10 +2438,10 @@
       </c>
       <c r="I27" s="19" t="inlineStr"/>
       <c r="J27" s="22" t="n">
-        <v>46282</v>
+        <v>46289</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46289</v>
+        <v>46293</v>
       </c>
       <c r="L27" s="23" t="inlineStr"/>
       <c r="M27" s="17" t="inlineStr">
@@ -2448,17 +2464,17 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>unesco:a4685014-44a0-4ec8-9b63-08df0ff5ff21</t>
+          <t>unesco:5f5ec6eb-c0e8-4e67-e28f-08df14acbbca</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ3051 - EDITAL 11/2026 (REPUBLICAÇÃO)</t>
+          <t>914BRZ1102- Edital nº 37/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr">
@@ -2479,10 +2495,10 @@
       </c>
       <c r="I28" s="11" t="inlineStr"/>
       <c r="J28" s="14" t="n">
-        <v>46285</v>
+        <v>46289</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="L28" s="15" t="inlineStr"/>
       <c r="M28" s="9" t="inlineStr">
@@ -2505,17 +2521,17 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>unesco:49fa6512-497b-43c7-9b65-08df0ff5ff21</t>
+          <t>unesco:dceb9c82-2a2c-4ba9-e290-08df14acbbca</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ1085 - Edital nº 04/2026 - 4 vagas - Consultores Individuais</t>
+          <t>914BRZ1102- Edital nº 38/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E29" s="20" t="inlineStr">
@@ -2526,7 +2542,7 @@
       <c r="F29" s="21" t="inlineStr"/>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Saúde</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
@@ -2536,10 +2552,10 @@
       </c>
       <c r="I29" s="19" t="inlineStr"/>
       <c r="J29" s="22" t="n">
-        <v>46287</v>
+        <v>46289</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="L29" s="23" t="inlineStr"/>
       <c r="M29" s="17" t="inlineStr">
@@ -2562,17 +2578,17 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>unesco:f0e2f0e3-b50c-4695-6d11-08df126138f3</t>
+          <t>unesco:7f118a1a-eb71-48a2-e28d-08df14acbbca</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ3051 - EDITAL 17/2026 (REPUBLICAÇÃO)</t>
+          <t>914BRZ1159 - Publicação Edital 40/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
@@ -2583,7 +2599,7 @@
       <c r="F30" s="13" t="inlineStr"/>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
@@ -2593,10 +2609,10 @@
       </c>
       <c r="I30" s="11" t="inlineStr"/>
       <c r="J30" s="14" t="n">
-        <v>46285</v>
+        <v>46289</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>46292</v>
+        <v>46295</v>
       </c>
       <c r="L30" s="15" t="inlineStr"/>
       <c r="M30" s="9" t="inlineStr">
@@ -2614,17 +2630,17 @@
     <row r="31">
       <c r="A31" s="17" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
+          <t>unesco:a4685014-44a0-4ec8-9b63-08df0ff5ff21</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
+          <t>Projeto 914BRZ3051 - EDITAL 11/2026 (REPUBLICAÇÃO)</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
@@ -2640,63 +2656,53 @@
       <c r="F31" s="21" t="inlineStr"/>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I31" s="19" t="inlineStr">
-        <is>
-          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I31" s="19" t="inlineStr"/>
       <c r="J31" s="22" t="n">
-        <v>46224</v>
+        <v>46285</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46233</v>
-      </c>
-      <c r="L31" s="23" t="n">
-        <v>288000</v>
-      </c>
+        <v>46292</v>
+      </c>
+      <c r="L31" s="23" t="inlineStr"/>
       <c r="M31" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N31" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N31" s="20" t="inlineStr"/>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
+          <t>unesco:49fa6512-497b-43c7-9b65-08df0ff5ff21</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
+          <t>Projeto 914BRZ1085 - Edital nº 04/2026 - 4 vagas - Consultores Individuais</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E32" s="12" t="inlineStr">
@@ -2707,63 +2713,53 @@
       <c r="F32" s="13" t="inlineStr"/>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Saúde</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I32" s="11" t="inlineStr">
-        <is>
-          <t>Remoto, Brasília - DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I32" s="11" t="inlineStr"/>
       <c r="J32" s="14" t="n">
-        <v>46232</v>
+        <v>46287</v>
       </c>
       <c r="K32" s="14" t="n">
-        <v>46238</v>
-      </c>
-      <c r="L32" s="15" t="n">
-        <v>30000</v>
-      </c>
+        <v>46292</v>
+      </c>
+      <c r="L32" s="15" t="inlineStr"/>
       <c r="M32" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N32" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N32" s="12" t="inlineStr"/>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="17" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
+          <t>unesco:f0e2f0e3-b50c-4695-6d11-08df126138f3</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
+          <t>Projeto 914BRZ3051 - EDITAL 17/2026 (REPUBLICAÇÃO)</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E33" s="20" t="inlineStr">
@@ -2774,41 +2770,31 @@
       <c r="F33" s="21" t="inlineStr"/>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I33" s="19" t="inlineStr">
-        <is>
-          <t>Remoto, Brasília - DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I33" s="19" t="inlineStr"/>
       <c r="J33" s="22" t="n">
-        <v>46232</v>
+        <v>46285</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46238</v>
-      </c>
-      <c r="L33" s="23" t="n">
-        <v>30000</v>
-      </c>
+        <v>46292</v>
+      </c>
+      <c r="L33" s="23" t="inlineStr"/>
       <c r="M33" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N33" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N33" s="20" t="inlineStr"/>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
@@ -2820,12 +2806,12 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -2846,19 +2832,19 @@
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
+          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
         </is>
       </c>
       <c r="J34" s="14" t="n">
-        <v>46232</v>
+        <v>46224</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46237</v>
+        <v>46233</v>
       </c>
       <c r="L34" s="15" t="n">
         <v>288000</v>
@@ -2875,7 +2861,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
         </is>
       </c>
     </row>
@@ -2887,17 +2873,17 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E35" s="20" t="inlineStr">
@@ -2908,7 +2894,7 @@
       <c r="F35" s="21" t="inlineStr"/>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
@@ -2918,17 +2904,17 @@
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46240</v>
+        <v>46232</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46245</v>
+        <v>46238</v>
       </c>
       <c r="L35" s="23" t="n">
-        <v>204000</v>
+        <v>30000</v>
       </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
@@ -2942,7 +2928,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
         </is>
       </c>
     </row>
@@ -2954,12 +2940,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -2975,7 +2961,7 @@
       <c r="F36" s="13" t="inlineStr"/>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
@@ -2985,17 +2971,17 @@
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46240</v>
+        <v>46232</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46245</v>
+        <v>46238</v>
       </c>
       <c r="L36" s="15" t="n">
-        <v>80000</v>
+        <v>30000</v>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
@@ -3009,7 +2995,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
         </is>
       </c>
     </row>
@@ -3021,12 +3007,12 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
@@ -3042,27 +3028,27 @@
       <c r="F37" s="21" t="inlineStr"/>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46240</v>
+        <v>46232</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46245</v>
+        <v>46237</v>
       </c>
       <c r="L37" s="23" t="n">
-        <v>204000</v>
+        <v>288000</v>
       </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
@@ -3076,7 +3062,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
         </is>
       </c>
     </row>
@@ -3088,12 +3074,12 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
@@ -3119,7 +3105,7 @@
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Brasília - Df</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
@@ -3129,7 +3115,7 @@
         <v>46245</v>
       </c>
       <c r="L38" s="15" t="n">
-        <v>80000</v>
+        <v>204000</v>
       </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
@@ -3143,7 +3129,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
         </is>
       </c>
     </row>
@@ -3155,12 +3141,12 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
@@ -3176,7 +3162,7 @@
       <c r="F39" s="21" t="inlineStr"/>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
@@ -3196,7 +3182,7 @@
         <v>46245</v>
       </c>
       <c r="L39" s="23" t="n">
-        <v>100000</v>
+        <v>204000</v>
       </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
@@ -3210,7 +3196,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
         </is>
       </c>
     </row>
@@ -3222,12 +3208,12 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
@@ -3243,27 +3229,27 @@
       <c r="F40" s="13" t="inlineStr"/>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46227</v>
+        <v>46240</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46252</v>
+        <v>46245</v>
       </c>
       <c r="L40" s="15" t="n">
-        <v>286000</v>
+        <v>80000</v>
       </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
@@ -3277,7 +3263,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
         </is>
       </c>
     </row>
@@ -3289,12 +3275,12 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
@@ -3310,27 +3296,27 @@
       <c r="F41" s="21" t="inlineStr"/>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Brasília - Df</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46246</v>
+        <v>46240</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46257</v>
+        <v>46245</v>
       </c>
       <c r="L41" s="23" t="n">
-        <v>54000</v>
+        <v>80000</v>
       </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
@@ -3344,7 +3330,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
         </is>
       </c>
     </row>
@@ -3356,12 +3342,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3377,27 +3363,27 @@
       <c r="F42" s="13" t="inlineStr"/>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46246</v>
+        <v>46240</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46257</v>
+        <v>46245</v>
       </c>
       <c r="L42" s="15" t="n">
-        <v>54000</v>
+        <v>100000</v>
       </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
@@ -3411,7 +3397,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
         </is>
       </c>
     </row>
@@ -3423,12 +3409,12 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
@@ -3444,29 +3430,31 @@
       <c r="F43" s="21" t="inlineStr"/>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46246</v>
+        <v>46227</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L43" s="23" t="inlineStr"/>
+        <v>46252</v>
+      </c>
+      <c r="L43" s="23" t="n">
+        <v>286000</v>
+      </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N43" s="20" t="inlineStr">
@@ -3476,7 +3464,7 @@
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
@@ -3488,17 +3476,17 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E44" s="12" t="inlineStr">
@@ -3509,31 +3497,29 @@
       <c r="F44" s="13" t="inlineStr"/>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46251</v>
+        <v>46246</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46256</v>
-      </c>
-      <c r="L44" s="15" t="n">
-        <v>50000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L44" s="15" t="inlineStr"/>
       <c r="M44" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N44" s="12" t="inlineStr">
@@ -3543,7 +3529,7 @@
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -3555,12 +3541,12 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
@@ -3576,7 +3562,7 @@
       <c r="F45" s="21" t="inlineStr"/>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
@@ -3586,17 +3572,17 @@
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46252</v>
+        <v>46246</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46259</v>
+        <v>46257</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>60000</v>
+        <v>54000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
@@ -3610,7 +3596,7 @@
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -3622,17 +3608,17 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E46" s="12" t="inlineStr">
@@ -3643,41 +3629,41 @@
       <c r="F46" s="13" t="inlineStr"/>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J46" s="14" t="n">
-        <v>46208</v>
+        <v>46246</v>
       </c>
       <c r="K46" s="14" t="n">
-        <v>46259</v>
+        <v>46257</v>
       </c>
       <c r="L46" s="15" t="n">
-        <v>500000</v>
+        <v>54000</v>
       </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N46" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -3689,17 +3675,17 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E47" s="20" t="inlineStr">
@@ -3710,7 +3696,7 @@
       <c r="F47" s="21" t="inlineStr"/>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
@@ -3720,21 +3706,21 @@
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J47" s="22" t="n">
-        <v>46246</v>
+        <v>46251</v>
       </c>
       <c r="K47" s="22" t="n">
-        <v>46272</v>
+        <v>46256</v>
       </c>
       <c r="L47" s="23" t="n">
-        <v>54000</v>
+        <v>50000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N47" s="20" t="inlineStr">
@@ -3744,7 +3730,7 @@
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -3756,17 +3742,17 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E48" s="12" t="inlineStr">
@@ -3777,27 +3763,27 @@
       <c r="F48" s="13" t="inlineStr"/>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J48" s="14" t="n">
-        <v>46265</v>
+        <v>46252</v>
       </c>
       <c r="K48" s="14" t="n">
-        <v>46270</v>
+        <v>46259</v>
       </c>
       <c r="L48" s="15" t="n">
-        <v>30000</v>
+        <v>60000</v>
       </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
@@ -3811,7 +3797,7 @@
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -3823,17 +3809,17 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E49" s="20" t="inlineStr">
@@ -3844,41 +3830,41 @@
       <c r="F49" s="21" t="inlineStr"/>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J49" s="22" t="n">
-        <v>46266</v>
+        <v>46208</v>
       </c>
       <c r="K49" s="22" t="n">
-        <v>46288</v>
+        <v>46259</v>
       </c>
       <c r="L49" s="23" t="n">
-        <v>70000</v>
+        <v>500000</v>
       </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N49" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -3890,12 +3876,12 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
@@ -3911,29 +3897,31 @@
       <c r="F50" s="13" t="inlineStr"/>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J50" s="14" t="n">
-        <v>46275</v>
+        <v>46246</v>
       </c>
       <c r="K50" s="14" t="n">
-        <v>46281</v>
-      </c>
-      <c r="L50" s="15" t="inlineStr"/>
+        <v>46272</v>
+      </c>
+      <c r="L50" s="15" t="n">
+        <v>54000</v>
+      </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N50" s="12" t="inlineStr">
@@ -3943,7 +3931,7 @@
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -3955,17 +3943,17 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E51" s="20" t="inlineStr">
@@ -3976,7 +3964,7 @@
       <c r="F51" s="21" t="inlineStr"/>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
@@ -3986,17 +3974,17 @@
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
-        <v>46275</v>
+        <v>46265</v>
       </c>
       <c r="K51" s="22" t="n">
-        <v>46280</v>
+        <v>46270</v>
       </c>
       <c r="L51" s="23" t="n">
-        <v>50000</v>
+        <v>30000</v>
       </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
@@ -4010,7 +3998,7 @@
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -4022,12 +4010,12 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
@@ -4057,25 +4045,27 @@
         </is>
       </c>
       <c r="J52" s="14" t="n">
-        <v>46278</v>
+        <v>46266</v>
       </c>
       <c r="K52" s="14" t="n">
-        <v>46289</v>
-      </c>
-      <c r="L52" s="15" t="inlineStr"/>
+        <v>46288</v>
+      </c>
+      <c r="L52" s="15" t="n">
+        <v>70000</v>
+      </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N52" s="12" t="inlineStr">
         <is>
-          <t>ugp@educacao.sp.gov.br</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
@@ -4087,17 +4077,17 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E53" s="20" t="inlineStr">
@@ -4108,7 +4098,7 @@
       <c r="F53" s="21" t="inlineStr"/>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
@@ -4118,17 +4108,17 @@
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>Dados Remoto</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
-        <v>46281</v>
+        <v>46275</v>
       </c>
       <c r="K53" s="22" t="n">
-        <v>46286</v>
+        <v>46280</v>
       </c>
       <c r="L53" s="23" t="n">
-        <v>110000</v>
+        <v>50000</v>
       </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
@@ -4142,7 +4132,7 @@
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
@@ -4154,12 +4144,12 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
@@ -4175,28 +4165,26 @@
       <c r="F54" s="13" t="inlineStr"/>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J54" s="14" t="n">
-        <v>46282</v>
+        <v>46275</v>
       </c>
       <c r="K54" s="14" t="n">
-        <v>46286</v>
-      </c>
-      <c r="L54" s="15" t="n">
-        <v>30000</v>
-      </c>
+        <v>46281</v>
+      </c>
+      <c r="L54" s="15" t="inlineStr"/>
       <c r="M54" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -4209,7 +4197,7 @@
       </c>
       <c r="O54" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
         </is>
       </c>
     </row>
@@ -4221,17 +4209,17 @@
       </c>
       <c r="B55" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
         </is>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E55" s="20" t="inlineStr">
@@ -4242,41 +4230,41 @@
       <c r="F55" s="21" t="inlineStr"/>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Dados Remoto</t>
         </is>
       </c>
       <c r="J55" s="22" t="n">
-        <v>46244</v>
+        <v>46281</v>
       </c>
       <c r="K55" s="22" t="n">
-        <v>46300</v>
+        <v>46286</v>
       </c>
       <c r="L55" s="23" t="n">
-        <v>350000</v>
+        <v>110000</v>
       </c>
       <c r="M55" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N55" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O55" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
         </is>
       </c>
     </row>
@@ -4288,17 +4276,17 @@
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E56" s="12" t="inlineStr">
@@ -4309,46 +4297,245 @@
       <c r="F56" s="13" t="inlineStr"/>
       <c r="G56" s="11" t="inlineStr">
         <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+        </is>
+      </c>
+      <c r="H56" s="11" t="inlineStr">
+        <is>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I56" s="11" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="J56" s="14" t="n">
+        <v>46282</v>
+      </c>
+      <c r="K56" s="14" t="n">
+        <v>46286</v>
+      </c>
+      <c r="L56" s="15" t="n">
+        <v>30000</v>
+      </c>
+      <c r="M56" s="9" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N56" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O56" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B57" s="18" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+        </is>
+      </c>
+      <c r="C57" s="19" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+        </is>
+      </c>
+      <c r="D57" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E57" s="20" t="inlineStr">
+        <is>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F57" s="21" t="inlineStr"/>
+      <c r="G57" s="19" t="inlineStr">
+        <is>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+        </is>
+      </c>
+      <c r="H57" s="19" t="inlineStr">
+        <is>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I57" s="19" t="inlineStr">
+        <is>
+          <t>São Paulo - SP</t>
+        </is>
+      </c>
+      <c r="J57" s="22" t="n">
+        <v>46278</v>
+      </c>
+      <c r="K57" s="22" t="n">
+        <v>46289</v>
+      </c>
+      <c r="L57" s="23" t="inlineStr"/>
+      <c r="M57" s="17" t="inlineStr">
+        <is>
+          <t>En presentación</t>
+        </is>
+      </c>
+      <c r="N57" s="20" t="inlineStr">
+        <is>
+          <t>ugp@educacao.sp.gov.br</t>
+        </is>
+      </c>
+      <c r="O57" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="9" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B58" s="10" t="inlineStr">
+        <is>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+        </is>
+      </c>
+      <c r="C58" s="11" t="inlineStr">
+        <is>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+        </is>
+      </c>
+      <c r="D58" s="11" t="inlineStr">
+        <is>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+        </is>
+      </c>
+      <c r="E58" s="12" t="inlineStr">
+        <is>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F58" s="13" t="inlineStr"/>
+      <c r="G58" s="11" t="inlineStr">
+        <is>
           <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
-      <c r="H56" s="11" t="inlineStr">
+      <c r="H58" s="11" t="inlineStr">
         <is>
           <t>OEI/MDHC</t>
         </is>
       </c>
-      <c r="I56" s="11" t="inlineStr">
+      <c r="I58" s="11" t="inlineStr">
         <is>
           <t>Nacional</t>
         </is>
       </c>
-      <c r="J56" s="14" t="n">
+      <c r="J58" s="14" t="n">
         <v>46244</v>
       </c>
-      <c r="K56" s="14" t="n">
+      <c r="K58" s="14" t="n">
         <v>46296</v>
       </c>
-      <c r="L56" s="15" t="n">
+      <c r="L58" s="15" t="n">
         <v>935000</v>
       </c>
-      <c r="M56" s="9" t="inlineStr">
+      <c r="M58" s="9" t="inlineStr">
         <is>
           <t>En fase de apresentação</t>
         </is>
       </c>
-      <c r="N56" s="12" t="inlineStr">
+      <c r="N58" s="12" t="inlineStr">
         <is>
           <t>compras.bra@oei.int</t>
         </is>
       </c>
-      <c r="O56" s="16" t="inlineStr">
+      <c r="O58" s="16" t="inlineStr">
         <is>
           <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B59" s="18" t="inlineStr">
+        <is>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+        </is>
+      </c>
+      <c r="C59" s="19" t="inlineStr">
+        <is>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+        </is>
+      </c>
+      <c r="D59" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+        </is>
+      </c>
+      <c r="E59" s="20" t="inlineStr">
+        <is>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F59" s="21" t="inlineStr"/>
+      <c r="G59" s="19" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+        </is>
+      </c>
+      <c r="H59" s="19" t="inlineStr">
+        <is>
+          <t>OEI/MDHC</t>
+        </is>
+      </c>
+      <c r="I59" s="19" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="J59" s="22" t="n">
+        <v>46244</v>
+      </c>
+      <c r="K59" s="22" t="n">
+        <v>46300</v>
+      </c>
+      <c r="L59" s="23" t="n">
+        <v>350000</v>
+      </c>
+      <c r="M59" s="17" t="inlineStr">
+        <is>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N59" s="20" t="inlineStr">
+        <is>
+          <t>compras.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O59" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O56"/>
+  <autoFilter ref="A1:O59"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -4405,6 +4592,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId58"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -4449,21 +4639,21 @@
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Unesco</t>
+          <t>Pnud</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Pnud</t>
+          <t>Unesco</t>
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -4505,7 +4695,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -4547,7 +4737,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3">
@@ -4619,7 +4809,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3">
@@ -4629,7 +4819,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4">
@@ -4639,7 +4829,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5">
@@ -4731,7 +4921,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3">
@@ -4761,7 +4951,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -4801,7 +4991,7 @@
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-09-29 18:02
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$62</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 28/09/2026 às 21:10</t>
+          <t>Gerado em 29/09/2026 às 18:02</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6">
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="17">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>140806.0606060606</v>
+        <v>137241.1428571429</v>
       </c>
     </row>
     <row r="20">
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="25">
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O63"/>
+  <dimension ref="A1:O62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1049,7 +1049,7 @@
         <v>46280</v>
       </c>
       <c r="K4" s="14" t="n">
-        <v>46295</v>
+        <v>46310</v>
       </c>
       <c r="L4" s="15" t="n">
         <v>120000</v>
@@ -1116,7 +1116,7 @@
         <v>46280</v>
       </c>
       <c r="K5" s="22" t="n">
-        <v>46295</v>
+        <v>46310</v>
       </c>
       <c r="L5" s="23" t="n">
         <v>120000</v>
@@ -2933,12 +2933,12 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>unesco:6c8e0acd-2d12-4dc7-e28e-08df14acbbca</t>
+          <t>unesco:7f118a1a-eb71-48a2-e28d-08df14acbbca</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1102- Edital nº 36/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ1159 - Publicação Edital 40/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -2952,11 +2952,11 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.437</v>
+        <v>0.585</v>
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Educação / Ensino, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
@@ -2969,7 +2969,7 @@
         <v>46289</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46293</v>
+        <v>46295</v>
       </c>
       <c r="L34" s="15" t="inlineStr"/>
       <c r="M34" s="9" t="inlineStr">
@@ -2992,30 +2992,30 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>unesco:5f5ec6eb-c0e8-4e67-e28f-08df14acbbca</t>
+          <t>unesco:80185502-579b-44a1-e3c6-08df13ea9ffe</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1102- Edital nº 37/2026 - 01 vaga - Consultor Individual</t>
+          <t>Projeto 914BRZ3051 - EDITAL 22/2026</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E35" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F35" s="21" t="n">
-        <v>0.437</v>
+        <v>0.341</v>
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Educação / Ensino, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
@@ -3025,10 +3025,10 @@
       </c>
       <c r="I35" s="19" t="inlineStr"/>
       <c r="J35" s="22" t="n">
-        <v>46289</v>
+        <v>46292</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46293</v>
+        <v>46299</v>
       </c>
       <c r="L35" s="23" t="inlineStr"/>
       <c r="M35" s="17" t="inlineStr">
@@ -3046,22 +3046,22 @@
     <row r="36">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>unesco:dceb9c82-2a2c-4ba9-e290-08df14acbbca</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1102- Edital nº 38/2026 - 01 vaga - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E36" s="12" t="inlineStr">
@@ -3070,111 +3070,131 @@
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>0.437</v>
+        <v>0.569</v>
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Educação / Ensino, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Cultura, Trabalho / Emprego, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I36" s="11" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I36" s="11" t="inlineStr">
+        <is>
+          <t>Brasília - Df</t>
+        </is>
+      </c>
       <c r="J36" s="14" t="n">
-        <v>46289</v>
+        <v>46240</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46293</v>
-      </c>
-      <c r="L36" s="15" t="inlineStr"/>
+        <v>46245</v>
+      </c>
+      <c r="L36" s="15" t="n">
+        <v>80000</v>
+      </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N36" s="12" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N36" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>unesco:7f118a1a-eb71-48a2-e28d-08df14acbbca</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 40/2026 - 1 vaga - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E37" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F37" s="21" t="n">
-        <v>0.585</v>
+        <v>0.433</v>
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I37" s="19" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I37" s="19" t="inlineStr">
+        <is>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+        </is>
+      </c>
       <c r="J37" s="22" t="n">
-        <v>46289</v>
+        <v>46227</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46295</v>
-      </c>
-      <c r="L37" s="23" t="inlineStr"/>
+        <v>46252</v>
+      </c>
+      <c r="L37" s="23" t="n">
+        <v>286000</v>
+      </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N37" s="20" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N37" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>unesco:80185502-579b-44a1-e3c6-08df13ea9ffe</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ3051 - EDITAL 22/2026</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
@@ -3184,39 +3204,49 @@
       </c>
       <c r="E38" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.341</v>
+        <v>0.492</v>
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Cultura, Desenvolvimento Social / Políticas Públicas</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I38" s="11" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I38" s="11" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J38" s="14" t="n">
-        <v>46292</v>
+        <v>46240</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46299</v>
-      </c>
-      <c r="L38" s="15" t="inlineStr"/>
+        <v>46245</v>
+      </c>
+      <c r="L38" s="15" t="n">
+        <v>100000</v>
+      </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N38" s="12" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N38" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
         </is>
       </c>
     </row>
@@ -3228,12 +3258,12 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
@@ -3247,11 +3277,11 @@
         </is>
       </c>
       <c r="F39" s="21" t="n">
-        <v>0.569</v>
+        <v>0.511</v>
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Cultura, Trabalho / Emprego, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Cultura</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
@@ -3261,7 +3291,7 @@
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Brasília - Df</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
@@ -3271,7 +3301,7 @@
         <v>46245</v>
       </c>
       <c r="L39" s="23" t="n">
-        <v>80000</v>
+        <v>204000</v>
       </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
@@ -3285,7 +3315,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
         </is>
       </c>
     </row>
@@ -3366,12 +3396,12 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
@@ -3381,15 +3411,15 @@
       </c>
       <c r="E41" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F41" s="21" t="n">
-        <v>0.492</v>
+        <v>0.481</v>
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Cultura, Desenvolvimento Social / Políticas Públicas</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
@@ -3409,7 +3439,7 @@
         <v>46245</v>
       </c>
       <c r="L41" s="23" t="n">
-        <v>100000</v>
+        <v>204000</v>
       </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
@@ -3423,7 +3453,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
         </is>
       </c>
     </row>
@@ -3435,12 +3465,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3454,31 +3484,31 @@
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.511</v>
+        <v>0.569</v>
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Cultura</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46245</v>
+        <v>46257</v>
       </c>
       <c r="L42" s="15" t="n">
-        <v>204000</v>
+        <v>54000</v>
       </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
@@ -3492,7 +3522,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -3504,12 +3534,12 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
@@ -3519,39 +3549,37 @@
       </c>
       <c r="E43" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F43" s="21" t="n">
-        <v>0.433</v>
+        <v>0.492</v>
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46227</v>
+        <v>46246</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46252</v>
-      </c>
-      <c r="L43" s="23" t="n">
-        <v>286000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L43" s="23" t="inlineStr"/>
       <c r="M43" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N43" s="20" t="inlineStr">
@@ -3561,7 +3589,7 @@
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -3573,12 +3601,12 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
@@ -3588,35 +3616,35 @@
       </c>
       <c r="E44" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>0.481</v>
+        <v>0.569</v>
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46245</v>
+        <v>46257</v>
       </c>
       <c r="L44" s="15" t="n">
-        <v>204000</v>
+        <v>54000</v>
       </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
@@ -3630,7 +3658,7 @@
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -3642,17 +3670,17 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E45" s="20" t="inlineStr">
@@ -3661,33 +3689,35 @@
         </is>
       </c>
       <c r="F45" s="21" t="n">
-        <v>0.492</v>
+        <v>0.593</v>
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46246</v>
+        <v>46251</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L45" s="23" t="inlineStr"/>
+        <v>46256</v>
+      </c>
+      <c r="L45" s="23" t="n">
+        <v>50000</v>
+      </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N45" s="20" t="inlineStr">
@@ -3697,7 +3727,7 @@
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -3709,12 +3739,12 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -3728,11 +3758,11 @@
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.569</v>
+        <v>0.46</v>
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Educação / Ensino</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
@@ -3742,17 +3772,17 @@
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J46" s="14" t="n">
-        <v>46246</v>
+        <v>46252</v>
       </c>
       <c r="K46" s="14" t="n">
-        <v>46257</v>
+        <v>46259</v>
       </c>
       <c r="L46" s="15" t="n">
-        <v>54000</v>
+        <v>60000</v>
       </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
@@ -3766,7 +3796,7 @@
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -3778,50 +3808,50 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E47" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F47" s="21" t="n">
-        <v>0.569</v>
+        <v>0.451</v>
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J47" s="22" t="n">
-        <v>46246</v>
+        <v>46265</v>
       </c>
       <c r="K47" s="22" t="n">
-        <v>46257</v>
+        <v>46270</v>
       </c>
       <c r="L47" s="23" t="n">
-        <v>54000</v>
+        <v>30000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
@@ -3835,7 +3865,7 @@
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -3847,30 +3877,30 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E48" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F48" s="13" t="n">
-        <v>0.593</v>
+        <v>0.492</v>
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Educação / Ensino</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
@@ -3880,21 +3910,21 @@
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J48" s="14" t="n">
-        <v>46251</v>
+        <v>46246</v>
       </c>
       <c r="K48" s="14" t="n">
-        <v>46256</v>
+        <v>46272</v>
       </c>
       <c r="L48" s="15" t="n">
-        <v>50000</v>
+        <v>54000</v>
       </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N48" s="12" t="inlineStr">
@@ -3904,7 +3934,7 @@
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -3916,64 +3946,64 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E49" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F49" s="21" t="n">
-        <v>0.46</v>
+        <v>0.464</v>
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J49" s="22" t="n">
-        <v>46252</v>
+        <v>46208</v>
       </c>
       <c r="K49" s="22" t="n">
         <v>46259</v>
       </c>
       <c r="L49" s="23" t="n">
-        <v>60000</v>
+        <v>500000</v>
       </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N49" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -3985,64 +4015,64 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E50" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>0.464</v>
+        <v>0.527</v>
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J50" s="14" t="n">
-        <v>46208</v>
+        <v>46266</v>
       </c>
       <c r="K50" s="14" t="n">
-        <v>46259</v>
+        <v>46288</v>
       </c>
       <c r="L50" s="15" t="n">
-        <v>500000</v>
+        <v>70000</v>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N50" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
@@ -4054,12 +4084,12 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
@@ -4069,39 +4099,39 @@
       </c>
       <c r="E51" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F51" s="21" t="n">
-        <v>0.492</v>
+        <v>0.3</v>
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
-        <v>46246</v>
+        <v>46275</v>
       </c>
       <c r="K51" s="22" t="n">
-        <v>46272</v>
+        <v>46280</v>
       </c>
       <c r="L51" s="23" t="n">
-        <v>54000</v>
+        <v>50000</v>
       </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N51" s="20" t="inlineStr">
@@ -4111,7 +4141,7 @@
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
@@ -4123,64 +4153,64 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E52" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F52" s="13" t="n">
-        <v>0.451</v>
+        <v>0.493</v>
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Desenvolvimento Social / Políticas Públicas</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J52" s="14" t="n">
-        <v>46265</v>
+        <v>46244</v>
       </c>
       <c r="K52" s="14" t="n">
-        <v>46270</v>
+        <v>46296</v>
       </c>
       <c r="L52" s="15" t="n">
-        <v>30000</v>
+        <v>935000</v>
       </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N52" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -4192,17 +4222,17 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E53" s="20" t="inlineStr">
@@ -4211,31 +4241,31 @@
         </is>
       </c>
       <c r="F53" s="21" t="n">
-        <v>0.527</v>
+        <v>0.493</v>
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Ciência / Tecnologia e Inovação, Engenharia / Infraestrutura</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Dados Remoto</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
-        <v>46266</v>
+        <v>46281</v>
       </c>
       <c r="K53" s="22" t="n">
-        <v>46288</v>
+        <v>46286</v>
       </c>
       <c r="L53" s="23" t="n">
-        <v>70000</v>
+        <v>110000</v>
       </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
@@ -4249,7 +4279,7 @@
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
         </is>
       </c>
     </row>
@@ -4261,12 +4291,12 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
@@ -4276,34 +4306,36 @@
       </c>
       <c r="E54" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F54" s="13" t="n">
-        <v>0.2</v>
+        <v>0.451</v>
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J54" s="14" t="n">
-        <v>46275</v>
+        <v>46282</v>
       </c>
       <c r="K54" s="14" t="n">
-        <v>46281</v>
-      </c>
-      <c r="L54" s="15" t="inlineStr"/>
+        <v>46286</v>
+      </c>
+      <c r="L54" s="15" t="n">
+        <v>30000</v>
+      </c>
       <c r="M54" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -4316,7 +4348,7 @@
       </c>
       <c r="O54" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
         </is>
       </c>
     </row>
@@ -4328,17 +4360,17 @@
       </c>
       <c r="B55" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
         </is>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E55" s="20" t="inlineStr">
@@ -4347,11 +4379,11 @@
         </is>
       </c>
       <c r="F55" s="21" t="n">
-        <v>0.493</v>
+        <v>0.2</v>
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Ciência / Tecnologia e Inovação, Engenharia / Infraestrutura</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
@@ -4361,18 +4393,16 @@
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>Dados Remoto</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J55" s="22" t="n">
+        <v>46275</v>
+      </c>
+      <c r="K55" s="22" t="n">
         <v>46281</v>
       </c>
-      <c r="K55" s="22" t="n">
-        <v>46286</v>
-      </c>
-      <c r="L55" s="23" t="n">
-        <v>110000</v>
-      </c>
+      <c r="L55" s="23" t="inlineStr"/>
       <c r="M55" s="17" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -4385,7 +4415,7 @@
       </c>
       <c r="O55" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
         </is>
       </c>
     </row>
@@ -4397,12 +4427,12 @@
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
@@ -4416,45 +4446,43 @@
         </is>
       </c>
       <c r="F56" s="13" t="n">
-        <v>0.3</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="G56" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H56" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I56" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J56" s="14" t="n">
-        <v>46275</v>
+        <v>46278</v>
       </c>
       <c r="K56" s="14" t="n">
-        <v>46280</v>
-      </c>
-      <c r="L56" s="15" t="n">
-        <v>50000</v>
-      </c>
+        <v>46295</v>
+      </c>
+      <c r="L56" s="15" t="inlineStr"/>
       <c r="M56" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N56" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>ugp@educacao.sp.gov.br</t>
         </is>
       </c>
       <c r="O56" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
         </is>
       </c>
     </row>
@@ -4466,17 +4494,17 @@
       </c>
       <c r="B57" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
         </is>
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
         </is>
       </c>
       <c r="D57" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E57" s="20" t="inlineStr">
@@ -4485,45 +4513,43 @@
         </is>
       </c>
       <c r="F57" s="21" t="n">
-        <v>0.493</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="G57" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Desenvolvimento Social / Políticas Públicas</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Trabalho / Emprego, Segurança</t>
         </is>
       </c>
       <c r="H57" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I57" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J57" s="22" t="n">
-        <v>46244</v>
+        <v>46290</v>
       </c>
       <c r="K57" s="22" t="n">
-        <v>46296</v>
-      </c>
-      <c r="L57" s="23" t="n">
-        <v>935000</v>
-      </c>
+        <v>46294</v>
+      </c>
+      <c r="L57" s="23" t="inlineStr"/>
       <c r="M57" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N57" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O57" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
         </is>
       </c>
     </row>
@@ -4535,62 +4561,64 @@
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E58" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F58" s="13" t="n">
-        <v>0.5639999999999999</v>
+        <v>0.464</v>
       </c>
       <c r="G58" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Trabalho / Emprego, Segurança</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H58" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I58" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J58" s="14" t="n">
-        <v>46290</v>
+        <v>46244</v>
       </c>
       <c r="K58" s="14" t="n">
-        <v>46294</v>
-      </c>
-      <c r="L58" s="15" t="inlineStr"/>
+        <v>46300</v>
+      </c>
+      <c r="L58" s="15" t="n">
+        <v>350000</v>
+      </c>
       <c r="M58" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N58" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O58" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -4602,12 +4630,12 @@
       </c>
       <c r="B59" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
         </is>
       </c>
       <c r="C59" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
         </is>
       </c>
       <c r="D59" s="19" t="inlineStr">
@@ -4617,11 +4645,11 @@
       </c>
       <c r="E59" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F59" s="21" t="n">
-        <v>0.451</v>
+        <v>0.232</v>
       </c>
       <c r="G59" s="19" t="inlineStr">
         <is>
@@ -4635,14 +4663,14 @@
       </c>
       <c r="I59" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
         </is>
       </c>
       <c r="J59" s="22" t="n">
-        <v>46282</v>
+        <v>46293</v>
       </c>
       <c r="K59" s="22" t="n">
-        <v>46286</v>
+        <v>46298</v>
       </c>
       <c r="L59" s="23" t="n">
         <v>30000</v>
@@ -4659,7 +4687,7 @@
       </c>
       <c r="O59" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
         </is>
       </c>
     </row>
@@ -4671,12 +4699,12 @@
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
+          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
         </is>
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
+          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
         </is>
       </c>
       <c r="D60" s="11" t="inlineStr">
@@ -4686,35 +4714,35 @@
       </c>
       <c r="E60" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F60" s="13" t="n">
-        <v>0.2</v>
+        <v>0.175</v>
       </c>
       <c r="G60" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Educação / Ensino, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Direitos Humanos / Cidadania</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Engenharia / Infraestrutura</t>
         </is>
       </c>
       <c r="H60" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I60" s="11" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Rio Grande do Norte</t>
+          <t>Remota e/ou presencial em Brasília - DF</t>
         </is>
       </c>
       <c r="J60" s="14" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="K60" s="14" t="n">
-        <v>46298</v>
+        <v>46297</v>
       </c>
       <c r="L60" s="15" t="n">
-        <v>21000</v>
+        <v>600000</v>
       </c>
       <c r="M60" s="9" t="inlineStr">
         <is>
@@ -4728,7 +4756,7 @@
       </c>
       <c r="O60" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
         </is>
       </c>
     </row>
@@ -4740,12 +4768,12 @@
       </c>
       <c r="B61" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
         </is>
       </c>
       <c r="C61" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
         </is>
       </c>
       <c r="D61" s="19" t="inlineStr">
@@ -4755,15 +4783,15 @@
       </c>
       <c r="E61" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F61" s="21" t="n">
-        <v>0.5639999999999999</v>
+        <v>0.2</v>
       </c>
       <c r="G61" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Educação / Ensino, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Direitos Humanos / Cidadania</t>
         </is>
       </c>
       <c r="H61" s="19" t="inlineStr">
@@ -4773,29 +4801,31 @@
       </c>
       <c r="I61" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Articulação Estadual - Rio Grande do Norte</t>
         </is>
       </c>
       <c r="J61" s="22" t="n">
-        <v>46278</v>
+        <v>46293</v>
       </c>
       <c r="K61" s="22" t="n">
-        <v>46295</v>
-      </c>
-      <c r="L61" s="23" t="inlineStr"/>
+        <v>46298</v>
+      </c>
+      <c r="L61" s="23" t="n">
+        <v>21000</v>
+      </c>
       <c r="M61" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N61" s="20" t="inlineStr">
         <is>
-          <t>ugp@educacao.sp.gov.br</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O61" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
         </is>
       </c>
     </row>
@@ -4807,12 +4837,12 @@
       </c>
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
         </is>
       </c>
       <c r="C62" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
         </is>
       </c>
       <c r="D62" s="11" t="inlineStr">
@@ -4826,11 +4856,11 @@
         </is>
       </c>
       <c r="F62" s="13" t="n">
-        <v>0.232</v>
+        <v>0.355</v>
       </c>
       <c r="G62" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Educação / Ensino</t>
         </is>
       </c>
       <c r="H62" s="11" t="inlineStr">
@@ -4840,17 +4870,17 @@
       </c>
       <c r="I62" s="11" t="inlineStr">
         <is>
-          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J62" s="14" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="K62" s="14" t="n">
-        <v>46298</v>
+        <v>46305</v>
       </c>
       <c r="L62" s="15" t="n">
-        <v>30000</v>
+        <v>60000</v>
       </c>
       <c r="M62" s="9" t="inlineStr">
         <is>
@@ -4864,81 +4894,12 @@
       </c>
       <c r="O62" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="17" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B63" s="18" t="inlineStr">
-        <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
-        </is>
-      </c>
-      <c r="C63" s="19" t="inlineStr">
-        <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
-        </is>
-      </c>
-      <c r="D63" s="19" t="inlineStr">
-        <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
-        </is>
-      </c>
-      <c r="E63" s="20" t="inlineStr">
-        <is>
-          <t>Consultoria Diversidade Inclusao</t>
-        </is>
-      </c>
-      <c r="F63" s="21" t="n">
-        <v>0.464</v>
-      </c>
-      <c r="G63" s="19" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
-        </is>
-      </c>
-      <c r="H63" s="19" t="inlineStr">
-        <is>
-          <t>OEI/MDHC</t>
-        </is>
-      </c>
-      <c r="I63" s="19" t="inlineStr">
-        <is>
-          <t>Nacional</t>
-        </is>
-      </c>
-      <c r="J63" s="22" t="n">
-        <v>46244</v>
-      </c>
-      <c r="K63" s="22" t="n">
-        <v>46300</v>
-      </c>
-      <c r="L63" s="23" t="n">
-        <v>350000</v>
-      </c>
-      <c r="M63" s="17" t="inlineStr">
-        <is>
-          <t>En fase de apresentação</t>
-        </is>
-      </c>
-      <c r="N63" s="20" t="inlineStr">
-        <is>
-          <t>compras.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O63" s="24" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O63"/>
+  <autoFilter ref="A1:O62"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -5001,7 +4962,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId59"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId60"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId62"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -5040,7 +5000,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3">
@@ -5060,7 +5020,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -5112,7 +5072,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4">
@@ -5164,7 +5124,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3">
@@ -5174,7 +5134,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
@@ -5236,7 +5196,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3">
@@ -5246,7 +5206,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4">
@@ -5266,23 +5226,23 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>Ciência / Tecnologia e Inovação</t>
+          <t>Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>Meio Ambiente / Clima / Geografia</t>
+          <t>Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="B7" s="18" t="n">
@@ -5368,7 +5328,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3">
@@ -5388,7 +5348,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5">
@@ -5398,7 +5358,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6">
@@ -5486,7 +5446,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -5501,7 +5461,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-09-30 17:57
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$61</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 29/09/2026 às 18:02</t>
+          <t>Gerado em 30/09/2026 às 17:56</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6">
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="17">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>137241.1428571429</v>
+        <v>134956.6666666667</v>
       </c>
     </row>
     <row r="20">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="24">
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="25">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O62"/>
+  <dimension ref="A1:O61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2638,12 +2638,12 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>unesco:5028b251-6c79-4f6d-f98d-08df189e5e5f</t>
+          <t>unesco:31acdc9f-bf0b-43fe-5017-08df1966cd05</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1102- Edital nº 39/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ1161.2 - Edital nº 01/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
@@ -2653,15 +2653,15 @@
       </c>
       <c r="E29" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F29" s="21" t="n">
-        <v>0.569</v>
+        <v>0.393</v>
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Educação / Ensino</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
@@ -2674,7 +2674,7 @@
         <v>46290</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="L29" s="23" t="inlineStr"/>
       <c r="M29" s="17" t="inlineStr">
@@ -2697,12 +2697,12 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>unesco:31acdc9f-bf0b-43fe-5017-08df1966cd05</t>
+          <t>unesco:4d25520a-6684-41e6-3080-08df1a5635e8</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1161.2 - Edital nº 01/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ1161.2 - Edital nº 02/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
@@ -2716,11 +2716,11 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.393</v>
+        <v>0.25</v>
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
@@ -2730,7 +2730,7 @@
       </c>
       <c r="I30" s="11" t="inlineStr"/>
       <c r="J30" s="14" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="K30" s="14" t="n">
         <v>46295</v>
@@ -2756,12 +2756,12 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>unesco:4d25520a-6684-41e6-3080-08df1a5635e8</t>
+          <t>unesco:c0a1d55e-84e2-4c98-3081-08df1a5635e8</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1161.2 - Edital nº 02/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ1161.2 - Edital nº 03/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
@@ -2779,7 +2779,7 @@
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Educação / Ensino</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
@@ -2815,12 +2815,12 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>unesco:c0a1d55e-84e2-4c98-3081-08df1a5635e8</t>
+          <t>unesco:7f118a1a-eb71-48a2-e28d-08df14acbbca</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1161.2 - Edital nº 03/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ1159 - Publicação Edital 40/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
@@ -2830,15 +2830,15 @@
       </c>
       <c r="E32" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.25</v>
+        <v>0.585</v>
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
@@ -2848,7 +2848,7 @@
       </c>
       <c r="I32" s="11" t="inlineStr"/>
       <c r="J32" s="14" t="n">
-        <v>46291</v>
+        <v>46289</v>
       </c>
       <c r="K32" s="14" t="n">
         <v>46295</v>
@@ -2874,17 +2874,17 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>unesco:6277cc83-3d55-4575-091b-08df172a76c5</t>
+          <t>unesco:80185502-579b-44a1-e3c6-08df13ea9ffe</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>14BRZ1163 - Publicação -  Edital 69/2026 - 01 Vaga consultor Individual</t>
+          <t>Projeto 914BRZ3051 - EDITAL 22/2026</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E33" s="20" t="inlineStr">
@@ -2893,11 +2893,11 @@
         </is>
       </c>
       <c r="F33" s="21" t="n">
-        <v>0.536</v>
+        <v>0.341</v>
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
@@ -2907,10 +2907,10 @@
       </c>
       <c r="I33" s="19" t="inlineStr"/>
       <c r="J33" s="22" t="n">
-        <v>46289</v>
+        <v>46292</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46294</v>
+        <v>46299</v>
       </c>
       <c r="L33" s="23" t="inlineStr"/>
       <c r="M33" s="17" t="inlineStr">
@@ -2928,22 +2928,22 @@
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>unesco:7f118a1a-eb71-48a2-e28d-08df14acbbca</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 40/2026 - 1 vaga - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E34" s="12" t="inlineStr">
@@ -2952,52 +2952,62 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.585</v>
+        <v>0.511</v>
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Cultura</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I34" s="11" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I34" s="11" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J34" s="14" t="n">
-        <v>46289</v>
+        <v>46240</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46295</v>
-      </c>
-      <c r="L34" s="15" t="inlineStr"/>
+        <v>46245</v>
+      </c>
+      <c r="L34" s="15" t="n">
+        <v>204000</v>
+      </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N34" s="12" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N34" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>unesco:80185502-579b-44a1-e3c6-08df13ea9ffe</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ3051 - EDITAL 22/2026</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
@@ -3011,35 +3021,45 @@
         </is>
       </c>
       <c r="F35" s="21" t="n">
-        <v>0.341</v>
+        <v>0.462</v>
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Cultura, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I35" s="19" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I35" s="19" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J35" s="22" t="n">
-        <v>46292</v>
+        <v>46240</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46299</v>
-      </c>
-      <c r="L35" s="23" t="inlineStr"/>
+        <v>46245</v>
+      </c>
+      <c r="L35" s="23" t="n">
+        <v>80000</v>
+      </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N35" s="20" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N35" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
         </is>
       </c>
     </row>
@@ -3051,12 +3071,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -3066,35 +3086,35 @@
       </c>
       <c r="E36" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>0.569</v>
+        <v>0.433</v>
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Cultura, Trabalho / Emprego, Ciência / Tecnologia e Inovação</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>Brasília - Df</t>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46240</v>
+        <v>46227</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46245</v>
+        <v>46252</v>
       </c>
       <c r="L36" s="15" t="n">
-        <v>80000</v>
+        <v>286000</v>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
@@ -3108,7 +3128,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
@@ -3120,12 +3140,12 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
@@ -3139,31 +3159,31 @@
         </is>
       </c>
       <c r="F37" s="21" t="n">
-        <v>0.433</v>
+        <v>0.481</v>
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46227</v>
+        <v>46240</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46252</v>
+        <v>46245</v>
       </c>
       <c r="L37" s="23" t="n">
-        <v>286000</v>
+        <v>204000</v>
       </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
@@ -3177,7 +3197,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
         </is>
       </c>
     </row>
@@ -3189,12 +3209,12 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
@@ -3208,11 +3228,11 @@
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.492</v>
+        <v>0.569</v>
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Cultura, Desenvolvimento Social / Políticas Públicas</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Cultura, Trabalho / Emprego, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
@@ -3222,7 +3242,7 @@
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Brasília - Df</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
@@ -3232,7 +3252,7 @@
         <v>46245</v>
       </c>
       <c r="L38" s="15" t="n">
-        <v>100000</v>
+        <v>80000</v>
       </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
@@ -3246,7 +3266,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
         </is>
       </c>
     </row>
@@ -3258,12 +3278,12 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
@@ -3277,11 +3297,11 @@
         </is>
       </c>
       <c r="F39" s="21" t="n">
-        <v>0.511</v>
+        <v>0.492</v>
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Cultura</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Cultura, Desenvolvimento Social / Políticas Públicas</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
@@ -3301,7 +3321,7 @@
         <v>46245</v>
       </c>
       <c r="L39" s="23" t="n">
-        <v>204000</v>
+        <v>100000</v>
       </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
@@ -3315,7 +3335,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
         </is>
       </c>
     </row>
@@ -3327,12 +3347,12 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
@@ -3342,15 +3362,15 @@
       </c>
       <c r="E40" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.462</v>
+        <v>0.492</v>
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Cultura, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
@@ -3360,21 +3380,19 @@
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46245</v>
-      </c>
-      <c r="L40" s="15" t="n">
-        <v>80000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L40" s="15" t="inlineStr"/>
       <c r="M40" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N40" s="12" t="inlineStr">
@@ -3384,7 +3402,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -3396,12 +3414,12 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
@@ -3411,35 +3429,35 @@
       </c>
       <c r="E41" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F41" s="21" t="n">
-        <v>0.481</v>
+        <v>0.569</v>
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46245</v>
+        <v>46257</v>
       </c>
       <c r="L41" s="23" t="n">
-        <v>204000</v>
+        <v>54000</v>
       </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
@@ -3453,7 +3471,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -3534,12 +3552,12 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
@@ -3553,33 +3571,35 @@
         </is>
       </c>
       <c r="F43" s="21" t="n">
-        <v>0.492</v>
+        <v>0.46</v>
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Educação / Ensino</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46246</v>
+        <v>46252</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L43" s="23" t="inlineStr"/>
+        <v>46259</v>
+      </c>
+      <c r="L43" s="23" t="n">
+        <v>60000</v>
+      </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N43" s="20" t="inlineStr">
@@ -3589,7 +3609,7 @@
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -3601,17 +3621,17 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E44" s="12" t="inlineStr">
@@ -3620,11 +3640,11 @@
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>0.569</v>
+        <v>0.593</v>
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
@@ -3634,17 +3654,17 @@
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46246</v>
+        <v>46251</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46257</v>
+        <v>46256</v>
       </c>
       <c r="L44" s="15" t="n">
-        <v>54000</v>
+        <v>50000</v>
       </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
@@ -3658,7 +3678,7 @@
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -3670,64 +3690,64 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E45" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F45" s="21" t="n">
-        <v>0.593</v>
+        <v>0.464</v>
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46251</v>
+        <v>46208</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46256</v>
+        <v>46259</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>50000</v>
+        <v>500000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N45" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -3739,50 +3759,50 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E46" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.46</v>
+        <v>0.451</v>
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J46" s="14" t="n">
-        <v>46252</v>
+        <v>46265</v>
       </c>
       <c r="K46" s="14" t="n">
-        <v>46259</v>
+        <v>46270</v>
       </c>
       <c r="L46" s="15" t="n">
-        <v>60000</v>
+        <v>30000</v>
       </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
@@ -3796,7 +3816,7 @@
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -3808,17 +3828,17 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E47" s="20" t="inlineStr">
@@ -3827,35 +3847,35 @@
         </is>
       </c>
       <c r="F47" s="21" t="n">
-        <v>0.451</v>
+        <v>0.492</v>
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Educação / Ensino</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J47" s="22" t="n">
-        <v>46265</v>
+        <v>46246</v>
       </c>
       <c r="K47" s="22" t="n">
-        <v>46270</v>
+        <v>46272</v>
       </c>
       <c r="L47" s="23" t="n">
-        <v>30000</v>
+        <v>54000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N47" s="20" t="inlineStr">
@@ -3865,7 +3885,7 @@
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -3877,12 +3897,12 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
@@ -3892,15 +3912,15 @@
       </c>
       <c r="E48" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F48" s="13" t="n">
-        <v>0.492</v>
+        <v>0.527</v>
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Educação / Ensino</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
@@ -3910,21 +3930,21 @@
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J48" s="14" t="n">
-        <v>46246</v>
+        <v>46266</v>
       </c>
       <c r="K48" s="14" t="n">
-        <v>46272</v>
+        <v>46288</v>
       </c>
       <c r="L48" s="15" t="n">
-        <v>54000</v>
+        <v>70000</v>
       </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N48" s="12" t="inlineStr">
@@ -3934,7 +3954,7 @@
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
@@ -3946,64 +3966,64 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E49" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F49" s="21" t="n">
-        <v>0.464</v>
+        <v>0.3</v>
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J49" s="22" t="n">
-        <v>46208</v>
+        <v>46275</v>
       </c>
       <c r="K49" s="22" t="n">
-        <v>46259</v>
+        <v>46280</v>
       </c>
       <c r="L49" s="23" t="n">
-        <v>500000</v>
+        <v>50000</v>
       </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N49" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
@@ -4015,12 +4035,12 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
@@ -4034,32 +4054,30 @@
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>0.527</v>
+        <v>0.2</v>
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J50" s="14" t="n">
-        <v>46266</v>
+        <v>46275</v>
       </c>
       <c r="K50" s="14" t="n">
-        <v>46288</v>
-      </c>
-      <c r="L50" s="15" t="n">
-        <v>70000</v>
-      </c>
+        <v>46281</v>
+      </c>
+      <c r="L50" s="15" t="inlineStr"/>
       <c r="M50" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -4072,7 +4090,7 @@
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
         </is>
       </c>
     </row>
@@ -4084,17 +4102,17 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E51" s="20" t="inlineStr">
@@ -4103,11 +4121,11 @@
         </is>
       </c>
       <c r="F51" s="21" t="n">
-        <v>0.3</v>
+        <v>0.493</v>
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Ciência / Tecnologia e Inovação, Engenharia / Infraestrutura</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
@@ -4117,17 +4135,17 @@
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Dados Remoto</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
-        <v>46275</v>
+        <v>46281</v>
       </c>
       <c r="K51" s="22" t="n">
-        <v>46280</v>
+        <v>46286</v>
       </c>
       <c r="L51" s="23" t="n">
-        <v>50000</v>
+        <v>110000</v>
       </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
@@ -4141,7 +4159,7 @@
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
         </is>
       </c>
     </row>
@@ -4153,64 +4171,64 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E52" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F52" s="13" t="n">
-        <v>0.493</v>
+        <v>0.451</v>
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Desenvolvimento Social / Políticas Públicas</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J52" s="14" t="n">
-        <v>46244</v>
+        <v>46282</v>
       </c>
       <c r="K52" s="14" t="n">
-        <v>46296</v>
+        <v>46286</v>
       </c>
       <c r="L52" s="15" t="n">
-        <v>935000</v>
+        <v>30000</v>
       </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N52" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
         </is>
       </c>
     </row>
@@ -4222,17 +4240,17 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E53" s="20" t="inlineStr">
@@ -4241,11 +4259,11 @@
         </is>
       </c>
       <c r="F53" s="21" t="n">
-        <v>0.493</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Ciência / Tecnologia e Inovação, Engenharia / Infraestrutura</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Trabalho / Emprego, Segurança</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
@@ -4255,18 +4273,16 @@
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>Dados Remoto</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
-        <v>46281</v>
+        <v>46290</v>
       </c>
       <c r="K53" s="22" t="n">
-        <v>46286</v>
-      </c>
-      <c r="L53" s="23" t="n">
-        <v>110000</v>
-      </c>
+        <v>46294</v>
+      </c>
+      <c r="L53" s="23" t="inlineStr"/>
       <c r="M53" s="17" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -4279,7 +4295,7 @@
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
         </is>
       </c>
     </row>
@@ -4291,12 +4307,12 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
@@ -4306,15 +4322,15 @@
       </c>
       <c r="E54" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F54" s="13" t="n">
-        <v>0.451</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
@@ -4324,31 +4340,29 @@
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J54" s="14" t="n">
-        <v>46282</v>
+        <v>46278</v>
       </c>
       <c r="K54" s="14" t="n">
-        <v>46286</v>
-      </c>
-      <c r="L54" s="15" t="n">
-        <v>30000</v>
-      </c>
+        <v>46295</v>
+      </c>
+      <c r="L54" s="15" t="inlineStr"/>
       <c r="M54" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N54" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>ugp@educacao.sp.gov.br</t>
         </is>
       </c>
       <c r="O54" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
         </is>
       </c>
     </row>
@@ -4360,17 +4374,17 @@
       </c>
       <c r="B55" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E55" s="20" t="inlineStr">
@@ -4379,43 +4393,45 @@
         </is>
       </c>
       <c r="F55" s="21" t="n">
-        <v>0.2</v>
+        <v>0.493</v>
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Desenvolvimento Social / Políticas Públicas</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J55" s="22" t="n">
-        <v>46275</v>
+        <v>46244</v>
       </c>
       <c r="K55" s="22" t="n">
-        <v>46281</v>
-      </c>
-      <c r="L55" s="23" t="inlineStr"/>
+        <v>46296</v>
+      </c>
+      <c r="L55" s="23" t="n">
+        <v>935000</v>
+      </c>
       <c r="M55" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N55" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O55" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -4427,62 +4443,64 @@
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E56" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F56" s="13" t="n">
-        <v>0.5639999999999999</v>
+        <v>0.464</v>
       </c>
       <c r="G56" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H56" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I56" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J56" s="14" t="n">
-        <v>46278</v>
+        <v>46244</v>
       </c>
       <c r="K56" s="14" t="n">
-        <v>46295</v>
-      </c>
-      <c r="L56" s="15" t="inlineStr"/>
+        <v>46300</v>
+      </c>
+      <c r="L56" s="15" t="n">
+        <v>350000</v>
+      </c>
       <c r="M56" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N56" s="12" t="inlineStr">
         <is>
-          <t>ugp@educacao.sp.gov.br</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O56" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -4494,52 +4512,54 @@
       </c>
       <c r="B57" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
         </is>
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
         </is>
       </c>
       <c r="D57" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E57" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F57" s="21" t="n">
-        <v>0.5639999999999999</v>
+        <v>0.2</v>
       </c>
       <c r="G57" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Trabalho / Emprego, Segurança</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Educação / Ensino, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Direitos Humanos / Cidadania</t>
         </is>
       </c>
       <c r="H57" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I57" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Articulação Estadual - Rio Grande do Norte</t>
         </is>
       </c>
       <c r="J57" s="22" t="n">
-        <v>46290</v>
+        <v>46293</v>
       </c>
       <c r="K57" s="22" t="n">
-        <v>46294</v>
-      </c>
-      <c r="L57" s="23" t="inlineStr"/>
+        <v>46298</v>
+      </c>
+      <c r="L57" s="23" t="n">
+        <v>21000</v>
+      </c>
       <c r="M57" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N57" s="20" t="inlineStr">
@@ -4549,7 +4569,7 @@
       </c>
       <c r="O57" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
         </is>
       </c>
     </row>
@@ -4561,50 +4581,50 @@
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E58" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F58" s="13" t="n">
-        <v>0.464</v>
+        <v>0.175</v>
       </c>
       <c r="G58" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Engenharia / Infraestrutura</t>
         </is>
       </c>
       <c r="H58" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I58" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Remota e/ou presencial em Brasília - DF</t>
         </is>
       </c>
       <c r="J58" s="14" t="n">
-        <v>46244</v>
+        <v>46294</v>
       </c>
       <c r="K58" s="14" t="n">
-        <v>46300</v>
+        <v>46297</v>
       </c>
       <c r="L58" s="15" t="n">
-        <v>350000</v>
+        <v>600000</v>
       </c>
       <c r="M58" s="9" t="inlineStr">
         <is>
@@ -4613,12 +4633,12 @@
       </c>
       <c r="N58" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O58" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
         </is>
       </c>
     </row>
@@ -4699,12 +4719,12 @@
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
         </is>
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
         </is>
       </c>
       <c r="D60" s="11" t="inlineStr">
@@ -4714,39 +4734,39 @@
       </c>
       <c r="E60" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Não Classificado</t>
         </is>
       </c>
       <c r="F60" s="13" t="n">
-        <v>0.175</v>
+        <v>0.077</v>
       </c>
       <c r="G60" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Engenharia / Infraestrutura</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H60" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I60" s="11" t="inlineStr">
         <is>
-          <t>Remota e/ou presencial em Brasília - DF</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J60" s="14" t="n">
         <v>46294</v>
       </c>
       <c r="K60" s="14" t="n">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="L60" s="15" t="n">
-        <v>600000</v>
+        <v>55000</v>
       </c>
       <c r="M60" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N60" s="12" t="inlineStr">
@@ -4756,7 +4776,7 @@
       </c>
       <c r="O60" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
         </is>
       </c>
     </row>
@@ -4768,12 +4788,12 @@
       </c>
       <c r="B61" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
         </is>
       </c>
       <c r="C61" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
         </is>
       </c>
       <c r="D61" s="19" t="inlineStr">
@@ -4783,15 +4803,15 @@
       </c>
       <c r="E61" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F61" s="21" t="n">
-        <v>0.2</v>
+        <v>0.355</v>
       </c>
       <c r="G61" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Educação / Ensino, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Direitos Humanos / Cidadania</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Educação / Ensino</t>
         </is>
       </c>
       <c r="H61" s="19" t="inlineStr">
@@ -4801,21 +4821,21 @@
       </c>
       <c r="I61" s="19" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Rio Grande do Norte</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J61" s="22" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="K61" s="22" t="n">
-        <v>46298</v>
+        <v>46302</v>
       </c>
       <c r="L61" s="23" t="n">
-        <v>21000</v>
+        <v>60000</v>
       </c>
       <c r="M61" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N61" s="20" t="inlineStr">
@@ -4825,81 +4845,12 @@
       </c>
       <c r="O61" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="9" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B62" s="10" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
-        </is>
-      </c>
-      <c r="C62" s="11" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
-        </is>
-      </c>
-      <c r="D62" s="11" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E62" s="12" t="inlineStr">
-        <is>
-          <t>Engenharia Processos Analytics</t>
-        </is>
-      </c>
-      <c r="F62" s="13" t="n">
-        <v>0.355</v>
-      </c>
-      <c r="G62" s="11" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Educação / Ensino</t>
-        </is>
-      </c>
-      <c r="H62" s="11" t="inlineStr">
-        <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I62" s="11" t="inlineStr">
-        <is>
-          <t>São Paulo - SP</t>
-        </is>
-      </c>
-      <c r="J62" s="14" t="n">
-        <v>46294</v>
-      </c>
-      <c r="K62" s="14" t="n">
-        <v>46305</v>
-      </c>
-      <c r="L62" s="15" t="n">
-        <v>60000</v>
-      </c>
-      <c r="M62" s="9" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N62" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O62" s="16" t="inlineStr">
-        <is>
           <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O62"/>
+  <autoFilter ref="A1:O61"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -4961,7 +4912,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId59"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId61"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -5000,7 +4950,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3">
@@ -5020,7 +4970,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -5062,7 +5012,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3">
@@ -5072,7 +5022,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4">
@@ -5082,7 +5032,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -5124,7 +5074,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3">
@@ -5134,7 +5084,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4">
@@ -5196,7 +5146,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3">
@@ -5216,7 +5166,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5">
@@ -5226,7 +5176,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6">
@@ -5324,7 +5274,7 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
@@ -5354,11 +5304,11 @@
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6">
@@ -5446,7 +5396,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -5461,7 +5411,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-10-01 18:28
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$62</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 30/09/2026 às 17:56</t>
+          <t>Gerado em 01/10/2026 às 18:27</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6">
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>36</v>
+        <v>41</v>
       </c>
     </row>
     <row r="17">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>134956.6666666667</v>
+        <v>123620.4878048781</v>
       </c>
     </row>
     <row r="20">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>93500</v>
+        <v>86800</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="25">
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O61"/>
+  <dimension ref="A1:O62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -943,11 +943,11 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>146373</v>
+        <v>146374</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edital nº 26/2026 – Contratação de Consultoria Individual para aprimoramento de soluções analíticas e computacionais aplicadas ao Modelo de Mensuração de Custos da Digitalização de Serviços Públicos </t>
+          <t>Edital nº 27/2026 – Contratação de Consultoria Individual II - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Servidões de Passagem para Orlas e Praias</t>
         </is>
       </c>
       <c r="D3" s="19" t="inlineStr">
@@ -957,11 +957,11 @@
       </c>
       <c r="E3" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F3" s="21" t="n">
-        <v>0.5</v>
+        <v>0.494</v>
       </c>
       <c r="G3" s="19" t="inlineStr">
         <is>
@@ -982,10 +982,10 @@
         <v>46280</v>
       </c>
       <c r="K3" s="22" t="n">
-        <v>46295</v>
+        <v>46310</v>
       </c>
       <c r="L3" s="23" t="n">
-        <v>108000</v>
+        <v>120000</v>
       </c>
       <c r="M3" s="17" t="inlineStr">
         <is>
@@ -1010,11 +1010,11 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>146374</v>
+        <v>146375</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>Edital nº 27/2026 – Contratação de Consultoria Individual II - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Servidões de Passagem para Orlas e Praias</t>
+          <t>Edital nº 28/2026 - Contratação de Consultoria Individual I - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Acessibilidade em Orlas e Praias</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
@@ -1042,7 +1042,7 @@
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>REMOTO</t>
         </is>
       </c>
       <c r="J4" s="14" t="n">
@@ -1077,11 +1077,11 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>146375</v>
+        <v>146384</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t>Edital nº 28/2026 - Contratação de Consultoria Individual I - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Acessibilidade em Orlas e Praias</t>
+          <t>Edital 05/2026 - Estudos e análises para o fortalecimento da perspectiva de gênero nas políticas públicas de direitos humanos</t>
         </is>
       </c>
       <c r="D5" s="19" t="inlineStr">
@@ -1091,32 +1091,32 @@
       </c>
       <c r="E5" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Não Classificado</t>
         </is>
       </c>
       <c r="F5" s="21" t="n">
-        <v>0.494</v>
+        <v>0.116</v>
       </c>
       <c r="G5" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Desenvolvimento Social / Políticas Públicas, Direitos Humanos / Cidadania</t>
         </is>
       </c>
       <c r="H5" s="19" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I5" s="19" t="inlineStr">
         <is>
-          <t>REMOTO</t>
+          <t>Território Nacional</t>
         </is>
       </c>
       <c r="J5" s="22" t="n">
-        <v>46280</v>
+        <v>46283</v>
       </c>
       <c r="K5" s="22" t="n">
-        <v>46310</v>
+        <v>46296</v>
       </c>
       <c r="L5" s="23" t="n">
         <v>120000</v>
@@ -1128,7 +1128,7 @@
       </c>
       <c r="N5" s="20" t="inlineStr">
         <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
+          <t>dirp@mdh.gov.br</t>
         </is>
       </c>
       <c r="O5" s="24" t="inlineStr">
@@ -1144,11 +1144,11 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>146384</v>
+        <v>146385</v>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>Edital 05/2026 - Estudos e análises para o fortalecimento da perspectiva de gênero nas políticas públicas de direitos humanos</t>
+          <t>Contratação de consultor para elaborar o Caderno Temático de Referência: Investigação de Crimes contra Jornalistas e Comunicadores</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
@@ -1158,15 +1158,15 @@
       </c>
       <c r="E6" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.116</v>
+        <v>0.407</v>
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Desenvolvimento Social / Políticas Públicas, Direitos Humanos / Cidadania</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr">
@@ -1176,17 +1176,17 @@
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>Território Nacional</t>
+          <t>Home-based</t>
         </is>
       </c>
       <c r="J6" s="14" t="n">
-        <v>46283</v>
+        <v>46289</v>
       </c>
       <c r="K6" s="14" t="n">
-        <v>46296</v>
+        <v>46311</v>
       </c>
       <c r="L6" s="15" t="n">
-        <v>120000</v>
+        <v>100000</v>
       </c>
       <c r="M6" s="9" t="inlineStr">
         <is>
@@ -1195,7 +1195,7 @@
       </c>
       <c r="N6" s="12" t="inlineStr">
         <is>
-          <t>dirp@mdh.gov.br</t>
+          <t>prodocbra016@mj.gov.br</t>
         </is>
       </c>
       <c r="O6" s="16" t="inlineStr">
@@ -1211,11 +1211,11 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>146385</v>
+        <v>146380</v>
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor para elaborar o Caderno Temático de Referência: Investigação de Crimes contra Jornalistas e Comunicadores</t>
+          <t>PROJETO BRA 23/023 - TR 138/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A PROPOSIÇÃO DE PLATAFORMAS E DASHBOARDS DE VISUALIZAÇÃO DE DADOS PARA A AGENDA DE DESENVOLVIMENTO HUMANO</t>
         </is>
       </c>
       <c r="D7" s="19" t="inlineStr">
@@ -1225,35 +1225,35 @@
       </c>
       <c r="E7" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F7" s="21" t="n">
-        <v>0.407</v>
+        <v>0.511</v>
       </c>
       <c r="G7" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H7" s="19" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>IBGE</t>
         </is>
       </c>
       <c r="I7" s="19" t="inlineStr">
         <is>
-          <t>Home-based</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J7" s="22" t="n">
-        <v>46289</v>
+        <v>46287</v>
       </c>
       <c r="K7" s="22" t="n">
-        <v>46311</v>
+        <v>46296</v>
       </c>
       <c r="L7" s="23" t="n">
-        <v>100000</v>
+        <v>126500</v>
       </c>
       <c r="M7" s="17" t="inlineStr">
         <is>
@@ -1262,7 +1262,7 @@
       </c>
       <c r="N7" s="20" t="inlineStr">
         <is>
-          <t>prodocbra016@mj.gov.br</t>
+          <t>projetos.especiais@ibge.gov.br</t>
         </is>
       </c>
       <c r="O7" s="24" t="inlineStr">
@@ -1278,11 +1278,11 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>146380</v>
+        <v>146381</v>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 138/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A PROPOSIÇÃO DE PLATAFORMAS E DASHBOARDS DE VISUALIZAÇÃO DE DADOS PARA A AGENDA DE DESENVOLVIMENTO HUMANO</t>
+          <t>PROJETO BRA 23/023 - TR 139/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A SISTEMATIZAÇÃO E ELABORAÇÃO DO DOSSIÊ INSTITUCIONAL DA SÉRIE DIÁLOGOS NACIONAIS PARA O DESENVOLVIMENTO.</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
@@ -1292,11 +1292,11 @@
       </c>
       <c r="E8" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.511</v>
+        <v>0.464</v>
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
@@ -1345,11 +1345,11 @@
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>146381</v>
+        <v>146383</v>
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 139/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A SISTEMATIZAÇÃO E ELABORAÇÃO DO DOSSIÊ INSTITUCIONAL DA SÉRIE DIÁLOGOS NACIONAIS PARA O DESENVOLVIMENTO.</t>
+          <t>PROJETO BRA 23/023 - TR 145/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA DESENVOLVIMENTO DE PROPOSTA DE ALGORITMO DE GEOCODIFICAÇÃO DE ENDEREÇOS BRASILEIROS.</t>
         </is>
       </c>
       <c r="D9" s="19" t="inlineStr">
@@ -1363,11 +1363,11 @@
         </is>
       </c>
       <c r="F9" s="21" t="n">
-        <v>0.464</v>
+        <v>0.462</v>
       </c>
       <c r="G9" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H9" s="19" t="inlineStr">
@@ -1387,7 +1387,7 @@
         <v>46296</v>
       </c>
       <c r="L9" s="23" t="n">
-        <v>126500</v>
+        <v>86800</v>
       </c>
       <c r="M9" s="17" t="inlineStr">
         <is>
@@ -1412,29 +1412,29 @@
         </is>
       </c>
       <c r="B10" s="10" t="n">
-        <v>146383</v>
+        <v>146354</v>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 145/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA DESENVOLVIMENTO DE PROPOSTA DE ALGORITMO DE GEOCODIFICAÇÃO DE ENDEREÇOS BRASILEIROS.</t>
+          <t>PROJETO BRA 23/023 - TR 88/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA PROPOSIÇÃO DE SOLUÇÕES DE CIÊNCIA DE DADOS EM SENSORIAMENTO REMOTO.</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E10" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.462</v>
+        <v>0.411</v>
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
@@ -1448,13 +1448,13 @@
         </is>
       </c>
       <c r="J10" s="14" t="n">
-        <v>46287</v>
+        <v>46293</v>
       </c>
       <c r="K10" s="14" t="n">
-        <v>46296</v>
+        <v>46307</v>
       </c>
       <c r="L10" s="15" t="n">
-        <v>86800</v>
+        <v>93500</v>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
@@ -1479,11 +1479,11 @@
         </is>
       </c>
       <c r="B11" s="18" t="n">
-        <v>146354</v>
+        <v>146357</v>
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 88/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA PROPOSIÇÃO DE SOLUÇÕES DE CIÊNCIA DE DADOS EM SENSORIAMENTO REMOTO.</t>
+          <t>PROJETO BRA 23/023 - TR 141/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE METODOLOGIA DE MODELAGEM PREDITIVA PARA ANÁLISE TERRITORIAL DO DESENVOLVIMENTO HUMANO.</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
@@ -1493,15 +1493,15 @@
       </c>
       <c r="E11" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F11" s="21" t="n">
-        <v>0.411</v>
+        <v>0.464</v>
       </c>
       <c r="G11" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H11" s="19" t="inlineStr">
@@ -1515,13 +1515,13 @@
         </is>
       </c>
       <c r="J11" s="22" t="n">
-        <v>46293</v>
+        <v>46287</v>
       </c>
       <c r="K11" s="22" t="n">
-        <v>46307</v>
+        <v>46296</v>
       </c>
       <c r="L11" s="23" t="n">
-        <v>93500</v>
+        <v>126500</v>
       </c>
       <c r="M11" s="17" t="inlineStr">
         <is>
@@ -1546,11 +1546,11 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>146357</v>
+        <v>146358</v>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 141/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE METODOLOGIA DE MODELAGEM PREDITIVA PARA ANÁLISE TERRITORIAL DO DESENVOLVIMENTO HUMANO.</t>
+          <t>PROJETO BRA 23/023 - TR 142/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE METODOLOGIA DE MODELAGEM PREDITIVA COM FOCO NO PROCESSAMENTO E INTEGRAÇÃO DE DADOS GEOESPACIAIS.</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
@@ -1564,7 +1564,7 @@
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.464</v>
+        <v>0.481</v>
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
@@ -1613,29 +1613,29 @@
         </is>
       </c>
       <c r="B13" s="18" t="n">
-        <v>146358</v>
+        <v>146382</v>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 142/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE METODOLOGIA DE MODELAGEM PREDITIVA COM FOCO NO PROCESSAMENTO E INTEGRAÇÃO DE DADOS GEOESPACIAIS.</t>
+          <t>PROJETO BRA 23/023 - TR 140/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A AVALIAÇÃO DA OPERAÇÕES CENSITÁRIAS EM TERRAS INDÍGENAS DE RORAIMA.</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E13" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F13" s="21" t="n">
-        <v>0.481</v>
+        <v>0.378</v>
       </c>
       <c r="G13" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Logística / Operações</t>
         </is>
       </c>
       <c r="H13" s="19" t="inlineStr">
@@ -1649,13 +1649,13 @@
         </is>
       </c>
       <c r="J13" s="22" t="n">
-        <v>46287</v>
+        <v>46293</v>
       </c>
       <c r="K13" s="22" t="n">
-        <v>46296</v>
+        <v>46307</v>
       </c>
       <c r="L13" s="23" t="n">
-        <v>126500</v>
+        <v>91500</v>
       </c>
       <c r="M13" s="17" t="inlineStr">
         <is>
@@ -1680,29 +1680,29 @@
         </is>
       </c>
       <c r="B14" s="10" t="n">
-        <v>146382</v>
+        <v>146379</v>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 140/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A AVALIAÇÃO DA OPERAÇÕES CENSITÁRIAS EM TERRAS INDÍGENAS DE RORAIMA.</t>
+          <t>PROJETO BRA 23/023 - TR 132/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA ANÁLISE DOS MÉTODOS DE ROTEAMENTO PARA OPERAÇÕES DE PESQUISA EM CAMPO.</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.378</v>
+        <v>0.165</v>
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Logística / Operações</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Logística / Operações</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
@@ -1722,7 +1722,7 @@
         <v>46307</v>
       </c>
       <c r="L14" s="15" t="n">
-        <v>91500</v>
+        <v>121500</v>
       </c>
       <c r="M14" s="9" t="inlineStr">
         <is>
@@ -1747,11 +1747,11 @@
         </is>
       </c>
       <c r="B15" s="18" t="n">
-        <v>146379</v>
+        <v>146378</v>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 132/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA ANÁLISE DOS MÉTODOS DE ROTEAMENTO PARA OPERAÇÕES DE PESQUISA EM CAMPO.</t>
+          <t>PROJETO BRA 23/023 - TR 131/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE GEOPROCESSAMENTO.</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
@@ -1761,11 +1761,11 @@
       </c>
       <c r="E15" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F15" s="21" t="n">
-        <v>0.165</v>
+        <v>0.29</v>
       </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
@@ -1814,11 +1814,11 @@
         </is>
       </c>
       <c r="B16" s="10" t="n">
-        <v>146378</v>
+        <v>146377</v>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 131/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE GEOPROCESSAMENTO.</t>
+          <t>PROJETO BRA 23/023 - TR 130/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE CIÊNCIA DE DADOS E SENSORIAMENTO REMOTO.</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -1832,11 +1832,11 @@
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.29</v>
+        <v>0.224</v>
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Logística / Operações</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Cultura, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
@@ -1856,7 +1856,7 @@
         <v>46307</v>
       </c>
       <c r="L16" s="15" t="n">
-        <v>121500</v>
+        <v>93500</v>
       </c>
       <c r="M16" s="9" t="inlineStr">
         <is>
@@ -1881,11 +1881,11 @@
         </is>
       </c>
       <c r="B17" s="18" t="n">
-        <v>146377</v>
+        <v>146355</v>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 130/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE CIÊNCIA DE DADOS E SENSORIAMENTO REMOTO.</t>
+          <t>PROJETO BRA 23/023 - TR 119/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA DESENVOLVIMENTO DE PROPOSTA DE APRIMORAMENTO DO SISTEMA INTEGRADO DE PESQUISAS DOMICILIARES.</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1895,15 +1895,15 @@
       </c>
       <c r="E17" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F17" s="21" t="n">
-        <v>0.224</v>
+        <v>0.294</v>
       </c>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Cultura, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
@@ -1948,11 +1948,11 @@
         </is>
       </c>
       <c r="B18" s="10" t="n">
-        <v>146355</v>
+        <v>146376</v>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 119/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA DESENVOLVIMENTO DE PROPOSTA DE APRIMORAMENTO DO SISTEMA INTEGRADO DE PESQUISAS DOMICILIARES.</t>
+          <t>PROJETO BRA 23/023 - TR 116/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA MAPEAMENTO DE INOVAÇÕES NO PROCESSO DE PRODUÇÃO ESTATÍSTICA.</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -1962,15 +1962,15 @@
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.294</v>
+        <v>0.378</v>
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -1990,7 +1990,7 @@
         <v>46307</v>
       </c>
       <c r="L18" s="15" t="n">
-        <v>93500</v>
+        <v>86800</v>
       </c>
       <c r="M18" s="9" t="inlineStr">
         <is>
@@ -2015,11 +2015,11 @@
         </is>
       </c>
       <c r="B19" s="18" t="n">
-        <v>146376</v>
+        <v>146390</v>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 116/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA MAPEAMENTO DE INOVAÇÕES NO PROCESSO DE PRODUÇÃO ESTATÍSTICA.</t>
+          <t>BRA/24/018 - CONTRATAÇÃO DE CONSULTOR ESPECIALIZADO EM POLÍTICA DE INOVAÇÃO E DE TRANSFORMAÇÃO DIGITAL</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
@@ -2033,31 +2033,31 @@
         </is>
       </c>
       <c r="F19" s="21" t="n">
-        <v>0.378</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
         <is>
-          <t>IBGE</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I19" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Salvador/BA</t>
         </is>
       </c>
       <c r="J19" s="22" t="n">
-        <v>46293</v>
+        <v>46282</v>
       </c>
       <c r="K19" s="22" t="n">
-        <v>46307</v>
+        <v>46296</v>
       </c>
       <c r="L19" s="23" t="n">
-        <v>86800</v>
+        <v>49580</v>
       </c>
       <c r="M19" s="17" t="inlineStr">
         <is>
@@ -2066,7 +2066,7 @@
       </c>
       <c r="N19" s="20" t="inlineStr">
         <is>
-          <t>projetos.especiais@ibge.gov.br</t>
+          <t>selecaopnud0326@pge.ba.gov.br</t>
         </is>
       </c>
       <c r="O19" s="24" t="inlineStr">
@@ -2082,16 +2082,16 @@
         </is>
       </c>
       <c r="B20" s="10" t="n">
-        <v>146390</v>
+        <v>146394</v>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>BRA/24/018 - CONTRATAÇÃO DE CONSULTOR ESPECIALIZADO EM POLÍTICA DE INOVAÇÃO E DE TRANSFORMAÇÃO DIGITAL</t>
+          <t>Edital nº 30/2026 – Contratação de Consultoria Individual para realizar estudo de caso sobre a Secretaria de Serviços Compartilhados</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
@@ -2100,31 +2100,31 @@
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.5639999999999999</v>
+        <v>0.483</v>
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Ciência / Tecnologia e Inovação</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>MGI</t>
         </is>
       </c>
       <c r="I20" s="11" t="inlineStr">
         <is>
-          <t>Salvador/BA</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J20" s="14" t="n">
-        <v>46282</v>
+        <v>46289</v>
       </c>
       <c r="K20" s="14" t="n">
-        <v>46296</v>
+        <v>46304</v>
       </c>
       <c r="L20" s="15" t="n">
-        <v>49580</v>
+        <v>90000</v>
       </c>
       <c r="M20" s="9" t="inlineStr">
         <is>
@@ -2133,7 +2133,7 @@
       </c>
       <c r="N20" s="12" t="inlineStr">
         <is>
-          <t>selecaopnud0326@pge.ba.gov.br</t>
+          <t>prodoc.mgi@gestao.gov.br</t>
         </is>
       </c>
       <c r="O20" s="16" t="inlineStr">
@@ -2149,11 +2149,11 @@
         </is>
       </c>
       <c r="B21" s="18" t="n">
-        <v>146394</v>
+        <v>146396</v>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>Edital nº 30/2026 – Contratação de Consultoria Individual para realizar estudo de caso sobre a Secretaria de Serviços Compartilhados</t>
+          <t>BRA/25/024 - Edital nº 013/2026 – Contratação de consultoria especializada (pessoa física) para desenvolvimento de estudo e análise sobre os efeitos econômicos e sociais dos recursos mobilizados pelo FAT e pelo FGTS</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
@@ -2163,35 +2163,35 @@
       </c>
       <c r="E21" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F21" s="21" t="n">
-        <v>0.483</v>
+        <v>0.474</v>
       </c>
       <c r="G21" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>MTE</t>
         </is>
       </c>
       <c r="I21" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Brasília, com disponibilidade para viagens</t>
         </is>
       </c>
       <c r="J21" s="22" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="K21" s="22" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="L21" s="23" t="n">
-        <v>90000</v>
+        <v>208966.53</v>
       </c>
       <c r="M21" s="17" t="inlineStr">
         <is>
@@ -2200,7 +2200,7 @@
       </c>
       <c r="N21" s="20" t="inlineStr">
         <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
+          <t>selecao.spt@trabalho.gov.br</t>
         </is>
       </c>
       <c r="O21" s="24" t="inlineStr">
@@ -2212,15 +2212,17 @@
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B22" s="10" t="n">
-        <v>146396</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
+        </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>BRA/25/024 - Edital nº 013/2026 – Contratação de consultoria especializada (pessoa física) para desenvolvimento de estudo e análise sobre os efeitos econômicos e sociais dos recursos mobilizados pelo FAT e pelo FGTS</t>
+          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -2234,45 +2236,35 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.474</v>
+        <v>0.464</v>
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Arquitetura / Design</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
         <is>
-          <t>MTE</t>
-        </is>
-      </c>
-      <c r="I22" s="11" t="inlineStr">
-        <is>
-          <t>Brasília, com disponibilidade para viagens</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I22" s="11" t="inlineStr"/>
       <c r="J22" s="14" t="n">
-        <v>46290</v>
+        <v>46286</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46303</v>
-      </c>
-      <c r="L22" s="15" t="n">
-        <v>208966.53</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L22" s="15" t="inlineStr"/>
       <c r="M22" s="9" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N22" s="12" t="inlineStr">
-        <is>
-          <t>selecao.spt@trabalho.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N22" s="12" t="inlineStr"/>
       <c r="O22" s="16" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
@@ -2284,12 +2276,12 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
+          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
+          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
@@ -2307,7 +2299,7 @@
       </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Arquitetura / Design</t>
+          <t>Tecnologia da Informação / Dados, Ciências Sociais / Participação Social</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
@@ -2343,12 +2335,12 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
+          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
+          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -2362,11 +2354,11 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.464</v>
+        <v>0.423</v>
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Ciências Sociais / Participação Social</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
@@ -2402,12 +2394,12 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
+          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
+          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
@@ -2421,11 +2413,11 @@
         </is>
       </c>
       <c r="F25" s="21" t="n">
-        <v>0.423</v>
+        <v>0.464</v>
       </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Ciências Sociais / Participação Social</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
@@ -2461,12 +2453,12 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
+          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
+          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -2480,7 +2472,7 @@
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.464</v>
+        <v>0.423</v>
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
@@ -2520,12 +2512,12 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
+          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
+          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
@@ -2543,7 +2535,7 @@
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Ciências Sociais / Participação Social</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
@@ -2579,17 +2571,17 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
+          <t>unesco:ec486dce-4c41-4830-4e64-08df1817d7a0</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
+          <t>Projeto 914BRZ1085 - Edital nº 05/2026 - 02 vagas - Consultores Individuais</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr">
@@ -2598,11 +2590,11 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.423</v>
+        <v>0.3</v>
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Saúde, Estatística / Pesquisa / Metodologia, Cultura, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
@@ -2612,10 +2604,10 @@
       </c>
       <c r="I28" s="11" t="inlineStr"/>
       <c r="J28" s="14" t="n">
-        <v>46286</v>
+        <v>46296</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46316</v>
+        <v>46303</v>
       </c>
       <c r="L28" s="15" t="inlineStr"/>
       <c r="M28" s="9" t="inlineStr">
@@ -2638,17 +2630,17 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>unesco:31acdc9f-bf0b-43fe-5017-08df1966cd05</t>
+          <t>unesco:80185502-579b-44a1-e3c6-08df13ea9ffe</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1161.2 - Edital nº 01/2026 - 01 vaga - Consultor Individual</t>
+          <t>Projeto 914BRZ3051 - EDITAL 22/2026</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E29" s="20" t="inlineStr">
@@ -2657,11 +2649,11 @@
         </is>
       </c>
       <c r="F29" s="21" t="n">
-        <v>0.393</v>
+        <v>0.341</v>
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
@@ -2671,10 +2663,10 @@
       </c>
       <c r="I29" s="19" t="inlineStr"/>
       <c r="J29" s="22" t="n">
-        <v>46290</v>
+        <v>46292</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46295</v>
+        <v>46299</v>
       </c>
       <c r="L29" s="23" t="inlineStr"/>
       <c r="M29" s="17" t="inlineStr">
@@ -2692,22 +2684,22 @@
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>unesco:4d25520a-6684-41e6-3080-08df1a5635e8</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1161.2 - Edital nº 02/2026 - 01 vaga - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
@@ -2716,116 +2708,136 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.25</v>
+        <v>0.462</v>
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Cultura, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I30" s="11" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I30" s="11" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J30" s="14" t="n">
-        <v>46291</v>
+        <v>46240</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>46295</v>
-      </c>
-      <c r="L30" s="15" t="inlineStr"/>
+        <v>46245</v>
+      </c>
+      <c r="L30" s="15" t="n">
+        <v>80000</v>
+      </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N30" s="12" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N30" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>unesco:c0a1d55e-84e2-4c98-3081-08df1a5635e8</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1161.2 - Edital nº 03/2026 - 01 vaga - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E31" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F31" s="21" t="n">
-        <v>0.25</v>
+        <v>0.569</v>
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Cultura, Trabalho / Emprego, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I31" s="19" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I31" s="19" t="inlineStr">
+        <is>
+          <t>Brasília - Df</t>
+        </is>
+      </c>
       <c r="J31" s="22" t="n">
-        <v>46291</v>
+        <v>46240</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46295</v>
-      </c>
-      <c r="L31" s="23" t="inlineStr"/>
+        <v>46245</v>
+      </c>
+      <c r="L31" s="23" t="n">
+        <v>80000</v>
+      </c>
       <c r="M31" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N31" s="20" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N31" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>unesco:7f118a1a-eb71-48a2-e28d-08df14acbbca</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 40/2026 - 1 vaga - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E32" s="12" t="inlineStr">
@@ -2834,52 +2846,62 @@
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.585</v>
+        <v>0.492</v>
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Cultura, Desenvolvimento Social / Políticas Públicas</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I32" s="11" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I32" s="11" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J32" s="14" t="n">
-        <v>46289</v>
+        <v>46240</v>
       </c>
       <c r="K32" s="14" t="n">
-        <v>46295</v>
-      </c>
-      <c r="L32" s="15" t="inlineStr"/>
+        <v>46245</v>
+      </c>
+      <c r="L32" s="15" t="n">
+        <v>100000</v>
+      </c>
       <c r="M32" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N32" s="12" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N32" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>unesco:80185502-579b-44a1-e3c6-08df13ea9ffe</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ3051 - EDITAL 22/2026</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
@@ -2893,35 +2915,45 @@
         </is>
       </c>
       <c r="F33" s="21" t="n">
-        <v>0.341</v>
+        <v>0.433</v>
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I33" s="19" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I33" s="19" t="inlineStr">
+        <is>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+        </is>
+      </c>
       <c r="J33" s="22" t="n">
-        <v>46292</v>
+        <v>46227</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46299</v>
-      </c>
-      <c r="L33" s="23" t="inlineStr"/>
+        <v>46252</v>
+      </c>
+      <c r="L33" s="23" t="n">
+        <v>286000</v>
+      </c>
       <c r="M33" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N33" s="20" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N33" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
@@ -3002,12 +3034,12 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
@@ -3021,11 +3053,11 @@
         </is>
       </c>
       <c r="F35" s="21" t="n">
-        <v>0.462</v>
+        <v>0.481</v>
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Cultura, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
@@ -3045,7 +3077,7 @@
         <v>46245</v>
       </c>
       <c r="L35" s="23" t="n">
-        <v>80000</v>
+        <v>204000</v>
       </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
@@ -3059,7 +3091,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
         </is>
       </c>
     </row>
@@ -3071,12 +3103,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -3086,15 +3118,15 @@
       </c>
       <c r="E36" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>0.433</v>
+        <v>0.569</v>
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
@@ -3104,17 +3136,17 @@
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46227</v>
+        <v>46246</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46252</v>
+        <v>46257</v>
       </c>
       <c r="L36" s="15" t="n">
-        <v>286000</v>
+        <v>54000</v>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
@@ -3128,7 +3160,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -3140,12 +3172,12 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
@@ -3155,35 +3187,35 @@
       </c>
       <c r="E37" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F37" s="21" t="n">
-        <v>0.481</v>
+        <v>0.569</v>
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46245</v>
+        <v>46257</v>
       </c>
       <c r="L37" s="23" t="n">
-        <v>204000</v>
+        <v>54000</v>
       </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
@@ -3197,7 +3229,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -3209,12 +3241,12 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
@@ -3228,11 +3260,11 @@
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.569</v>
+        <v>0.492</v>
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Cultura, Trabalho / Emprego, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
@@ -3242,21 +3274,19 @@
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Brasília - Df</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46245</v>
-      </c>
-      <c r="L38" s="15" t="n">
-        <v>80000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L38" s="15" t="inlineStr"/>
       <c r="M38" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N38" s="12" t="inlineStr">
@@ -3266,7 +3296,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -3278,17 +3308,17 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E39" s="20" t="inlineStr">
@@ -3297,31 +3327,31 @@
         </is>
       </c>
       <c r="F39" s="21" t="n">
-        <v>0.492</v>
+        <v>0.593</v>
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Cultura, Desenvolvimento Social / Políticas Públicas</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46240</v>
+        <v>46251</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46245</v>
+        <v>46256</v>
       </c>
       <c r="L39" s="23" t="n">
-        <v>100000</v>
+        <v>50000</v>
       </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
@@ -3335,7 +3365,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -3347,12 +3377,12 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
@@ -3366,33 +3396,35 @@
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.492</v>
+        <v>0.46</v>
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Educação / Ensino</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46246</v>
+        <v>46252</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L40" s="15" t="inlineStr"/>
+        <v>46259</v>
+      </c>
+      <c r="L40" s="15" t="n">
+        <v>60000</v>
+      </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N40" s="12" t="inlineStr">
@@ -3402,7 +3434,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -3414,50 +3446,50 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E41" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F41" s="21" t="n">
-        <v>0.569</v>
+        <v>0.451</v>
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46246</v>
+        <v>46265</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46257</v>
+        <v>46270</v>
       </c>
       <c r="L41" s="23" t="n">
-        <v>54000</v>
+        <v>30000</v>
       </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
@@ -3471,7 +3503,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -3483,12 +3515,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3498,15 +3530,15 @@
       </c>
       <c r="E42" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.569</v>
+        <v>0.492</v>
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Educação / Ensino</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
@@ -3523,14 +3555,14 @@
         <v>46246</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46257</v>
+        <v>46272</v>
       </c>
       <c r="L42" s="15" t="n">
         <v>54000</v>
       </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N42" s="12" t="inlineStr">
@@ -3540,7 +3572,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -3552,64 +3584,64 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E43" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F43" s="21" t="n">
-        <v>0.46</v>
+        <v>0.464</v>
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46252</v>
+        <v>46208</v>
       </c>
       <c r="K43" s="22" t="n">
         <v>46259</v>
       </c>
       <c r="L43" s="23" t="n">
-        <v>60000</v>
+        <v>500000</v>
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N43" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -3621,17 +3653,17 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E44" s="12" t="inlineStr">
@@ -3640,11 +3672,11 @@
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>0.593</v>
+        <v>0.527</v>
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
@@ -3654,17 +3686,17 @@
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46251</v>
+        <v>46266</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46256</v>
+        <v>46288</v>
       </c>
       <c r="L44" s="15" t="n">
-        <v>50000</v>
+        <v>70000</v>
       </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
@@ -3678,7 +3710,7 @@
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
@@ -3690,64 +3722,64 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E45" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F45" s="21" t="n">
-        <v>0.464</v>
+        <v>0.3</v>
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46208</v>
+        <v>46275</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46259</v>
+        <v>46280</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>500000</v>
+        <v>50000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N45" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
@@ -3759,12 +3791,12 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -3774,15 +3806,15 @@
       </c>
       <c r="E46" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.451</v>
+        <v>0.493</v>
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Ciência / Tecnologia e Inovação, Engenharia / Infraestrutura</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
@@ -3792,17 +3824,17 @@
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Dados Remoto</t>
         </is>
       </c>
       <c r="J46" s="14" t="n">
-        <v>46265</v>
+        <v>46281</v>
       </c>
       <c r="K46" s="14" t="n">
-        <v>46270</v>
+        <v>46286</v>
       </c>
       <c r="L46" s="15" t="n">
-        <v>30000</v>
+        <v>110000</v>
       </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
@@ -3816,7 +3848,7 @@
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
         </is>
       </c>
     </row>
@@ -3828,12 +3860,12 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
@@ -3843,39 +3875,37 @@
       </c>
       <c r="E47" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F47" s="21" t="n">
-        <v>0.492</v>
+        <v>0.2</v>
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J47" s="22" t="n">
-        <v>46246</v>
+        <v>46275</v>
       </c>
       <c r="K47" s="22" t="n">
-        <v>46272</v>
-      </c>
-      <c r="L47" s="23" t="n">
-        <v>54000</v>
-      </c>
+        <v>46281</v>
+      </c>
+      <c r="L47" s="23" t="inlineStr"/>
       <c r="M47" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N47" s="20" t="inlineStr">
@@ -3885,7 +3915,7 @@
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
         </is>
       </c>
     </row>
@@ -3897,17 +3927,17 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E48" s="12" t="inlineStr">
@@ -3916,32 +3946,30 @@
         </is>
       </c>
       <c r="F48" s="13" t="n">
-        <v>0.527</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Trabalho / Emprego, Segurança</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J48" s="14" t="n">
-        <v>46266</v>
+        <v>46290</v>
       </c>
       <c r="K48" s="14" t="n">
-        <v>46288</v>
-      </c>
-      <c r="L48" s="15" t="n">
-        <v>70000</v>
-      </c>
+        <v>46294</v>
+      </c>
+      <c r="L48" s="15" t="inlineStr"/>
       <c r="M48" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3954,7 +3982,7 @@
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
         </is>
       </c>
     </row>
@@ -3966,12 +3994,12 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
@@ -3981,35 +4009,35 @@
       </c>
       <c r="E49" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F49" s="21" t="n">
-        <v>0.3</v>
+        <v>0.451</v>
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J49" s="22" t="n">
-        <v>46275</v>
+        <v>46282</v>
       </c>
       <c r="K49" s="22" t="n">
-        <v>46280</v>
+        <v>46286</v>
       </c>
       <c r="L49" s="23" t="n">
-        <v>50000</v>
+        <v>30000</v>
       </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
@@ -4023,7 +4051,7 @@
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
         </is>
       </c>
     </row>
@@ -4035,62 +4063,64 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E50" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>0.2</v>
+        <v>0.464</v>
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J50" s="14" t="n">
-        <v>46275</v>
+        <v>46244</v>
       </c>
       <c r="K50" s="14" t="n">
-        <v>46281</v>
-      </c>
-      <c r="L50" s="15" t="inlineStr"/>
+        <v>46300</v>
+      </c>
+      <c r="L50" s="15" t="n">
+        <v>350000</v>
+      </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N50" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -4102,17 +4132,17 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E51" s="20" t="inlineStr">
@@ -4121,45 +4151,43 @@
         </is>
       </c>
       <c r="F51" s="21" t="n">
-        <v>0.493</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Ciência / Tecnologia e Inovação, Engenharia / Infraestrutura</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>Dados Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
-        <v>46281</v>
+        <v>46278</v>
       </c>
       <c r="K51" s="22" t="n">
-        <v>46286</v>
-      </c>
-      <c r="L51" s="23" t="n">
-        <v>110000</v>
-      </c>
+        <v>46295</v>
+      </c>
+      <c r="L51" s="23" t="inlineStr"/>
       <c r="M51" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N51" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>ugp@educacao.sp.gov.br</t>
         </is>
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
         </is>
       </c>
     </row>
@@ -4171,12 +4199,12 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
+          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
+          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
@@ -4186,39 +4214,39 @@
       </c>
       <c r="E52" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F52" s="13" t="n">
-        <v>0.451</v>
+        <v>0.175</v>
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Engenharia / Infraestrutura</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Remota e/ou presencial em Brasília - DF</t>
         </is>
       </c>
       <c r="J52" s="14" t="n">
-        <v>46282</v>
+        <v>46294</v>
       </c>
       <c r="K52" s="14" t="n">
-        <v>46286</v>
+        <v>46297</v>
       </c>
       <c r="L52" s="15" t="n">
-        <v>30000</v>
+        <v>600000</v>
       </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N52" s="12" t="inlineStr">
@@ -4228,7 +4256,7 @@
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
         </is>
       </c>
     </row>
@@ -4240,17 +4268,17 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E53" s="20" t="inlineStr">
@@ -4259,30 +4287,32 @@
         </is>
       </c>
       <c r="F53" s="21" t="n">
-        <v>0.5639999999999999</v>
+        <v>0.232</v>
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Trabalho / Emprego, Segurança</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
-        <v>46290</v>
+        <v>46293</v>
       </c>
       <c r="K53" s="22" t="n">
-        <v>46294</v>
-      </c>
-      <c r="L53" s="23" t="inlineStr"/>
+        <v>46298</v>
+      </c>
+      <c r="L53" s="23" t="n">
+        <v>30000</v>
+      </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -4295,7 +4325,7 @@
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
         </is>
       </c>
     </row>
@@ -4307,12 +4337,12 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
@@ -4322,15 +4352,15 @@
       </c>
       <c r="E54" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F54" s="13" t="n">
-        <v>0.5639999999999999</v>
+        <v>0.2</v>
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Educação / Ensino, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Direitos Humanos / Cidadania</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
@@ -4340,29 +4370,31 @@
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Articulação Estadual - Rio Grande do Norte</t>
         </is>
       </c>
       <c r="J54" s="14" t="n">
-        <v>46278</v>
+        <v>46293</v>
       </c>
       <c r="K54" s="14" t="n">
-        <v>46295</v>
-      </c>
-      <c r="L54" s="15" t="inlineStr"/>
+        <v>46298</v>
+      </c>
+      <c r="L54" s="15" t="n">
+        <v>21000</v>
+      </c>
       <c r="M54" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N54" s="12" t="inlineStr">
         <is>
-          <t>ugp@educacao.sp.gov.br</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O54" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
         </is>
       </c>
     </row>
@@ -4374,64 +4406,64 @@
       </c>
       <c r="B55" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
         </is>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E55" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Não Classificado</t>
         </is>
       </c>
       <c r="F55" s="21" t="n">
-        <v>0.493</v>
+        <v>0.077</v>
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Desenvolvimento Social / Políticas Públicas</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J55" s="22" t="n">
-        <v>46244</v>
+        <v>46294</v>
       </c>
       <c r="K55" s="22" t="n">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="L55" s="23" t="n">
-        <v>935000</v>
+        <v>55000</v>
       </c>
       <c r="M55" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N55" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O55" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
         </is>
       </c>
     </row>
@@ -4443,64 +4475,64 @@
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E56" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F56" s="13" t="n">
-        <v>0.464</v>
+        <v>0.355</v>
       </c>
       <c r="G56" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Educação / Ensino</t>
         </is>
       </c>
       <c r="H56" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I56" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J56" s="14" t="n">
-        <v>46244</v>
+        <v>46294</v>
       </c>
       <c r="K56" s="14" t="n">
-        <v>46300</v>
+        <v>46302</v>
       </c>
       <c r="L56" s="15" t="n">
-        <v>350000</v>
+        <v>60000</v>
       </c>
       <c r="M56" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N56" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O56" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
         </is>
       </c>
     </row>
@@ -4512,12 +4544,12 @@
       </c>
       <c r="B57" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
         </is>
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
         </is>
       </c>
       <c r="D57" s="19" t="inlineStr">
@@ -4527,39 +4559,39 @@
       </c>
       <c r="E57" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F57" s="21" t="n">
-        <v>0.2</v>
+        <v>0.333</v>
       </c>
       <c r="G57" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Educação / Ensino, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Direitos Humanos / Cidadania</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Cultura, Segurança, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H57" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I57" s="19" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Rio Grande do Norte</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J57" s="22" t="n">
-        <v>46293</v>
+        <v>46296</v>
       </c>
       <c r="K57" s="22" t="n">
-        <v>46298</v>
+        <v>46300</v>
       </c>
       <c r="L57" s="23" t="n">
-        <v>21000</v>
+        <v>60000</v>
       </c>
       <c r="M57" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N57" s="20" t="inlineStr">
@@ -4569,7 +4601,7 @@
       </c>
       <c r="O57" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
         </is>
       </c>
     </row>
@@ -4581,12 +4613,12 @@
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
@@ -4600,35 +4632,35 @@
         </is>
       </c>
       <c r="F58" s="13" t="n">
-        <v>0.175</v>
+        <v>0.282</v>
       </c>
       <c r="G58" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Engenharia / Infraestrutura</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
         </is>
       </c>
       <c r="H58" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I58" s="11" t="inlineStr">
         <is>
-          <t>Remota e/ou presencial em Brasília - DF</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J58" s="14" t="n">
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="K58" s="14" t="n">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="L58" s="15" t="n">
-        <v>600000</v>
+        <v>60000</v>
       </c>
       <c r="M58" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N58" s="12" t="inlineStr">
@@ -4638,7 +4670,7 @@
       </c>
       <c r="O58" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
         </is>
       </c>
     </row>
@@ -4650,12 +4682,12 @@
       </c>
       <c r="B59" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
         </is>
       </c>
       <c r="C59" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
         </is>
       </c>
       <c r="D59" s="19" t="inlineStr">
@@ -4665,35 +4697,35 @@
       </c>
       <c r="E59" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F59" s="21" t="n">
-        <v>0.232</v>
+        <v>0.216</v>
       </c>
       <c r="G59" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
+          <t>Tecnologia da Informação / Dados, Cultura, Comunicação, Arquitetura / Design</t>
         </is>
       </c>
       <c r="H59" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I59" s="19" t="inlineStr">
         <is>
-          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J59" s="22" t="n">
-        <v>46293</v>
+        <v>46296</v>
       </c>
       <c r="K59" s="22" t="n">
-        <v>46298</v>
+        <v>46300</v>
       </c>
       <c r="L59" s="23" t="n">
-        <v>30000</v>
+        <v>33000</v>
       </c>
       <c r="M59" s="17" t="inlineStr">
         <is>
@@ -4707,7 +4739,7 @@
       </c>
       <c r="O59" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
         </is>
       </c>
     </row>
@@ -4719,12 +4751,12 @@
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
         </is>
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
         </is>
       </c>
       <c r="D60" s="11" t="inlineStr">
@@ -4734,35 +4766,35 @@
       </c>
       <c r="E60" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F60" s="13" t="n">
-        <v>0.077</v>
+        <v>0.378</v>
       </c>
       <c r="G60" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Cultura, Comunicação</t>
         </is>
       </c>
       <c r="H60" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I60" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J60" s="14" t="n">
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="K60" s="14" t="n">
         <v>46300</v>
       </c>
       <c r="L60" s="15" t="n">
-        <v>55000</v>
+        <v>36000</v>
       </c>
       <c r="M60" s="9" t="inlineStr">
         <is>
@@ -4776,7 +4808,7 @@
       </c>
       <c r="O60" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
         </is>
       </c>
     </row>
@@ -4788,12 +4820,12 @@
       </c>
       <c r="B61" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
         </is>
       </c>
       <c r="C61" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
         </is>
       </c>
       <c r="D61" s="19" t="inlineStr">
@@ -4803,54 +4835,123 @@
       </c>
       <c r="E61" s="20" t="inlineStr">
         <is>
+          <t>Consultoria Diversidade Inclusao</t>
+        </is>
+      </c>
+      <c r="F61" s="21" t="n">
+        <v>0.178</v>
+      </c>
+      <c r="G61" s="19" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Cultura, Comunicação</t>
+        </is>
+      </c>
+      <c r="H61" s="19" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I61" s="19" t="inlineStr">
+        <is>
+          <t>Vitória - ES</t>
+        </is>
+      </c>
+      <c r="J61" s="22" t="n">
+        <v>46296</v>
+      </c>
+      <c r="K61" s="22" t="n">
+        <v>46300</v>
+      </c>
+      <c r="L61" s="23" t="n">
+        <v>21000</v>
+      </c>
+      <c r="M61" s="17" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N61" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O61" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="9" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B62" s="10" t="inlineStr">
+        <is>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+        </is>
+      </c>
+      <c r="C62" s="11" t="inlineStr">
+        <is>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+        </is>
+      </c>
+      <c r="D62" s="11" t="inlineStr">
+        <is>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+        </is>
+      </c>
+      <c r="E62" s="12" t="inlineStr">
+        <is>
           <t>Engenharia Processos Analytics</t>
         </is>
       </c>
-      <c r="F61" s="21" t="n">
-        <v>0.355</v>
-      </c>
-      <c r="G61" s="19" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Educação / Ensino</t>
-        </is>
-      </c>
-      <c r="H61" s="19" t="inlineStr">
-        <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I61" s="19" t="inlineStr">
-        <is>
-          <t>São Paulo - SP</t>
-        </is>
-      </c>
-      <c r="J61" s="22" t="n">
-        <v>46294</v>
-      </c>
-      <c r="K61" s="22" t="n">
-        <v>46302</v>
-      </c>
-      <c r="L61" s="23" t="n">
-        <v>60000</v>
-      </c>
-      <c r="M61" s="17" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N61" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O61" s="24" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
+      <c r="F62" s="13" t="n">
+        <v>0.493</v>
+      </c>
+      <c r="G62" s="11" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Desenvolvimento Social / Políticas Públicas</t>
+        </is>
+      </c>
+      <c r="H62" s="11" t="inlineStr">
+        <is>
+          <t>OEI/MDHC</t>
+        </is>
+      </c>
+      <c r="I62" s="11" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="J62" s="14" t="n">
+        <v>46244</v>
+      </c>
+      <c r="K62" s="14" t="n">
+        <v>46296</v>
+      </c>
+      <c r="L62" s="15" t="n">
+        <v>935000</v>
+      </c>
+      <c r="M62" s="9" t="inlineStr">
+        <is>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N62" s="12" t="inlineStr">
+        <is>
+          <t>compras.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O62" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O61"/>
+  <autoFilter ref="A1:O62"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -4912,6 +5013,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId59"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId61"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -4950,7 +5052,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3">
@@ -4960,7 +5062,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4">
@@ -4970,7 +5072,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -5022,7 +5124,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4">
@@ -5070,21 +5172,21 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4">
@@ -5146,7 +5248,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3">
@@ -5156,7 +5258,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4">
@@ -5166,13 +5268,13 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
-          <t>Educação / Ensino</t>
+          <t>Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="B5" s="18" t="n">
@@ -5186,47 +5288,47 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>Ciência / Tecnologia e Inovação</t>
+          <t>Cultura</t>
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>Desenvolvimento Social / Políticas Públicas</t>
+          <t>Educação / Ensino</t>
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="19" t="inlineStr">
         <is>
-          <t>Ciências Sociais / Participação Social</t>
+          <t>Desenvolvimento Social / Políticas Públicas</t>
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>Cultura</t>
+          <t>Ciências Sociais / Participação Social</t>
         </is>
       </c>
       <c r="B10" s="10" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11">
@@ -5236,7 +5338,7 @@
         </is>
       </c>
       <c r="B11" s="18" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -5274,27 +5376,27 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>IBGE</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>IBGE</t>
         </is>
       </c>
       <c r="B4" s="10" t="n">
@@ -5308,7 +5410,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6">
@@ -5318,7 +5420,7 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -5411,7 +5513,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-10-03 16:07
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$56</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 01/10/2026 às 18:27</t>
+          <t>Gerado em 03/10/2026 às 16:06</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>61</v>
+        <v>55</v>
       </c>
     </row>
     <row r="6">
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="17">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>123620.4878048781</v>
+        <v>121990.5263157895</v>
       </c>
     </row>
     <row r="20">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>86800</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
@@ -730,21 +730,21 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="25">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O62"/>
+  <dimension ref="A1:O56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -876,11 +876,11 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>146370</v>
+        <v>146374</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edital nº 25/2026 – Contratação de Consultoria Individual para avaliar os efeitos de intervenções comportamentais (políticas fiscais e de arquitetura de escolha) em mercado experimental para promover escolhas alimentares mais saudáveis. </t>
+          <t>Edital nº 27/2026 – Contratação de Consultoria Individual II - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Servidões de Passagem para Orlas e Praias</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
@@ -894,11 +894,11 @@
         </is>
       </c>
       <c r="F2" s="13" t="n">
-        <v>0.411</v>
+        <v>0.494</v>
       </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>Arquitetura / Design</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H2" s="11" t="inlineStr">
@@ -908,17 +908,17 @@
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>REMOTO</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J2" s="14" t="n">
-        <v>46276</v>
+        <v>46280</v>
       </c>
       <c r="K2" s="14" t="n">
-        <v>46297</v>
+        <v>46310</v>
       </c>
       <c r="L2" s="15" t="n">
-        <v>126000</v>
+        <v>120000</v>
       </c>
       <c r="M2" s="9" t="inlineStr">
         <is>
@@ -943,11 +943,11 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>146374</v>
+        <v>146375</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
-          <t>Edital nº 27/2026 – Contratação de Consultoria Individual II - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Servidões de Passagem para Orlas e Praias</t>
+          <t>Edital nº 28/2026 - Contratação de Consultoria Individual I - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Acessibilidade em Orlas e Praias</t>
         </is>
       </c>
       <c r="D3" s="19" t="inlineStr">
@@ -975,7 +975,7 @@
       </c>
       <c r="I3" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>REMOTO</t>
         </is>
       </c>
       <c r="J3" s="22" t="n">
@@ -1010,11 +1010,11 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>146375</v>
+        <v>146385</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>Edital nº 28/2026 - Contratação de Consultoria Individual I - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Acessibilidade em Orlas e Praias</t>
+          <t>Contratação de consultor para elaborar o Caderno Temático de Referência: Investigação de Crimes contra Jornalistas e Comunicadores</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
@@ -1028,7 +1028,7 @@
         </is>
       </c>
       <c r="F4" s="13" t="n">
-        <v>0.494</v>
+        <v>0.407</v>
       </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
@@ -1037,22 +1037,22 @@
       </c>
       <c r="H4" s="11" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>REMOTO</t>
+          <t>Home-based</t>
         </is>
       </c>
       <c r="J4" s="14" t="n">
-        <v>46280</v>
+        <v>46289</v>
       </c>
       <c r="K4" s="14" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="L4" s="15" t="n">
-        <v>120000</v>
+        <v>100000</v>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
@@ -1061,7 +1061,7 @@
       </c>
       <c r="N4" s="12" t="inlineStr">
         <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
+          <t>prodocbra016@mj.gov.br</t>
         </is>
       </c>
       <c r="O4" s="16" t="inlineStr">
@@ -1077,49 +1077,49 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>146384</v>
+        <v>146354</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t>Edital 05/2026 - Estudos e análises para o fortalecimento da perspectiva de gênero nas políticas públicas de direitos humanos</t>
+          <t>PROJETO BRA 23/023 - TR 88/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA PROPOSIÇÃO DE SOLUÇÕES DE CIÊNCIA DE DADOS EM SENSORIAMENTO REMOTO.</t>
         </is>
       </c>
       <c r="D5" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E5" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F5" s="21" t="n">
-        <v>0.116</v>
+        <v>0.411</v>
       </c>
       <c r="G5" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Desenvolvimento Social / Políticas Públicas, Direitos Humanos / Cidadania</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H5" s="19" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>IBGE</t>
         </is>
       </c>
       <c r="I5" s="19" t="inlineStr">
         <is>
-          <t>Território Nacional</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J5" s="22" t="n">
-        <v>46283</v>
+        <v>46293</v>
       </c>
       <c r="K5" s="22" t="n">
-        <v>46296</v>
+        <v>46307</v>
       </c>
       <c r="L5" s="23" t="n">
-        <v>120000</v>
+        <v>93500</v>
       </c>
       <c r="M5" s="17" t="inlineStr">
         <is>
@@ -1128,7 +1128,7 @@
       </c>
       <c r="N5" s="20" t="inlineStr">
         <is>
-          <t>dirp@mdh.gov.br</t>
+          <t>projetos.especiais@ibge.gov.br</t>
         </is>
       </c>
       <c r="O5" s="24" t="inlineStr">
@@ -1144,11 +1144,11 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>146385</v>
+        <v>146382</v>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor para elaborar o Caderno Temático de Referência: Investigação de Crimes contra Jornalistas e Comunicadores</t>
+          <t>PROJETO BRA 23/023 - TR 140/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A AVALIAÇÃO DA OPERAÇÕES CENSITÁRIAS EM TERRAS INDÍGENAS DE RORAIMA.</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
@@ -1158,35 +1158,35 @@
       </c>
       <c r="E6" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.407</v>
+        <v>0.378</v>
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Logística / Operações</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>IBGE</t>
         </is>
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>Home-based</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J6" s="14" t="n">
-        <v>46289</v>
+        <v>46293</v>
       </c>
       <c r="K6" s="14" t="n">
-        <v>46311</v>
+        <v>46307</v>
       </c>
       <c r="L6" s="15" t="n">
-        <v>100000</v>
+        <v>91500</v>
       </c>
       <c r="M6" s="9" t="inlineStr">
         <is>
@@ -1195,7 +1195,7 @@
       </c>
       <c r="N6" s="12" t="inlineStr">
         <is>
-          <t>prodocbra016@mj.gov.br</t>
+          <t>projetos.especiais@ibge.gov.br</t>
         </is>
       </c>
       <c r="O6" s="16" t="inlineStr">
@@ -1211,29 +1211,29 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>146380</v>
+        <v>146379</v>
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 138/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A PROPOSIÇÃO DE PLATAFORMAS E DASHBOARDS DE VISUALIZAÇÃO DE DADOS PARA A AGENDA DE DESENVOLVIMENTO HUMANO</t>
+          <t>PROJETO BRA 23/023 - TR 132/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA ANÁLISE DOS MÉTODOS DE ROTEAMENTO PARA OPERAÇÕES DE PESQUISA EM CAMPO.</t>
         </is>
       </c>
       <c r="D7" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E7" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F7" s="21" t="n">
-        <v>0.511</v>
+        <v>0.165</v>
       </c>
       <c r="G7" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Logística / Operações</t>
         </is>
       </c>
       <c r="H7" s="19" t="inlineStr">
@@ -1247,13 +1247,13 @@
         </is>
       </c>
       <c r="J7" s="22" t="n">
-        <v>46287</v>
+        <v>46293</v>
       </c>
       <c r="K7" s="22" t="n">
-        <v>46296</v>
+        <v>46307</v>
       </c>
       <c r="L7" s="23" t="n">
-        <v>126500</v>
+        <v>121500</v>
       </c>
       <c r="M7" s="17" t="inlineStr">
         <is>
@@ -1278,29 +1278,29 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>146381</v>
+        <v>146378</v>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 139/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A SISTEMATIZAÇÃO E ELABORAÇÃO DO DOSSIÊ INSTITUCIONAL DA SÉRIE DIÁLOGOS NACIONAIS PARA O DESENVOLVIMENTO.</t>
+          <t>PROJETO BRA 23/023 - TR 131/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE GEOPROCESSAMENTO.</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E8" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.464</v>
+        <v>0.29</v>
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Logística / Operações</t>
         </is>
       </c>
       <c r="H8" s="11" t="inlineStr">
@@ -1314,13 +1314,13 @@
         </is>
       </c>
       <c r="J8" s="14" t="n">
-        <v>46287</v>
+        <v>46293</v>
       </c>
       <c r="K8" s="14" t="n">
-        <v>46296</v>
+        <v>46307</v>
       </c>
       <c r="L8" s="15" t="n">
-        <v>126500</v>
+        <v>121500</v>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
@@ -1345,29 +1345,29 @@
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>146383</v>
+        <v>146377</v>
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 145/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA DESENVOLVIMENTO DE PROPOSTA DE ALGORITMO DE GEOCODIFICAÇÃO DE ENDEREÇOS BRASILEIROS.</t>
+          <t>PROJETO BRA 23/023 - TR 130/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE CIÊNCIA DE DADOS E SENSORIAMENTO REMOTO.</t>
         </is>
       </c>
       <c r="D9" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E9" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F9" s="21" t="n">
-        <v>0.462</v>
+        <v>0.224</v>
       </c>
       <c r="G9" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Cultura, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H9" s="19" t="inlineStr">
@@ -1381,13 +1381,13 @@
         </is>
       </c>
       <c r="J9" s="22" t="n">
-        <v>46287</v>
+        <v>46293</v>
       </c>
       <c r="K9" s="22" t="n">
-        <v>46296</v>
+        <v>46307</v>
       </c>
       <c r="L9" s="23" t="n">
-        <v>86800</v>
+        <v>93500</v>
       </c>
       <c r="M9" s="17" t="inlineStr">
         <is>
@@ -1412,11 +1412,11 @@
         </is>
       </c>
       <c r="B10" s="10" t="n">
-        <v>146354</v>
+        <v>146355</v>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 88/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA PROPOSIÇÃO DE SOLUÇÕES DE CIÊNCIA DE DADOS EM SENSORIAMENTO REMOTO.</t>
+          <t>PROJETO BRA 23/023 - TR 119/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA DESENVOLVIMENTO DE PROPOSTA DE APRIMORAMENTO DO SISTEMA INTEGRADO DE PESQUISAS DOMICILIARES.</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
@@ -1426,15 +1426,15 @@
       </c>
       <c r="E10" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.411</v>
+        <v>0.294</v>
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
@@ -1479,11 +1479,11 @@
         </is>
       </c>
       <c r="B11" s="18" t="n">
-        <v>146357</v>
+        <v>146376</v>
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 141/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE METODOLOGIA DE MODELAGEM PREDITIVA PARA ANÁLISE TERRITORIAL DO DESENVOLVIMENTO HUMANO.</t>
+          <t>PROJETO BRA 23/023 - TR 116/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA MAPEAMENTO DE INOVAÇÕES NO PROCESSO DE PRODUÇÃO ESTATÍSTICA.</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
@@ -1493,15 +1493,15 @@
       </c>
       <c r="E11" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F11" s="21" t="n">
-        <v>0.464</v>
+        <v>0.378</v>
       </c>
       <c r="G11" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H11" s="19" t="inlineStr">
@@ -1515,13 +1515,13 @@
         </is>
       </c>
       <c r="J11" s="22" t="n">
-        <v>46287</v>
+        <v>46293</v>
       </c>
       <c r="K11" s="22" t="n">
-        <v>46296</v>
+        <v>46307</v>
       </c>
       <c r="L11" s="23" t="n">
-        <v>126500</v>
+        <v>86800</v>
       </c>
       <c r="M11" s="17" t="inlineStr">
         <is>
@@ -1546,34 +1546,34 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>146358</v>
+        <v>146394</v>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 142/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE METODOLOGIA DE MODELAGEM PREDITIVA COM FOCO NO PROCESSAMENTO E INTEGRAÇÃO DE DADOS GEOESPACIAIS.</t>
+          <t>Edital nº 30/2026 – Contratação de Consultoria Individual para realizar estudo de caso sobre a Secretaria de Serviços Compartilhados</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E12" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.481</v>
+        <v>0.483</v>
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>IBGE</t>
+          <t>MGI</t>
         </is>
       </c>
       <c r="I12" s="11" t="inlineStr">
@@ -1582,13 +1582,13 @@
         </is>
       </c>
       <c r="J12" s="14" t="n">
-        <v>46287</v>
+        <v>46289</v>
       </c>
       <c r="K12" s="14" t="n">
-        <v>46296</v>
+        <v>46304</v>
       </c>
       <c r="L12" s="15" t="n">
-        <v>126500</v>
+        <v>90000</v>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
@@ -1597,7 +1597,7 @@
       </c>
       <c r="N12" s="12" t="inlineStr">
         <is>
-          <t>projetos.especiais@ibge.gov.br</t>
+          <t>prodoc.mgi@gestao.gov.br</t>
         </is>
       </c>
       <c r="O12" s="16" t="inlineStr">
@@ -1613,11 +1613,11 @@
         </is>
       </c>
       <c r="B13" s="18" t="n">
-        <v>146382</v>
+        <v>146396</v>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 140/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A AVALIAÇÃO DA OPERAÇÕES CENSITÁRIAS EM TERRAS INDÍGENAS DE RORAIMA.</t>
+          <t>BRA/25/024 - Edital nº 013/2026 – Contratação de consultoria especializada (pessoa física) para desenvolvimento de estudo e análise sobre os efeitos econômicos e sociais dos recursos mobilizados pelo FAT e pelo FGTS</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
@@ -1627,35 +1627,35 @@
       </c>
       <c r="E13" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F13" s="21" t="n">
-        <v>0.378</v>
+        <v>0.474</v>
       </c>
       <c r="G13" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Logística / Operações</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H13" s="19" t="inlineStr">
         <is>
-          <t>IBGE</t>
+          <t>MTE</t>
         </is>
       </c>
       <c r="I13" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Brasília, com disponibilidade para viagens</t>
         </is>
       </c>
       <c r="J13" s="22" t="n">
-        <v>46293</v>
+        <v>46290</v>
       </c>
       <c r="K13" s="22" t="n">
-        <v>46307</v>
+        <v>46303</v>
       </c>
       <c r="L13" s="23" t="n">
-        <v>91500</v>
+        <v>208966.53</v>
       </c>
       <c r="M13" s="17" t="inlineStr">
         <is>
@@ -1664,7 +1664,7 @@
       </c>
       <c r="N13" s="20" t="inlineStr">
         <is>
-          <t>projetos.especiais@ibge.gov.br</t>
+          <t>selecao.spt@trabalho.gov.br</t>
         </is>
       </c>
       <c r="O13" s="24" t="inlineStr">
@@ -1676,20 +1676,22 @@
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="n">
-        <v>146379</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
+        </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 132/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA ANÁLISE DOS MÉTODOS DE ROTEAMENTO PARA OPERAÇÕES DE PESQUISA EM CAMPO.</t>
+          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E14" s="12" t="inlineStr">
@@ -1698,199 +1700,175 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.165</v>
+        <v>0.464</v>
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Logística / Operações</t>
+          <t>Arquitetura / Design</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
         <is>
-          <t>IBGE</t>
-        </is>
-      </c>
-      <c r="I14" s="11" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I14" s="11" t="inlineStr"/>
       <c r="J14" s="14" t="n">
-        <v>46293</v>
+        <v>46286</v>
       </c>
       <c r="K14" s="14" t="n">
-        <v>46307</v>
-      </c>
-      <c r="L14" s="15" t="n">
-        <v>121500</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L14" s="15" t="inlineStr"/>
       <c r="M14" s="9" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N14" s="12" t="inlineStr">
-        <is>
-          <t>projetos.especiais@ibge.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N14" s="12" t="inlineStr"/>
       <c r="O14" s="16" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="17" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B15" s="18" t="n">
-        <v>146378</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
+        </is>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 131/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE GEOPROCESSAMENTO.</t>
+          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E15" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F15" s="21" t="n">
-        <v>0.29</v>
+        <v>0.464</v>
       </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Logística / Operações</t>
+          <t>Tecnologia da Informação / Dados, Ciências Sociais / Participação Social</t>
         </is>
       </c>
       <c r="H15" s="19" t="inlineStr">
         <is>
-          <t>IBGE</t>
-        </is>
-      </c>
-      <c r="I15" s="19" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I15" s="19" t="inlineStr"/>
       <c r="J15" s="22" t="n">
-        <v>46293</v>
+        <v>46286</v>
       </c>
       <c r="K15" s="22" t="n">
-        <v>46307</v>
-      </c>
-      <c r="L15" s="23" t="n">
-        <v>121500</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L15" s="23" t="inlineStr"/>
       <c r="M15" s="17" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N15" s="20" t="inlineStr">
-        <is>
-          <t>projetos.especiais@ibge.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N15" s="20" t="inlineStr"/>
       <c r="O15" s="24" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B16" s="10" t="n">
-        <v>146377</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
+        </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 130/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE CIÊNCIA DE DADOS E SENSORIAMENTO REMOTO.</t>
+          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E16" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.224</v>
+        <v>0.423</v>
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Cultura, Ciência / Tecnologia e Inovação</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
         <is>
-          <t>IBGE</t>
-        </is>
-      </c>
-      <c r="I16" s="11" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I16" s="11" t="inlineStr"/>
       <c r="J16" s="14" t="n">
-        <v>46293</v>
+        <v>46286</v>
       </c>
       <c r="K16" s="14" t="n">
-        <v>46307</v>
-      </c>
-      <c r="L16" s="15" t="n">
-        <v>93500</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L16" s="15" t="inlineStr"/>
       <c r="M16" s="9" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N16" s="12" t="inlineStr">
-        <is>
-          <t>projetos.especiais@ibge.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N16" s="12" t="inlineStr"/>
       <c r="O16" s="16" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="17" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B17" s="18" t="n">
-        <v>146355</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
+        </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 119/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA DESENVOLVIMENTO DE PROPOSTA DE APRIMORAMENTO DO SISTEMA INTEGRADO DE PESQUISAS DOMICILIARES.</t>
+          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E17" s="20" t="inlineStr">
@@ -1899,266 +1877,234 @@
         </is>
       </c>
       <c r="F17" s="21" t="n">
-        <v>0.294</v>
+        <v>0.464</v>
       </c>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Ciências Sociais / Participação Social</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
         <is>
-          <t>IBGE</t>
-        </is>
-      </c>
-      <c r="I17" s="19" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I17" s="19" t="inlineStr"/>
       <c r="J17" s="22" t="n">
-        <v>46293</v>
+        <v>46286</v>
       </c>
       <c r="K17" s="22" t="n">
-        <v>46307</v>
-      </c>
-      <c r="L17" s="23" t="n">
-        <v>93500</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L17" s="23" t="inlineStr"/>
       <c r="M17" s="17" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N17" s="20" t="inlineStr">
-        <is>
-          <t>projetos.especiais@ibge.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N17" s="20" t="inlineStr"/>
       <c r="O17" s="24" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B18" s="10" t="n">
-        <v>146376</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
+        </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 116/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA MAPEAMENTO DE INOVAÇÕES NO PROCESSO DE PRODUÇÃO ESTATÍSTICA.</t>
+          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.378</v>
+        <v>0.423</v>
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Ciências Sociais / Participação Social</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
         <is>
-          <t>IBGE</t>
-        </is>
-      </c>
-      <c r="I18" s="11" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I18" s="11" t="inlineStr"/>
       <c r="J18" s="14" t="n">
-        <v>46293</v>
+        <v>46286</v>
       </c>
       <c r="K18" s="14" t="n">
-        <v>46307</v>
-      </c>
-      <c r="L18" s="15" t="n">
-        <v>86800</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L18" s="15" t="inlineStr"/>
       <c r="M18" s="9" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N18" s="12" t="inlineStr">
-        <is>
-          <t>projetos.especiais@ibge.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N18" s="12" t="inlineStr"/>
       <c r="O18" s="16" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="17" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B19" s="18" t="n">
-        <v>146390</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
+        </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>BRA/24/018 - CONTRATAÇÃO DE CONSULTOR ESPECIALIZADO EM POLÍTICA DE INOVAÇÃO E DE TRANSFORMAÇÃO DIGITAL</t>
+          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E19" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F19" s="21" t="n">
-        <v>0.5639999999999999</v>
+        <v>0.423</v>
       </c>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Ciência / Tecnologia e Inovação</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
         <is>
-          <t>Não identificado</t>
-        </is>
-      </c>
-      <c r="I19" s="19" t="inlineStr">
-        <is>
-          <t>Salvador/BA</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I19" s="19" t="inlineStr"/>
       <c r="J19" s="22" t="n">
-        <v>46282</v>
+        <v>46286</v>
       </c>
       <c r="K19" s="22" t="n">
-        <v>46296</v>
-      </c>
-      <c r="L19" s="23" t="n">
-        <v>49580</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L19" s="23" t="inlineStr"/>
       <c r="M19" s="17" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N19" s="20" t="inlineStr">
-        <is>
-          <t>selecaopnud0326@pge.ba.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N19" s="20" t="inlineStr"/>
       <c r="O19" s="24" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B20" s="10" t="n">
-        <v>146394</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>unesco:ec486dce-4c41-4830-4e64-08df1817d7a0</t>
+        </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>Edital nº 30/2026 – Contratação de Consultoria Individual para realizar estudo de caso sobre a Secretaria de Serviços Compartilhados</t>
+          <t>Projeto 914BRZ1085 - Edital nº 05/2026 - 02 vagas - Consultores Individuais</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.483</v>
+        <v>0.3</v>
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Saúde, Estatística / Pesquisa / Metodologia, Cultura, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>MGI</t>
-        </is>
-      </c>
-      <c r="I20" s="11" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="inlineStr"/>
       <c r="J20" s="14" t="n">
-        <v>46289</v>
+        <v>46296</v>
       </c>
       <c r="K20" s="14" t="n">
-        <v>46304</v>
-      </c>
-      <c r="L20" s="15" t="n">
-        <v>90000</v>
-      </c>
+        <v>46303</v>
+      </c>
+      <c r="L20" s="15" t="inlineStr"/>
       <c r="M20" s="9" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N20" s="12" t="inlineStr">
-        <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N20" s="12" t="inlineStr"/>
       <c r="O20" s="16" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="17" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B21" s="18" t="n">
-        <v>146396</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>unesco:80185502-579b-44a1-e3c6-08df13ea9ffe</t>
+        </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>BRA/25/024 - Edital nº 013/2026 – Contratação de consultoria especializada (pessoa física) para desenvolvimento de estudo e análise sobre os efeitos econômicos e sociais dos recursos mobilizados pelo FAT e pelo FGTS</t>
+          <t>Projeto 914BRZ3051 - EDITAL 22/2026</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E21" s="20" t="inlineStr">
@@ -2167,67 +2113,57 @@
         </is>
       </c>
       <c r="F21" s="21" t="n">
-        <v>0.474</v>
+        <v>0.341</v>
       </c>
       <c r="G21" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
         <is>
-          <t>MTE</t>
-        </is>
-      </c>
-      <c r="I21" s="19" t="inlineStr">
-        <is>
-          <t>Brasília, com disponibilidade para viagens</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I21" s="19" t="inlineStr"/>
       <c r="J21" s="22" t="n">
-        <v>46290</v>
+        <v>46292</v>
       </c>
       <c r="K21" s="22" t="n">
-        <v>46303</v>
-      </c>
-      <c r="L21" s="23" t="n">
-        <v>208966.53</v>
-      </c>
+        <v>46299</v>
+      </c>
+      <c r="L21" s="23" t="inlineStr"/>
       <c r="M21" s="17" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N21" s="20" t="inlineStr">
-        <is>
-          <t>selecao.spt@trabalho.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N21" s="20" t="inlineStr"/>
       <c r="O21" s="24" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E22" s="12" t="inlineStr">
@@ -2236,116 +2172,136 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.464</v>
+        <v>0.481</v>
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Arquitetura / Design</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I22" s="11" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I22" s="11" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J22" s="14" t="n">
-        <v>46286</v>
+        <v>46240</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46316</v>
-      </c>
-      <c r="L22" s="15" t="inlineStr"/>
+        <v>46245</v>
+      </c>
+      <c r="L22" s="15" t="n">
+        <v>204000</v>
+      </c>
       <c r="M22" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N22" s="12" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N22" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O22" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E23" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F23" s="21" t="n">
-        <v>0.464</v>
+        <v>0.511</v>
       </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Ciências Sociais / Participação Social</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Cultura</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I23" s="19" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I23" s="19" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J23" s="22" t="n">
-        <v>46286</v>
+        <v>46240</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46316</v>
-      </c>
-      <c r="L23" s="23" t="inlineStr"/>
+        <v>46245</v>
+      </c>
+      <c r="L23" s="23" t="n">
+        <v>204000</v>
+      </c>
       <c r="M23" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N23" s="20" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N23" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O23" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E24" s="12" t="inlineStr">
@@ -2354,57 +2310,67 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.423</v>
+        <v>0.462</v>
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Cultura, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I24" s="11" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I24" s="11" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J24" s="14" t="n">
-        <v>46286</v>
+        <v>46240</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46316</v>
-      </c>
-      <c r="L24" s="15" t="inlineStr"/>
+        <v>46245</v>
+      </c>
+      <c r="L24" s="15" t="n">
+        <v>80000</v>
+      </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N24" s="12" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N24" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O24" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E25" s="20" t="inlineStr">
@@ -2413,170 +2379,200 @@
         </is>
       </c>
       <c r="F25" s="21" t="n">
-        <v>0.464</v>
+        <v>0.433</v>
       </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Ciências Sociais / Participação Social</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I25" s="19" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I25" s="19" t="inlineStr">
+        <is>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+        </is>
+      </c>
       <c r="J25" s="22" t="n">
-        <v>46286</v>
+        <v>46227</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46316</v>
-      </c>
-      <c r="L25" s="23" t="inlineStr"/>
+        <v>46252</v>
+      </c>
+      <c r="L25" s="23" t="n">
+        <v>286000</v>
+      </c>
       <c r="M25" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N25" s="20" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N25" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O25" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E26" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.423</v>
+        <v>0.492</v>
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Ciências Sociais / Participação Social</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Cultura, Desenvolvimento Social / Políticas Públicas</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I26" s="11" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I26" s="11" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J26" s="14" t="n">
-        <v>46286</v>
+        <v>46240</v>
       </c>
       <c r="K26" s="14" t="n">
-        <v>46316</v>
-      </c>
-      <c r="L26" s="15" t="inlineStr"/>
+        <v>46245</v>
+      </c>
+      <c r="L26" s="15" t="n">
+        <v>100000</v>
+      </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N26" s="12" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N26" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O26" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E27" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F27" s="21" t="n">
-        <v>0.423</v>
+        <v>0.569</v>
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Cultura, Trabalho / Emprego, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I27" s="19" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I27" s="19" t="inlineStr">
+        <is>
+          <t>Brasília - Df</t>
+        </is>
+      </c>
       <c r="J27" s="22" t="n">
-        <v>46286</v>
+        <v>46240</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46316</v>
-      </c>
-      <c r="L27" s="23" t="inlineStr"/>
+        <v>46245</v>
+      </c>
+      <c r="L27" s="23" t="n">
+        <v>80000</v>
+      </c>
       <c r="M27" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N27" s="20" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N27" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>unesco:ec486dce-4c41-4830-4e64-08df1817d7a0</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ1085 - Edital nº 05/2026 - 02 vagas - Consultores Individuais</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
@@ -2586,56 +2582,64 @@
       </c>
       <c r="E28" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.3</v>
+        <v>0.492</v>
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Saúde, Estatística / Pesquisa / Metodologia, Cultura, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I28" s="11" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I28" s="11" t="inlineStr">
+        <is>
+          <t>Brasília - DF | Híbrido</t>
+        </is>
+      </c>
       <c r="J28" s="14" t="n">
-        <v>46296</v>
+        <v>46246</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46303</v>
+        <v>46250</v>
       </c>
       <c r="L28" s="15" t="inlineStr"/>
       <c r="M28" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N28" s="12" t="inlineStr"/>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N28" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O28" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>unesco:80185502-579b-44a1-e3c6-08df13ea9ffe</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ3051 - EDITAL 22/2026</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
@@ -2645,39 +2649,49 @@
       </c>
       <c r="E29" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F29" s="21" t="n">
-        <v>0.341</v>
+        <v>0.569</v>
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I29" s="19" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I29" s="19" t="inlineStr">
+        <is>
+          <t>Porto Alegre/RS</t>
+        </is>
+      </c>
       <c r="J29" s="22" t="n">
-        <v>46292</v>
+        <v>46246</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46299</v>
-      </c>
-      <c r="L29" s="23" t="inlineStr"/>
+        <v>46257</v>
+      </c>
+      <c r="L29" s="23" t="n">
+        <v>54000</v>
+      </c>
       <c r="M29" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N29" s="20" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N29" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -2689,50 +2703,50 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.462</v>
+        <v>0.593</v>
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Cultura, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J30" s="14" t="n">
-        <v>46240</v>
+        <v>46251</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>46245</v>
+        <v>46256</v>
       </c>
       <c r="L30" s="15" t="n">
-        <v>80000</v>
+        <v>50000</v>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
@@ -2746,7 +2760,7 @@
       </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -2758,12 +2772,12 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
@@ -2781,27 +2795,27 @@
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Cultura, Trabalho / Emprego, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I31" s="19" t="inlineStr">
         <is>
-          <t>Brasília - Df</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J31" s="22" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46245</v>
+        <v>46257</v>
       </c>
       <c r="L31" s="23" t="n">
-        <v>80000</v>
+        <v>54000</v>
       </c>
       <c r="M31" s="17" t="inlineStr">
         <is>
@@ -2815,7 +2829,7 @@
       </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -2827,12 +2841,12 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
@@ -2846,31 +2860,31 @@
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.492</v>
+        <v>0.46</v>
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Cultura, Desenvolvimento Social / Políticas Públicas</t>
+          <t>Tecnologia da Informação / Dados, Educação / Ensino</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I32" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J32" s="14" t="n">
-        <v>46240</v>
+        <v>46252</v>
       </c>
       <c r="K32" s="14" t="n">
-        <v>46245</v>
+        <v>46259</v>
       </c>
       <c r="L32" s="15" t="n">
-        <v>100000</v>
+        <v>60000</v>
       </c>
       <c r="M32" s="9" t="inlineStr">
         <is>
@@ -2884,7 +2898,7 @@
       </c>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -2896,17 +2910,17 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E33" s="20" t="inlineStr">
@@ -2915,45 +2929,45 @@
         </is>
       </c>
       <c r="F33" s="21" t="n">
-        <v>0.433</v>
+        <v>0.464</v>
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J33" s="22" t="n">
-        <v>46227</v>
+        <v>46208</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46252</v>
+        <v>46259</v>
       </c>
       <c r="L33" s="23" t="n">
-        <v>286000</v>
+        <v>500000</v>
       </c>
       <c r="M33" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N33" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -2965,12 +2979,12 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -2980,39 +2994,39 @@
       </c>
       <c r="E34" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.511</v>
+        <v>0.492</v>
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Cultura</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Educação / Ensino</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J34" s="14" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46245</v>
+        <v>46272</v>
       </c>
       <c r="L34" s="15" t="n">
-        <v>204000</v>
+        <v>54000</v>
       </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N34" s="12" t="inlineStr">
@@ -3022,7 +3036,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -3034,17 +3048,17 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E35" s="20" t="inlineStr">
@@ -3053,11 +3067,11 @@
         </is>
       </c>
       <c r="F35" s="21" t="n">
-        <v>0.481</v>
+        <v>0.451</v>
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
@@ -3067,17 +3081,17 @@
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46240</v>
+        <v>46265</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46245</v>
+        <v>46270</v>
       </c>
       <c r="L35" s="23" t="n">
-        <v>204000</v>
+        <v>30000</v>
       </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
@@ -3091,7 +3105,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -3103,12 +3117,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -3122,31 +3136,31 @@
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>0.569</v>
+        <v>0.3</v>
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46246</v>
+        <v>46275</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46257</v>
+        <v>46280</v>
       </c>
       <c r="L36" s="15" t="n">
-        <v>54000</v>
+        <v>50000</v>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
@@ -3160,7 +3174,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
@@ -3172,12 +3186,12 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
@@ -3191,32 +3205,30 @@
         </is>
       </c>
       <c r="F37" s="21" t="n">
-        <v>0.569</v>
+        <v>0.2</v>
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46246</v>
+        <v>46275</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46257</v>
-      </c>
-      <c r="L37" s="23" t="n">
-        <v>54000</v>
-      </c>
+        <v>46281</v>
+      </c>
+      <c r="L37" s="23" t="inlineStr"/>
       <c r="M37" s="17" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3229,7 +3241,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
         </is>
       </c>
     </row>
@@ -3241,12 +3253,12 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
@@ -3260,33 +3272,35 @@
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.492</v>
+        <v>0.527</v>
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Ciência / Tecnologia e Inovação</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46246</v>
+        <v>46266</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L38" s="15" t="inlineStr"/>
+        <v>46288</v>
+      </c>
+      <c r="L38" s="15" t="n">
+        <v>70000</v>
+      </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N38" s="12" t="inlineStr">
@@ -3296,7 +3310,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
@@ -3308,17 +3322,17 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E39" s="20" t="inlineStr">
@@ -3327,31 +3341,31 @@
         </is>
       </c>
       <c r="F39" s="21" t="n">
-        <v>0.593</v>
+        <v>0.493</v>
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Ciência / Tecnologia e Inovação, Engenharia / Infraestrutura</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Dados Remoto</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46251</v>
+        <v>46281</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46256</v>
+        <v>46286</v>
       </c>
       <c r="L39" s="23" t="n">
-        <v>50000</v>
+        <v>110000</v>
       </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
@@ -3365,7 +3379,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
         </is>
       </c>
     </row>
@@ -3377,12 +3391,12 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
@@ -3392,15 +3406,15 @@
       </c>
       <c r="E40" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.46</v>
+        <v>0.451</v>
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
@@ -3410,17 +3424,17 @@
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46252</v>
+        <v>46282</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46259</v>
+        <v>46286</v>
       </c>
       <c r="L40" s="15" t="n">
-        <v>60000</v>
+        <v>30000</v>
       </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
@@ -3434,7 +3448,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
         </is>
       </c>
     </row>
@@ -3446,30 +3460,30 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E41" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F41" s="21" t="n">
-        <v>0.451</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Trabalho / Emprego, Segurança</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
@@ -3479,18 +3493,16 @@
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46265</v>
+        <v>46290</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46270</v>
-      </c>
-      <c r="L41" s="23" t="n">
-        <v>30000</v>
-      </c>
+        <v>46294</v>
+      </c>
+      <c r="L41" s="23" t="inlineStr"/>
       <c r="M41" s="17" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3503,7 +3515,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
         </is>
       </c>
     </row>
@@ -3515,12 +3527,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3530,15 +3542,15 @@
       </c>
       <c r="E42" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.492</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Educação / Ensino</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
@@ -3548,31 +3560,29 @@
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46246</v>
+        <v>46278</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46272</v>
-      </c>
-      <c r="L42" s="15" t="n">
-        <v>54000</v>
-      </c>
+        <v>46295</v>
+      </c>
+      <c r="L42" s="15" t="inlineStr"/>
       <c r="M42" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N42" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>ugp@educacao.sp.gov.br</t>
         </is>
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
         </is>
       </c>
     </row>
@@ -3584,64 +3594,64 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E43" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F43" s="21" t="n">
-        <v>0.464</v>
+        <v>0.232</v>
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46208</v>
+        <v>46293</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46259</v>
+        <v>46298</v>
       </c>
       <c r="L43" s="23" t="n">
-        <v>500000</v>
+        <v>30000</v>
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N43" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
         </is>
       </c>
     </row>
@@ -3653,12 +3663,12 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
@@ -3668,15 +3678,15 @@
       </c>
       <c r="E44" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>0.527</v>
+        <v>0.2</v>
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Educação / Ensino, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Direitos Humanos / Cidadania</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
@@ -3686,21 +3696,21 @@
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Articulação Estadual - Rio Grande do Norte</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46266</v>
+        <v>46293</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46288</v>
+        <v>46298</v>
       </c>
       <c r="L44" s="15" t="n">
-        <v>70000</v>
+        <v>21000</v>
       </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N44" s="12" t="inlineStr">
@@ -3710,7 +3720,7 @@
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
         </is>
       </c>
     </row>
@@ -3722,64 +3732,64 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E45" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F45" s="21" t="n">
-        <v>0.3</v>
+        <v>0.464</v>
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46275</v>
+        <v>46244</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46280</v>
+        <v>46300</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>50000</v>
+        <v>350000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N45" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -3791,50 +3801,50 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E46" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Não Classificado</t>
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.493</v>
+        <v>0.077</v>
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Ciência / Tecnologia e Inovação, Engenharia / Infraestrutura</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>Dados Remoto</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J46" s="14" t="n">
-        <v>46281</v>
+        <v>46294</v>
       </c>
       <c r="K46" s="14" t="n">
-        <v>46286</v>
+        <v>46300</v>
       </c>
       <c r="L46" s="15" t="n">
-        <v>110000</v>
+        <v>55000</v>
       </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
@@ -3848,7 +3858,7 @@
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
         </is>
       </c>
     </row>
@@ -3860,12 +3870,12 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
+          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
+          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
@@ -3879,11 +3889,11 @@
         </is>
       </c>
       <c r="F47" s="21" t="n">
-        <v>0.2</v>
+        <v>0.175</v>
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Engenharia / Infraestrutura</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
@@ -3893,19 +3903,21 @@
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Remota e/ou presencial em Brasília - DF</t>
         </is>
       </c>
       <c r="J47" s="22" t="n">
-        <v>46275</v>
+        <v>46294</v>
       </c>
       <c r="K47" s="22" t="n">
-        <v>46281</v>
-      </c>
-      <c r="L47" s="23" t="inlineStr"/>
+        <v>46297</v>
+      </c>
+      <c r="L47" s="23" t="n">
+        <v>600000</v>
+      </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N47" s="20" t="inlineStr">
@@ -3915,7 +3927,7 @@
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
         </is>
       </c>
     </row>
@@ -3927,17 +3939,17 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E48" s="12" t="inlineStr">
@@ -3946,30 +3958,32 @@
         </is>
       </c>
       <c r="F48" s="13" t="n">
-        <v>0.5639999999999999</v>
+        <v>0.355</v>
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Trabalho / Emprego, Segurança</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Educação / Ensino</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J48" s="14" t="n">
-        <v>46290</v>
+        <v>46294</v>
       </c>
       <c r="K48" s="14" t="n">
-        <v>46294</v>
-      </c>
-      <c r="L48" s="15" t="inlineStr"/>
+        <v>46302</v>
+      </c>
+      <c r="L48" s="15" t="n">
+        <v>60000</v>
+      </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3982,7 +3996,7 @@
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
         </is>
       </c>
     </row>
@@ -3994,12 +4008,12 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
@@ -4009,35 +4023,35 @@
       </c>
       <c r="E49" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F49" s="21" t="n">
-        <v>0.451</v>
+        <v>0.333</v>
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Cultura, Segurança, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J49" s="22" t="n">
-        <v>46282</v>
+        <v>46296</v>
       </c>
       <c r="K49" s="22" t="n">
-        <v>46286</v>
+        <v>46300</v>
       </c>
       <c r="L49" s="23" t="n">
-        <v>30000</v>
+        <v>60000</v>
       </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
@@ -4051,7 +4065,7 @@
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
         </is>
       </c>
     </row>
@@ -4063,17 +4077,17 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E50" s="12" t="inlineStr">
@@ -4082,45 +4096,45 @@
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>0.464</v>
+        <v>0.216</v>
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Cultura, Comunicação, Arquitetura / Design</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J50" s="14" t="n">
-        <v>46244</v>
+        <v>46296</v>
       </c>
       <c r="K50" s="14" t="n">
         <v>46300</v>
       </c>
       <c r="L50" s="15" t="n">
-        <v>350000</v>
+        <v>33000</v>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N50" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
         </is>
       </c>
     </row>
@@ -4132,12 +4146,12 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
@@ -4151,11 +4165,11 @@
         </is>
       </c>
       <c r="F51" s="21" t="n">
-        <v>0.5639999999999999</v>
+        <v>0.282</v>
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
@@ -4165,29 +4179,31 @@
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
-        <v>46278</v>
+        <v>46296</v>
       </c>
       <c r="K51" s="22" t="n">
-        <v>46295</v>
-      </c>
-      <c r="L51" s="23" t="inlineStr"/>
+        <v>46300</v>
+      </c>
+      <c r="L51" s="23" t="n">
+        <v>60000</v>
+      </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N51" s="20" t="inlineStr">
         <is>
-          <t>ugp@educacao.sp.gov.br</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
         </is>
       </c>
     </row>
@@ -4199,17 +4215,17 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E52" s="12" t="inlineStr">
@@ -4218,31 +4234,31 @@
         </is>
       </c>
       <c r="F52" s="13" t="n">
-        <v>0.175</v>
+        <v>0.493</v>
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Engenharia / Infraestrutura</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Desenvolvimento Social / Políticas Públicas</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>Remota e/ou presencial em Brasília - DF</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J52" s="14" t="n">
-        <v>46294</v>
+        <v>46244</v>
       </c>
       <c r="K52" s="14" t="n">
-        <v>46297</v>
+        <v>46296</v>
       </c>
       <c r="L52" s="15" t="n">
-        <v>600000</v>
+        <v>935000</v>
       </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
@@ -4251,12 +4267,12 @@
       </c>
       <c r="N52" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -4268,12 +4284,12 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
@@ -4283,35 +4299,35 @@
       </c>
       <c r="E53" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F53" s="21" t="n">
-        <v>0.232</v>
+        <v>0.178</v>
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
+          <t>Tecnologia da Informação / Dados, Cultura, Comunicação</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
-        <v>46293</v>
+        <v>46296</v>
       </c>
       <c r="K53" s="22" t="n">
-        <v>46298</v>
+        <v>46300</v>
       </c>
       <c r="L53" s="23" t="n">
-        <v>30000</v>
+        <v>21000</v>
       </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
@@ -4325,7 +4341,7 @@
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
         </is>
       </c>
     </row>
@@ -4337,12 +4353,12 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
@@ -4352,39 +4368,39 @@
       </c>
       <c r="E54" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F54" s="13" t="n">
-        <v>0.2</v>
+        <v>0.378</v>
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Educação / Ensino, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Direitos Humanos / Cidadania</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Cultura, Comunicação</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Rio Grande do Norte</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J54" s="14" t="n">
-        <v>46293</v>
+        <v>46296</v>
       </c>
       <c r="K54" s="14" t="n">
-        <v>46298</v>
+        <v>46300</v>
       </c>
       <c r="L54" s="15" t="n">
-        <v>21000</v>
+        <v>36000</v>
       </c>
       <c r="M54" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N54" s="12" t="inlineStr">
@@ -4394,7 +4410,7 @@
       </c>
       <c r="O54" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
         </is>
       </c>
     </row>
@@ -4406,12 +4422,12 @@
       </c>
       <c r="B55" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304</t>
         </is>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13304</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
@@ -4421,15 +4437,15 @@
       </c>
       <c r="E55" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F55" s="21" t="n">
-        <v>0.077</v>
+        <v>0.445</v>
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
@@ -4439,17 +4455,17 @@
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J55" s="22" t="n">
-        <v>46294</v>
+        <v>46297</v>
       </c>
       <c r="K55" s="22" t="n">
-        <v>46300</v>
+        <v>46311</v>
       </c>
       <c r="L55" s="23" t="n">
-        <v>55000</v>
+        <v>90000</v>
       </c>
       <c r="M55" s="17" t="inlineStr">
         <is>
@@ -4463,7 +4479,7 @@
       </c>
       <c r="O55" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304/</t>
         </is>
       </c>
     </row>
@@ -4475,12 +4491,12 @@
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13221</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
@@ -4494,11 +4510,11 @@
         </is>
       </c>
       <c r="F56" s="13" t="n">
-        <v>0.355</v>
+        <v>0.409</v>
       </c>
       <c r="G56" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H56" s="11" t="inlineStr">
@@ -4512,13 +4528,13 @@
         </is>
       </c>
       <c r="J56" s="14" t="n">
-        <v>46294</v>
+        <v>46297</v>
       </c>
       <c r="K56" s="14" t="n">
-        <v>46302</v>
+        <v>46311</v>
       </c>
       <c r="L56" s="15" t="n">
-        <v>60000</v>
+        <v>70000</v>
       </c>
       <c r="M56" s="9" t="inlineStr">
         <is>
@@ -4532,426 +4548,12 @@
       </c>
       <c r="O56" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="17" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B57" s="18" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
-        </is>
-      </c>
-      <c r="C57" s="19" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
-        </is>
-      </c>
-      <c r="D57" s="19" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E57" s="20" t="inlineStr">
-        <is>
-          <t>Engenharia Processos Analytics</t>
-        </is>
-      </c>
-      <c r="F57" s="21" t="n">
-        <v>0.333</v>
-      </c>
-      <c r="G57" s="19" t="inlineStr">
-        <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Cultura, Segurança, Ciência / Tecnologia e Inovação</t>
-        </is>
-      </c>
-      <c r="H57" s="19" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I57" s="19" t="inlineStr">
-        <is>
-          <t>Brasília - DF</t>
-        </is>
-      </c>
-      <c r="J57" s="22" t="n">
-        <v>46296</v>
-      </c>
-      <c r="K57" s="22" t="n">
-        <v>46300</v>
-      </c>
-      <c r="L57" s="23" t="n">
-        <v>60000</v>
-      </c>
-      <c r="M57" s="17" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N57" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O57" s="24" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="9" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B58" s="10" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
-        </is>
-      </c>
-      <c r="C58" s="11" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
-        </is>
-      </c>
-      <c r="D58" s="11" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E58" s="12" t="inlineStr">
-        <is>
-          <t>Engenharia Processos Analytics</t>
-        </is>
-      </c>
-      <c r="F58" s="13" t="n">
-        <v>0.282</v>
-      </c>
-      <c r="G58" s="11" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
-        </is>
-      </c>
-      <c r="H58" s="11" t="inlineStr">
-        <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I58" s="11" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="J58" s="14" t="n">
-        <v>46296</v>
-      </c>
-      <c r="K58" s="14" t="n">
-        <v>46300</v>
-      </c>
-      <c r="L58" s="15" t="n">
-        <v>60000</v>
-      </c>
-      <c r="M58" s="9" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N58" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O58" s="16" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="17" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B59" s="18" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
-        </is>
-      </c>
-      <c r="C59" s="19" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
-        </is>
-      </c>
-      <c r="D59" s="19" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E59" s="20" t="inlineStr">
-        <is>
-          <t>Consultoria Diversidade Inclusao</t>
-        </is>
-      </c>
-      <c r="F59" s="21" t="n">
-        <v>0.216</v>
-      </c>
-      <c r="G59" s="19" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Cultura, Comunicação, Arquitetura / Design</t>
-        </is>
-      </c>
-      <c r="H59" s="19" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I59" s="19" t="inlineStr">
-        <is>
-          <t>Vitória - ES</t>
-        </is>
-      </c>
-      <c r="J59" s="22" t="n">
-        <v>46296</v>
-      </c>
-      <c r="K59" s="22" t="n">
-        <v>46300</v>
-      </c>
-      <c r="L59" s="23" t="n">
-        <v>33000</v>
-      </c>
-      <c r="M59" s="17" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N59" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O59" s="24" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="9" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B60" s="10" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
-        </is>
-      </c>
-      <c r="C60" s="11" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
-        </is>
-      </c>
-      <c r="D60" s="11" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E60" s="12" t="inlineStr">
-        <is>
-          <t>Engenharia Processos Analytics</t>
-        </is>
-      </c>
-      <c r="F60" s="13" t="n">
-        <v>0.378</v>
-      </c>
-      <c r="G60" s="11" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Cultura, Comunicação</t>
-        </is>
-      </c>
-      <c r="H60" s="11" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I60" s="11" t="inlineStr">
-        <is>
-          <t>Vitória - ES</t>
-        </is>
-      </c>
-      <c r="J60" s="14" t="n">
-        <v>46296</v>
-      </c>
-      <c r="K60" s="14" t="n">
-        <v>46300</v>
-      </c>
-      <c r="L60" s="15" t="n">
-        <v>36000</v>
-      </c>
-      <c r="M60" s="9" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N60" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O60" s="16" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="17" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B61" s="18" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
-        </is>
-      </c>
-      <c r="C61" s="19" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
-        </is>
-      </c>
-      <c r="D61" s="19" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E61" s="20" t="inlineStr">
-        <is>
-          <t>Consultoria Diversidade Inclusao</t>
-        </is>
-      </c>
-      <c r="F61" s="21" t="n">
-        <v>0.178</v>
-      </c>
-      <c r="G61" s="19" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Cultura, Comunicação</t>
-        </is>
-      </c>
-      <c r="H61" s="19" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I61" s="19" t="inlineStr">
-        <is>
-          <t>Vitória - ES</t>
-        </is>
-      </c>
-      <c r="J61" s="22" t="n">
-        <v>46296</v>
-      </c>
-      <c r="K61" s="22" t="n">
-        <v>46300</v>
-      </c>
-      <c r="L61" s="23" t="n">
-        <v>21000</v>
-      </c>
-      <c r="M61" s="17" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N61" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O61" s="24" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="9" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B62" s="10" t="inlineStr">
-        <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
-        </is>
-      </c>
-      <c r="C62" s="11" t="inlineStr">
-        <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
-        </is>
-      </c>
-      <c r="D62" s="11" t="inlineStr">
-        <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
-        </is>
-      </c>
-      <c r="E62" s="12" t="inlineStr">
-        <is>
-          <t>Engenharia Processos Analytics</t>
-        </is>
-      </c>
-      <c r="F62" s="13" t="n">
-        <v>0.493</v>
-      </c>
-      <c r="G62" s="11" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Desenvolvimento Social / Políticas Públicas</t>
-        </is>
-      </c>
-      <c r="H62" s="11" t="inlineStr">
-        <is>
-          <t>OEI/MDHC</t>
-        </is>
-      </c>
-      <c r="I62" s="11" t="inlineStr">
-        <is>
-          <t>Nacional</t>
-        </is>
-      </c>
-      <c r="J62" s="14" t="n">
-        <v>46244</v>
-      </c>
-      <c r="K62" s="14" t="n">
-        <v>46296</v>
-      </c>
-      <c r="L62" s="15" t="n">
-        <v>935000</v>
-      </c>
-      <c r="M62" s="9" t="inlineStr">
-        <is>
-          <t>En fase de apresentação</t>
-        </is>
-      </c>
-      <c r="N62" s="12" t="inlineStr">
-        <is>
-          <t>compras.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O62" s="16" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O62"/>
+  <autoFilter ref="A1:O56"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -5008,12 +4610,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId61"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -5052,7 +4648,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3">
@@ -5062,7 +4658,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4">
@@ -5110,21 +4706,21 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4">
@@ -5134,7 +4730,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -5176,7 +4772,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3">
@@ -5186,7 +4782,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4">
@@ -5196,7 +4792,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
@@ -5248,7 +4844,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3">
@@ -5258,7 +4854,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4">
@@ -5268,43 +4864,43 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
-          <t>Ciência / Tecnologia e Inovação</t>
+          <t>Cultura</t>
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>Meio Ambiente / Clima / Geografia</t>
+          <t>Educação / Ensino</t>
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>Cultura</t>
+          <t>Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>Educação / Ensino</t>
+          <t>Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="B8" s="10" t="n">
@@ -5314,7 +4910,7 @@
     <row r="9">
       <c r="A9" s="19" t="inlineStr">
         <is>
-          <t>Desenvolvimento Social / Políticas Públicas</t>
+          <t>Ciências Sociais / Participação Social</t>
         </is>
       </c>
       <c r="B9" s="18" t="n">
@@ -5324,11 +4920,11 @@
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>Ciências Sociais / Participação Social</t>
+          <t>Desenvolvimento Social / Políticas Públicas</t>
         </is>
       </c>
       <c r="B10" s="10" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11">
@@ -5390,27 +4986,27 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>IBGE</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>IBGE</t>
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
@@ -5420,13 +5016,13 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="B7" s="18" t="n">
@@ -5436,11 +5032,11 @@
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -5498,7 +5094,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -5513,7 +5109,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-10-06 18:17
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$54</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -27,7 +27,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Por_Tipo'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Por_Area'!$A$1:$B$11</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Por_Area'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Por_Orgao'!$A$1:$B$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Por_Orgao'!$A$1:$B$10</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Por_Orgao'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Perfis'!$A$1:$C$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'Perfis'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 03/10/2026 às 16:06</t>
+          <t>Gerado em 06/10/2026 às 18:16</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6">
@@ -620,7 +620,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="17">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>121990.5263157895</v>
+        <v>116902.8988571428</v>
       </c>
     </row>
     <row r="20">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>80000</v>
+        <v>62500</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="24">
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
     </row>
     <row r="25">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O56"/>
+  <dimension ref="A1:O54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1676,17 +1676,15 @@
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="n">
+        <v>146401</v>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
+          <t>Edital 06/2026 - Programa de Privacidade e Segurança da Informação</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -1696,39 +1694,49 @@
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.464</v>
+        <v>0.175</v>
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Arquitetura / Design</t>
+          <t>Tecnologia da Informação / Dados, Segurança</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I14" s="11" t="inlineStr"/>
+          <t>Não identificado</t>
+        </is>
+      </c>
+      <c r="I14" s="11" t="inlineStr">
+        <is>
+          <t>Território Nacional</t>
+        </is>
+      </c>
       <c r="J14" s="14" t="n">
-        <v>46286</v>
+        <v>46301</v>
       </c>
       <c r="K14" s="14" t="n">
         <v>46316</v>
       </c>
-      <c r="L14" s="15" t="inlineStr"/>
+      <c r="L14" s="15" t="n">
+        <v>120000</v>
+      </c>
       <c r="M14" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N14" s="12" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N14" s="12" t="inlineStr">
+        <is>
+          <t>cgti@mdh.gov.br</t>
+        </is>
+      </c>
       <c r="O14" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
@@ -1740,12 +1748,12 @@
       </c>
       <c r="B15" s="18" t="inlineStr">
         <is>
-          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
+          <t>unesco:375ed309-bb72-44ae-7d86-08df1d6278dd</t>
         </is>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
+          <t>914BRZ1159 - Publicação Edital 41/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
@@ -1755,15 +1763,15 @@
       </c>
       <c r="E15" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F15" s="21" t="n">
-        <v>0.464</v>
+        <v>0.433</v>
       </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Ciências Sociais / Participação Social</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H15" s="19" t="inlineStr">
@@ -1773,10 +1781,10 @@
       </c>
       <c r="I15" s="19" t="inlineStr"/>
       <c r="J15" s="22" t="n">
-        <v>46286</v>
+        <v>46300</v>
       </c>
       <c r="K15" s="22" t="n">
-        <v>46316</v>
+        <v>46304</v>
       </c>
       <c r="L15" s="23" t="inlineStr"/>
       <c r="M15" s="17" t="inlineStr">
@@ -1799,12 +1807,12 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
+          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
+          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -1818,11 +1826,11 @@
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.423</v>
+        <v>0.464</v>
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Arquitetura / Design</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
@@ -1858,12 +1866,12 @@
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
+          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
         </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
+          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1881,7 +1889,7 @@
       </c>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>Ciências Sociais / Participação Social</t>
+          <t>Tecnologia da Informação / Dados, Ciências Sociais / Participação Social</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
@@ -1917,12 +1925,12 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
+          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
+          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -1940,7 +1948,7 @@
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Ciências Sociais / Participação Social</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -1976,12 +1984,12 @@
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
+          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
+          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
@@ -1995,11 +2003,11 @@
         </is>
       </c>
       <c r="F19" s="21" t="n">
-        <v>0.423</v>
+        <v>0.464</v>
       </c>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Ciências Sociais / Participação Social</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
@@ -2035,17 +2043,17 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>unesco:ec486dce-4c41-4830-4e64-08df1817d7a0</t>
+          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ1085 - Edital nº 05/2026 - 02 vagas - Consultores Individuais</t>
+          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
@@ -2054,11 +2062,11 @@
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.3</v>
+        <v>0.423</v>
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Saúde, Estatística / Pesquisa / Metodologia, Cultura, Ciência / Tecnologia e Inovação</t>
+          <t>Ciências Sociais / Participação Social</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
@@ -2068,10 +2076,10 @@
       </c>
       <c r="I20" s="11" t="inlineStr"/>
       <c r="J20" s="14" t="n">
-        <v>46296</v>
+        <v>46286</v>
       </c>
       <c r="K20" s="14" t="n">
-        <v>46303</v>
+        <v>46316</v>
       </c>
       <c r="L20" s="15" t="inlineStr"/>
       <c r="M20" s="9" t="inlineStr">
@@ -2094,17 +2102,17 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>unesco:80185502-579b-44a1-e3c6-08df13ea9ffe</t>
+          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ3051 - EDITAL 22/2026</t>
+          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E21" s="20" t="inlineStr">
@@ -2113,11 +2121,11 @@
         </is>
       </c>
       <c r="F21" s="21" t="n">
-        <v>0.341</v>
+        <v>0.423</v>
       </c>
       <c r="G21" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
@@ -2127,10 +2135,10 @@
       </c>
       <c r="I21" s="19" t="inlineStr"/>
       <c r="J21" s="22" t="n">
-        <v>46292</v>
+        <v>46286</v>
       </c>
       <c r="K21" s="22" t="n">
-        <v>46299</v>
+        <v>46316</v>
       </c>
       <c r="L21" s="23" t="inlineStr"/>
       <c r="M21" s="17" t="inlineStr">
@@ -2148,17 +2156,17 @@
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>unesco:ec486dce-4c41-4830-4e64-08df1817d7a0</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>Projeto 914BRZ1085 - Edital nº 05/2026 - 02 vagas - Consultores Individuais</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -2172,45 +2180,35 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.481</v>
+        <v>0.3</v>
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Saúde, Estatística / Pesquisa / Metodologia, Cultura, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I22" s="11" t="inlineStr">
-        <is>
-          <t>Brasília - DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I22" s="11" t="inlineStr"/>
       <c r="J22" s="14" t="n">
-        <v>46240</v>
+        <v>46296</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46245</v>
-      </c>
-      <c r="L22" s="15" t="n">
-        <v>204000</v>
-      </c>
+        <v>46303</v>
+      </c>
+      <c r="L22" s="15" t="inlineStr"/>
       <c r="M22" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N22" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N22" s="12" t="inlineStr"/>
       <c r="O22" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
@@ -2222,12 +2220,12 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
@@ -2237,35 +2235,35 @@
       </c>
       <c r="E23" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F23" s="21" t="n">
-        <v>0.511</v>
+        <v>0.433</v>
       </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Cultura</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I23" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
         </is>
       </c>
       <c r="J23" s="22" t="n">
-        <v>46240</v>
+        <v>46227</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46245</v>
+        <v>46252</v>
       </c>
       <c r="L23" s="23" t="n">
-        <v>204000</v>
+        <v>286000</v>
       </c>
       <c r="M23" s="17" t="inlineStr">
         <is>
@@ -2279,7 +2277,7 @@
       </c>
       <c r="O23" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
@@ -2291,12 +2289,12 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -2306,35 +2304,35 @@
       </c>
       <c r="E24" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.462</v>
+        <v>0.569</v>
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Cultura, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I24" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J24" s="14" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46245</v>
+        <v>46257</v>
       </c>
       <c r="L24" s="15" t="n">
-        <v>80000</v>
+        <v>54000</v>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
@@ -2348,7 +2346,7 @@
       </c>
       <c r="O24" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -2360,12 +2358,12 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
@@ -2375,15 +2373,15 @@
       </c>
       <c r="E25" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F25" s="21" t="n">
-        <v>0.433</v>
+        <v>0.569</v>
       </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
@@ -2393,17 +2391,17 @@
       </c>
       <c r="I25" s="19" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J25" s="22" t="n">
-        <v>46227</v>
+        <v>46246</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46252</v>
+        <v>46257</v>
       </c>
       <c r="L25" s="23" t="n">
-        <v>286000</v>
+        <v>54000</v>
       </c>
       <c r="M25" s="17" t="inlineStr">
         <is>
@@ -2417,7 +2415,7 @@
       </c>
       <c r="O25" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -2498,12 +2496,12 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
@@ -2517,11 +2515,11 @@
         </is>
       </c>
       <c r="F27" s="21" t="n">
-        <v>0.569</v>
+        <v>0.492</v>
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Cultura, Trabalho / Emprego, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
@@ -2531,21 +2529,19 @@
       </c>
       <c r="I27" s="19" t="inlineStr">
         <is>
-          <t>Brasília - Df</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J27" s="22" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46245</v>
-      </c>
-      <c r="L27" s="23" t="n">
-        <v>80000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L27" s="23" t="inlineStr"/>
       <c r="M27" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N27" s="20" t="inlineStr">
@@ -2555,7 +2551,7 @@
       </c>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -2567,17 +2563,17 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr">
@@ -2586,33 +2582,35 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.492</v>
+        <v>0.593</v>
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I28" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J28" s="14" t="n">
-        <v>46246</v>
+        <v>46251</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L28" s="15" t="inlineStr"/>
+        <v>46256</v>
+      </c>
+      <c r="L28" s="15" t="n">
+        <v>50000</v>
+      </c>
       <c r="M28" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N28" s="12" t="inlineStr">
@@ -2622,7 +2620,7 @@
       </c>
       <c r="O28" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -2634,12 +2632,12 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
@@ -2653,11 +2651,11 @@
         </is>
       </c>
       <c r="F29" s="21" t="n">
-        <v>0.569</v>
+        <v>0.46</v>
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Educação / Ensino</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
@@ -2667,17 +2665,17 @@
       </c>
       <c r="I29" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J29" s="22" t="n">
-        <v>46246</v>
+        <v>46252</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46257</v>
+        <v>46259</v>
       </c>
       <c r="L29" s="23" t="n">
-        <v>54000</v>
+        <v>60000</v>
       </c>
       <c r="M29" s="17" t="inlineStr">
         <is>
@@ -2691,7 +2689,7 @@
       </c>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -2703,30 +2701,30 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.593</v>
+        <v>0.492</v>
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Educação / Ensino</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
@@ -2736,21 +2734,21 @@
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J30" s="14" t="n">
-        <v>46251</v>
+        <v>46246</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>46256</v>
+        <v>46272</v>
       </c>
       <c r="L30" s="15" t="n">
-        <v>50000</v>
+        <v>54000</v>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N30" s="12" t="inlineStr">
@@ -2760,7 +2758,7 @@
       </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -2772,50 +2770,50 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E31" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F31" s="21" t="n">
-        <v>0.569</v>
+        <v>0.451</v>
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I31" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J31" s="22" t="n">
-        <v>46246</v>
+        <v>46265</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46257</v>
+        <v>46270</v>
       </c>
       <c r="L31" s="23" t="n">
-        <v>54000</v>
+        <v>30000</v>
       </c>
       <c r="M31" s="17" t="inlineStr">
         <is>
@@ -2829,7 +2827,7 @@
       </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -2841,12 +2839,12 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
@@ -2856,15 +2854,15 @@
       </c>
       <c r="E32" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.46</v>
+        <v>0.451</v>
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
@@ -2874,17 +2872,17 @@
       </c>
       <c r="I32" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J32" s="14" t="n">
-        <v>46252</v>
+        <v>46282</v>
       </c>
       <c r="K32" s="14" t="n">
-        <v>46259</v>
+        <v>46286</v>
       </c>
       <c r="L32" s="15" t="n">
-        <v>60000</v>
+        <v>30000</v>
       </c>
       <c r="M32" s="9" t="inlineStr">
         <is>
@@ -2898,7 +2896,7 @@
       </c>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
         </is>
       </c>
     </row>
@@ -2910,64 +2908,62 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E33" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F33" s="21" t="n">
-        <v>0.464</v>
+        <v>0.2</v>
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J33" s="22" t="n">
-        <v>46208</v>
+        <v>46275</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46259</v>
-      </c>
-      <c r="L33" s="23" t="n">
-        <v>500000</v>
-      </c>
+        <v>46281</v>
+      </c>
+      <c r="L33" s="23" t="inlineStr"/>
       <c r="M33" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N33" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
         </is>
       </c>
     </row>
@@ -2979,12 +2975,12 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -2994,15 +2990,15 @@
       </c>
       <c r="E34" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.492</v>
+        <v>0.527</v>
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Educação / Ensino</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
@@ -3012,21 +3008,21 @@
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J34" s="14" t="n">
-        <v>46246</v>
+        <v>46266</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46272</v>
+        <v>46288</v>
       </c>
       <c r="L34" s="15" t="n">
-        <v>54000</v>
+        <v>70000</v>
       </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N34" s="12" t="inlineStr">
@@ -3036,7 +3032,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
@@ -3048,12 +3044,12 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
@@ -3063,15 +3059,15 @@
       </c>
       <c r="E35" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F35" s="21" t="n">
-        <v>0.451</v>
+        <v>0.493</v>
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Ciência / Tecnologia e Inovação, Engenharia / Infraestrutura</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
@@ -3081,17 +3077,17 @@
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Dados Remoto</t>
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46265</v>
+        <v>46281</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46270</v>
+        <v>46286</v>
       </c>
       <c r="L35" s="23" t="n">
-        <v>30000</v>
+        <v>110000</v>
       </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
@@ -3105,7 +3101,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
         </is>
       </c>
     </row>
@@ -3186,17 +3182,17 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E37" s="20" t="inlineStr">
@@ -3205,11 +3201,11 @@
         </is>
       </c>
       <c r="F37" s="21" t="n">
-        <v>0.2</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Ciência / Tecnologia e Inovação</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Trabalho / Emprego, Segurança</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
@@ -3223,10 +3219,10 @@
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46275</v>
+        <v>46290</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46281</v>
+        <v>46294</v>
       </c>
       <c r="L37" s="23" t="inlineStr"/>
       <c r="M37" s="17" t="inlineStr">
@@ -3241,7 +3237,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
         </is>
       </c>
     </row>
@@ -3253,12 +3249,12 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
@@ -3272,11 +3268,11 @@
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.527</v>
+        <v>0.232</v>
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
@@ -3286,17 +3282,17 @@
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46266</v>
+        <v>46293</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46288</v>
+        <v>46298</v>
       </c>
       <c r="L38" s="15" t="n">
-        <v>70000</v>
+        <v>30000</v>
       </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
@@ -3310,7 +3306,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
         </is>
       </c>
     </row>
@@ -3322,17 +3318,17 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E39" s="20" t="inlineStr">
@@ -3341,45 +3337,43 @@
         </is>
       </c>
       <c r="F39" s="21" t="n">
-        <v>0.493</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Ciência / Tecnologia e Inovação, Engenharia / Infraestrutura</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Dados Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46281</v>
+        <v>46278</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46286</v>
-      </c>
-      <c r="L39" s="23" t="n">
-        <v>110000</v>
-      </c>
+        <v>46295</v>
+      </c>
+      <c r="L39" s="23" t="inlineStr"/>
       <c r="M39" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N39" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>ugp@educacao.sp.gov.br</t>
         </is>
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
         </is>
       </c>
     </row>
@@ -3391,12 +3385,12 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
@@ -3410,11 +3404,11 @@
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.451</v>
+        <v>0.2</v>
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Educação / Ensino, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Direitos Humanos / Cidadania</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
@@ -3424,21 +3418,21 @@
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Articulação Estadual - Rio Grande do Norte</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46282</v>
+        <v>46293</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46286</v>
+        <v>46298</v>
       </c>
       <c r="L40" s="15" t="n">
-        <v>30000</v>
+        <v>21000</v>
       </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N40" s="12" t="inlineStr">
@@ -3448,7 +3442,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
         </is>
       </c>
     </row>
@@ -3460,17 +3454,17 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E41" s="20" t="inlineStr">
@@ -3479,30 +3473,32 @@
         </is>
       </c>
       <c r="F41" s="21" t="n">
-        <v>0.5639999999999999</v>
+        <v>0.355</v>
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Trabalho / Emprego, Segurança</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Educação / Ensino</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46290</v>
+        <v>46294</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46294</v>
-      </c>
-      <c r="L41" s="23" t="inlineStr"/>
+        <v>46302</v>
+      </c>
+      <c r="L41" s="23" t="n">
+        <v>60000</v>
+      </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3515,7 +3511,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
         </is>
       </c>
     </row>
@@ -3527,12 +3523,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3542,15 +3538,15 @@
       </c>
       <c r="E42" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Não Classificado</t>
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.5639999999999999</v>
+        <v>0.077</v>
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
@@ -3560,29 +3556,31 @@
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46278</v>
+        <v>46294</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46295</v>
-      </c>
-      <c r="L42" s="15" t="inlineStr"/>
+        <v>46300</v>
+      </c>
+      <c r="L42" s="15" t="n">
+        <v>55000</v>
+      </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N42" s="12" t="inlineStr">
         <is>
-          <t>ugp@educacao.sp.gov.br</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
         </is>
       </c>
     </row>
@@ -3594,12 +3592,12 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
+          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
+          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
@@ -3613,35 +3611,35 @@
         </is>
       </c>
       <c r="F43" s="21" t="n">
-        <v>0.232</v>
+        <v>0.175</v>
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Engenharia / Infraestrutura</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
+          <t>Remota e/ou presencial em Brasília - DF</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46298</v>
+        <v>46297</v>
       </c>
       <c r="L43" s="23" t="n">
-        <v>30000</v>
+        <v>600000</v>
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N43" s="20" t="inlineStr">
@@ -3651,7 +3649,7 @@
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
         </is>
       </c>
     </row>
@@ -3663,12 +3661,12 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
@@ -3678,39 +3676,39 @@
       </c>
       <c r="E44" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>0.2</v>
+        <v>0.333</v>
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Educação / Ensino, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Direitos Humanos / Cidadania</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Cultura, Segurança, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Rio Grande do Norte</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46293</v>
+        <v>46296</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46298</v>
+        <v>46300</v>
       </c>
       <c r="L44" s="15" t="n">
-        <v>21000</v>
+        <v>60000</v>
       </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N44" s="12" t="inlineStr">
@@ -3720,7 +3718,7 @@
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
         </is>
       </c>
     </row>
@@ -3732,17 +3730,17 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E45" s="20" t="inlineStr">
@@ -3751,45 +3749,45 @@
         </is>
       </c>
       <c r="F45" s="21" t="n">
-        <v>0.464</v>
+        <v>0.216</v>
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Cultura, Comunicação, Arquitetura / Design</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46244</v>
+        <v>46296</v>
       </c>
       <c r="K45" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>350000</v>
+        <v>33000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N45" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
         </is>
       </c>
     </row>
@@ -3801,12 +3799,12 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -3816,15 +3814,15 @@
       </c>
       <c r="E46" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.077</v>
+        <v>0.282</v>
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
@@ -3838,13 +3836,13 @@
         </is>
       </c>
       <c r="J46" s="14" t="n">
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="K46" s="14" t="n">
         <v>46300</v>
       </c>
       <c r="L46" s="15" t="n">
-        <v>55000</v>
+        <v>60000</v>
       </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
@@ -3858,7 +3856,7 @@
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
         </is>
       </c>
     </row>
@@ -3870,12 +3868,12 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
@@ -3889,11 +3887,11 @@
         </is>
       </c>
       <c r="F47" s="21" t="n">
-        <v>0.175</v>
+        <v>0.378</v>
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Engenharia / Infraestrutura</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Cultura, Comunicação</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
@@ -3903,21 +3901,21 @@
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>Remota e/ou presencial em Brasília - DF</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J47" s="22" t="n">
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="K47" s="22" t="n">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="L47" s="23" t="n">
-        <v>600000</v>
+        <v>36000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N47" s="20" t="inlineStr">
@@ -3927,7 +3925,7 @@
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
         </is>
       </c>
     </row>
@@ -3939,12 +3937,12 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
@@ -3954,35 +3952,35 @@
       </c>
       <c r="E48" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F48" s="13" t="n">
-        <v>0.355</v>
+        <v>0.178</v>
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Cultura, Comunicação</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J48" s="14" t="n">
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="K48" s="14" t="n">
-        <v>46302</v>
+        <v>46300</v>
       </c>
       <c r="L48" s="15" t="n">
-        <v>60000</v>
+        <v>21000</v>
       </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
@@ -3996,7 +3994,7 @@
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
         </is>
       </c>
     </row>
@@ -4008,17 +4006,17 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E49" s="20" t="inlineStr">
@@ -4027,45 +4025,45 @@
         </is>
       </c>
       <c r="F49" s="21" t="n">
-        <v>0.333</v>
+        <v>0.493</v>
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Cultura, Segurança, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Desenvolvimento Social / Políticas Públicas</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J49" s="22" t="n">
+        <v>46244</v>
+      </c>
+      <c r="K49" s="22" t="n">
         <v>46296</v>
       </c>
-      <c r="K49" s="22" t="n">
-        <v>46300</v>
-      </c>
       <c r="L49" s="23" t="n">
-        <v>60000</v>
+        <v>935000</v>
       </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N49" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -4077,12 +4075,12 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13221</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
@@ -4092,35 +4090,35 @@
       </c>
       <c r="E50" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>0.216</v>
+        <v>0.409</v>
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Cultura, Comunicação, Arquitetura / Design</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J50" s="14" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="K50" s="14" t="n">
-        <v>46300</v>
+        <v>46311</v>
       </c>
       <c r="L50" s="15" t="n">
-        <v>33000</v>
+        <v>70000</v>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
@@ -4134,7 +4132,7 @@
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221/</t>
         </is>
       </c>
     </row>
@@ -4146,12 +4144,12 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13304</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
@@ -4165,11 +4163,11 @@
         </is>
       </c>
       <c r="F51" s="21" t="n">
-        <v>0.282</v>
+        <v>0.445</v>
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
@@ -4179,21 +4177,21 @@
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="K51" s="22" t="n">
-        <v>46300</v>
+        <v>46311</v>
       </c>
       <c r="L51" s="23" t="n">
-        <v>60000</v>
+        <v>90000</v>
       </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>Suspendida</t>
         </is>
       </c>
       <c r="N51" s="20" t="inlineStr">
@@ -4203,7 +4201,7 @@
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304/</t>
         </is>
       </c>
     </row>
@@ -4215,12 +4213,12 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
@@ -4230,15 +4228,15 @@
       </c>
       <c r="E52" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F52" s="13" t="n">
-        <v>0.493</v>
+        <v>0.464</v>
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Desenvolvimento Social / Políticas Públicas</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
@@ -4255,10 +4253,10 @@
         <v>46244</v>
       </c>
       <c r="K52" s="14" t="n">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="L52" s="15" t="n">
-        <v>935000</v>
+        <v>350000</v>
       </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
@@ -4272,7 +4270,7 @@
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -4284,64 +4282,64 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
+          <t>oei:procedimento-simplificado-no-13307-2026-oei-secult-es</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
+          <t>Procedimento Simplificado nº 13307/2026 – OEI/SECULT-ES</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E53" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Não Classificado</t>
         </is>
       </c>
       <c r="F53" s="21" t="n">
-        <v>0.178</v>
+        <v>0.125</v>
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Cultura, Comunicação</t>
+          <t>Tecnologia da Informação / Dados, Cultura</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/SECULT</t>
         </is>
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>Vitória/ES</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
-        <v>46296</v>
+        <v>46301</v>
       </c>
       <c r="K53" s="22" t="n">
-        <v>46300</v>
+        <v>46315</v>
       </c>
       <c r="L53" s="23" t="n">
-        <v>21000</v>
+        <v>600000</v>
       </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N53" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13307-2026-oei-secult-es/</t>
         </is>
       </c>
     </row>
@@ -4353,17 +4351,17 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E54" s="12" t="inlineStr">
@@ -4376,7 +4374,7 @@
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Cultura, Comunicação</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Comunicação</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
@@ -4386,17 +4384,17 @@
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
         </is>
       </c>
       <c r="J54" s="14" t="n">
-        <v>46296</v>
+        <v>46301</v>
       </c>
       <c r="K54" s="14" t="n">
-        <v>46300</v>
+        <v>46305</v>
       </c>
       <c r="L54" s="15" t="n">
-        <v>36000</v>
+        <v>62500</v>
       </c>
       <c r="M54" s="9" t="inlineStr">
         <is>
@@ -4410,150 +4408,12 @@
       </c>
       <c r="O54" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="17" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B55" s="18" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304</t>
-        </is>
-      </c>
-      <c r="C55" s="19" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13304</t>
-        </is>
-      </c>
-      <c r="D55" s="19" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E55" s="20" t="inlineStr">
-        <is>
-          <t>Engenharia Processos Analytics</t>
-        </is>
-      </c>
-      <c r="F55" s="21" t="n">
-        <v>0.445</v>
-      </c>
-      <c r="G55" s="19" t="inlineStr">
-        <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
-        </is>
-      </c>
-      <c r="H55" s="19" t="inlineStr">
-        <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I55" s="19" t="inlineStr">
-        <is>
-          <t>São Paulo - SP</t>
-        </is>
-      </c>
-      <c r="J55" s="22" t="n">
-        <v>46297</v>
-      </c>
-      <c r="K55" s="22" t="n">
-        <v>46311</v>
-      </c>
-      <c r="L55" s="23" t="n">
-        <v>90000</v>
-      </c>
-      <c r="M55" s="17" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N55" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O55" s="24" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304/</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="9" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B56" s="10" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221</t>
-        </is>
-      </c>
-      <c r="C56" s="11" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13221</t>
-        </is>
-      </c>
-      <c r="D56" s="11" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E56" s="12" t="inlineStr">
-        <is>
-          <t>Engenharia Processos Analytics</t>
-        </is>
-      </c>
-      <c r="F56" s="13" t="n">
-        <v>0.409</v>
-      </c>
-      <c r="G56" s="11" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
-        </is>
-      </c>
-      <c r="H56" s="11" t="inlineStr">
-        <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I56" s="11" t="inlineStr">
-        <is>
-          <t>São Paulo - SP</t>
-        </is>
-      </c>
-      <c r="J56" s="14" t="n">
-        <v>46297</v>
-      </c>
-      <c r="K56" s="14" t="n">
-        <v>46311</v>
-      </c>
-      <c r="L56" s="15" t="n">
-        <v>70000</v>
-      </c>
-      <c r="M56" s="9" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N56" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O56" s="16" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O56"/>
+  <autoFilter ref="A1:O54"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -4608,8 +4468,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId51"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId55"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -4648,7 +4506,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3">
@@ -4658,7 +4516,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4">
@@ -4710,7 +4568,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3">
@@ -4720,7 +4578,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
@@ -4730,7 +4588,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -4772,7 +4630,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3">
@@ -4782,7 +4640,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4">
@@ -4844,7 +4702,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3">
@@ -4854,7 +4712,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4">
@@ -4870,17 +4728,17 @@
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
-          <t>Cultura</t>
+          <t>Educação / Ensino</t>
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>Educação / Ensino</t>
+          <t>Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="B6" s="10" t="n">
@@ -4890,21 +4748,21 @@
     <row r="7">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>Ciência / Tecnologia e Inovação</t>
+          <t>Cultura</t>
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>Meio Ambiente / Clima / Geografia</t>
+          <t>Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9">
@@ -4934,7 +4792,7 @@
         </is>
       </c>
       <c r="B11" s="18" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -4950,7 +4808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4972,7 +4830,7 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
@@ -4982,11 +4840,11 @@
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4">
@@ -5022,21 +4880,21 @@
     <row r="7">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -5049,8 +4907,18 @@
         <v>1</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>OEI/SECULT</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B9"/>
+  <autoFilter ref="A1:B10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -5094,7 +4962,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -5109,7 +4977,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-10-07 18:50
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 06/10/2026 às 18:16</t>
+          <t>Gerado em 07/10/2026 às 18:49</t>
         </is>
       </c>
     </row>
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>116902.8988571428</v>
+        <v>118045.756</v>
       </c>
     </row>
     <row r="20">
@@ -2220,30 +2220,30 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E23" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F23" s="21" t="n">
-        <v>0.433</v>
+        <v>0.593</v>
       </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
@@ -2253,17 +2253,17 @@
       </c>
       <c r="I23" s="19" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J23" s="22" t="n">
-        <v>46227</v>
+        <v>46251</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46252</v>
+        <v>46256</v>
       </c>
       <c r="L23" s="23" t="n">
-        <v>286000</v>
+        <v>50000</v>
       </c>
       <c r="M23" s="17" t="inlineStr">
         <is>
@@ -2277,7 +2277,7 @@
       </c>
       <c r="O23" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -2289,12 +2289,12 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -2304,15 +2304,15 @@
       </c>
       <c r="E24" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.569</v>
+        <v>0.433</v>
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
@@ -2322,17 +2322,17 @@
       </c>
       <c r="I24" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
         </is>
       </c>
       <c r="J24" s="14" t="n">
-        <v>46246</v>
+        <v>46227</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46257</v>
+        <v>46252</v>
       </c>
       <c r="L24" s="15" t="n">
-        <v>54000</v>
+        <v>286000</v>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
@@ -2346,7 +2346,7 @@
       </c>
       <c r="O24" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
@@ -2427,12 +2427,12 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -2450,7 +2450,7 @@
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Cultura, Desenvolvimento Social / Políticas Públicas</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
@@ -2460,21 +2460,19 @@
       </c>
       <c r="I26" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J26" s="14" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K26" s="14" t="n">
-        <v>46245</v>
-      </c>
-      <c r="L26" s="15" t="n">
-        <v>100000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L26" s="15" t="inlineStr"/>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N26" s="12" t="inlineStr">
@@ -2484,7 +2482,7 @@
       </c>
       <c r="O26" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -2496,12 +2494,12 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
@@ -2515,33 +2513,35 @@
         </is>
       </c>
       <c r="F27" s="21" t="n">
-        <v>0.492</v>
+        <v>0.569</v>
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I27" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J27" s="22" t="n">
         <v>46246</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L27" s="23" t="inlineStr"/>
+        <v>46257</v>
+      </c>
+      <c r="L27" s="23" t="n">
+        <v>54000</v>
+      </c>
       <c r="M27" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N27" s="20" t="inlineStr">
@@ -2551,7 +2551,7 @@
       </c>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -2563,17 +2563,17 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr">
@@ -2582,11 +2582,11 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.593</v>
+        <v>0.46</v>
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Educação / Ensino</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
@@ -2596,17 +2596,17 @@
       </c>
       <c r="I28" s="11" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J28" s="14" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46256</v>
+        <v>46259</v>
       </c>
       <c r="L28" s="15" t="n">
-        <v>50000</v>
+        <v>60000</v>
       </c>
       <c r="M28" s="9" t="inlineStr">
         <is>
@@ -2620,7 +2620,7 @@
       </c>
       <c r="O28" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -2632,12 +2632,12 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
@@ -2647,15 +2647,15 @@
       </c>
       <c r="E29" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F29" s="21" t="n">
-        <v>0.46</v>
+        <v>0.492</v>
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Educação / Ensino</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Educação / Ensino</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
@@ -2665,21 +2665,21 @@
       </c>
       <c r="I29" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J29" s="22" t="n">
-        <v>46252</v>
+        <v>46246</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46259</v>
+        <v>46272</v>
       </c>
       <c r="L29" s="23" t="n">
-        <v>60000</v>
+        <v>54000</v>
       </c>
       <c r="M29" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N29" s="20" t="inlineStr">
@@ -2689,7 +2689,7 @@
       </c>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -2701,17 +2701,17 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
@@ -2720,35 +2720,35 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.492</v>
+        <v>0.451</v>
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J30" s="14" t="n">
-        <v>46246</v>
+        <v>46265</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>46272</v>
+        <v>46270</v>
       </c>
       <c r="L30" s="15" t="n">
-        <v>54000</v>
+        <v>30000</v>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N30" s="12" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -2770,50 +2770,50 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E31" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F31" s="21" t="n">
-        <v>0.451</v>
+        <v>0.527</v>
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I31" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J31" s="22" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46270</v>
+        <v>46288</v>
       </c>
       <c r="L31" s="23" t="n">
-        <v>30000</v>
+        <v>70000</v>
       </c>
       <c r="M31" s="17" t="inlineStr">
         <is>
@@ -2827,7 +2827,7 @@
       </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
@@ -2839,50 +2839,50 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E32" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.451</v>
+        <v>0.493</v>
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Ciência / Tecnologia e Inovação, Engenharia / Infraestrutura</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I32" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Dados Remoto</t>
         </is>
       </c>
       <c r="J32" s="14" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="K32" s="14" t="n">
         <v>46286</v>
       </c>
       <c r="L32" s="15" t="n">
-        <v>30000</v>
+        <v>110000</v>
       </c>
       <c r="M32" s="9" t="inlineStr">
         <is>
@@ -2896,7 +2896,7 @@
       </c>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
         </is>
       </c>
     </row>
@@ -2975,12 +2975,12 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -2994,31 +2994,31 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.527</v>
+        <v>0.3</v>
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J34" s="14" t="n">
-        <v>46266</v>
+        <v>46275</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46288</v>
+        <v>46280</v>
       </c>
       <c r="L34" s="15" t="n">
-        <v>70000</v>
+        <v>50000</v>
       </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
@@ -3032,7 +3032,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
@@ -3044,17 +3044,17 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E35" s="20" t="inlineStr">
@@ -3063,11 +3063,11 @@
         </is>
       </c>
       <c r="F35" s="21" t="n">
-        <v>0.493</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Ciência / Tecnologia e Inovação, Engenharia / Infraestrutura</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Trabalho / Emprego, Segurança</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
@@ -3077,18 +3077,16 @@
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>Dados Remoto</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46281</v>
+        <v>46290</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46286</v>
-      </c>
-      <c r="L35" s="23" t="n">
-        <v>110000</v>
-      </c>
+        <v>46294</v>
+      </c>
+      <c r="L35" s="23" t="inlineStr"/>
       <c r="M35" s="17" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3101,7 +3099,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
         </is>
       </c>
     </row>
@@ -3113,12 +3111,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -3128,35 +3126,35 @@
       </c>
       <c r="E36" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>0.3</v>
+        <v>0.451</v>
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46275</v>
+        <v>46282</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46280</v>
+        <v>46286</v>
       </c>
       <c r="L36" s="15" t="n">
-        <v>50000</v>
+        <v>30000</v>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
@@ -3170,7 +3168,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
         </is>
       </c>
     </row>
@@ -3182,17 +3180,17 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E37" s="20" t="inlineStr">
@@ -3205,39 +3203,39 @@
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Trabalho / Emprego, Segurança</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46290</v>
+        <v>46278</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="L37" s="23" t="inlineStr"/>
       <c r="M37" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N37" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>ugp@educacao.sp.gov.br</t>
         </is>
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
         </is>
       </c>
     </row>
@@ -3249,12 +3247,12 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
@@ -3264,15 +3262,15 @@
       </c>
       <c r="E38" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.232</v>
+        <v>0.2</v>
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Educação / Ensino, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Direitos Humanos / Cidadania</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
@@ -3282,7 +3280,7 @@
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
+          <t>Articulação Estadual - Rio Grande do Norte</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
@@ -3292,11 +3290,11 @@
         <v>46298</v>
       </c>
       <c r="L38" s="15" t="n">
-        <v>30000</v>
+        <v>21000</v>
       </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N38" s="12" t="inlineStr">
@@ -3306,7 +3304,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
         </is>
       </c>
     </row>
@@ -3318,12 +3316,12 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
@@ -3337,43 +3335,45 @@
         </is>
       </c>
       <c r="F39" s="21" t="n">
-        <v>0.5639999999999999</v>
+        <v>0.175</v>
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Engenharia / Infraestrutura</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remota e/ou presencial em Brasília - DF</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46278</v>
+        <v>46294</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46295</v>
-      </c>
-      <c r="L39" s="23" t="inlineStr"/>
+        <v>46297</v>
+      </c>
+      <c r="L39" s="23" t="n">
+        <v>600000</v>
+      </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N39" s="20" t="inlineStr">
         <is>
-          <t>ugp@educacao.sp.gov.br</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
         </is>
       </c>
     </row>
@@ -3385,12 +3385,12 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
@@ -3400,15 +3400,15 @@
       </c>
       <c r="E40" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.2</v>
+        <v>0.232</v>
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Educação / Ensino, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Direitos Humanos / Cidadania</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
@@ -3418,7 +3418,7 @@
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Rio Grande do Norte</t>
+          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
@@ -3428,11 +3428,11 @@
         <v>46298</v>
       </c>
       <c r="L40" s="15" t="n">
-        <v>21000</v>
+        <v>30000</v>
       </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N40" s="12" t="inlineStr">
@@ -3442,7 +3442,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
         </is>
       </c>
     </row>
@@ -3454,12 +3454,12 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
@@ -3469,15 +3469,15 @@
       </c>
       <c r="E41" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Não Classificado</t>
         </is>
       </c>
       <c r="F41" s="21" t="n">
-        <v>0.355</v>
+        <v>0.077</v>
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
@@ -3487,17 +3487,17 @@
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
         <v>46294</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46302</v>
+        <v>46300</v>
       </c>
       <c r="L41" s="23" t="n">
-        <v>60000</v>
+        <v>55000</v>
       </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
@@ -3511,7 +3511,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
         </is>
       </c>
     </row>
@@ -3523,12 +3523,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3538,15 +3538,15 @@
       </c>
       <c r="E42" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.077</v>
+        <v>0.355</v>
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Educação / Ensino</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
@@ -3556,17 +3556,17 @@
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
         <v>46294</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46300</v>
+        <v>46302</v>
       </c>
       <c r="L42" s="15" t="n">
-        <v>55000</v>
+        <v>60000</v>
       </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
@@ -3580,7 +3580,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
         </is>
       </c>
     </row>
@@ -3592,12 +3592,12 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
@@ -3611,11 +3611,11 @@
         </is>
       </c>
       <c r="F43" s="21" t="n">
-        <v>0.175</v>
+        <v>0.333</v>
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Engenharia / Infraestrutura</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Cultura, Segurança, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
@@ -3625,21 +3625,21 @@
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Remota e/ou presencial em Brasília - DF</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="L43" s="23" t="n">
-        <v>600000</v>
+        <v>60000</v>
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N43" s="20" t="inlineStr">
@@ -3649,7 +3649,7 @@
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
         </is>
       </c>
     </row>
@@ -3661,12 +3661,12 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
@@ -3680,21 +3680,21 @@
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>0.333</v>
+        <v>0.282</v>
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Cultura, Segurança, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
         </is>
       </c>
     </row>
@@ -3799,12 +3799,12 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -3814,25 +3814,25 @@
       </c>
       <c r="E46" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.282</v>
+        <v>0.178</v>
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
+          <t>Tecnologia da Informação / Dados, Cultura, Comunicação</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J46" s="14" t="n">
@@ -3842,7 +3842,7 @@
         <v>46300</v>
       </c>
       <c r="L46" s="15" t="n">
-        <v>60000</v>
+        <v>21000</v>
       </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
@@ -3856,7 +3856,7 @@
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
         </is>
       </c>
     </row>
@@ -3868,17 +3868,17 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E47" s="20" t="inlineStr">
@@ -3887,45 +3887,45 @@
         </is>
       </c>
       <c r="F47" s="21" t="n">
-        <v>0.378</v>
+        <v>0.493</v>
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Cultura, Comunicação</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Desenvolvimento Social / Políticas Públicas</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J47" s="22" t="n">
+        <v>46244</v>
+      </c>
+      <c r="K47" s="22" t="n">
         <v>46296</v>
       </c>
-      <c r="K47" s="22" t="n">
-        <v>46300</v>
-      </c>
       <c r="L47" s="23" t="n">
-        <v>36000</v>
+        <v>935000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N47" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -3937,12 +3937,12 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
@@ -3952,15 +3952,15 @@
       </c>
       <c r="E48" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F48" s="13" t="n">
-        <v>0.178</v>
+        <v>0.378</v>
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Cultura, Comunicação</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Cultura, Comunicação</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
@@ -3980,7 +3980,7 @@
         <v>46300</v>
       </c>
       <c r="L48" s="15" t="n">
-        <v>21000</v>
+        <v>36000</v>
       </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
@@ -3994,7 +3994,7 @@
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
         </is>
       </c>
     </row>
@@ -4006,17 +4006,17 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13221</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E49" s="20" t="inlineStr">
@@ -4025,45 +4025,45 @@
         </is>
       </c>
       <c r="F49" s="21" t="n">
-        <v>0.493</v>
+        <v>0.409</v>
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Desenvolvimento Social / Políticas Públicas</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J49" s="22" t="n">
-        <v>46244</v>
+        <v>46297</v>
       </c>
       <c r="K49" s="22" t="n">
-        <v>46296</v>
+        <v>46311</v>
       </c>
       <c r="L49" s="23" t="n">
-        <v>935000</v>
+        <v>70000</v>
       </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N49" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221/</t>
         </is>
       </c>
     </row>
@@ -4075,12 +4075,12 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13221</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13304</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
@@ -4094,11 +4094,11 @@
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>0.409</v>
+        <v>0.445</v>
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
@@ -4118,11 +4118,11 @@
         <v>46311</v>
       </c>
       <c r="L50" s="15" t="n">
-        <v>70000</v>
+        <v>90000</v>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>Suspendida</t>
         </is>
       </c>
       <c r="N50" s="12" t="inlineStr">
@@ -4132,7 +4132,7 @@
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304/</t>
         </is>
       </c>
     </row>
@@ -4144,64 +4144,64 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13304</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E51" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F51" s="21" t="n">
-        <v>0.445</v>
+        <v>0.464</v>
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
-        <v>46297</v>
+        <v>46244</v>
       </c>
       <c r="K51" s="22" t="n">
-        <v>46311</v>
+        <v>46300</v>
       </c>
       <c r="L51" s="23" t="n">
-        <v>90000</v>
+        <v>350000</v>
       </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
-          <t>Suspendida</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N51" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -4213,12 +4213,12 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:procedimento-simplificado-no-13307-2026-oei-secult-es</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Procedimento Simplificado nº 13307/2026 – OEI/SECULT-ES</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
@@ -4228,35 +4228,35 @@
       </c>
       <c r="E52" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Não Classificado</t>
         </is>
       </c>
       <c r="F52" s="13" t="n">
-        <v>0.464</v>
+        <v>0.125</v>
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Cultura</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/SECULT</t>
         </is>
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Vitória/ES</t>
         </is>
       </c>
       <c r="J52" s="14" t="n">
-        <v>46244</v>
+        <v>46301</v>
       </c>
       <c r="K52" s="14" t="n">
-        <v>46300</v>
+        <v>46315</v>
       </c>
       <c r="L52" s="15" t="n">
-        <v>350000</v>
+        <v>600000</v>
       </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
@@ -4270,7 +4270,7 @@
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13307-2026-oei-secult-es/</t>
         </is>
       </c>
     </row>
@@ -4282,64 +4282,64 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:procedimento-simplificado-no-13307-2026-oei-secult-es</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Procedimento Simplificado nº 13307/2026 – OEI/SECULT-ES</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E53" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F53" s="21" t="n">
-        <v>0.125</v>
+        <v>0.378</v>
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Cultura</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Comunicação</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
         <is>
-          <t>OEI/SECULT</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>Vitória/ES</t>
+          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
         <v>46301</v>
       </c>
       <c r="K53" s="22" t="n">
-        <v>46315</v>
+        <v>46305</v>
       </c>
       <c r="L53" s="23" t="n">
-        <v>600000</v>
+        <v>62500</v>
       </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N53" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13307-2026-oei-secult-es/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
         </is>
       </c>
     </row>
@@ -4351,17 +4351,17 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13288</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E54" s="12" t="inlineStr">
@@ -4370,31 +4370,31 @@
         </is>
       </c>
       <c r="F54" s="13" t="n">
-        <v>0.378</v>
+        <v>0.433</v>
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Comunicação</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
+          <t>Consultor especialista em Gestão de Processos Secretaria de Estado da Educação  SEED-PR</t>
         </is>
       </c>
       <c r="J54" s="14" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="K54" s="14" t="n">
-        <v>46305</v>
+        <v>46307</v>
       </c>
       <c r="L54" s="15" t="n">
-        <v>62500</v>
+        <v>140000</v>
       </c>
       <c r="M54" s="9" t="inlineStr">
         <is>
@@ -4408,7 +4408,7 @@
       </c>
       <c r="O54" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288/</t>
         </is>
       </c>
     </row>
@@ -4630,7 +4630,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3">
@@ -4650,7 +4650,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
@@ -4702,7 +4702,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3">
@@ -4712,7 +4712,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4">
@@ -4722,7 +4722,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5">
@@ -4748,17 +4748,17 @@
     <row r="7">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>Cultura</t>
+          <t>Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>Ciência / Tecnologia e Inovação</t>
+          <t>Cultura</t>
         </is>
       </c>
       <c r="B8" s="10" t="n">
@@ -4782,7 +4782,7 @@
         </is>
       </c>
       <c r="B10" s="10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
@@ -4834,7 +4834,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3">
@@ -4844,7 +4844,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
🤖 Daily run: 2026-10-08 18:47
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$58</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -27,7 +27,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Por_Tipo'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Por_Area'!$A$1:$B$11</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Por_Area'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Por_Orgao'!$A$1:$B$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Por_Orgao'!$A$1:$B$11</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Por_Orgao'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Perfis'!$A$1:$C$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'Perfis'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 07/10/2026 às 18:49</t>
+          <t>Gerado em 08/10/2026 às 18:47</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6">
@@ -620,7 +620,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="17">
@@ -696,7 +696,7 @@
         </is>
       </c>
       <c r="B18" s="7" t="n">
-        <v>935000</v>
+        <v>2778901.38</v>
       </c>
     </row>
     <row r="19">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>118045.756</v>
+        <v>186276.3905263158</v>
       </c>
     </row>
     <row r="20">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>62500</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="24">
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="25">
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O54"/>
+  <dimension ref="A1:O58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1748,12 +1748,12 @@
       </c>
       <c r="B15" s="18" t="inlineStr">
         <is>
-          <t>unesco:375ed309-bb72-44ae-7d86-08df1d6278dd</t>
+          <t>unesco:8e654be2-3b1f-4782-d2b4-08df1fb02468</t>
         </is>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 41/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 57/2026 - 3 vagas - Consultor Individual</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
@@ -1763,15 +1763,15 @@
       </c>
       <c r="E15" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F15" s="21" t="n">
-        <v>0.433</v>
+        <v>0.222</v>
       </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Educação / Ensino, Direitos Humanos / Cidadania</t>
         </is>
       </c>
       <c r="H15" s="19" t="inlineStr">
@@ -1781,10 +1781,10 @@
       </c>
       <c r="I15" s="19" t="inlineStr"/>
       <c r="J15" s="22" t="n">
-        <v>46300</v>
+        <v>46303</v>
       </c>
       <c r="K15" s="22" t="n">
-        <v>46304</v>
+        <v>46309</v>
       </c>
       <c r="L15" s="23" t="inlineStr"/>
       <c r="M15" s="17" t="inlineStr">
@@ -1807,12 +1807,12 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
+          <t>unesco:375ed309-bb72-44ae-7d86-08df1d6278dd</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
+          <t>914BRZ1159 - Publicação Edital 41/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -1822,15 +1822,15 @@
       </c>
       <c r="E16" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.464</v>
+        <v>0.433</v>
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Arquitetura / Design</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
@@ -1840,10 +1840,10 @@
       </c>
       <c r="I16" s="11" t="inlineStr"/>
       <c r="J16" s="14" t="n">
-        <v>46286</v>
+        <v>46300</v>
       </c>
       <c r="K16" s="14" t="n">
-        <v>46316</v>
+        <v>46304</v>
       </c>
       <c r="L16" s="15" t="inlineStr"/>
       <c r="M16" s="9" t="inlineStr">
@@ -1866,12 +1866,12 @@
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
+          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
         </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
+          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1889,7 +1889,7 @@
       </c>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Ciências Sociais / Participação Social</t>
+          <t>Arquitetura / Design</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
@@ -1925,12 +1925,12 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
+          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
+          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -1944,11 +1944,11 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.423</v>
+        <v>0.464</v>
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Tecnologia da Informação / Dados, Ciências Sociais / Participação Social</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -1984,12 +1984,12 @@
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
+          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
+          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
@@ -2003,11 +2003,11 @@
         </is>
       </c>
       <c r="F19" s="21" t="n">
-        <v>0.464</v>
+        <v>0.423</v>
       </c>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Ciências Sociais / Participação Social</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
@@ -2043,12 +2043,12 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
+          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
+          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -2062,7 +2062,7 @@
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.423</v>
+        <v>0.464</v>
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
@@ -2102,12 +2102,12 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
+          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
+          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
@@ -2125,7 +2125,7 @@
       </c>
       <c r="G21" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Ciências Sociais / Participação Social</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
@@ -2161,17 +2161,17 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>unesco:ec486dce-4c41-4830-4e64-08df1817d7a0</t>
+          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ1085 - Edital nº 05/2026 - 02 vagas - Consultores Individuais</t>
+          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E22" s="12" t="inlineStr">
@@ -2180,11 +2180,11 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.3</v>
+        <v>0.423</v>
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Saúde, Estatística / Pesquisa / Metodologia, Cultura, Ciência / Tecnologia e Inovação</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
@@ -2194,10 +2194,10 @@
       </c>
       <c r="I22" s="11" t="inlineStr"/>
       <c r="J22" s="14" t="n">
-        <v>46296</v>
+        <v>46286</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46303</v>
+        <v>46316</v>
       </c>
       <c r="L22" s="15" t="inlineStr"/>
       <c r="M22" s="9" t="inlineStr">
@@ -2215,69 +2215,59 @@
     <row r="23">
       <c r="A23" s="17" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>unesco:ec486dce-4c41-4830-4e64-08df1817d7a0</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Projeto 914BRZ1085 - Edital nº 05/2026 - 02 vagas - Consultores Individuais</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E23" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F23" s="21" t="n">
-        <v>0.593</v>
+        <v>0.3</v>
       </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Saúde, Estatística / Pesquisa / Metodologia, Cultura, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I23" s="19" t="inlineStr">
-        <is>
-          <t>Recife - PE</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I23" s="19" t="inlineStr"/>
       <c r="J23" s="22" t="n">
-        <v>46251</v>
+        <v>46296</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46256</v>
-      </c>
-      <c r="L23" s="23" t="n">
-        <v>50000</v>
-      </c>
+        <v>46303</v>
+      </c>
+      <c r="L23" s="23" t="inlineStr"/>
       <c r="M23" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N23" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N23" s="20" t="inlineStr"/>
       <c r="O23" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
@@ -2358,12 +2348,12 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
@@ -2377,35 +2367,33 @@
         </is>
       </c>
       <c r="F25" s="21" t="n">
-        <v>0.569</v>
+        <v>0.492</v>
       </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I25" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J25" s="22" t="n">
         <v>46246</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46257</v>
-      </c>
-      <c r="L25" s="23" t="n">
-        <v>54000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L25" s="23" t="inlineStr"/>
       <c r="M25" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N25" s="20" t="inlineStr">
@@ -2415,7 +2403,7 @@
       </c>
       <c r="O25" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -2427,12 +2415,12 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -2446,33 +2434,35 @@
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.492</v>
+        <v>0.569</v>
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I26" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J26" s="14" t="n">
         <v>46246</v>
       </c>
       <c r="K26" s="14" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L26" s="15" t="inlineStr"/>
+        <v>46257</v>
+      </c>
+      <c r="L26" s="15" t="n">
+        <v>54000</v>
+      </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N26" s="12" t="inlineStr">
@@ -2482,7 +2472,7 @@
       </c>
       <c r="O26" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -2494,12 +2484,12 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
@@ -2517,7 +2507,7 @@
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
@@ -2551,7 +2541,7 @@
       </c>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -2563,17 +2553,17 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr">
@@ -2582,11 +2572,11 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.46</v>
+        <v>0.593</v>
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
@@ -2596,17 +2586,17 @@
       </c>
       <c r="I28" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J28" s="14" t="n">
-        <v>46252</v>
+        <v>46251</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46259</v>
+        <v>46256</v>
       </c>
       <c r="L28" s="15" t="n">
-        <v>60000</v>
+        <v>50000</v>
       </c>
       <c r="M28" s="9" t="inlineStr">
         <is>
@@ -2620,7 +2610,7 @@
       </c>
       <c r="O28" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -2632,12 +2622,12 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
@@ -2647,15 +2637,15 @@
       </c>
       <c r="E29" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F29" s="21" t="n">
-        <v>0.492</v>
+        <v>0.46</v>
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Educação / Ensino</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
@@ -2665,21 +2655,21 @@
       </c>
       <c r="I29" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J29" s="22" t="n">
-        <v>46246</v>
+        <v>46252</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46272</v>
+        <v>46259</v>
       </c>
       <c r="L29" s="23" t="n">
-        <v>54000</v>
+        <v>60000</v>
       </c>
       <c r="M29" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N29" s="20" t="inlineStr">
@@ -2689,7 +2679,7 @@
       </c>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -2701,17 +2691,17 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
@@ -2720,35 +2710,35 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.451</v>
+        <v>0.492</v>
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Educação / Ensino</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J30" s="14" t="n">
-        <v>46265</v>
+        <v>46246</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>46270</v>
+        <v>46272</v>
       </c>
       <c r="L30" s="15" t="n">
-        <v>30000</v>
+        <v>54000</v>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N30" s="12" t="inlineStr">
@@ -2758,7 +2748,7 @@
       </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -2770,50 +2760,50 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E31" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F31" s="21" t="n">
-        <v>0.527</v>
+        <v>0.451</v>
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I31" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J31" s="22" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46288</v>
+        <v>46270</v>
       </c>
       <c r="L31" s="23" t="n">
-        <v>70000</v>
+        <v>30000</v>
       </c>
       <c r="M31" s="17" t="inlineStr">
         <is>
@@ -2827,7 +2817,7 @@
       </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -2839,17 +2829,17 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E32" s="12" t="inlineStr">
@@ -2858,31 +2848,31 @@
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.493</v>
+        <v>0.527</v>
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Ciência / Tecnologia e Inovação, Engenharia / Infraestrutura</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I32" s="11" t="inlineStr">
         <is>
-          <t>Dados Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J32" s="14" t="n">
-        <v>46281</v>
+        <v>46266</v>
       </c>
       <c r="K32" s="14" t="n">
-        <v>46286</v>
+        <v>46288</v>
       </c>
       <c r="L32" s="15" t="n">
-        <v>110000</v>
+        <v>70000</v>
       </c>
       <c r="M32" s="9" t="inlineStr">
         <is>
@@ -2896,7 +2886,7 @@
       </c>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
@@ -2908,12 +2898,12 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
@@ -2927,11 +2917,11 @@
         </is>
       </c>
       <c r="F33" s="21" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
@@ -2941,16 +2931,18 @@
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J33" s="22" t="n">
         <v>46275</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46281</v>
-      </c>
-      <c r="L33" s="23" t="inlineStr"/>
+        <v>46280</v>
+      </c>
+      <c r="L33" s="23" t="n">
+        <v>50000</v>
+      </c>
       <c r="M33" s="17" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -2963,7 +2955,7 @@
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
@@ -2975,12 +2967,12 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -2994,11 +2986,11 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
@@ -3008,18 +3000,16 @@
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J34" s="14" t="n">
         <v>46275</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46280</v>
-      </c>
-      <c r="L34" s="15" t="n">
-        <v>50000</v>
-      </c>
+        <v>46281</v>
+      </c>
+      <c r="L34" s="15" t="inlineStr"/>
       <c r="M34" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3032,7 +3022,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
         </is>
       </c>
     </row>
@@ -3044,49 +3034,51 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E35" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F35" s="21" t="n">
-        <v>0.5639999999999999</v>
+        <v>0.451</v>
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Trabalho / Emprego, Segurança</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46290</v>
+        <v>46282</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46294</v>
-      </c>
-      <c r="L35" s="23" t="inlineStr"/>
+        <v>46286</v>
+      </c>
+      <c r="L35" s="23" t="n">
+        <v>30000</v>
+      </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3099,7 +3091,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
         </is>
       </c>
     </row>
@@ -3111,51 +3103,49 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E36" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>0.451</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Trabalho / Emprego, Segurança</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46282</v>
+        <v>46290</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46286</v>
-      </c>
-      <c r="L36" s="15" t="n">
-        <v>30000</v>
-      </c>
+        <v>46294</v>
+      </c>
+      <c r="L36" s="15" t="inlineStr"/>
       <c r="M36" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3168,7 +3158,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
         </is>
       </c>
     </row>
@@ -3180,17 +3170,17 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E37" s="20" t="inlineStr">
@@ -3199,43 +3189,45 @@
         </is>
       </c>
       <c r="F37" s="21" t="n">
-        <v>0.5639999999999999</v>
+        <v>0.493</v>
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Ciência / Tecnologia e Inovação, Engenharia / Infraestrutura</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Dados Remoto</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46278</v>
+        <v>46281</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46295</v>
-      </c>
-      <c r="L37" s="23" t="inlineStr"/>
+        <v>46286</v>
+      </c>
+      <c r="L37" s="23" t="n">
+        <v>110000</v>
+      </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N37" s="20" t="inlineStr">
         <is>
-          <t>ugp@educacao.sp.gov.br</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
         </is>
       </c>
     </row>
@@ -3247,12 +3239,12 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
@@ -3262,15 +3254,15 @@
       </c>
       <c r="E38" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.2</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Educação / Ensino, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Direitos Humanos / Cidadania</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
@@ -3280,18 +3272,16 @@
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Rio Grande do Norte</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46293</v>
+        <v>46278</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46298</v>
-      </c>
-      <c r="L38" s="15" t="n">
-        <v>21000</v>
-      </c>
+        <v>46295</v>
+      </c>
+      <c r="L38" s="15" t="inlineStr"/>
       <c r="M38" s="9" t="inlineStr">
         <is>
           <t>En fase de apresentação</t>
@@ -3299,12 +3289,12 @@
       </c>
       <c r="N38" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>ugp@educacao.sp.gov.br</t>
         </is>
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
         </is>
       </c>
     </row>
@@ -3316,12 +3306,12 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
@@ -3331,35 +3321,35 @@
       </c>
       <c r="E39" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F39" s="21" t="n">
-        <v>0.175</v>
+        <v>0.2</v>
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Engenharia / Infraestrutura</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Educação / Ensino, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Direitos Humanos / Cidadania</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Remota e/ou presencial em Brasília - DF</t>
+          <t>Articulação Estadual - Rio Grande do Norte</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="L39" s="23" t="n">
-        <v>600000</v>
+        <v>21000</v>
       </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
@@ -3373,7 +3363,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
         </is>
       </c>
     </row>
@@ -3454,12 +3444,12 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
+          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
+          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
@@ -3469,39 +3459,39 @@
       </c>
       <c r="E41" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F41" s="21" t="n">
-        <v>0.077</v>
+        <v>0.175</v>
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Engenharia / Infraestrutura</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Remota e/ou presencial em Brasília - DF</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
         <v>46294</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46300</v>
+        <v>46297</v>
       </c>
       <c r="L41" s="23" t="n">
-        <v>55000</v>
+        <v>600000</v>
       </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N41" s="20" t="inlineStr">
@@ -3511,7 +3501,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
         </is>
       </c>
     </row>
@@ -3523,12 +3513,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3538,15 +3528,15 @@
       </c>
       <c r="E42" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Não Classificado</t>
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.355</v>
+        <v>0.077</v>
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
@@ -3556,17 +3546,17 @@
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
         <v>46294</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46302</v>
+        <v>46300</v>
       </c>
       <c r="L42" s="15" t="n">
-        <v>60000</v>
+        <v>55000</v>
       </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
@@ -3580,7 +3570,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
         </is>
       </c>
     </row>
@@ -3592,12 +3582,12 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
@@ -3611,28 +3601,28 @@
         </is>
       </c>
       <c r="F43" s="21" t="n">
-        <v>0.333</v>
+        <v>0.355</v>
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Cultura, Segurança, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Educação / Ensino</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46296</v>
+        <v>46294</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46300</v>
+        <v>46302</v>
       </c>
       <c r="L43" s="23" t="n">
         <v>60000</v>
@@ -3649,7 +3639,7 @@
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
         </is>
       </c>
     </row>
@@ -3661,12 +3651,12 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
@@ -3680,21 +3670,21 @@
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>0.282</v>
+        <v>0.333</v>
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Cultura, Segurança, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
@@ -3718,7 +3708,7 @@
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
         </is>
       </c>
     </row>
@@ -3730,12 +3720,12 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
@@ -3745,25 +3735,25 @@
       </c>
       <c r="E45" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F45" s="21" t="n">
-        <v>0.216</v>
+        <v>0.282</v>
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Cultura, Comunicação, Arquitetura / Design</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
@@ -3773,7 +3763,7 @@
         <v>46300</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>33000</v>
+        <v>60000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
@@ -3787,7 +3777,7 @@
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
         </is>
       </c>
     </row>
@@ -3799,12 +3789,12 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -3818,11 +3808,11 @@
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.178</v>
+        <v>0.216</v>
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Cultura, Comunicação</t>
+          <t>Tecnologia da Informação / Dados, Cultura, Comunicação, Arquitetura / Design</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
@@ -3842,7 +3832,7 @@
         <v>46300</v>
       </c>
       <c r="L46" s="15" t="n">
-        <v>21000</v>
+        <v>33000</v>
       </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
@@ -3856,7 +3846,7 @@
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
         </is>
       </c>
     </row>
@@ -3868,64 +3858,64 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E47" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F47" s="21" t="n">
-        <v>0.493</v>
+        <v>0.178</v>
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Desenvolvimento Social / Políticas Públicas</t>
+          <t>Tecnologia da Informação / Dados, Cultura, Comunicação</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J47" s="22" t="n">
-        <v>46244</v>
+        <v>46296</v>
       </c>
       <c r="K47" s="22" t="n">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="L47" s="23" t="n">
-        <v>935000</v>
+        <v>21000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N47" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
         </is>
       </c>
     </row>
@@ -3937,17 +3927,17 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E48" s="12" t="inlineStr">
@@ -3956,45 +3946,45 @@
         </is>
       </c>
       <c r="F48" s="13" t="n">
-        <v>0.378</v>
+        <v>0.493</v>
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Cultura, Comunicação</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Desenvolvimento Social / Políticas Públicas</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J48" s="14" t="n">
+        <v>46244</v>
+      </c>
+      <c r="K48" s="14" t="n">
         <v>46296</v>
       </c>
-      <c r="K48" s="14" t="n">
-        <v>46300</v>
-      </c>
       <c r="L48" s="15" t="n">
-        <v>36000</v>
+        <v>935000</v>
       </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N48" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -4006,12 +3996,12 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13221</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
@@ -4025,31 +4015,31 @@
         </is>
       </c>
       <c r="F49" s="21" t="n">
-        <v>0.409</v>
+        <v>0.378</v>
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Cultura, Comunicação</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J49" s="22" t="n">
-        <v>46297</v>
+        <v>46296</v>
       </c>
       <c r="K49" s="22" t="n">
-        <v>46311</v>
+        <v>46300</v>
       </c>
       <c r="L49" s="23" t="n">
-        <v>70000</v>
+        <v>36000</v>
       </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
@@ -4063,7 +4053,7 @@
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
         </is>
       </c>
     </row>
@@ -4075,12 +4065,12 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13304</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13221</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
@@ -4094,11 +4084,11 @@
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>0.445</v>
+        <v>0.409</v>
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
@@ -4118,11 +4108,11 @@
         <v>46311</v>
       </c>
       <c r="L50" s="15" t="n">
-        <v>90000</v>
+        <v>70000</v>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>Suspendida</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N50" s="12" t="inlineStr">
@@ -4132,7 +4122,7 @@
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221/</t>
         </is>
       </c>
     </row>
@@ -4213,64 +4203,64 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:procedimento-simplificado-no-13307-2026-oei-secult-es</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Procedimento Simplificado nº 13307/2026 – OEI/SECULT-ES</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13304</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E52" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F52" s="13" t="n">
-        <v>0.125</v>
+        <v>0.445</v>
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Cultura</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
-          <t>OEI/SECULT</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>Vitória/ES</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J52" s="14" t="n">
-        <v>46301</v>
+        <v>46297</v>
       </c>
       <c r="K52" s="14" t="n">
-        <v>46315</v>
+        <v>46311</v>
       </c>
       <c r="L52" s="15" t="n">
-        <v>600000</v>
+        <v>90000</v>
       </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>Suspendida</t>
         </is>
       </c>
       <c r="N52" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13307-2026-oei-secult-es/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304/</t>
         </is>
       </c>
     </row>
@@ -4282,64 +4272,64 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
+          <t>oei:procedimento-simplificado-no-13307-2026-oei-secult-es</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
+          <t>Procedimento Simplificado nº 13307/2026 – OEI/SECULT-ES</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E53" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Não Classificado</t>
         </is>
       </c>
       <c r="F53" s="21" t="n">
-        <v>0.378</v>
+        <v>0.125</v>
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Comunicação</t>
+          <t>Tecnologia da Informação / Dados, Cultura</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/SECULT</t>
         </is>
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
+          <t>Vitória/ES</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
         <v>46301</v>
       </c>
       <c r="K53" s="22" t="n">
-        <v>46305</v>
+        <v>46315</v>
       </c>
       <c r="L53" s="23" t="n">
-        <v>62500</v>
+        <v>600000</v>
       </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N53" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13307-2026-oei-secult-es/</t>
         </is>
       </c>
     </row>
@@ -4351,69 +4341,345 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
+        </is>
+      </c>
+      <c r="C54" s="11" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
+        </is>
+      </c>
+      <c r="D54" s="11" t="inlineStr">
+        <is>
+          <t>Consultoria Pessoa Física (PF)</t>
+        </is>
+      </c>
+      <c r="E54" s="12" t="inlineStr">
+        <is>
+          <t>Engenharia Processos Analytics</t>
+        </is>
+      </c>
+      <c r="F54" s="13" t="n">
+        <v>0.378</v>
+      </c>
+      <c r="G54" s="11" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Comunicação</t>
+        </is>
+      </c>
+      <c r="H54" s="11" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I54" s="11" t="inlineStr">
+        <is>
+          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
+        </is>
+      </c>
+      <c r="J54" s="14" t="n">
+        <v>46301</v>
+      </c>
+      <c r="K54" s="14" t="n">
+        <v>46305</v>
+      </c>
+      <c r="L54" s="15" t="n">
+        <v>62500</v>
+      </c>
+      <c r="M54" s="9" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N54" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O54" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B55" s="18" t="inlineStr">
+        <is>
+          <t>oei:licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco</t>
+        </is>
+      </c>
+      <c r="C55" s="19" t="inlineStr">
+        <is>
+          <t>LICITAÇÃO Nº 13292/2026- OEI/FPOS MELHOR TÉCNICA E MENOR PREÇO</t>
+        </is>
+      </c>
+      <c r="D55" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+        </is>
+      </c>
+      <c r="E55" s="20" t="inlineStr">
+        <is>
+          <t>Consultoria Diversidade Inclusao</t>
+        </is>
+      </c>
+      <c r="F55" s="21" t="n">
+        <v>0.175</v>
+      </c>
+      <c r="G55" s="19" t="inlineStr">
+        <is>
+          <t>Meio Ambiente / Clima / Geografia, Cultura, Engenharia / Infraestrutura</t>
+        </is>
+      </c>
+      <c r="H55" s="19" t="inlineStr">
+        <is>
+          <t>OEI/FPOS</t>
+        </is>
+      </c>
+      <c r="I55" s="19" t="inlineStr">
+        <is>
+          <t>Território Nacional</t>
+        </is>
+      </c>
+      <c r="J55" s="22" t="n">
+        <v>46302</v>
+      </c>
+      <c r="K55" s="22" t="n">
+        <v>46322</v>
+      </c>
+      <c r="L55" s="23" t="n">
+        <v>2778901.38</v>
+      </c>
+      <c r="M55" s="17" t="inlineStr">
+        <is>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N55" s="20" t="inlineStr">
+        <is>
+          <t>compras.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O55" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco/</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="9" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B56" s="10" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321</t>
+        </is>
+      </c>
+      <c r="C56" s="11" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO FP-26-05 – Brasil em Rede – TR13321</t>
+        </is>
+      </c>
+      <c r="D56" s="11" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E56" s="12" t="inlineStr">
+        <is>
+          <t>Engenharia Processos Analytics</t>
+        </is>
+      </c>
+      <c r="F56" s="13" t="n">
+        <v>0.352</v>
+      </c>
+      <c r="G56" s="11" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+        </is>
+      </c>
+      <c r="H56" s="11" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I56" s="11" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="J56" s="14" t="n">
+        <v>46302</v>
+      </c>
+      <c r="K56" s="14" t="n">
+        <v>46307</v>
+      </c>
+      <c r="L56" s="15" t="n">
+        <v>27000</v>
+      </c>
+      <c r="M56" s="9" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N56" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O56" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321/</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B57" s="18" t="inlineStr">
+        <is>
           <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288</t>
         </is>
       </c>
-      <c r="C54" s="11" t="inlineStr">
+      <c r="C57" s="19" t="inlineStr">
         <is>
           <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13288</t>
         </is>
       </c>
-      <c r="D54" s="11" t="inlineStr">
+      <c r="D57" s="19" t="inlineStr">
         <is>
           <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
-      <c r="E54" s="12" t="inlineStr">
+      <c r="E57" s="20" t="inlineStr">
         <is>
           <t>Engenharia Processos Analytics</t>
         </is>
       </c>
-      <c r="F54" s="13" t="n">
+      <c r="F57" s="21" t="n">
         <v>0.433</v>
       </c>
-      <c r="G54" s="11" t="inlineStr">
+      <c r="G57" s="19" t="inlineStr">
         <is>
           <t>Gestão / Administração Pública</t>
         </is>
       </c>
-      <c r="H54" s="11" t="inlineStr">
+      <c r="H57" s="19" t="inlineStr">
         <is>
           <t>OEI/BRA</t>
         </is>
       </c>
-      <c r="I54" s="11" t="inlineStr">
+      <c r="I57" s="19" t="inlineStr">
         <is>
           <t>Consultor especialista em Gestão de Processos Secretaria de Estado da Educação  SEED-PR</t>
         </is>
       </c>
-      <c r="J54" s="14" t="n">
+      <c r="J57" s="22" t="n">
         <v>46302</v>
       </c>
-      <c r="K54" s="14" t="n">
+      <c r="K57" s="22" t="n">
         <v>46307</v>
       </c>
-      <c r="L54" s="15" t="n">
+      <c r="L57" s="23" t="n">
         <v>140000</v>
       </c>
-      <c r="M54" s="9" t="inlineStr">
+      <c r="M57" s="17" t="inlineStr">
         <is>
           <t>En evaluación</t>
         </is>
       </c>
-      <c r="N54" s="12" t="inlineStr">
+      <c r="N57" s="20" t="inlineStr">
         <is>
           <t>selecao.bra@oei.int</t>
         </is>
       </c>
-      <c r="O54" s="16" t="inlineStr">
+      <c r="O57" s="24" t="inlineStr">
         <is>
           <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288/</t>
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" s="9" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B58" s="10" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13312</t>
+        </is>
+      </c>
+      <c r="C58" s="11" t="inlineStr">
+        <is>
+          <t>Contratação de consultor PROJETO ABDI – TR 13312</t>
+        </is>
+      </c>
+      <c r="D58" s="11" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E58" s="12" t="inlineStr">
+        <is>
+          <t>Engenharia Processos Analytics</t>
+        </is>
+      </c>
+      <c r="F58" s="13" t="n">
+        <v>0.267</v>
+      </c>
+      <c r="G58" s="11" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+        </is>
+      </c>
+      <c r="H58" s="11" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I58" s="11" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="J58" s="14" t="n">
+        <v>46303</v>
+      </c>
+      <c r="K58" s="14" t="n">
+        <v>46307</v>
+      </c>
+      <c r="L58" s="15" t="n">
+        <v>600000</v>
+      </c>
+      <c r="M58" s="9" t="inlineStr">
+        <is>
+          <t>En presentación</t>
+        </is>
+      </c>
+      <c r="N58" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O58" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13312/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O54"/>
+  <autoFilter ref="A1:O58"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -4468,6 +4734,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId51"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId57"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -4506,7 +4776,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3">
@@ -4526,7 +4796,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -4568,7 +4838,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3">
@@ -4578,7 +4848,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4">
@@ -4630,7 +4900,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3">
@@ -4640,7 +4910,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4">
@@ -4660,7 +4930,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -4702,7 +4972,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3">
@@ -4712,7 +4982,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4">
@@ -4722,43 +4992,43 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
-          <t>Educação / Ensino</t>
+          <t>Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>Meio Ambiente / Clima / Geografia</t>
+          <t>Educação / Ensino</t>
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>Ciência / Tecnologia e Inovação</t>
+          <t>Cultura</t>
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>Cultura</t>
+          <t>Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="B8" s="10" t="n">
@@ -4808,7 +5078,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4844,7 +5114,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4">
@@ -4854,7 +5124,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
@@ -4917,8 +5187,18 @@
         <v>1</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>OEI/FPOS</t>
+        </is>
+      </c>
+      <c r="B11" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B10"/>
+  <autoFilter ref="A1:B11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -4962,7 +5242,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -4977,7 +5257,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-10-09 18:18
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$58</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$60</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -27,7 +27,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Por_Tipo'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Por_Area'!$A$1:$B$11</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Por_Area'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Por_Orgao'!$A$1:$B$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Por_Orgao'!$A$1:$B$10</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Por_Orgao'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Perfis'!$A$1:$C$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'Perfis'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 08/10/2026 às 18:47</t>
+          <t>Gerado em 09/10/2026 às 18:17</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6">
@@ -620,7 +620,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="24">
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="25">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O58"/>
+  <dimension ref="A1:O60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1116,7 +1116,7 @@
         <v>46293</v>
       </c>
       <c r="K5" s="22" t="n">
-        <v>46307</v>
+        <v>46313</v>
       </c>
       <c r="L5" s="23" t="n">
         <v>93500</v>
@@ -1183,7 +1183,7 @@
         <v>46293</v>
       </c>
       <c r="K6" s="14" t="n">
-        <v>46307</v>
+        <v>46313</v>
       </c>
       <c r="L6" s="15" t="n">
         <v>91500</v>
@@ -1250,7 +1250,7 @@
         <v>46293</v>
       </c>
       <c r="K7" s="22" t="n">
-        <v>46307</v>
+        <v>46313</v>
       </c>
       <c r="L7" s="23" t="n">
         <v>121500</v>
@@ -1317,7 +1317,7 @@
         <v>46293</v>
       </c>
       <c r="K8" s="14" t="n">
-        <v>46307</v>
+        <v>46313</v>
       </c>
       <c r="L8" s="15" t="n">
         <v>121500</v>
@@ -1384,7 +1384,7 @@
         <v>46293</v>
       </c>
       <c r="K9" s="22" t="n">
-        <v>46307</v>
+        <v>46313</v>
       </c>
       <c r="L9" s="23" t="n">
         <v>93500</v>
@@ -1451,7 +1451,7 @@
         <v>46293</v>
       </c>
       <c r="K10" s="14" t="n">
-        <v>46307</v>
+        <v>46313</v>
       </c>
       <c r="L10" s="15" t="n">
         <v>93500</v>
@@ -1518,7 +1518,7 @@
         <v>46293</v>
       </c>
       <c r="K11" s="22" t="n">
-        <v>46307</v>
+        <v>46313</v>
       </c>
       <c r="L11" s="23" t="n">
         <v>86800</v>
@@ -1613,11 +1613,11 @@
         </is>
       </c>
       <c r="B13" s="18" t="n">
-        <v>146396</v>
+        <v>146401</v>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>BRA/25/024 - Edital nº 013/2026 – Contratação de consultoria especializada (pessoa física) para desenvolvimento de estudo e análise sobre os efeitos econômicos e sociais dos recursos mobilizados pelo FAT e pelo FGTS</t>
+          <t>Edital 06/2026 - Programa de Privacidade e Segurança da Informação</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
@@ -1627,35 +1627,35 @@
       </c>
       <c r="E13" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F13" s="21" t="n">
-        <v>0.474</v>
+        <v>0.175</v>
       </c>
       <c r="G13" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Segurança</t>
         </is>
       </c>
       <c r="H13" s="19" t="inlineStr">
         <is>
-          <t>MTE</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I13" s="19" t="inlineStr">
         <is>
-          <t>Brasília, com disponibilidade para viagens</t>
+          <t>Território Nacional</t>
         </is>
       </c>
       <c r="J13" s="22" t="n">
-        <v>46290</v>
+        <v>46301</v>
       </c>
       <c r="K13" s="22" t="n">
-        <v>46303</v>
+        <v>46316</v>
       </c>
       <c r="L13" s="23" t="n">
-        <v>208966.53</v>
+        <v>120000</v>
       </c>
       <c r="M13" s="17" t="inlineStr">
         <is>
@@ -1664,7 +1664,7 @@
       </c>
       <c r="N13" s="20" t="inlineStr">
         <is>
-          <t>selecao.spt@trabalho.gov.br</t>
+          <t>cgti@mdh.gov.br</t>
         </is>
       </c>
       <c r="O13" s="24" t="inlineStr">
@@ -1676,15 +1676,17 @@
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="n">
-        <v>146401</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>unesco:8e654be2-3b1f-4782-d2b4-08df1fb02468</t>
+        </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>Edital 06/2026 - Programa de Privacidade e Segurança da Informação</t>
+          <t>914BRZ1155 - EDITAL Nº 57/2026 - 3 vagas - Consultor Individual</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -1694,49 +1696,39 @@
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.175</v>
+        <v>0.222</v>
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Segurança</t>
+          <t>Educação / Ensino, Direitos Humanos / Cidadania</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
         <is>
-          <t>Não identificado</t>
-        </is>
-      </c>
-      <c r="I14" s="11" t="inlineStr">
-        <is>
-          <t>Território Nacional</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I14" s="11" t="inlineStr"/>
       <c r="J14" s="14" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="K14" s="14" t="n">
-        <v>46316</v>
-      </c>
-      <c r="L14" s="15" t="n">
-        <v>120000</v>
-      </c>
+        <v>46309</v>
+      </c>
+      <c r="L14" s="15" t="inlineStr"/>
       <c r="M14" s="9" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N14" s="12" t="inlineStr">
-        <is>
-          <t>cgti@mdh.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N14" s="12" t="inlineStr"/>
       <c r="O14" s="16" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
@@ -1748,12 +1740,12 @@
       </c>
       <c r="B15" s="18" t="inlineStr">
         <is>
-          <t>unesco:8e654be2-3b1f-4782-d2b4-08df1fb02468</t>
+          <t>unesco:d8649b2a-6267-450d-bf98-08df23ad085e</t>
         </is>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 57/2026 - 3 vagas - Consultor Individual</t>
+          <t>914BRZ4027 - Edital 56/2026 - Arquitetura e Urbanismo - Iphan-SP</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
@@ -1763,15 +1755,15 @@
       </c>
       <c r="E15" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F15" s="21" t="n">
-        <v>0.222</v>
+        <v>0.333</v>
       </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
-          <t>Educação / Ensino, Direitos Humanos / Cidadania</t>
+          <t>Gestão / Administração Pública, Cultura, Arquitetura / Design</t>
         </is>
       </c>
       <c r="H15" s="19" t="inlineStr">
@@ -1781,7 +1773,7 @@
       </c>
       <c r="I15" s="19" t="inlineStr"/>
       <c r="J15" s="22" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="K15" s="22" t="n">
         <v>46309</v>
@@ -1807,12 +1799,12 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>unesco:375ed309-bb72-44ae-7d86-08df1d6278dd</t>
+          <t>unesco:ec3e284f-74b2-4ad2-bf99-08df23ad085e</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 41/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ4027 - Edital 57/2026 - Arquitetura e Urbanismo - Centro Vivo</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -1822,15 +1814,15 @@
       </c>
       <c r="E16" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Não Classificado</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.433</v>
+        <v>0.143</v>
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Gestão / Administração Pública, Cultura, Arquitetura / Design</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
@@ -1840,10 +1832,10 @@
       </c>
       <c r="I16" s="11" t="inlineStr"/>
       <c r="J16" s="14" t="n">
-        <v>46300</v>
+        <v>46304</v>
       </c>
       <c r="K16" s="14" t="n">
-        <v>46304</v>
+        <v>46309</v>
       </c>
       <c r="L16" s="15" t="inlineStr"/>
       <c r="M16" s="9" t="inlineStr">
@@ -1866,12 +1858,12 @@
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
+          <t>unesco:fb72c64e-511e-4325-60e3-08df20839863</t>
         </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
+          <t>914BRZ1162 - Edital 05/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1881,15 +1873,15 @@
       </c>
       <c r="E17" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F17" s="21" t="n">
-        <v>0.464</v>
+        <v>0.175</v>
       </c>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>Arquitetura / Design</t>
+          <t>Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
@@ -1899,10 +1891,10 @@
       </c>
       <c r="I17" s="19" t="inlineStr"/>
       <c r="J17" s="22" t="n">
-        <v>46286</v>
+        <v>46304</v>
       </c>
       <c r="K17" s="22" t="n">
-        <v>46316</v>
+        <v>46310</v>
       </c>
       <c r="L17" s="23" t="inlineStr"/>
       <c r="M17" s="17" t="inlineStr">
@@ -1925,12 +1917,12 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
+          <t>unesco:df21a7d3-d7d5-44ad-60e4-08df20839863</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
+          <t>914BRZ1162 - Edital 06/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -1940,15 +1932,15 @@
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.464</v>
+        <v>0.3</v>
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Ciências Sociais / Participação Social</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -1958,10 +1950,10 @@
       </c>
       <c r="I18" s="11" t="inlineStr"/>
       <c r="J18" s="14" t="n">
-        <v>46286</v>
+        <v>46304</v>
       </c>
       <c r="K18" s="14" t="n">
-        <v>46316</v>
+        <v>46310</v>
       </c>
       <c r="L18" s="15" t="inlineStr"/>
       <c r="M18" s="9" t="inlineStr">
@@ -1984,12 +1976,12 @@
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
+          <t>unesco:375ed309-bb72-44ae-7d86-08df1d6278dd</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
+          <t>914BRZ1159 - Publicação Edital 41/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
@@ -1999,15 +1991,15 @@
       </c>
       <c r="E19" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F19" s="21" t="n">
-        <v>0.423</v>
+        <v>0.433</v>
       </c>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
@@ -2017,10 +2009,10 @@
       </c>
       <c r="I19" s="19" t="inlineStr"/>
       <c r="J19" s="22" t="n">
-        <v>46286</v>
+        <v>46300</v>
       </c>
       <c r="K19" s="22" t="n">
-        <v>46316</v>
+        <v>46304</v>
       </c>
       <c r="L19" s="23" t="inlineStr"/>
       <c r="M19" s="17" t="inlineStr">
@@ -2043,12 +2035,12 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
+          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
+          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -2066,7 +2058,7 @@
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Ciências Sociais / Participação Social</t>
+          <t>Arquitetura / Design</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
@@ -2102,12 +2094,12 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
+          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
+          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
@@ -2121,11 +2113,11 @@
         </is>
       </c>
       <c r="F21" s="21" t="n">
-        <v>0.423</v>
+        <v>0.464</v>
       </c>
       <c r="G21" s="19" t="inlineStr">
         <is>
-          <t>Ciências Sociais / Participação Social</t>
+          <t>Tecnologia da Informação / Dados, Ciências Sociais / Participação Social</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
@@ -2161,12 +2153,12 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
+          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
+          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -2184,7 +2176,7 @@
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
@@ -2220,17 +2212,17 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>unesco:ec486dce-4c41-4830-4e64-08df1817d7a0</t>
+          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ1085 - Edital nº 05/2026 - 02 vagas - Consultores Individuais</t>
+          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E23" s="20" t="inlineStr">
@@ -2239,11 +2231,11 @@
         </is>
       </c>
       <c r="F23" s="21" t="n">
-        <v>0.3</v>
+        <v>0.464</v>
       </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Saúde, Estatística / Pesquisa / Metodologia, Cultura, Ciência / Tecnologia e Inovação</t>
+          <t>Ciências Sociais / Participação Social</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
@@ -2253,10 +2245,10 @@
       </c>
       <c r="I23" s="19" t="inlineStr"/>
       <c r="J23" s="22" t="n">
-        <v>46296</v>
+        <v>46286</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46303</v>
+        <v>46316</v>
       </c>
       <c r="L23" s="23" t="inlineStr"/>
       <c r="M23" s="17" t="inlineStr">
@@ -2274,22 +2266,22 @@
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E24" s="12" t="inlineStr">
@@ -2298,112 +2290,94 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.433</v>
+        <v>0.423</v>
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Ciências Sociais / Participação Social</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I24" s="11" t="inlineStr">
-        <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I24" s="11" t="inlineStr"/>
       <c r="J24" s="14" t="n">
-        <v>46227</v>
+        <v>46286</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46252</v>
-      </c>
-      <c r="L24" s="15" t="n">
-        <v>286000</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L24" s="15" t="inlineStr"/>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N24" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N24" s="12" t="inlineStr"/>
       <c r="O24" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="17" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E25" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F25" s="21" t="n">
-        <v>0.492</v>
+        <v>0.423</v>
       </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Ciência / Tecnologia e Inovação</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I25" s="19" t="inlineStr">
-        <is>
-          <t>Brasília - DF | Híbrido</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I25" s="19" t="inlineStr"/>
       <c r="J25" s="22" t="n">
-        <v>46246</v>
+        <v>46286</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46250</v>
+        <v>46316</v>
       </c>
       <c r="L25" s="23" t="inlineStr"/>
       <c r="M25" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
-        </is>
-      </c>
-      <c r="N25" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N25" s="20" t="inlineStr"/>
       <c r="O25" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
@@ -2415,12 +2389,12 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -2438,7 +2412,7 @@
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
@@ -2472,7 +2446,7 @@
       </c>
       <c r="O26" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -2484,12 +2458,12 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
@@ -2499,15 +2473,15 @@
       </c>
       <c r="E27" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F27" s="21" t="n">
-        <v>0.569</v>
+        <v>0.433</v>
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
@@ -2517,17 +2491,17 @@
       </c>
       <c r="I27" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
         </is>
       </c>
       <c r="J27" s="22" t="n">
-        <v>46246</v>
+        <v>46227</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46257</v>
+        <v>46252</v>
       </c>
       <c r="L27" s="23" t="n">
-        <v>54000</v>
+        <v>286000</v>
       </c>
       <c r="M27" s="17" t="inlineStr">
         <is>
@@ -2541,7 +2515,7 @@
       </c>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
@@ -2553,17 +2527,17 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr">
@@ -2572,35 +2546,33 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.593</v>
+        <v>0.492</v>
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I28" s="11" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J28" s="14" t="n">
-        <v>46251</v>
+        <v>46246</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46256</v>
-      </c>
-      <c r="L28" s="15" t="n">
-        <v>50000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L28" s="15" t="inlineStr"/>
       <c r="M28" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N28" s="12" t="inlineStr">
@@ -2610,7 +2582,7 @@
       </c>
       <c r="O28" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -2622,12 +2594,12 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
@@ -2641,11 +2613,11 @@
         </is>
       </c>
       <c r="F29" s="21" t="n">
-        <v>0.46</v>
+        <v>0.569</v>
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
@@ -2655,17 +2627,17 @@
       </c>
       <c r="I29" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J29" s="22" t="n">
-        <v>46252</v>
+        <v>46246</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46259</v>
+        <v>46257</v>
       </c>
       <c r="L29" s="23" t="n">
-        <v>60000</v>
+        <v>54000</v>
       </c>
       <c r="M29" s="17" t="inlineStr">
         <is>
@@ -2679,7 +2651,7 @@
       </c>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -2691,30 +2663,30 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.492</v>
+        <v>0.593</v>
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
@@ -2724,21 +2696,21 @@
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J30" s="14" t="n">
-        <v>46246</v>
+        <v>46251</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>46272</v>
+        <v>46256</v>
       </c>
       <c r="L30" s="15" t="n">
-        <v>54000</v>
+        <v>50000</v>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N30" s="12" t="inlineStr">
@@ -2748,7 +2720,7 @@
       </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -2760,50 +2732,50 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E31" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F31" s="21" t="n">
-        <v>0.451</v>
+        <v>0.46</v>
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Educação / Ensino</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I31" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J31" s="22" t="n">
-        <v>46265</v>
+        <v>46252</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46270</v>
+        <v>46259</v>
       </c>
       <c r="L31" s="23" t="n">
-        <v>30000</v>
+        <v>60000</v>
       </c>
       <c r="M31" s="17" t="inlineStr">
         <is>
@@ -2817,7 +2789,7 @@
       </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -2898,30 +2870,30 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E33" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F33" s="21" t="n">
-        <v>0.3</v>
+        <v>0.451</v>
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
@@ -2931,17 +2903,17 @@
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J33" s="22" t="n">
-        <v>46275</v>
+        <v>46265</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46280</v>
+        <v>46270</v>
       </c>
       <c r="L33" s="23" t="n">
-        <v>50000</v>
+        <v>30000</v>
       </c>
       <c r="M33" s="17" t="inlineStr">
         <is>
@@ -2955,7 +2927,7 @@
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -2967,12 +2939,12 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -2982,37 +2954,39 @@
       </c>
       <c r="E34" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.2</v>
+        <v>0.492</v>
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Ciência / Tecnologia e Inovação</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Educação / Ensino</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J34" s="14" t="n">
-        <v>46275</v>
+        <v>46246</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46281</v>
-      </c>
-      <c r="L34" s="15" t="inlineStr"/>
+        <v>46272</v>
+      </c>
+      <c r="L34" s="15" t="n">
+        <v>54000</v>
+      </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N34" s="12" t="inlineStr">
@@ -3022,7 +2996,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -3034,12 +3008,12 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
@@ -3049,35 +3023,35 @@
       </c>
       <c r="E35" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F35" s="21" t="n">
-        <v>0.451</v>
+        <v>0.3</v>
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46282</v>
+        <v>46275</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46286</v>
+        <v>46280</v>
       </c>
       <c r="L35" s="23" t="n">
-        <v>30000</v>
+        <v>50000</v>
       </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
@@ -3091,7 +3065,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
@@ -3103,49 +3077,51 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E36" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>0.5639999999999999</v>
+        <v>0.451</v>
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Trabalho / Emprego, Segurança</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46290</v>
+        <v>46282</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46294</v>
-      </c>
-      <c r="L36" s="15" t="inlineStr"/>
+        <v>46286</v>
+      </c>
+      <c r="L36" s="15" t="n">
+        <v>30000</v>
+      </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3158,7 +3134,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
         </is>
       </c>
     </row>
@@ -3170,17 +3146,17 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E37" s="20" t="inlineStr">
@@ -3189,11 +3165,11 @@
         </is>
       </c>
       <c r="F37" s="21" t="n">
-        <v>0.493</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Ciência / Tecnologia e Inovação, Engenharia / Infraestrutura</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Trabalho / Emprego, Segurança</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
@@ -3203,18 +3179,16 @@
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Dados Remoto</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46281</v>
+        <v>46290</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46286</v>
-      </c>
-      <c r="L37" s="23" t="n">
-        <v>110000</v>
-      </c>
+        <v>46294</v>
+      </c>
+      <c r="L37" s="23" t="inlineStr"/>
       <c r="M37" s="17" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3227,7 +3201,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
         </is>
       </c>
     </row>
@@ -3239,12 +3213,12 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
@@ -3258,43 +3232,43 @@
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.5639999999999999</v>
+        <v>0.2</v>
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46278</v>
+        <v>46275</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46295</v>
+        <v>46281</v>
       </c>
       <c r="L38" s="15" t="inlineStr"/>
       <c r="M38" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N38" s="12" t="inlineStr">
         <is>
-          <t>ugp@educacao.sp.gov.br</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
         </is>
       </c>
     </row>
@@ -3306,54 +3280,54 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E39" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F39" s="21" t="n">
-        <v>0.2</v>
+        <v>0.493</v>
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Educação / Ensino, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Direitos Humanos / Cidadania</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Ciência / Tecnologia e Inovação, Engenharia / Infraestrutura</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Rio Grande do Norte</t>
+          <t>Dados Remoto</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46293</v>
+        <v>46281</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46298</v>
+        <v>46286</v>
       </c>
       <c r="L39" s="23" t="n">
-        <v>21000</v>
+        <v>110000</v>
       </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N39" s="20" t="inlineStr">
@@ -3363,7 +3337,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
         </is>
       </c>
     </row>
@@ -3375,12 +3349,12 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
@@ -3394,11 +3368,11 @@
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.232</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
@@ -3408,31 +3382,29 @@
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46293</v>
+        <v>46278</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46298</v>
-      </c>
-      <c r="L40" s="15" t="n">
-        <v>30000</v>
-      </c>
+        <v>46295</v>
+      </c>
+      <c r="L40" s="15" t="inlineStr"/>
       <c r="M40" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N40" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>ugp@educacao.sp.gov.br</t>
         </is>
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
         </is>
       </c>
     </row>
@@ -3444,12 +3416,12 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
@@ -3459,35 +3431,35 @@
       </c>
       <c r="E41" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F41" s="21" t="n">
-        <v>0.175</v>
+        <v>0.2</v>
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Engenharia / Infraestrutura</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Educação / Ensino, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Direitos Humanos / Cidadania</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Remota e/ou presencial em Brasília - DF</t>
+          <t>Articulação Estadual - Rio Grande do Norte</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="L41" s="23" t="n">
-        <v>600000</v>
+        <v>21000</v>
       </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
@@ -3501,7 +3473,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
         </is>
       </c>
     </row>
@@ -3582,12 +3554,12 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
@@ -3601,11 +3573,11 @@
         </is>
       </c>
       <c r="F43" s="21" t="n">
-        <v>0.355</v>
+        <v>0.232</v>
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
@@ -3615,17 +3587,17 @@
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46302</v>
+        <v>46298</v>
       </c>
       <c r="L43" s="23" t="n">
-        <v>60000</v>
+        <v>30000</v>
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
@@ -3639,7 +3611,7 @@
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
         </is>
       </c>
     </row>
@@ -3651,12 +3623,12 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
+          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
+          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
@@ -3670,11 +3642,11 @@
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>0.333</v>
+        <v>0.175</v>
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Cultura, Segurança, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Engenharia / Infraestrutura</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
@@ -3684,21 +3656,21 @@
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remota e/ou presencial em Brasília - DF</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46296</v>
+        <v>46294</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46300</v>
+        <v>46297</v>
       </c>
       <c r="L44" s="15" t="n">
-        <v>60000</v>
+        <v>600000</v>
       </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N44" s="12" t="inlineStr">
@@ -3708,7 +3680,7 @@
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
         </is>
       </c>
     </row>
@@ -3720,12 +3692,12 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
@@ -3739,11 +3711,11 @@
         </is>
       </c>
       <c r="F45" s="21" t="n">
-        <v>0.282</v>
+        <v>0.355</v>
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Educação / Ensino</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
@@ -3753,14 +3725,14 @@
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46296</v>
+        <v>46294</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46300</v>
+        <v>46302</v>
       </c>
       <c r="L45" s="23" t="n">
         <v>60000</v>
@@ -3777,7 +3749,7 @@
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
         </is>
       </c>
     </row>
@@ -3789,12 +3761,12 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -3804,15 +3776,15 @@
       </c>
       <c r="E46" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.216</v>
+        <v>0.333</v>
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Cultura, Comunicação, Arquitetura / Design</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Cultura, Segurança, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
@@ -3822,7 +3794,7 @@
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J46" s="14" t="n">
@@ -3832,7 +3804,7 @@
         <v>46300</v>
       </c>
       <c r="L46" s="15" t="n">
-        <v>33000</v>
+        <v>60000</v>
       </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
@@ -3846,7 +3818,7 @@
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
         </is>
       </c>
     </row>
@@ -3858,12 +3830,12 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
@@ -3873,25 +3845,25 @@
       </c>
       <c r="E47" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F47" s="21" t="n">
-        <v>0.178</v>
+        <v>0.282</v>
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Cultura, Comunicação</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J47" s="22" t="n">
@@ -3901,7 +3873,7 @@
         <v>46300</v>
       </c>
       <c r="L47" s="23" t="n">
-        <v>21000</v>
+        <v>60000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
@@ -3915,7 +3887,7 @@
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
         </is>
       </c>
     </row>
@@ -3927,64 +3899,64 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E48" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F48" s="13" t="n">
-        <v>0.493</v>
+        <v>0.178</v>
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Desenvolvimento Social / Políticas Públicas</t>
+          <t>Tecnologia da Informação / Dados, Cultura, Comunicação</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J48" s="14" t="n">
-        <v>46244</v>
+        <v>46296</v>
       </c>
       <c r="K48" s="14" t="n">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="L48" s="15" t="n">
-        <v>935000</v>
+        <v>21000</v>
       </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N48" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
         </is>
       </c>
     </row>
@@ -3996,12 +3968,12 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
@@ -4011,15 +3983,15 @@
       </c>
       <c r="E49" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F49" s="21" t="n">
-        <v>0.378</v>
+        <v>0.216</v>
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Cultura, Comunicação</t>
+          <t>Tecnologia da Informação / Dados, Cultura, Comunicação, Arquitetura / Design</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
@@ -4039,7 +4011,7 @@
         <v>46300</v>
       </c>
       <c r="L49" s="23" t="n">
-        <v>36000</v>
+        <v>33000</v>
       </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
@@ -4053,7 +4025,7 @@
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
         </is>
       </c>
     </row>
@@ -4065,17 +4037,17 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13221</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E50" s="12" t="inlineStr">
@@ -4084,45 +4056,45 @@
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>0.409</v>
+        <v>0.493</v>
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Desenvolvimento Social / Políticas Públicas</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J50" s="14" t="n">
-        <v>46297</v>
+        <v>46244</v>
       </c>
       <c r="K50" s="14" t="n">
-        <v>46311</v>
+        <v>46296</v>
       </c>
       <c r="L50" s="15" t="n">
-        <v>70000</v>
+        <v>935000</v>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N50" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -4134,64 +4106,64 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E51" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F51" s="21" t="n">
-        <v>0.464</v>
+        <v>0.378</v>
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Cultura, Comunicação</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
-        <v>46244</v>
+        <v>46296</v>
       </c>
       <c r="K51" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="L51" s="23" t="n">
-        <v>350000</v>
+        <v>36000</v>
       </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N51" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
         </is>
       </c>
     </row>
@@ -4203,12 +4175,12 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13304</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13221</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
@@ -4222,11 +4194,11 @@
         </is>
       </c>
       <c r="F52" s="13" t="n">
-        <v>0.445</v>
+        <v>0.409</v>
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
@@ -4246,11 +4218,11 @@
         <v>46311</v>
       </c>
       <c r="L52" s="15" t="n">
-        <v>90000</v>
+        <v>70000</v>
       </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
-          <t>Suspendida</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N52" s="12" t="inlineStr">
@@ -4260,7 +4232,7 @@
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221/</t>
         </is>
       </c>
     </row>
@@ -4272,12 +4244,12 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:procedimento-simplificado-no-13307-2026-oei-secult-es</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Procedimento Simplificado nº 13307/2026 – OEI/SECULT-ES</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
@@ -4287,35 +4259,35 @@
       </c>
       <c r="E53" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F53" s="21" t="n">
-        <v>0.125</v>
+        <v>0.464</v>
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Cultura</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
         <is>
-          <t>OEI/SECULT</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>Vitória/ES</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
-        <v>46301</v>
+        <v>46244</v>
       </c>
       <c r="K53" s="22" t="n">
-        <v>46315</v>
+        <v>46300</v>
       </c>
       <c r="L53" s="23" t="n">
-        <v>600000</v>
+        <v>350000</v>
       </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
@@ -4329,7 +4301,7 @@
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13307-2026-oei-secult-es/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -4341,17 +4313,17 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13304</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E54" s="12" t="inlineStr">
@@ -4360,35 +4332,35 @@
         </is>
       </c>
       <c r="F54" s="13" t="n">
-        <v>0.378</v>
+        <v>0.445</v>
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Comunicação</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J54" s="14" t="n">
-        <v>46301</v>
+        <v>46297</v>
       </c>
       <c r="K54" s="14" t="n">
-        <v>46305</v>
+        <v>46311</v>
       </c>
       <c r="L54" s="15" t="n">
-        <v>62500</v>
+        <v>90000</v>
       </c>
       <c r="M54" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>Suspendida</t>
         </is>
       </c>
       <c r="N54" s="12" t="inlineStr">
@@ -4398,7 +4370,7 @@
       </c>
       <c r="O54" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304/</t>
         </is>
       </c>
     </row>
@@ -4479,64 +4451,64 @@
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321</t>
+          <t>oei:procedimento-simplificado-no-13307-2026-oei-secult-es</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO FP-26-05 – Brasil em Rede – TR13321</t>
+          <t>Procedimento Simplificado nº 13307/2026 – OEI/SECULT-ES</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E56" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Não Classificado</t>
         </is>
       </c>
       <c r="F56" s="13" t="n">
-        <v>0.352</v>
+        <v>0.125</v>
       </c>
       <c r="G56" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Cultura</t>
         </is>
       </c>
       <c r="H56" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/SECULT</t>
         </is>
       </c>
       <c r="I56" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Vitória/ES</t>
         </is>
       </c>
       <c r="J56" s="14" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="K56" s="14" t="n">
-        <v>46307</v>
+        <v>46315</v>
       </c>
       <c r="L56" s="15" t="n">
-        <v>27000</v>
+        <v>600000</v>
       </c>
       <c r="M56" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N56" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O56" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13307-2026-oei-secult-es/</t>
         </is>
       </c>
     </row>
@@ -4548,17 +4520,17 @@
       </c>
       <c r="B57" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
         </is>
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13288</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
         </is>
       </c>
       <c r="D57" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E57" s="20" t="inlineStr">
@@ -4567,31 +4539,31 @@
         </is>
       </c>
       <c r="F57" s="21" t="n">
-        <v>0.433</v>
+        <v>0.378</v>
       </c>
       <c r="G57" s="19" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Comunicação</t>
         </is>
       </c>
       <c r="H57" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I57" s="19" t="inlineStr">
         <is>
-          <t>Consultor especialista em Gestão de Processos Secretaria de Estado da Educação  SEED-PR</t>
+          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
         </is>
       </c>
       <c r="J57" s="22" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="K57" s="22" t="n">
-        <v>46307</v>
+        <v>46305</v>
       </c>
       <c r="L57" s="23" t="n">
-        <v>140000</v>
+        <v>62500</v>
       </c>
       <c r="M57" s="17" t="inlineStr">
         <is>
@@ -4605,7 +4577,7 @@
       </c>
       <c r="O57" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
         </is>
       </c>
     </row>
@@ -4617,17 +4589,17 @@
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13312</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO ABDI – TR 13312</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13288</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E58" s="12" t="inlineStr">
@@ -4636,50 +4608,188 @@
         </is>
       </c>
       <c r="F58" s="13" t="n">
-        <v>0.267</v>
+        <v>0.433</v>
       </c>
       <c r="G58" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H58" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I58" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Consultor especialista em Gestão de Processos Secretaria de Estado da Educação  SEED-PR</t>
         </is>
       </c>
       <c r="J58" s="14" t="n">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="K58" s="14" t="n">
         <v>46307</v>
       </c>
       <c r="L58" s="15" t="n">
+        <v>140000</v>
+      </c>
+      <c r="M58" s="9" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N58" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O58" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288/</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B59" s="18" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321</t>
+        </is>
+      </c>
+      <c r="C59" s="19" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO FP-26-05 – Brasil em Rede – TR13321</t>
+        </is>
+      </c>
+      <c r="D59" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E59" s="20" t="inlineStr">
+        <is>
+          <t>Engenharia Processos Analytics</t>
+        </is>
+      </c>
+      <c r="F59" s="21" t="n">
+        <v>0.352</v>
+      </c>
+      <c r="G59" s="19" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+        </is>
+      </c>
+      <c r="H59" s="19" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I59" s="19" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="J59" s="22" t="n">
+        <v>46302</v>
+      </c>
+      <c r="K59" s="22" t="n">
+        <v>46307</v>
+      </c>
+      <c r="L59" s="23" t="n">
+        <v>27000</v>
+      </c>
+      <c r="M59" s="17" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N59" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O59" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321/</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="9" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B60" s="10" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13312</t>
+        </is>
+      </c>
+      <c r="C60" s="11" t="inlineStr">
+        <is>
+          <t>Contratação de consultor PROJETO ABDI – TR 13312</t>
+        </is>
+      </c>
+      <c r="D60" s="11" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E60" s="12" t="inlineStr">
+        <is>
+          <t>Engenharia Processos Analytics</t>
+        </is>
+      </c>
+      <c r="F60" s="13" t="n">
+        <v>0.267</v>
+      </c>
+      <c r="G60" s="11" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+        </is>
+      </c>
+      <c r="H60" s="11" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I60" s="11" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="J60" s="14" t="n">
+        <v>46303</v>
+      </c>
+      <c r="K60" s="14" t="n">
+        <v>46307</v>
+      </c>
+      <c r="L60" s="15" t="n">
         <v>600000</v>
       </c>
-      <c r="M58" s="9" t="inlineStr">
+      <c r="M60" s="9" t="inlineStr">
         <is>
           <t>En presentación</t>
         </is>
       </c>
-      <c r="N58" s="12" t="inlineStr">
+      <c r="N60" s="12" t="inlineStr">
         <is>
           <t>selecao.bra@oei.int</t>
         </is>
       </c>
-      <c r="O58" s="16" t="inlineStr">
+      <c r="O60" s="16" t="inlineStr">
         <is>
           <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13312/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O58"/>
+  <autoFilter ref="A1:O60"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -4738,6 +4848,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId55"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId56"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId59"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -4786,7 +4898,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4">
@@ -4796,7 +4908,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -4838,7 +4950,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3">
@@ -4848,7 +4960,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
@@ -4858,7 +4970,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -4900,7 +5012,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3">
@@ -4910,7 +5022,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
@@ -4972,7 +5084,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3">
@@ -4982,7 +5094,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4">
@@ -4992,23 +5104,23 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
-          <t>Meio Ambiente / Clima / Geografia</t>
+          <t>Educação / Ensino</t>
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>Educação / Ensino</t>
+          <t>Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="B6" s="10" t="n">
@@ -5022,13 +5134,13 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>Ciência / Tecnologia e Inovação</t>
+          <t>Ciências Sociais / Participação Social</t>
         </is>
       </c>
       <c r="B8" s="10" t="n">
@@ -5038,11 +5150,11 @@
     <row r="9">
       <c r="A9" s="19" t="inlineStr">
         <is>
-          <t>Ciências Sociais / Participação Social</t>
+          <t>Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10">
@@ -5058,7 +5170,7 @@
     <row r="11">
       <c r="A11" s="19" t="inlineStr">
         <is>
-          <t>Trabalho / Emprego</t>
+          <t>Arquitetura / Design</t>
         </is>
       </c>
       <c r="B11" s="18" t="n">
@@ -5078,7 +5190,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5124,7 +5236,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5">
@@ -5170,7 +5282,7 @@
     <row r="9">
       <c r="A9" s="19" t="inlineStr">
         <is>
-          <t>MTE</t>
+          <t>OEI/FPOS</t>
         </is>
       </c>
       <c r="B9" s="18" t="n">
@@ -5187,18 +5299,8 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="19" t="inlineStr">
-        <is>
-          <t>OEI/FPOS</t>
-        </is>
-      </c>
-      <c r="B11" s="18" t="n">
-        <v>1</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:B11"/>
+  <autoFilter ref="A1:B10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -5242,7 +5344,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -5257,7 +5359,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-10-10 17:16
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$62</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 09/10/2026 às 18:17</t>
+          <t>Gerado em 10/10/2026 às 17:16</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6">
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="17">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>186276.3905263158</v>
+        <v>183581.1578378378</v>
       </c>
     </row>
     <row r="20">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>70000</v>
+        <v>62500</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="24">
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="25">
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O60"/>
+  <dimension ref="A1:O62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1546,11 +1546,11 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>146394</v>
+        <v>146401</v>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>Edital nº 30/2026 – Contratação de Consultoria Individual para realizar estudo de caso sobre a Secretaria de Serviços Compartilhados</t>
+          <t>Edital 06/2026 - Programa de Privacidade e Segurança da Informação</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
@@ -1564,31 +1564,31 @@
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.483</v>
+        <v>0.175</v>
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Segurança</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I12" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Território Nacional</t>
         </is>
       </c>
       <c r="J12" s="14" t="n">
-        <v>46289</v>
+        <v>46301</v>
       </c>
       <c r="K12" s="14" t="n">
-        <v>46304</v>
+        <v>46316</v>
       </c>
       <c r="L12" s="15" t="n">
-        <v>90000</v>
+        <v>120000</v>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
@@ -1597,7 +1597,7 @@
       </c>
       <c r="N12" s="12" t="inlineStr">
         <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
+          <t>cgti@mdh.gov.br</t>
         </is>
       </c>
       <c r="O12" s="16" t="inlineStr">
@@ -1613,11 +1613,11 @@
         </is>
       </c>
       <c r="B13" s="18" t="n">
-        <v>146401</v>
+        <v>146421</v>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>Edital 06/2026 - Programa de Privacidade e Segurança da Informação</t>
+          <t>Edital 9/2026 - Levantamento SIGAP - SENAD/MJSP</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
@@ -1631,11 +1631,11 @@
         </is>
       </c>
       <c r="F13" s="21" t="n">
-        <v>0.175</v>
+        <v>0.44</v>
       </c>
       <c r="G13" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Segurança</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H13" s="19" t="inlineStr">
@@ -1645,17 +1645,17 @@
       </c>
       <c r="I13" s="19" t="inlineStr">
         <is>
-          <t>Território Nacional</t>
+          <t>Híbrido</t>
         </is>
       </c>
       <c r="J13" s="22" t="n">
-        <v>46301</v>
+        <v>46304</v>
       </c>
       <c r="K13" s="22" t="n">
-        <v>46316</v>
+        <v>46313</v>
       </c>
       <c r="L13" s="23" t="n">
-        <v>120000</v>
+        <v>100000</v>
       </c>
       <c r="M13" s="17" t="inlineStr">
         <is>
@@ -1664,7 +1664,7 @@
       </c>
       <c r="N13" s="20" t="inlineStr">
         <is>
-          <t>cgti@mdh.gov.br</t>
+          <t>dga@mj.gov.br</t>
         </is>
       </c>
       <c r="O13" s="24" t="inlineStr">
@@ -1676,17 +1676,15 @@
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>unesco:8e654be2-3b1f-4782-d2b4-08df1fb02468</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="n">
+        <v>146422</v>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 57/2026 - 3 vagas - Consultor Individual</t>
+          <t>Edital 10/2026 - Reformulação painéis POWER BI</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -1696,61 +1694,69 @@
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.222</v>
+        <v>0.302</v>
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Educação / Ensino, Direitos Humanos / Cidadania</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I14" s="11" t="inlineStr"/>
+          <t>Não identificado</t>
+        </is>
+      </c>
+      <c r="I14" s="11" t="inlineStr">
+        <is>
+          <t>Híbrido</t>
+        </is>
+      </c>
       <c r="J14" s="14" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="K14" s="14" t="n">
-        <v>46309</v>
-      </c>
-      <c r="L14" s="15" t="inlineStr"/>
+        <v>46313</v>
+      </c>
+      <c r="L14" s="15" t="n">
+        <v>60000</v>
+      </c>
       <c r="M14" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N14" s="12" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N14" s="12" t="inlineStr">
+        <is>
+          <t>dga@mj.gov.br</t>
+        </is>
+      </c>
       <c r="O14" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B15" s="18" t="inlineStr">
-        <is>
-          <t>unesco:d8649b2a-6267-450d-bf98-08df23ad085e</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="n">
+        <v>146423</v>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>914BRZ4027 - Edital 56/2026 - Arquitetura e Urbanismo - Iphan-SP</t>
+          <t>EDITAL 11/2026 - Padrões decisões judiciais destinação bens FUNAD</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E15" s="20" t="inlineStr">
@@ -1759,52 +1765,60 @@
         </is>
       </c>
       <c r="F15" s="21" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública, Cultura, Arquitetura / Design</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H15" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I15" s="19" t="inlineStr"/>
+          <t>Não identificado</t>
+        </is>
+      </c>
+      <c r="I15" s="19" t="inlineStr">
+        <is>
+          <t>Híbrido</t>
+        </is>
+      </c>
       <c r="J15" s="22" t="n">
         <v>46304</v>
       </c>
       <c r="K15" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="L15" s="23" t="inlineStr"/>
+        <v>46313</v>
+      </c>
+      <c r="L15" s="23" t="n">
+        <v>102000</v>
+      </c>
       <c r="M15" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N15" s="20" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N15" s="20" t="inlineStr">
+        <is>
+          <t>dga@mj.gov.br</t>
+        </is>
+      </c>
       <c r="O15" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B16" s="10" t="inlineStr">
-        <is>
-          <t>unesco:ec3e284f-74b2-4ad2-bf99-08df23ad085e</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="n">
+        <v>146424</v>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>914BRZ4027 - Edital 57/2026 - Arquitetura e Urbanismo - Centro Vivo</t>
+          <t>EDITAL 12/2026 - DIAGNÓSTICO COMPARADO RELACIONADO À DESTINAÇÃO DE BENS FUNAD</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -1814,56 +1828,64 @@
       </c>
       <c r="E16" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.143</v>
+        <v>0.378</v>
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública, Cultura, Arquitetura / Design</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Desenvolvimento Social / Políticas Públicas</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I16" s="11" t="inlineStr"/>
+          <t>Não identificado</t>
+        </is>
+      </c>
+      <c r="I16" s="11" t="inlineStr">
+        <is>
+          <t>Híbrido</t>
+        </is>
+      </c>
       <c r="J16" s="14" t="n">
         <v>46304</v>
       </c>
       <c r="K16" s="14" t="n">
-        <v>46309</v>
-      </c>
-      <c r="L16" s="15" t="inlineStr"/>
+        <v>46313</v>
+      </c>
+      <c r="L16" s="15" t="n">
+        <v>60000</v>
+      </c>
       <c r="M16" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N16" s="12" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N16" s="12" t="inlineStr">
+        <is>
+          <t>dga@mj.gov.br</t>
+        </is>
+      </c>
       <c r="O16" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B17" s="18" t="inlineStr">
-        <is>
-          <t>unesco:fb72c64e-511e-4325-60e3-08df20839863</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="n">
+        <v>146425</v>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1162 - Edital 05/2026 - 01 vaga - Consultor Individual</t>
+          <t>EDITAL 13/2026 - Metodologia realização do Levantamento Nacional de Álcool e Drogas (LENAD)</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1877,35 +1899,45 @@
         </is>
       </c>
       <c r="F17" s="21" t="n">
-        <v>0.175</v>
+        <v>0.355</v>
       </c>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I17" s="19" t="inlineStr"/>
+          <t>Não identificado</t>
+        </is>
+      </c>
+      <c r="I17" s="19" t="inlineStr">
+        <is>
+          <t>Híbrido</t>
+        </is>
+      </c>
       <c r="J17" s="22" t="n">
         <v>46304</v>
       </c>
       <c r="K17" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="L17" s="23" t="inlineStr"/>
+        <v>46313</v>
+      </c>
+      <c r="L17" s="23" t="n">
+        <v>40000</v>
+      </c>
       <c r="M17" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N17" s="20" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N17" s="20" t="inlineStr">
+        <is>
+          <t>dpagi@mj.gov.br</t>
+        </is>
+      </c>
       <c r="O17" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
@@ -1917,12 +1949,12 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>unesco:df21a7d3-d7d5-44ad-60e4-08df20839863</t>
+          <t>unesco:8e654be2-3b1f-4782-d2b4-08df1fb02468</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1162 - Edital 06/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 57/2026 - 3 vagas - Consultor Individual</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -1932,15 +1964,15 @@
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.3</v>
+        <v>0.222</v>
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Educação / Ensino, Direitos Humanos / Cidadania</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -1950,10 +1982,10 @@
       </c>
       <c r="I18" s="11" t="inlineStr"/>
       <c r="J18" s="14" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="K18" s="14" t="n">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="L18" s="15" t="inlineStr"/>
       <c r="M18" s="9" t="inlineStr">
@@ -1976,12 +2008,12 @@
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>unesco:375ed309-bb72-44ae-7d86-08df1d6278dd</t>
+          <t>unesco:d8649b2a-6267-450d-bf98-08df23ad085e</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 41/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ4027 - Edital 56/2026 - Arquitetura e Urbanismo - Iphan-SP</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
@@ -1995,11 +2027,11 @@
         </is>
       </c>
       <c r="F19" s="21" t="n">
-        <v>0.433</v>
+        <v>0.333</v>
       </c>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Gestão / Administração Pública, Cultura, Arquitetura / Design</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
@@ -2009,10 +2041,10 @@
       </c>
       <c r="I19" s="19" t="inlineStr"/>
       <c r="J19" s="22" t="n">
-        <v>46300</v>
+        <v>46304</v>
       </c>
       <c r="K19" s="22" t="n">
-        <v>46304</v>
+        <v>46309</v>
       </c>
       <c r="L19" s="23" t="inlineStr"/>
       <c r="M19" s="17" t="inlineStr">
@@ -2035,12 +2067,12 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
+          <t>unesco:ec3e284f-74b2-4ad2-bf99-08df23ad085e</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
+          <t>914BRZ4027 - Edital 57/2026 - Arquitetura e Urbanismo - Centro Vivo</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -2050,15 +2082,15 @@
       </c>
       <c r="E20" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Não Classificado</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.464</v>
+        <v>0.143</v>
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Arquitetura / Design</t>
+          <t>Gestão / Administração Pública, Cultura, Arquitetura / Design</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
@@ -2068,10 +2100,10 @@
       </c>
       <c r="I20" s="11" t="inlineStr"/>
       <c r="J20" s="14" t="n">
-        <v>46286</v>
+        <v>46304</v>
       </c>
       <c r="K20" s="14" t="n">
-        <v>46316</v>
+        <v>46309</v>
       </c>
       <c r="L20" s="15" t="inlineStr"/>
       <c r="M20" s="9" t="inlineStr">
@@ -2094,12 +2126,12 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
+          <t>unesco:fb72c64e-511e-4325-60e3-08df20839863</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
+          <t>914BRZ1162 - Edital 05/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
@@ -2109,15 +2141,15 @@
       </c>
       <c r="E21" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F21" s="21" t="n">
-        <v>0.464</v>
+        <v>0.175</v>
       </c>
       <c r="G21" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Ciências Sociais / Participação Social</t>
+          <t>Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
@@ -2127,10 +2159,10 @@
       </c>
       <c r="I21" s="19" t="inlineStr"/>
       <c r="J21" s="22" t="n">
-        <v>46286</v>
+        <v>46304</v>
       </c>
       <c r="K21" s="22" t="n">
-        <v>46316</v>
+        <v>46310</v>
       </c>
       <c r="L21" s="23" t="inlineStr"/>
       <c r="M21" s="17" t="inlineStr">
@@ -2153,12 +2185,12 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
+          <t>unesco:df21a7d3-d7d5-44ad-60e4-08df20839863</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
+          <t>914BRZ1162 - Edital 06/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -2168,15 +2200,15 @@
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.423</v>
+        <v>0.3</v>
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
@@ -2186,10 +2218,10 @@
       </c>
       <c r="I22" s="11" t="inlineStr"/>
       <c r="J22" s="14" t="n">
-        <v>46286</v>
+        <v>46304</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46316</v>
+        <v>46310</v>
       </c>
       <c r="L22" s="15" t="inlineStr"/>
       <c r="M22" s="9" t="inlineStr">
@@ -2212,12 +2244,12 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
+          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
+          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
@@ -2235,7 +2267,7 @@
       </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Ciências Sociais / Participação Social</t>
+          <t>Arquitetura / Design</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
@@ -2271,12 +2303,12 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
+          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
+          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -2290,11 +2322,11 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.423</v>
+        <v>0.464</v>
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Ciências Sociais / Participação Social</t>
+          <t>Tecnologia da Informação / Dados, Ciências Sociais / Participação Social</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
@@ -2330,12 +2362,12 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
+          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
+          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
@@ -2353,7 +2385,7 @@
       </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
@@ -2384,91 +2416,81 @@
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E26" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.569</v>
+        <v>0.464</v>
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Ciências Sociais / Participação Social</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I26" s="11" t="inlineStr">
-        <is>
-          <t>Porto Alegre/RS</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I26" s="11" t="inlineStr"/>
       <c r="J26" s="14" t="n">
-        <v>46246</v>
+        <v>46286</v>
       </c>
       <c r="K26" s="14" t="n">
-        <v>46257</v>
-      </c>
-      <c r="L26" s="15" t="n">
-        <v>54000</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L26" s="15" t="inlineStr"/>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N26" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N26" s="12" t="inlineStr"/>
       <c r="O26" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="17" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E27" s="20" t="inlineStr">
@@ -2477,112 +2499,94 @@
         </is>
       </c>
       <c r="F27" s="21" t="n">
-        <v>0.433</v>
+        <v>0.423</v>
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Ciências Sociais / Participação Social</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I27" s="19" t="inlineStr">
-        <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I27" s="19" t="inlineStr"/>
       <c r="J27" s="22" t="n">
-        <v>46227</v>
+        <v>46286</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46252</v>
-      </c>
-      <c r="L27" s="23" t="n">
-        <v>286000</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L27" s="23" t="inlineStr"/>
       <c r="M27" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N27" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N27" s="20" t="inlineStr"/>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.492</v>
+        <v>0.423</v>
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Ciência / Tecnologia e Inovação</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I28" s="11" t="inlineStr">
-        <is>
-          <t>Brasília - DF | Híbrido</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I28" s="11" t="inlineStr"/>
       <c r="J28" s="14" t="n">
-        <v>46246</v>
+        <v>46286</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46250</v>
+        <v>46316</v>
       </c>
       <c r="L28" s="15" t="inlineStr"/>
       <c r="M28" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
-        </is>
-      </c>
-      <c r="N28" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N28" s="12" t="inlineStr"/>
       <c r="O28" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
@@ -2594,17 +2598,17 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E29" s="20" t="inlineStr">
@@ -2613,11 +2617,11 @@
         </is>
       </c>
       <c r="F29" s="21" t="n">
-        <v>0.569</v>
+        <v>0.593</v>
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
@@ -2627,17 +2631,17 @@
       </c>
       <c r="I29" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J29" s="22" t="n">
-        <v>46246</v>
+        <v>46251</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46257</v>
+        <v>46256</v>
       </c>
       <c r="L29" s="23" t="n">
-        <v>54000</v>
+        <v>50000</v>
       </c>
       <c r="M29" s="17" t="inlineStr">
         <is>
@@ -2651,7 +2655,7 @@
       </c>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -2663,17 +2667,17 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
@@ -2682,11 +2686,11 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.593</v>
+        <v>0.569</v>
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
@@ -2696,17 +2700,17 @@
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J30" s="14" t="n">
-        <v>46251</v>
+        <v>46246</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="L30" s="15" t="n">
-        <v>50000</v>
+        <v>54000</v>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
@@ -2720,7 +2724,7 @@
       </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -2801,12 +2805,12 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
@@ -2820,35 +2824,33 @@
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.527</v>
+        <v>0.492</v>
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I32" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J32" s="14" t="n">
-        <v>46266</v>
+        <v>46246</v>
       </c>
       <c r="K32" s="14" t="n">
-        <v>46288</v>
-      </c>
-      <c r="L32" s="15" t="n">
-        <v>70000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L32" s="15" t="inlineStr"/>
       <c r="M32" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N32" s="12" t="inlineStr">
@@ -2858,7 +2860,7 @@
       </c>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -2870,50 +2872,50 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E33" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F33" s="21" t="n">
-        <v>0.451</v>
+        <v>0.569</v>
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J33" s="22" t="n">
-        <v>46265</v>
+        <v>46246</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46270</v>
+        <v>46257</v>
       </c>
       <c r="L33" s="23" t="n">
-        <v>30000</v>
+        <v>54000</v>
       </c>
       <c r="M33" s="17" t="inlineStr">
         <is>
@@ -2927,7 +2929,7 @@
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -2939,17 +2941,17 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E34" s="12" t="inlineStr">
@@ -2958,35 +2960,35 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.492</v>
+        <v>0.451</v>
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J34" s="14" t="n">
-        <v>46246</v>
+        <v>46265</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46272</v>
+        <v>46270</v>
       </c>
       <c r="L34" s="15" t="n">
-        <v>54000</v>
+        <v>30000</v>
       </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N34" s="12" t="inlineStr">
@@ -2996,7 +2998,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -3008,12 +3010,12 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
@@ -3023,39 +3025,39 @@
       </c>
       <c r="E35" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F35" s="21" t="n">
-        <v>0.3</v>
+        <v>0.492</v>
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Educação / Ensino</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46275</v>
+        <v>46246</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46280</v>
+        <v>46272</v>
       </c>
       <c r="L35" s="23" t="n">
-        <v>50000</v>
+        <v>54000</v>
       </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N35" s="20" t="inlineStr">
@@ -3065,7 +3067,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -3077,12 +3079,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -3092,15 +3094,15 @@
       </c>
       <c r="E36" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>0.451</v>
+        <v>0.527</v>
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
@@ -3110,17 +3112,17 @@
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46282</v>
+        <v>46266</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46286</v>
+        <v>46288</v>
       </c>
       <c r="L36" s="15" t="n">
-        <v>30000</v>
+        <v>70000</v>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
@@ -3134,7 +3136,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
@@ -3146,17 +3148,17 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E37" s="20" t="inlineStr">
@@ -3165,11 +3167,11 @@
         </is>
       </c>
       <c r="F37" s="21" t="n">
-        <v>0.5639999999999999</v>
+        <v>0.3</v>
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Trabalho / Emprego, Segurança</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
@@ -3179,16 +3181,18 @@
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46290</v>
+        <v>46275</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46294</v>
-      </c>
-      <c r="L37" s="23" t="inlineStr"/>
+        <v>46280</v>
+      </c>
+      <c r="L37" s="23" t="n">
+        <v>50000</v>
+      </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3201,7 +3205,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
@@ -3349,12 +3353,12 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
@@ -3364,15 +3368,15 @@
       </c>
       <c r="E40" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.5639999999999999</v>
+        <v>0.451</v>
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
@@ -3382,29 +3386,31 @@
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46278</v>
+        <v>46282</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46295</v>
-      </c>
-      <c r="L40" s="15" t="inlineStr"/>
+        <v>46286</v>
+      </c>
+      <c r="L40" s="15" t="n">
+        <v>30000</v>
+      </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N40" s="12" t="inlineStr">
         <is>
-          <t>ugp@educacao.sp.gov.br</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
         </is>
       </c>
     </row>
@@ -3416,54 +3422,52 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E41" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F41" s="21" t="n">
-        <v>0.2</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Educação / Ensino, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Direitos Humanos / Cidadania</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Trabalho / Emprego, Segurança</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Rio Grande do Norte</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46293</v>
+        <v>46290</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46298</v>
-      </c>
-      <c r="L41" s="23" t="n">
-        <v>21000</v>
-      </c>
+        <v>46294</v>
+      </c>
+      <c r="L41" s="23" t="inlineStr"/>
       <c r="M41" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N41" s="20" t="inlineStr">
@@ -3473,7 +3477,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
         </is>
       </c>
     </row>
@@ -3485,12 +3489,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3500,15 +3504,15 @@
       </c>
       <c r="E42" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.077</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
@@ -3518,31 +3522,29 @@
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46294</v>
+        <v>46278</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46300</v>
-      </c>
-      <c r="L42" s="15" t="n">
-        <v>55000</v>
-      </c>
+        <v>46295</v>
+      </c>
+      <c r="L42" s="15" t="inlineStr"/>
       <c r="M42" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N42" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>ugp@educacao.sp.gov.br</t>
         </is>
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
         </is>
       </c>
     </row>
@@ -3623,12 +3625,12 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
@@ -3638,35 +3640,35 @@
       </c>
       <c r="E44" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>0.175</v>
+        <v>0.2</v>
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Engenharia / Infraestrutura</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Educação / Ensino, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Direitos Humanos / Cidadania</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Remota e/ou presencial em Brasília - DF</t>
+          <t>Articulação Estadual - Rio Grande do Norte</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="L44" s="15" t="n">
-        <v>600000</v>
+        <v>21000</v>
       </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
@@ -3680,7 +3682,7 @@
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
         </is>
       </c>
     </row>
@@ -3692,12 +3694,12 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
+          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
+          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
@@ -3711,35 +3713,35 @@
         </is>
       </c>
       <c r="F45" s="21" t="n">
-        <v>0.355</v>
+        <v>0.175</v>
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Engenharia / Infraestrutura</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remota e/ou presencial em Brasília - DF</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
         <v>46294</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46302</v>
+        <v>46297</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>60000</v>
+        <v>600000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N45" s="20" t="inlineStr">
@@ -3749,7 +3751,7 @@
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
         </is>
       </c>
     </row>
@@ -3761,12 +3763,12 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -3780,28 +3782,28 @@
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.333</v>
+        <v>0.355</v>
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Cultura, Segurança, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Educação / Ensino</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J46" s="14" t="n">
-        <v>46296</v>
+        <v>46294</v>
       </c>
       <c r="K46" s="14" t="n">
-        <v>46300</v>
+        <v>46302</v>
       </c>
       <c r="L46" s="15" t="n">
         <v>60000</v>
@@ -3818,7 +3820,7 @@
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
         </is>
       </c>
     </row>
@@ -3830,12 +3832,12 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
@@ -3845,15 +3847,15 @@
       </c>
       <c r="E47" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Não Classificado</t>
         </is>
       </c>
       <c r="F47" s="21" t="n">
-        <v>0.282</v>
+        <v>0.077</v>
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
@@ -3867,13 +3869,13 @@
         </is>
       </c>
       <c r="J47" s="22" t="n">
-        <v>46296</v>
+        <v>46294</v>
       </c>
       <c r="K47" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="L47" s="23" t="n">
-        <v>60000</v>
+        <v>55000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
@@ -3887,7 +3889,7 @@
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
         </is>
       </c>
     </row>
@@ -3899,12 +3901,12 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
@@ -3914,15 +3916,15 @@
       </c>
       <c r="E48" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F48" s="13" t="n">
-        <v>0.178</v>
+        <v>0.333</v>
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Cultura, Comunicação</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Cultura, Segurança, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
@@ -3932,7 +3934,7 @@
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J48" s="14" t="n">
@@ -3942,7 +3944,7 @@
         <v>46300</v>
       </c>
       <c r="L48" s="15" t="n">
-        <v>21000</v>
+        <v>60000</v>
       </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
@@ -3956,7 +3958,7 @@
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
         </is>
       </c>
     </row>
@@ -4037,64 +4039,64 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E50" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>0.493</v>
+        <v>0.178</v>
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Desenvolvimento Social / Políticas Públicas</t>
+          <t>Tecnologia da Informação / Dados, Cultura, Comunicação</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J50" s="14" t="n">
-        <v>46244</v>
+        <v>46296</v>
       </c>
       <c r="K50" s="14" t="n">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="L50" s="15" t="n">
-        <v>935000</v>
+        <v>21000</v>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N50" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
         </is>
       </c>
     </row>
@@ -4106,12 +4108,12 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
@@ -4125,21 +4127,21 @@
         </is>
       </c>
       <c r="F51" s="21" t="n">
-        <v>0.378</v>
+        <v>0.282</v>
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Cultura, Comunicação</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
@@ -4149,7 +4151,7 @@
         <v>46300</v>
       </c>
       <c r="L51" s="23" t="n">
-        <v>36000</v>
+        <v>60000</v>
       </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
@@ -4163,7 +4165,7 @@
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
         </is>
       </c>
     </row>
@@ -4175,17 +4177,17 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13221</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E52" s="12" t="inlineStr">
@@ -4194,45 +4196,45 @@
         </is>
       </c>
       <c r="F52" s="13" t="n">
-        <v>0.409</v>
+        <v>0.493</v>
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Desenvolvimento Social / Políticas Públicas</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J52" s="14" t="n">
-        <v>46297</v>
+        <v>46244</v>
       </c>
       <c r="K52" s="14" t="n">
-        <v>46311</v>
+        <v>46296</v>
       </c>
       <c r="L52" s="15" t="n">
-        <v>70000</v>
+        <v>935000</v>
       </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N52" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -4244,64 +4246,64 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E53" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F53" s="21" t="n">
-        <v>0.464</v>
+        <v>0.378</v>
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Cultura, Comunicação</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
-        <v>46244</v>
+        <v>46296</v>
       </c>
       <c r="K53" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="L53" s="23" t="n">
-        <v>350000</v>
+        <v>36000</v>
       </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N53" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
         </is>
       </c>
     </row>
@@ -4313,12 +4315,12 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13304</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13221</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
@@ -4332,11 +4334,11 @@
         </is>
       </c>
       <c r="F54" s="13" t="n">
-        <v>0.445</v>
+        <v>0.409</v>
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
@@ -4356,11 +4358,11 @@
         <v>46311</v>
       </c>
       <c r="L54" s="15" t="n">
-        <v>90000</v>
+        <v>70000</v>
       </c>
       <c r="M54" s="9" t="inlineStr">
         <is>
-          <t>Suspendida</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N54" s="12" t="inlineStr">
@@ -4370,7 +4372,7 @@
       </c>
       <c r="O54" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221/</t>
         </is>
       </c>
     </row>
@@ -4382,64 +4384,64 @@
       </c>
       <c r="B55" s="18" t="inlineStr">
         <is>
-          <t>oei:licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304</t>
         </is>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>LICITAÇÃO Nº 13292/2026- OEI/FPOS MELHOR TÉCNICA E MENOR PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13304</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E55" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F55" s="21" t="n">
-        <v>0.175</v>
+        <v>0.445</v>
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Meio Ambiente / Clima / Geografia, Cultura, Engenharia / Infraestrutura</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
         <is>
-          <t>OEI/FPOS</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>Território Nacional</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J55" s="22" t="n">
-        <v>46302</v>
+        <v>46297</v>
       </c>
       <c r="K55" s="22" t="n">
-        <v>46322</v>
+        <v>46311</v>
       </c>
       <c r="L55" s="23" t="n">
-        <v>2778901.38</v>
+        <v>90000</v>
       </c>
       <c r="M55" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>Suspendida</t>
         </is>
       </c>
       <c r="N55" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O55" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304/</t>
         </is>
       </c>
     </row>
@@ -4451,12 +4453,12 @@
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>oei:procedimento-simplificado-no-13307-2026-oei-secult-es</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>Procedimento Simplificado nº 13307/2026 – OEI/SECULT-ES</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
@@ -4466,35 +4468,35 @@
       </c>
       <c r="E56" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F56" s="13" t="n">
-        <v>0.125</v>
+        <v>0.464</v>
       </c>
       <c r="G56" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Cultura</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H56" s="11" t="inlineStr">
         <is>
-          <t>OEI/SECULT</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I56" s="11" t="inlineStr">
         <is>
-          <t>Vitória/ES</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J56" s="14" t="n">
-        <v>46301</v>
+        <v>46244</v>
       </c>
       <c r="K56" s="14" t="n">
-        <v>46315</v>
+        <v>46300</v>
       </c>
       <c r="L56" s="15" t="n">
-        <v>600000</v>
+        <v>350000</v>
       </c>
       <c r="M56" s="9" t="inlineStr">
         <is>
@@ -4508,7 +4510,7 @@
       </c>
       <c r="O56" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13307-2026-oei-secult-es/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -4520,64 +4522,64 @@
       </c>
       <c r="B57" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
+          <t>oei:procedimento-simplificado-no-13307-2026-oei-secult-es</t>
         </is>
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
+          <t>Procedimento Simplificado nº 13307/2026 – OEI/SECULT-ES</t>
         </is>
       </c>
       <c r="D57" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E57" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Não Classificado</t>
         </is>
       </c>
       <c r="F57" s="21" t="n">
-        <v>0.378</v>
+        <v>0.125</v>
       </c>
       <c r="G57" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Comunicação</t>
+          <t>Tecnologia da Informação / Dados, Cultura</t>
         </is>
       </c>
       <c r="H57" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/SECULT</t>
         </is>
       </c>
       <c r="I57" s="19" t="inlineStr">
         <is>
-          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
+          <t>Vitória/ES</t>
         </is>
       </c>
       <c r="J57" s="22" t="n">
         <v>46301</v>
       </c>
       <c r="K57" s="22" t="n">
-        <v>46305</v>
+        <v>46315</v>
       </c>
       <c r="L57" s="23" t="n">
-        <v>62500</v>
+        <v>600000</v>
       </c>
       <c r="M57" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N57" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O57" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13307-2026-oei-secult-es/</t>
         </is>
       </c>
     </row>
@@ -4658,64 +4660,64 @@
       </c>
       <c r="B59" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321</t>
+          <t>oei:licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco</t>
         </is>
       </c>
       <c r="C59" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO FP-26-05 – Brasil em Rede – TR13321</t>
+          <t>LICITAÇÃO Nº 13292/2026- OEI/FPOS MELHOR TÉCNICA E MENOR PREÇO</t>
         </is>
       </c>
       <c r="D59" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E59" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F59" s="21" t="n">
-        <v>0.352</v>
+        <v>0.175</v>
       </c>
       <c r="G59" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Meio Ambiente / Clima / Geografia, Cultura, Engenharia / Infraestrutura</t>
         </is>
       </c>
       <c r="H59" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/FPOS</t>
         </is>
       </c>
       <c r="I59" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Território Nacional</t>
         </is>
       </c>
       <c r="J59" s="22" t="n">
         <v>46302</v>
       </c>
       <c r="K59" s="22" t="n">
-        <v>46307</v>
+        <v>46322</v>
       </c>
       <c r="L59" s="23" t="n">
-        <v>27000</v>
+        <v>2778901.38</v>
       </c>
       <c r="M59" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N59" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O59" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco/</t>
         </is>
       </c>
     </row>
@@ -4727,69 +4729,207 @@
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
+        </is>
+      </c>
+      <c r="C60" s="11" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
+        </is>
+      </c>
+      <c r="D60" s="11" t="inlineStr">
+        <is>
+          <t>Consultoria Pessoa Física (PF)</t>
+        </is>
+      </c>
+      <c r="E60" s="12" t="inlineStr">
+        <is>
+          <t>Engenharia Processos Analytics</t>
+        </is>
+      </c>
+      <c r="F60" s="13" t="n">
+        <v>0.378</v>
+      </c>
+      <c r="G60" s="11" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Comunicação</t>
+        </is>
+      </c>
+      <c r="H60" s="11" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I60" s="11" t="inlineStr">
+        <is>
+          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
+        </is>
+      </c>
+      <c r="J60" s="14" t="n">
+        <v>46301</v>
+      </c>
+      <c r="K60" s="14" t="n">
+        <v>46305</v>
+      </c>
+      <c r="L60" s="15" t="n">
+        <v>62500</v>
+      </c>
+      <c r="M60" s="9" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N60" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O60" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B61" s="18" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321</t>
+        </is>
+      </c>
+      <c r="C61" s="19" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO FP-26-05 – Brasil em Rede – TR13321</t>
+        </is>
+      </c>
+      <c r="D61" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E61" s="20" t="inlineStr">
+        <is>
+          <t>Engenharia Processos Analytics</t>
+        </is>
+      </c>
+      <c r="F61" s="21" t="n">
+        <v>0.352</v>
+      </c>
+      <c r="G61" s="19" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+        </is>
+      </c>
+      <c r="H61" s="19" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I61" s="19" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="J61" s="22" t="n">
+        <v>46302</v>
+      </c>
+      <c r="K61" s="22" t="n">
+        <v>46307</v>
+      </c>
+      <c r="L61" s="23" t="n">
+        <v>27000</v>
+      </c>
+      <c r="M61" s="17" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N61" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O61" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321/</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="9" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B62" s="10" t="inlineStr">
+        <is>
           <t>oei:contratacao-de-consultor-projeto-abdi-tr-13312</t>
         </is>
       </c>
-      <c r="C60" s="11" t="inlineStr">
+      <c r="C62" s="11" t="inlineStr">
         <is>
           <t>Contratação de consultor PROJETO ABDI – TR 13312</t>
         </is>
       </c>
-      <c r="D60" s="11" t="inlineStr">
+      <c r="D62" s="11" t="inlineStr">
         <is>
           <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
-      <c r="E60" s="12" t="inlineStr">
+      <c r="E62" s="12" t="inlineStr">
         <is>
           <t>Engenharia Processos Analytics</t>
         </is>
       </c>
-      <c r="F60" s="13" t="n">
+      <c r="F62" s="13" t="n">
         <v>0.267</v>
       </c>
-      <c r="G60" s="11" t="inlineStr">
+      <c r="G62" s="11" t="inlineStr">
         <is>
           <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
-      <c r="H60" s="11" t="inlineStr">
+      <c r="H62" s="11" t="inlineStr">
         <is>
           <t>OEI</t>
         </is>
       </c>
-      <c r="I60" s="11" t="inlineStr">
+      <c r="I62" s="11" t="inlineStr">
         <is>
           <t>Remoto</t>
         </is>
       </c>
-      <c r="J60" s="14" t="n">
+      <c r="J62" s="14" t="n">
         <v>46303</v>
       </c>
-      <c r="K60" s="14" t="n">
+      <c r="K62" s="14" t="n">
         <v>46307</v>
       </c>
-      <c r="L60" s="15" t="n">
+      <c r="L62" s="15" t="n">
         <v>600000</v>
       </c>
-      <c r="M60" s="9" t="inlineStr">
+      <c r="M62" s="9" t="inlineStr">
         <is>
           <t>En presentación</t>
         </is>
       </c>
-      <c r="N60" s="12" t="inlineStr">
+      <c r="N62" s="12" t="inlineStr">
         <is>
           <t>selecao.bra@oei.int</t>
         </is>
       </c>
-      <c r="O60" s="16" t="inlineStr">
+      <c r="O62" s="16" t="inlineStr">
         <is>
           <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13312/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O60"/>
+  <autoFilter ref="A1:O62"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -4850,6 +4990,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId57"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId61"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -4888,7 +5030,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3">
@@ -4898,7 +5040,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4">
@@ -4908,7 +5050,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -4950,7 +5092,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3">
@@ -4960,7 +5102,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4">
@@ -5022,7 +5164,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4">
@@ -5084,7 +5226,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3">
@@ -5094,7 +5236,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4">
@@ -5114,7 +5256,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6">
@@ -5140,7 +5282,7 @@
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>Ciências Sociais / Participação Social</t>
+          <t>Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="B8" s="10" t="n">
@@ -5150,11 +5292,11 @@
     <row r="9">
       <c r="A9" s="19" t="inlineStr">
         <is>
-          <t>Ciência / Tecnologia e Inovação</t>
+          <t>Ciências Sociais / Participação Social</t>
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
@@ -5164,13 +5306,13 @@
         </is>
       </c>
       <c r="B10" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="19" t="inlineStr">
         <is>
-          <t>Arquitetura / Design</t>
+          <t>Direito / Jurídico</t>
         </is>
       </c>
       <c r="B11" s="18" t="n">
@@ -5216,7 +5358,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3">
@@ -5236,13 +5378,13 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
-          <t>IBGE</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="B5" s="18" t="n">
@@ -5252,17 +5394,17 @@
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>IBGE</t>
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>MGI</t>
         </is>
       </c>
       <c r="B7" s="18" t="n">
@@ -5282,7 +5424,7 @@
     <row r="9">
       <c r="A9" s="19" t="inlineStr">
         <is>
-          <t>OEI/FPOS</t>
+          <t>OEI/SECULT</t>
         </is>
       </c>
       <c r="B9" s="18" t="n">
@@ -5292,7 +5434,7 @@
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>OEI/SECULT</t>
+          <t>OEI/FPOS</t>
         </is>
       </c>
       <c r="B10" s="10" t="n">
@@ -5344,7 +5486,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -5359,7 +5501,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-10-13 19:12
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$63</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 10/10/2026 às 17:16</t>
+          <t>Gerado em 13/10/2026 às 19:12</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6">
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="17">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>183581.1578378378</v>
+        <v>197696.8566666667</v>
       </c>
     </row>
     <row r="20">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>62500</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="24">
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="25">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O62"/>
+  <dimension ref="A1:O63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1944,22 +1944,20 @@
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B18" s="10" t="inlineStr">
-        <is>
-          <t>unesco:8e654be2-3b1f-4782-d2b4-08df1fb02468</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="n">
+        <v>146427</v>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 57/2026 - 3 vagas - Consultor Individual</t>
+          <t>BRA/23/006 - CONSULTORIA TÉCNICA EM COMUNICAÇÃO E PRODUÇÃO DE CONTEÚDO</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
@@ -1968,94 +1966,112 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.222</v>
+        <v>0.486</v>
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Educação / Ensino, Direitos Humanos / Cidadania</t>
+          <t>Comunicação</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I18" s="11" t="inlineStr"/>
+          <t>Não identificado</t>
+        </is>
+      </c>
+      <c r="I18" s="11" t="inlineStr">
+        <is>
+          <t>HOME OFFICE</t>
+        </is>
+      </c>
       <c r="J18" s="14" t="n">
-        <v>46303</v>
+        <v>46308</v>
       </c>
       <c r="K18" s="14" t="n">
-        <v>46309</v>
-      </c>
-      <c r="L18" s="15" t="inlineStr"/>
+        <v>46316</v>
+      </c>
+      <c r="L18" s="15" t="n">
+        <v>208000</v>
+      </c>
       <c r="M18" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N18" s="12" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N18" s="12" t="inlineStr">
+        <is>
+          <t>curriculos@consorcionordeste.gov.br</t>
+        </is>
+      </c>
       <c r="O18" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B19" s="18" t="inlineStr">
-        <is>
-          <t>unesco:d8649b2a-6267-450d-bf98-08df23ad085e</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="n">
+        <v>146428</v>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>914BRZ4027 - Edital 56/2026 - Arquitetura e Urbanismo - Iphan-SP</t>
+          <t>BRA/23/006 - CONSULTORIA TÉCNICA EM PRODUÇÃO EDITORIAL, DESIGN E DIAGRAMAÇÃO DE PUBLICAÇÕES INSTITUCIONAIS</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E19" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F19" s="21" t="n">
-        <v>0.333</v>
+        <v>0.494</v>
       </c>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública, Cultura, Arquitetura / Design</t>
+          <t>Arquitetura / Design</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I19" s="19" t="inlineStr"/>
+          <t>Não identificado</t>
+        </is>
+      </c>
+      <c r="I19" s="19" t="inlineStr">
+        <is>
+          <t>HOME OFFICE</t>
+        </is>
+      </c>
       <c r="J19" s="22" t="n">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="K19" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="L19" s="23" t="inlineStr"/>
+        <v>46316</v>
+      </c>
+      <c r="L19" s="23" t="n">
+        <v>28000</v>
+      </c>
       <c r="M19" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N19" s="20" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N19" s="20" t="inlineStr">
+        <is>
+          <t>curriculos@consorcionordeste.gov.br</t>
+        </is>
+      </c>
       <c r="O19" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
@@ -2067,12 +2083,12 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>unesco:ec3e284f-74b2-4ad2-bf99-08df23ad085e</t>
+          <t>unesco:1b397c59-629f-47bf-bf95-08df23ad085e</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>914BRZ4027 - Edital 57/2026 - Arquitetura e Urbanismo - Centro Vivo</t>
+          <t>914BRZ1159 - Republicação - Edital 33/2026 - 2 vagas - Consultor Individual</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -2082,15 +2098,15 @@
       </c>
       <c r="E20" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.143</v>
+        <v>0.175</v>
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública, Cultura, Arquitetura / Design</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
@@ -2100,10 +2116,10 @@
       </c>
       <c r="I20" s="11" t="inlineStr"/>
       <c r="J20" s="14" t="n">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="K20" s="14" t="n">
-        <v>46309</v>
+        <v>46313</v>
       </c>
       <c r="L20" s="15" t="inlineStr"/>
       <c r="M20" s="9" t="inlineStr">
@@ -2126,12 +2142,12 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>unesco:fb72c64e-511e-4325-60e3-08df20839863</t>
+          <t>unesco:8e654be2-3b1f-4782-d2b4-08df1fb02468</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1162 - Edital 05/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 57/2026 - 3 vagas - Consultor Individual</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
@@ -2141,15 +2157,15 @@
       </c>
       <c r="E21" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F21" s="21" t="n">
-        <v>0.175</v>
+        <v>0.222</v>
       </c>
       <c r="G21" s="19" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Educação / Ensino, Direitos Humanos / Cidadania</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
@@ -2159,10 +2175,10 @@
       </c>
       <c r="I21" s="19" t="inlineStr"/>
       <c r="J21" s="22" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="K21" s="22" t="n">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="L21" s="23" t="inlineStr"/>
       <c r="M21" s="17" t="inlineStr">
@@ -2185,12 +2201,12 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>unesco:df21a7d3-d7d5-44ad-60e4-08df20839863</t>
+          <t>unesco:d8649b2a-6267-450d-bf98-08df23ad085e</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1162 - Edital 06/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ4027 - Edital 56/2026 - Arquitetura e Urbanismo - Iphan-SP</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -2204,11 +2220,11 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.3</v>
+        <v>0.333</v>
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Gestão / Administração Pública, Cultura, Arquitetura / Design</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
@@ -2221,7 +2237,7 @@
         <v>46304</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="L22" s="15" t="inlineStr"/>
       <c r="M22" s="9" t="inlineStr">
@@ -2244,12 +2260,12 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
+          <t>unesco:ec3e284f-74b2-4ad2-bf99-08df23ad085e</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
+          <t>914BRZ4027 - Edital 57/2026 - Arquitetura e Urbanismo - Centro Vivo</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
@@ -2259,15 +2275,15 @@
       </c>
       <c r="E23" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Não Classificado</t>
         </is>
       </c>
       <c r="F23" s="21" t="n">
-        <v>0.464</v>
+        <v>0.143</v>
       </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Arquitetura / Design</t>
+          <t>Gestão / Administração Pública, Cultura, Arquitetura / Design</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
@@ -2277,10 +2293,10 @@
       </c>
       <c r="I23" s="19" t="inlineStr"/>
       <c r="J23" s="22" t="n">
-        <v>46286</v>
+        <v>46304</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46316</v>
+        <v>46309</v>
       </c>
       <c r="L23" s="23" t="inlineStr"/>
       <c r="M23" s="17" t="inlineStr">
@@ -2303,12 +2319,12 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
+          <t>unesco:fb72c64e-511e-4325-60e3-08df20839863</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
+          <t>914BRZ1162 - Edital 05/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -2318,15 +2334,15 @@
       </c>
       <c r="E24" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.464</v>
+        <v>0.175</v>
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Ciências Sociais / Participação Social</t>
+          <t>Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
@@ -2336,10 +2352,10 @@
       </c>
       <c r="I24" s="11" t="inlineStr"/>
       <c r="J24" s="14" t="n">
-        <v>46286</v>
+        <v>46304</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46316</v>
+        <v>46310</v>
       </c>
       <c r="L24" s="15" t="inlineStr"/>
       <c r="M24" s="9" t="inlineStr">
@@ -2362,12 +2378,12 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
+          <t>unesco:df21a7d3-d7d5-44ad-60e4-08df20839863</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
+          <t>914BRZ1162 - Edital 06/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
@@ -2377,15 +2393,15 @@
       </c>
       <c r="E25" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F25" s="21" t="n">
-        <v>0.423</v>
+        <v>0.3</v>
       </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
@@ -2395,10 +2411,10 @@
       </c>
       <c r="I25" s="19" t="inlineStr"/>
       <c r="J25" s="22" t="n">
-        <v>46286</v>
+        <v>46304</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46316</v>
+        <v>46310</v>
       </c>
       <c r="L25" s="23" t="inlineStr"/>
       <c r="M25" s="17" t="inlineStr">
@@ -2421,12 +2437,12 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
+          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
+          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -2444,7 +2460,7 @@
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Ciências Sociais / Participação Social</t>
+          <t>Arquitetura / Design</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
@@ -2480,12 +2496,12 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
+          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
+          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
@@ -2499,11 +2515,11 @@
         </is>
       </c>
       <c r="F27" s="21" t="n">
-        <v>0.423</v>
+        <v>0.464</v>
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Ciências Sociais / Participação Social</t>
+          <t>Tecnologia da Informação / Dados, Ciências Sociais / Participação Social</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
@@ -2539,12 +2555,12 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
+          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
+          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
@@ -2562,7 +2578,7 @@
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
@@ -2593,207 +2609,177 @@
     <row r="29">
       <c r="A29" s="17" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E29" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F29" s="21" t="n">
-        <v>0.593</v>
+        <v>0.464</v>
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Ciências Sociais / Participação Social</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I29" s="19" t="inlineStr">
-        <is>
-          <t>Recife - PE</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I29" s="19" t="inlineStr"/>
       <c r="J29" s="22" t="n">
-        <v>46251</v>
+        <v>46286</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46256</v>
-      </c>
-      <c r="L29" s="23" t="n">
-        <v>50000</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L29" s="23" t="inlineStr"/>
       <c r="M29" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N29" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N29" s="20" t="inlineStr"/>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.569</v>
+        <v>0.423</v>
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Ciências Sociais / Participação Social</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I30" s="11" t="inlineStr">
-        <is>
-          <t>Porto Alegre/RS</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I30" s="11" t="inlineStr"/>
       <c r="J30" s="14" t="n">
-        <v>46246</v>
+        <v>46286</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>46257</v>
-      </c>
-      <c r="L30" s="15" t="n">
-        <v>54000</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L30" s="15" t="inlineStr"/>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N30" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N30" s="12" t="inlineStr"/>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="17" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E31" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F31" s="21" t="n">
-        <v>0.46</v>
+        <v>0.423</v>
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Educação / Ensino</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I31" s="19" t="inlineStr">
-        <is>
-          <t>São Paulo - SP</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I31" s="19" t="inlineStr"/>
       <c r="J31" s="22" t="n">
-        <v>46252</v>
+        <v>46286</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46259</v>
-      </c>
-      <c r="L31" s="23" t="n">
-        <v>60000</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L31" s="23" t="inlineStr"/>
       <c r="M31" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N31" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N31" s="20" t="inlineStr"/>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
@@ -2805,12 +2791,12 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
@@ -2824,33 +2810,35 @@
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.492</v>
+        <v>0.46</v>
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Educação / Ensino</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I32" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J32" s="14" t="n">
-        <v>46246</v>
+        <v>46252</v>
       </c>
       <c r="K32" s="14" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L32" s="15" t="inlineStr"/>
+        <v>46259</v>
+      </c>
+      <c r="L32" s="15" t="n">
+        <v>60000</v>
+      </c>
       <c r="M32" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N32" s="12" t="inlineStr">
@@ -2860,7 +2848,7 @@
       </c>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -2872,17 +2860,17 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E33" s="20" t="inlineStr">
@@ -2891,11 +2879,11 @@
         </is>
       </c>
       <c r="F33" s="21" t="n">
-        <v>0.569</v>
+        <v>0.593</v>
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
@@ -2905,17 +2893,17 @@
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J33" s="22" t="n">
-        <v>46246</v>
+        <v>46251</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46257</v>
+        <v>46256</v>
       </c>
       <c r="L33" s="23" t="n">
-        <v>54000</v>
+        <v>50000</v>
       </c>
       <c r="M33" s="17" t="inlineStr">
         <is>
@@ -2929,7 +2917,7 @@
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -2941,17 +2929,17 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E34" s="12" t="inlineStr">
@@ -2960,35 +2948,35 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.451</v>
+        <v>0.492</v>
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Educação / Ensino</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J34" s="14" t="n">
-        <v>46265</v>
+        <v>46246</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46270</v>
+        <v>46272</v>
       </c>
       <c r="L34" s="15" t="n">
-        <v>30000</v>
+        <v>54000</v>
       </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N34" s="12" t="inlineStr">
@@ -2998,7 +2986,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -3010,17 +2998,17 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E35" s="20" t="inlineStr">
@@ -3029,35 +3017,35 @@
         </is>
       </c>
       <c r="F35" s="21" t="n">
-        <v>0.492</v>
+        <v>0.451</v>
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46246</v>
+        <v>46265</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46272</v>
+        <v>46270</v>
       </c>
       <c r="L35" s="23" t="n">
-        <v>54000</v>
+        <v>30000</v>
       </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N35" s="20" t="inlineStr">
@@ -3067,7 +3055,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -3353,51 +3341,49 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E40" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.451</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Trabalho / Emprego, Segurança</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46282</v>
+        <v>46290</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46286</v>
-      </c>
-      <c r="L40" s="15" t="n">
-        <v>30000</v>
-      </c>
+        <v>46294</v>
+      </c>
+      <c r="L40" s="15" t="inlineStr"/>
       <c r="M40" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3410,7 +3396,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
         </is>
       </c>
     </row>
@@ -3422,17 +3408,17 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E41" s="20" t="inlineStr">
@@ -3445,39 +3431,39 @@
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Trabalho / Emprego, Segurança</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46290</v>
+        <v>46278</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="L41" s="23" t="inlineStr"/>
       <c r="M41" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N41" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>ugp@educacao.sp.gov.br</t>
         </is>
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
         </is>
       </c>
     </row>
@@ -3489,12 +3475,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3504,15 +3490,15 @@
       </c>
       <c r="E42" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.5639999999999999</v>
+        <v>0.451</v>
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
@@ -3522,29 +3508,31 @@
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46278</v>
+        <v>46282</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46295</v>
-      </c>
-      <c r="L42" s="15" t="inlineStr"/>
+        <v>46286</v>
+      </c>
+      <c r="L42" s="15" t="n">
+        <v>30000</v>
+      </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N42" s="12" t="inlineStr">
         <is>
-          <t>ugp@educacao.sp.gov.br</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
         </is>
       </c>
     </row>
@@ -3763,12 +3751,12 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -3778,15 +3766,15 @@
       </c>
       <c r="E46" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Não Classificado</t>
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.355</v>
+        <v>0.077</v>
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
@@ -3796,17 +3784,17 @@
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J46" s="14" t="n">
         <v>46294</v>
       </c>
       <c r="K46" s="14" t="n">
-        <v>46302</v>
+        <v>46300</v>
       </c>
       <c r="L46" s="15" t="n">
-        <v>60000</v>
+        <v>55000</v>
       </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
@@ -3820,7 +3808,7 @@
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
         </is>
       </c>
     </row>
@@ -3832,12 +3820,12 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
@@ -3847,15 +3835,15 @@
       </c>
       <c r="E47" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F47" s="21" t="n">
-        <v>0.077</v>
+        <v>0.355</v>
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Educação / Ensino</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
@@ -3865,17 +3853,17 @@
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J47" s="22" t="n">
         <v>46294</v>
       </c>
       <c r="K47" s="22" t="n">
-        <v>46300</v>
+        <v>46302</v>
       </c>
       <c r="L47" s="23" t="n">
-        <v>55000</v>
+        <v>60000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
@@ -3889,7 +3877,7 @@
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
         </is>
       </c>
     </row>
@@ -4039,12 +4027,12 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
@@ -4054,25 +4042,25 @@
       </c>
       <c r="E50" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>0.178</v>
+        <v>0.282</v>
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Cultura, Comunicação</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J50" s="14" t="n">
@@ -4082,7 +4070,7 @@
         <v>46300</v>
       </c>
       <c r="L50" s="15" t="n">
-        <v>21000</v>
+        <v>60000</v>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
@@ -4096,7 +4084,7 @@
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
         </is>
       </c>
     </row>
@@ -4108,12 +4096,12 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
@@ -4123,25 +4111,25 @@
       </c>
       <c r="E51" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F51" s="21" t="n">
-        <v>0.282</v>
+        <v>0.178</v>
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
+          <t>Tecnologia da Informação / Dados, Cultura, Comunicação</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
@@ -4151,7 +4139,7 @@
         <v>46300</v>
       </c>
       <c r="L51" s="23" t="n">
-        <v>60000</v>
+        <v>21000</v>
       </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
@@ -4165,7 +4153,7 @@
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
         </is>
       </c>
     </row>
@@ -4384,64 +4372,64 @@
       </c>
       <c r="B55" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13304</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E55" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F55" s="21" t="n">
-        <v>0.445</v>
+        <v>0.464</v>
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J55" s="22" t="n">
-        <v>46297</v>
+        <v>46244</v>
       </c>
       <c r="K55" s="22" t="n">
-        <v>46311</v>
+        <v>46300</v>
       </c>
       <c r="L55" s="23" t="n">
-        <v>90000</v>
+        <v>350000</v>
       </c>
       <c r="M55" s="17" t="inlineStr">
         <is>
-          <t>Suspendida</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N55" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O55" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -4453,64 +4441,64 @@
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13304</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E56" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F56" s="13" t="n">
-        <v>0.464</v>
+        <v>0.445</v>
       </c>
       <c r="G56" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H56" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I56" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J56" s="14" t="n">
-        <v>46244</v>
+        <v>46297</v>
       </c>
       <c r="K56" s="14" t="n">
-        <v>46300</v>
+        <v>46311</v>
       </c>
       <c r="L56" s="15" t="n">
-        <v>350000</v>
+        <v>90000</v>
       </c>
       <c r="M56" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>Suspendida</t>
         </is>
       </c>
       <c r="N56" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O56" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304/</t>
         </is>
       </c>
     </row>
@@ -4591,17 +4579,17 @@
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13288</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E58" s="12" t="inlineStr">
@@ -4610,31 +4598,31 @@
         </is>
       </c>
       <c r="F58" s="13" t="n">
-        <v>0.433</v>
+        <v>0.378</v>
       </c>
       <c r="G58" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Comunicação</t>
         </is>
       </c>
       <c r="H58" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I58" s="11" t="inlineStr">
         <is>
-          <t>Consultor especialista em Gestão de Processos Secretaria de Estado da Educação  SEED-PR</t>
+          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
         </is>
       </c>
       <c r="J58" s="14" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="K58" s="14" t="n">
-        <v>46307</v>
+        <v>46305</v>
       </c>
       <c r="L58" s="15" t="n">
-        <v>140000</v>
+        <v>62500</v>
       </c>
       <c r="M58" s="9" t="inlineStr">
         <is>
@@ -4648,7 +4636,7 @@
       </c>
       <c r="O58" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
         </is>
       </c>
     </row>
@@ -4660,64 +4648,64 @@
       </c>
       <c r="B59" s="18" t="inlineStr">
         <is>
-          <t>oei:licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288</t>
         </is>
       </c>
       <c r="C59" s="19" t="inlineStr">
         <is>
-          <t>LICITAÇÃO Nº 13292/2026- OEI/FPOS MELHOR TÉCNICA E MENOR PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13288</t>
         </is>
       </c>
       <c r="D59" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E59" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F59" s="21" t="n">
-        <v>0.175</v>
+        <v>0.433</v>
       </c>
       <c r="G59" s="19" t="inlineStr">
         <is>
-          <t>Meio Ambiente / Clima / Geografia, Cultura, Engenharia / Infraestrutura</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H59" s="19" t="inlineStr">
         <is>
-          <t>OEI/FPOS</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I59" s="19" t="inlineStr">
         <is>
-          <t>Território Nacional</t>
+          <t>Consultor especialista em Gestão de Processos Secretaria de Estado da Educação  SEED-PR</t>
         </is>
       </c>
       <c r="J59" s="22" t="n">
         <v>46302</v>
       </c>
       <c r="K59" s="22" t="n">
-        <v>46322</v>
+        <v>46307</v>
       </c>
       <c r="L59" s="23" t="n">
-        <v>2778901.38</v>
+        <v>140000</v>
       </c>
       <c r="M59" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N59" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O59" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288/</t>
         </is>
       </c>
     </row>
@@ -4729,64 +4717,64 @@
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
+          <t>oei:licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco</t>
         </is>
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
+          <t>LICITAÇÃO Nº 13292/2026- OEI/FPOS MELHOR TÉCNICA E MENOR PREÇO</t>
         </is>
       </c>
       <c r="D60" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E60" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F60" s="13" t="n">
-        <v>0.378</v>
+        <v>0.175</v>
       </c>
       <c r="G60" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Comunicação</t>
+          <t>Meio Ambiente / Clima / Geografia, Cultura, Engenharia / Infraestrutura</t>
         </is>
       </c>
       <c r="H60" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/FPOS</t>
         </is>
       </c>
       <c r="I60" s="11" t="inlineStr">
         <is>
-          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
+          <t>Território Nacional</t>
         </is>
       </c>
       <c r="J60" s="14" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="K60" s="14" t="n">
-        <v>46305</v>
+        <v>46322</v>
       </c>
       <c r="L60" s="15" t="n">
-        <v>62500</v>
+        <v>2778901.38</v>
       </c>
       <c r="M60" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N60" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O60" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco/</t>
         </is>
       </c>
     </row>
@@ -4928,8 +4916,77 @@
         </is>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B63" s="18" t="inlineStr">
+        <is>
+          <t>oei:procedimento-simplificado-no-13340-2026-oei-secult-es-menor-preco</t>
+        </is>
+      </c>
+      <c r="C63" s="19" t="inlineStr">
+        <is>
+          <t>PROCEDIMENTO SIMPLIFICADO Nº 13340/2026- OEI/SECULT-ES MENOR PREÇO</t>
+        </is>
+      </c>
+      <c r="D63" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+        </is>
+      </c>
+      <c r="E63" s="20" t="inlineStr">
+        <is>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F63" s="21" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="G63" s="19" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Cultura, Trabalho / Emprego</t>
+        </is>
+      </c>
+      <c r="H63" s="19" t="inlineStr">
+        <is>
+          <t>OEI/SECULT</t>
+        </is>
+      </c>
+      <c r="I63" s="19" t="inlineStr">
+        <is>
+          <t>Vitória/ES.</t>
+        </is>
+      </c>
+      <c r="J63" s="22" t="n">
+        <v>46308</v>
+      </c>
+      <c r="K63" s="22" t="n">
+        <v>46321</v>
+      </c>
+      <c r="L63" s="23" t="n">
+        <v>600000</v>
+      </c>
+      <c r="M63" s="17" t="inlineStr">
+        <is>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N63" s="20" t="inlineStr">
+        <is>
+          <t>compras.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O63" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13340-2026-oei-secult-es-menor-preco/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O62"/>
+  <autoFilter ref="A1:O63"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -4992,6 +5049,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId59"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId60"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId62"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -5030,7 +5088,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3">
@@ -5040,7 +5098,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4">
@@ -5050,7 +5108,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -5092,7 +5150,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3">
@@ -5102,7 +5160,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4">
@@ -5112,7 +5170,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -5150,21 +5208,21 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4">
@@ -5174,7 +5232,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5">
@@ -5184,7 +5242,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -5226,7 +5284,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3">
@@ -5236,7 +5294,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4">
@@ -5246,27 +5304,27 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
-          <t>Educação / Ensino</t>
+          <t>Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>Meio Ambiente / Clima / Geografia</t>
+          <t>Educação / Ensino</t>
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7">
@@ -5276,13 +5334,13 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>Ciência / Tecnologia e Inovação</t>
+          <t>Ciências Sociais / Participação Social</t>
         </is>
       </c>
       <c r="B8" s="10" t="n">
@@ -5292,11 +5350,11 @@
     <row r="9">
       <c r="A9" s="19" t="inlineStr">
         <is>
-          <t>Ciências Sociais / Participação Social</t>
+          <t>Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10">
@@ -5312,11 +5370,11 @@
     <row r="11">
       <c r="A11" s="19" t="inlineStr">
         <is>
-          <t>Direito / Jurídico</t>
+          <t>Comunicação</t>
         </is>
       </c>
       <c r="B11" s="18" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -5358,7 +5416,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
@@ -5368,7 +5426,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4">
@@ -5378,7 +5436,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5">
@@ -5388,7 +5446,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
@@ -5428,7 +5486,7 @@
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -5486,7 +5544,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-10-14 17:01
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$65</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 13/10/2026 às 19:12</t>
+          <t>Gerado em 14/10/2026 às 17:01</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="24">
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O63"/>
+  <dimension ref="A1:O65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2083,12 +2083,12 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>unesco:1b397c59-629f-47bf-bf95-08df23ad085e</t>
+          <t>unesco:048a1d3b-843f-4613-60de-08df20839863</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Republicação - Edital 33/2026 - 2 vagas - Consultor Individual</t>
+          <t>914BRZ1159 - Publicação Edital 42/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -2102,11 +2102,11 @@
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.175</v>
+        <v>0.378</v>
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Gestão / Administração Pública, Comunicação</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
@@ -2116,10 +2116,10 @@
       </c>
       <c r="I20" s="11" t="inlineStr"/>
       <c r="J20" s="14" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="K20" s="14" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="L20" s="15" t="inlineStr"/>
       <c r="M20" s="9" t="inlineStr">
@@ -2142,12 +2142,12 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>unesco:8e654be2-3b1f-4782-d2b4-08df1fb02468</t>
+          <t>unesco:28aedd59-87d7-4b85-60e5-08df20839863</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 57/2026 - 3 vagas - Consultor Individual</t>
+          <t>914BRZ1162 - Edital 07/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
@@ -2157,15 +2157,15 @@
       </c>
       <c r="E21" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F21" s="21" t="n">
-        <v>0.222</v>
+        <v>0.175</v>
       </c>
       <c r="G21" s="19" t="inlineStr">
         <is>
-          <t>Educação / Ensino, Direitos Humanos / Cidadania</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Educação / Ensino</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
@@ -2175,10 +2175,10 @@
       </c>
       <c r="I21" s="19" t="inlineStr"/>
       <c r="J21" s="22" t="n">
-        <v>46303</v>
+        <v>46309</v>
       </c>
       <c r="K21" s="22" t="n">
-        <v>46309</v>
+        <v>46315</v>
       </c>
       <c r="L21" s="23" t="inlineStr"/>
       <c r="M21" s="17" t="inlineStr">
@@ -2201,12 +2201,12 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>unesco:d8649b2a-6267-450d-bf98-08df23ad085e</t>
+          <t>unesco:1b397c59-629f-47bf-bf95-08df23ad085e</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>914BRZ4027 - Edital 56/2026 - Arquitetura e Urbanismo - Iphan-SP</t>
+          <t>914BRZ1159 - Republicação - Edital 33/2026 - 2 vagas - Consultor Individual</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -2220,11 +2220,11 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.333</v>
+        <v>0.175</v>
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública, Cultura, Arquitetura / Design</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
@@ -2234,10 +2234,10 @@
       </c>
       <c r="I22" s="11" t="inlineStr"/>
       <c r="J22" s="14" t="n">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46309</v>
+        <v>46313</v>
       </c>
       <c r="L22" s="15" t="inlineStr"/>
       <c r="M22" s="9" t="inlineStr">
@@ -2260,12 +2260,12 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>unesco:ec3e284f-74b2-4ad2-bf99-08df23ad085e</t>
+          <t>unesco:8e654be2-3b1f-4782-d2b4-08df1fb02468</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>914BRZ4027 - Edital 57/2026 - Arquitetura e Urbanismo - Centro Vivo</t>
+          <t>914BRZ1155 - EDITAL Nº 57/2026 - 3 vagas - Consultor Individual</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
@@ -2275,15 +2275,15 @@
       </c>
       <c r="E23" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F23" s="21" t="n">
-        <v>0.143</v>
+        <v>0.222</v>
       </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública, Cultura, Arquitetura / Design</t>
+          <t>Educação / Ensino, Direitos Humanos / Cidadania</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
@@ -2293,7 +2293,7 @@
       </c>
       <c r="I23" s="19" t="inlineStr"/>
       <c r="J23" s="22" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="K23" s="22" t="n">
         <v>46309</v>
@@ -2319,12 +2319,12 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>unesco:fb72c64e-511e-4325-60e3-08df20839863</t>
+          <t>unesco:d8649b2a-6267-450d-bf98-08df23ad085e</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1162 - Edital 05/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ4027 - Edital 56/2026 - Arquitetura e Urbanismo - Iphan-SP</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -2338,11 +2338,11 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.175</v>
+        <v>0.333</v>
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Gestão / Administração Pública, Cultura, Arquitetura / Design</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
@@ -2355,7 +2355,7 @@
         <v>46304</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="L24" s="15" t="inlineStr"/>
       <c r="M24" s="9" t="inlineStr">
@@ -2378,12 +2378,12 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>unesco:df21a7d3-d7d5-44ad-60e4-08df20839863</t>
+          <t>unesco:ec3e284f-74b2-4ad2-bf99-08df23ad085e</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1162 - Edital 06/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ4027 - Edital 57/2026 - Arquitetura e Urbanismo - Centro Vivo</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
@@ -2393,15 +2393,15 @@
       </c>
       <c r="E25" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Não Classificado</t>
         </is>
       </c>
       <c r="F25" s="21" t="n">
-        <v>0.3</v>
+        <v>0.143</v>
       </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Gestão / Administração Pública, Cultura, Arquitetura / Design</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
@@ -2414,7 +2414,7 @@
         <v>46304</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="L25" s="23" t="inlineStr"/>
       <c r="M25" s="17" t="inlineStr">
@@ -2437,12 +2437,12 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
+          <t>unesco:fb72c64e-511e-4325-60e3-08df20839863</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
+          <t>914BRZ1162 - Edital 05/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -2452,15 +2452,15 @@
       </c>
       <c r="E26" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.464</v>
+        <v>0.175</v>
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Arquitetura / Design</t>
+          <t>Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
@@ -2470,10 +2470,10 @@
       </c>
       <c r="I26" s="11" t="inlineStr"/>
       <c r="J26" s="14" t="n">
-        <v>46286</v>
+        <v>46304</v>
       </c>
       <c r="K26" s="14" t="n">
-        <v>46316</v>
+        <v>46310</v>
       </c>
       <c r="L26" s="15" t="inlineStr"/>
       <c r="M26" s="9" t="inlineStr">
@@ -2496,12 +2496,12 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
+          <t>unesco:df21a7d3-d7d5-44ad-60e4-08df20839863</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
+          <t>914BRZ1162 - Edital 06/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
@@ -2511,15 +2511,15 @@
       </c>
       <c r="E27" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F27" s="21" t="n">
-        <v>0.464</v>
+        <v>0.3</v>
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Ciências Sociais / Participação Social</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
@@ -2529,10 +2529,10 @@
       </c>
       <c r="I27" s="19" t="inlineStr"/>
       <c r="J27" s="22" t="n">
-        <v>46286</v>
+        <v>46304</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46316</v>
+        <v>46310</v>
       </c>
       <c r="L27" s="23" t="inlineStr"/>
       <c r="M27" s="17" t="inlineStr">
@@ -2555,12 +2555,12 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
+          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
+          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
@@ -2574,11 +2574,11 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.423</v>
+        <v>0.464</v>
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Arquitetura / Design</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
@@ -2614,12 +2614,12 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
+          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
+          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
@@ -2637,7 +2637,7 @@
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Ciências Sociais / Participação Social</t>
+          <t>Tecnologia da Informação / Dados, Ciências Sociais / Participação Social</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
@@ -2673,12 +2673,12 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
+          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
+          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
@@ -2696,7 +2696,7 @@
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Ciências Sociais / Participação Social</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
@@ -2732,12 +2732,12 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
+          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
+          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
@@ -2751,11 +2751,11 @@
         </is>
       </c>
       <c r="F31" s="21" t="n">
-        <v>0.423</v>
+        <v>0.464</v>
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Ciências Sociais / Participação Social</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
@@ -2786,138 +2786,118 @@
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E32" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.46</v>
+        <v>0.423</v>
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Educação / Ensino</t>
+          <t>Ciências Sociais / Participação Social</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I32" s="11" t="inlineStr">
-        <is>
-          <t>São Paulo - SP</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I32" s="11" t="inlineStr"/>
       <c r="J32" s="14" t="n">
-        <v>46252</v>
+        <v>46286</v>
       </c>
       <c r="K32" s="14" t="n">
-        <v>46259</v>
-      </c>
-      <c r="L32" s="15" t="n">
-        <v>60000</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L32" s="15" t="inlineStr"/>
       <c r="M32" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N32" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N32" s="12" t="inlineStr"/>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="17" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E33" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F33" s="21" t="n">
-        <v>0.593</v>
+        <v>0.423</v>
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I33" s="19" t="inlineStr">
-        <is>
-          <t>Recife - PE</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I33" s="19" t="inlineStr"/>
       <c r="J33" s="22" t="n">
-        <v>46251</v>
+        <v>46286</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46256</v>
-      </c>
-      <c r="L33" s="23" t="n">
-        <v>50000</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L33" s="23" t="inlineStr"/>
       <c r="M33" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N33" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N33" s="20" t="inlineStr"/>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
@@ -2929,30 +2909,30 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E34" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.492</v>
+        <v>0.593</v>
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
@@ -2962,21 +2942,21 @@
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J34" s="14" t="n">
-        <v>46246</v>
+        <v>46251</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46272</v>
+        <v>46256</v>
       </c>
       <c r="L34" s="15" t="n">
-        <v>54000</v>
+        <v>50000</v>
       </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N34" s="12" t="inlineStr">
@@ -2986,7 +2966,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -2998,50 +2978,50 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E35" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F35" s="21" t="n">
-        <v>0.451</v>
+        <v>0.46</v>
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Educação / Ensino</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46265</v>
+        <v>46252</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46270</v>
+        <v>46259</v>
       </c>
       <c r="L35" s="23" t="n">
-        <v>30000</v>
+        <v>60000</v>
       </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
@@ -3055,7 +3035,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -3067,12 +3047,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -3082,15 +3062,15 @@
       </c>
       <c r="E36" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>0.527</v>
+        <v>0.492</v>
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Educação / Ensino</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
@@ -3100,21 +3080,21 @@
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46266</v>
+        <v>46246</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46288</v>
+        <v>46272</v>
       </c>
       <c r="L36" s="15" t="n">
-        <v>70000</v>
+        <v>54000</v>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N36" s="12" t="inlineStr">
@@ -3124,7 +3104,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -3136,12 +3116,12 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
@@ -3155,31 +3135,31 @@
         </is>
       </c>
       <c r="F37" s="21" t="n">
-        <v>0.3</v>
+        <v>0.527</v>
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46275</v>
+        <v>46266</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46280</v>
+        <v>46288</v>
       </c>
       <c r="L37" s="23" t="n">
-        <v>50000</v>
+        <v>70000</v>
       </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
@@ -3193,7 +3173,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
@@ -3205,17 +3185,17 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E38" s="12" t="inlineStr">
@@ -3224,11 +3204,11 @@
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.2</v>
+        <v>0.493</v>
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Ciência / Tecnologia e Inovação, Engenharia / Infraestrutura</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
@@ -3238,16 +3218,18 @@
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Dados Remoto</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46275</v>
+        <v>46281</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46281</v>
-      </c>
-      <c r="L38" s="15" t="inlineStr"/>
+        <v>46286</v>
+      </c>
+      <c r="L38" s="15" t="n">
+        <v>110000</v>
+      </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3260,7 +3242,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
         </is>
       </c>
     </row>
@@ -3272,17 +3254,17 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E39" s="20" t="inlineStr">
@@ -3291,11 +3273,11 @@
         </is>
       </c>
       <c r="F39" s="21" t="n">
-        <v>0.493</v>
+        <v>0.2</v>
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Ciência / Tecnologia e Inovação, Engenharia / Infraestrutura</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
@@ -3305,18 +3287,16 @@
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Dados Remoto</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
+        <v>46275</v>
+      </c>
+      <c r="K39" s="22" t="n">
         <v>46281</v>
       </c>
-      <c r="K39" s="22" t="n">
-        <v>46286</v>
-      </c>
-      <c r="L39" s="23" t="n">
-        <v>110000</v>
-      </c>
+      <c r="L39" s="23" t="inlineStr"/>
       <c r="M39" s="17" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3329,7 +3309,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
         </is>
       </c>
     </row>
@@ -3341,17 +3321,17 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E40" s="12" t="inlineStr">
@@ -3360,11 +3340,11 @@
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.5639999999999999</v>
+        <v>0.3</v>
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Trabalho / Emprego, Segurança</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
@@ -3374,16 +3354,18 @@
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46290</v>
+        <v>46275</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46294</v>
-      </c>
-      <c r="L40" s="15" t="inlineStr"/>
+        <v>46280</v>
+      </c>
+      <c r="L40" s="15" t="n">
+        <v>50000</v>
+      </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3396,7 +3378,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
@@ -3408,12 +3390,12 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
@@ -3423,15 +3405,15 @@
       </c>
       <c r="E41" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F41" s="21" t="n">
-        <v>0.5639999999999999</v>
+        <v>0.451</v>
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
@@ -3441,29 +3423,31 @@
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46278</v>
+        <v>46282</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46295</v>
-      </c>
-      <c r="L41" s="23" t="inlineStr"/>
+        <v>46286</v>
+      </c>
+      <c r="L41" s="23" t="n">
+        <v>30000</v>
+      </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N41" s="20" t="inlineStr">
         <is>
-          <t>ugp@educacao.sp.gov.br</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
         </is>
       </c>
     </row>
@@ -3475,17 +3459,17 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E42" s="12" t="inlineStr">
@@ -3498,12 +3482,12 @@
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I42" s="11" t="inlineStr">
@@ -3512,10 +3496,10 @@
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46282</v>
+        <v>46265</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46286</v>
+        <v>46270</v>
       </c>
       <c r="L42" s="15" t="n">
         <v>30000</v>
@@ -3532,7 +3516,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -3544,17 +3528,17 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E43" s="20" t="inlineStr">
@@ -3563,32 +3547,30 @@
         </is>
       </c>
       <c r="F43" s="21" t="n">
-        <v>0.232</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Trabalho / Emprego, Segurança</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46293</v>
+        <v>46290</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46298</v>
-      </c>
-      <c r="L43" s="23" t="n">
-        <v>30000</v>
-      </c>
+        <v>46294</v>
+      </c>
+      <c r="L43" s="23" t="inlineStr"/>
       <c r="M43" s="17" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3601,7 +3583,7 @@
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
         </is>
       </c>
     </row>
@@ -3613,12 +3595,12 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
@@ -3628,15 +3610,15 @@
       </c>
       <c r="E44" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>0.2</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Educação / Ensino, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Direitos Humanos / Cidadania</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
@@ -3646,18 +3628,16 @@
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Rio Grande do Norte</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46293</v>
+        <v>46278</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46298</v>
-      </c>
-      <c r="L44" s="15" t="n">
-        <v>21000</v>
-      </c>
+        <v>46295</v>
+      </c>
+      <c r="L44" s="15" t="inlineStr"/>
       <c r="M44" s="9" t="inlineStr">
         <is>
           <t>En fase de apresentação</t>
@@ -3665,12 +3645,12 @@
       </c>
       <c r="N44" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>ugp@educacao.sp.gov.br</t>
         </is>
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
         </is>
       </c>
     </row>
@@ -3682,12 +3662,12 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
@@ -3697,35 +3677,35 @@
       </c>
       <c r="E45" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F45" s="21" t="n">
-        <v>0.175</v>
+        <v>0.2</v>
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Engenharia / Infraestrutura</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Educação / Ensino, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Direitos Humanos / Cidadania</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Remota e/ou presencial em Brasília - DF</t>
+          <t>Articulação Estadual - Rio Grande do Norte</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>600000</v>
+        <v>21000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
@@ -3739,7 +3719,7 @@
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
         </is>
       </c>
     </row>
@@ -3751,12 +3731,12 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -3766,15 +3746,15 @@
       </c>
       <c r="E46" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.077</v>
+        <v>0.232</v>
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
@@ -3784,17 +3764,17 @@
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
         </is>
       </c>
       <c r="J46" s="14" t="n">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="K46" s="14" t="n">
-        <v>46300</v>
+        <v>46298</v>
       </c>
       <c r="L46" s="15" t="n">
-        <v>55000</v>
+        <v>30000</v>
       </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
@@ -3808,7 +3788,7 @@
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
         </is>
       </c>
     </row>
@@ -3820,12 +3800,12 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
+          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
+          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
@@ -3839,35 +3819,35 @@
         </is>
       </c>
       <c r="F47" s="21" t="n">
-        <v>0.355</v>
+        <v>0.175</v>
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Engenharia / Infraestrutura</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remota e/ou presencial em Brasília - DF</t>
         </is>
       </c>
       <c r="J47" s="22" t="n">
         <v>46294</v>
       </c>
       <c r="K47" s="22" t="n">
-        <v>46302</v>
+        <v>46297</v>
       </c>
       <c r="L47" s="23" t="n">
-        <v>60000</v>
+        <v>600000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N47" s="20" t="inlineStr">
@@ -3877,7 +3857,7 @@
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
         </is>
       </c>
     </row>
@@ -3889,12 +3869,12 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
@@ -3904,35 +3884,35 @@
       </c>
       <c r="E48" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Não Classificado</t>
         </is>
       </c>
       <c r="F48" s="13" t="n">
-        <v>0.333</v>
+        <v>0.077</v>
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Cultura, Segurança, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J48" s="14" t="n">
-        <v>46296</v>
+        <v>46294</v>
       </c>
       <c r="K48" s="14" t="n">
         <v>46300</v>
       </c>
       <c r="L48" s="15" t="n">
-        <v>60000</v>
+        <v>55000</v>
       </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
@@ -3946,7 +3926,7 @@
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
         </is>
       </c>
     </row>
@@ -3958,12 +3938,12 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
@@ -3973,15 +3953,15 @@
       </c>
       <c r="E49" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F49" s="21" t="n">
-        <v>0.216</v>
+        <v>0.333</v>
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Cultura, Comunicação, Arquitetura / Design</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Cultura, Segurança, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
@@ -3991,7 +3971,7 @@
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J49" s="22" t="n">
@@ -4001,7 +3981,7 @@
         <v>46300</v>
       </c>
       <c r="L49" s="23" t="n">
-        <v>33000</v>
+        <v>60000</v>
       </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
@@ -4015,7 +3995,7 @@
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
         </is>
       </c>
     </row>
@@ -4096,12 +4076,12 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
@@ -4111,35 +4091,35 @@
       </c>
       <c r="E51" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F51" s="21" t="n">
-        <v>0.178</v>
+        <v>0.355</v>
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Cultura, Comunicação</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Educação / Ensino</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
-        <v>46296</v>
+        <v>46294</v>
       </c>
       <c r="K51" s="22" t="n">
-        <v>46300</v>
+        <v>46302</v>
       </c>
       <c r="L51" s="23" t="n">
-        <v>21000</v>
+        <v>60000</v>
       </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
@@ -4153,7 +4133,7 @@
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
         </is>
       </c>
     </row>
@@ -4165,64 +4145,64 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E52" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F52" s="13" t="n">
-        <v>0.493</v>
+        <v>0.216</v>
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Desenvolvimento Social / Políticas Públicas</t>
+          <t>Tecnologia da Informação / Dados, Cultura, Comunicação, Arquitetura / Design</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J52" s="14" t="n">
-        <v>46244</v>
+        <v>46296</v>
       </c>
       <c r="K52" s="14" t="n">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="L52" s="15" t="n">
-        <v>935000</v>
+        <v>33000</v>
       </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N52" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
         </is>
       </c>
     </row>
@@ -4234,12 +4214,12 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
@@ -4249,15 +4229,15 @@
       </c>
       <c r="E53" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F53" s="21" t="n">
-        <v>0.378</v>
+        <v>0.178</v>
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Cultura, Comunicação</t>
+          <t>Tecnologia da Informação / Dados, Cultura, Comunicação</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
@@ -4277,7 +4257,7 @@
         <v>46300</v>
       </c>
       <c r="L53" s="23" t="n">
-        <v>36000</v>
+        <v>21000</v>
       </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
@@ -4291,7 +4271,7 @@
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
         </is>
       </c>
     </row>
@@ -4303,17 +4283,17 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13221</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E54" s="12" t="inlineStr">
@@ -4322,45 +4302,45 @@
         </is>
       </c>
       <c r="F54" s="13" t="n">
-        <v>0.409</v>
+        <v>0.493</v>
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Desenvolvimento Social / Políticas Públicas</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J54" s="14" t="n">
-        <v>46297</v>
+        <v>46244</v>
       </c>
       <c r="K54" s="14" t="n">
-        <v>46311</v>
+        <v>46296</v>
       </c>
       <c r="L54" s="15" t="n">
-        <v>70000</v>
+        <v>935000</v>
       </c>
       <c r="M54" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N54" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O54" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -4372,64 +4352,64 @@
       </c>
       <c r="B55" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221</t>
         </is>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13221</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E55" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F55" s="21" t="n">
-        <v>0.464</v>
+        <v>0.409</v>
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J55" s="22" t="n">
-        <v>46244</v>
+        <v>46297</v>
       </c>
       <c r="K55" s="22" t="n">
-        <v>46300</v>
+        <v>46311</v>
       </c>
       <c r="L55" s="23" t="n">
-        <v>350000</v>
+        <v>70000</v>
       </c>
       <c r="M55" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N55" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O55" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221/</t>
         </is>
       </c>
     </row>
@@ -4441,12 +4421,12 @@
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13304</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
@@ -4460,35 +4440,35 @@
         </is>
       </c>
       <c r="F56" s="13" t="n">
-        <v>0.445</v>
+        <v>0.378</v>
       </c>
       <c r="G56" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Cultura, Comunicação</t>
         </is>
       </c>
       <c r="H56" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I56" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J56" s="14" t="n">
-        <v>46297</v>
+        <v>46296</v>
       </c>
       <c r="K56" s="14" t="n">
-        <v>46311</v>
+        <v>46300</v>
       </c>
       <c r="L56" s="15" t="n">
-        <v>90000</v>
+        <v>36000</v>
       </c>
       <c r="M56" s="9" t="inlineStr">
         <is>
-          <t>Suspendida</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N56" s="12" t="inlineStr">
@@ -4498,7 +4478,7 @@
       </c>
       <c r="O56" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
         </is>
       </c>
     </row>
@@ -4510,12 +4490,12 @@
       </c>
       <c r="B57" s="18" t="inlineStr">
         <is>
-          <t>oei:procedimento-simplificado-no-13307-2026-oei-secult-es</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>Procedimento Simplificado nº 13307/2026 – OEI/SECULT-ES</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D57" s="19" t="inlineStr">
@@ -4525,35 +4505,35 @@
       </c>
       <c r="E57" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F57" s="21" t="n">
-        <v>0.125</v>
+        <v>0.464</v>
       </c>
       <c r="G57" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Cultura</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H57" s="19" t="inlineStr">
         <is>
-          <t>OEI/SECULT</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I57" s="19" t="inlineStr">
         <is>
-          <t>Vitória/ES</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J57" s="22" t="n">
-        <v>46301</v>
+        <v>46244</v>
       </c>
       <c r="K57" s="22" t="n">
-        <v>46315</v>
+        <v>46300</v>
       </c>
       <c r="L57" s="23" t="n">
-        <v>600000</v>
+        <v>350000</v>
       </c>
       <c r="M57" s="17" t="inlineStr">
         <is>
@@ -4567,7 +4547,7 @@
       </c>
       <c r="O57" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13307-2026-oei-secult-es/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -4579,64 +4559,64 @@
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
+          <t>oei:procedimento-simplificado-no-13307-2026-oei-secult-es</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
+          <t>Procedimento Simplificado nº 13307/2026 – OEI/SECULT-ES</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E58" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Não Classificado</t>
         </is>
       </c>
       <c r="F58" s="13" t="n">
-        <v>0.378</v>
+        <v>0.125</v>
       </c>
       <c r="G58" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Comunicação</t>
+          <t>Tecnologia da Informação / Dados, Cultura</t>
         </is>
       </c>
       <c r="H58" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/SECULT</t>
         </is>
       </c>
       <c r="I58" s="11" t="inlineStr">
         <is>
-          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
+          <t>Vitória/ES</t>
         </is>
       </c>
       <c r="J58" s="14" t="n">
         <v>46301</v>
       </c>
       <c r="K58" s="14" t="n">
-        <v>46305</v>
+        <v>46315</v>
       </c>
       <c r="L58" s="15" t="n">
-        <v>62500</v>
+        <v>600000</v>
       </c>
       <c r="M58" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N58" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O58" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13307-2026-oei-secult-es/</t>
         </is>
       </c>
     </row>
@@ -4648,17 +4628,17 @@
       </c>
       <c r="B59" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
         </is>
       </c>
       <c r="C59" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13288</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
         </is>
       </c>
       <c r="D59" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E59" s="20" t="inlineStr">
@@ -4667,31 +4647,31 @@
         </is>
       </c>
       <c r="F59" s="21" t="n">
-        <v>0.433</v>
+        <v>0.378</v>
       </c>
       <c r="G59" s="19" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Comunicação</t>
         </is>
       </c>
       <c r="H59" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I59" s="19" t="inlineStr">
         <is>
-          <t>Consultor especialista em Gestão de Processos Secretaria de Estado da Educação  SEED-PR</t>
+          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
         </is>
       </c>
       <c r="J59" s="22" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="K59" s="22" t="n">
-        <v>46307</v>
+        <v>46305</v>
       </c>
       <c r="L59" s="23" t="n">
-        <v>140000</v>
+        <v>62500</v>
       </c>
       <c r="M59" s="17" t="inlineStr">
         <is>
@@ -4705,7 +4685,7 @@
       </c>
       <c r="O59" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
         </is>
       </c>
     </row>
@@ -4717,64 +4697,64 @@
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t>oei:licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304</t>
         </is>
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>LICITAÇÃO Nº 13292/2026- OEI/FPOS MELHOR TÉCNICA E MENOR PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13304</t>
         </is>
       </c>
       <c r="D60" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E60" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F60" s="13" t="n">
-        <v>0.175</v>
+        <v>0.445</v>
       </c>
       <c r="G60" s="11" t="inlineStr">
         <is>
-          <t>Meio Ambiente / Clima / Geografia, Cultura, Engenharia / Infraestrutura</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H60" s="11" t="inlineStr">
         <is>
-          <t>OEI/FPOS</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I60" s="11" t="inlineStr">
         <is>
-          <t>Território Nacional</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J60" s="14" t="n">
-        <v>46302</v>
+        <v>46297</v>
       </c>
       <c r="K60" s="14" t="n">
-        <v>46322</v>
+        <v>46311</v>
       </c>
       <c r="L60" s="15" t="n">
-        <v>2778901.38</v>
+        <v>90000</v>
       </c>
       <c r="M60" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>Suspendida</t>
         </is>
       </c>
       <c r="N60" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O60" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304/</t>
         </is>
       </c>
     </row>
@@ -4786,64 +4766,64 @@
       </c>
       <c r="B61" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321</t>
+          <t>oei:licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco</t>
         </is>
       </c>
       <c r="C61" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO FP-26-05 – Brasil em Rede – TR13321</t>
+          <t>LICITAÇÃO Nº 13292/2026- OEI/FPOS MELHOR TÉCNICA E MENOR PREÇO</t>
         </is>
       </c>
       <c r="D61" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E61" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F61" s="21" t="n">
-        <v>0.352</v>
+        <v>0.175</v>
       </c>
       <c r="G61" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Meio Ambiente / Clima / Geografia, Cultura, Engenharia / Infraestrutura</t>
         </is>
       </c>
       <c r="H61" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/FPOS</t>
         </is>
       </c>
       <c r="I61" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Território Nacional</t>
         </is>
       </c>
       <c r="J61" s="22" t="n">
         <v>46302</v>
       </c>
       <c r="K61" s="22" t="n">
-        <v>46307</v>
+        <v>46322</v>
       </c>
       <c r="L61" s="23" t="n">
-        <v>27000</v>
+        <v>2778901.38</v>
       </c>
       <c r="M61" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N61" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O61" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco/</t>
         </is>
       </c>
     </row>
@@ -4855,17 +4835,17 @@
       </c>
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13312</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288</t>
         </is>
       </c>
       <c r="C62" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO ABDI – TR 13312</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13288</t>
         </is>
       </c>
       <c r="D62" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E62" s="12" t="inlineStr">
@@ -4874,35 +4854,35 @@
         </is>
       </c>
       <c r="F62" s="13" t="n">
-        <v>0.267</v>
+        <v>0.433</v>
       </c>
       <c r="G62" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H62" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I62" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Consultor especialista em Gestão de Processos Secretaria de Estado da Educação  SEED-PR</t>
         </is>
       </c>
       <c r="J62" s="14" t="n">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="K62" s="14" t="n">
         <v>46307</v>
       </c>
       <c r="L62" s="15" t="n">
-        <v>600000</v>
+        <v>140000</v>
       </c>
       <c r="M62" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N62" s="12" t="inlineStr">
@@ -4912,7 +4892,7 @@
       </c>
       <c r="O62" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13312/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288/</t>
         </is>
       </c>
     </row>
@@ -4924,69 +4904,207 @@
       </c>
       <c r="B63" s="18" t="inlineStr">
         <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321</t>
+        </is>
+      </c>
+      <c r="C63" s="19" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO FP-26-05 – Brasil em Rede – TR13321</t>
+        </is>
+      </c>
+      <c r="D63" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E63" s="20" t="inlineStr">
+        <is>
+          <t>Engenharia Processos Analytics</t>
+        </is>
+      </c>
+      <c r="F63" s="21" t="n">
+        <v>0.352</v>
+      </c>
+      <c r="G63" s="19" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+        </is>
+      </c>
+      <c r="H63" s="19" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I63" s="19" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="J63" s="22" t="n">
+        <v>46302</v>
+      </c>
+      <c r="K63" s="22" t="n">
+        <v>46307</v>
+      </c>
+      <c r="L63" s="23" t="n">
+        <v>27000</v>
+      </c>
+      <c r="M63" s="17" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N63" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O63" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321/</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="9" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B64" s="10" t="inlineStr">
+        <is>
           <t>oei:procedimento-simplificado-no-13340-2026-oei-secult-es-menor-preco</t>
         </is>
       </c>
-      <c r="C63" s="19" t="inlineStr">
+      <c r="C64" s="11" t="inlineStr">
         <is>
           <t>PROCEDIMENTO SIMPLIFICADO Nº 13340/2026- OEI/SECULT-ES MENOR PREÇO</t>
         </is>
       </c>
-      <c r="D63" s="19" t="inlineStr">
+      <c r="D64" s="11" t="inlineStr">
         <is>
           <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
-      <c r="E63" s="20" t="inlineStr">
+      <c r="E64" s="12" t="inlineStr">
         <is>
           <t>Não Classificado</t>
         </is>
       </c>
-      <c r="F63" s="21" t="n">
+      <c r="F64" s="13" t="n">
         <v>0.125</v>
       </c>
-      <c r="G63" s="19" t="inlineStr">
+      <c r="G64" s="11" t="inlineStr">
         <is>
           <t>Tecnologia da Informação / Dados, Cultura, Trabalho / Emprego</t>
         </is>
       </c>
-      <c r="H63" s="19" t="inlineStr">
+      <c r="H64" s="11" t="inlineStr">
         <is>
           <t>OEI/SECULT</t>
         </is>
       </c>
-      <c r="I63" s="19" t="inlineStr">
+      <c r="I64" s="11" t="inlineStr">
         <is>
           <t>Vitória/ES.</t>
         </is>
       </c>
-      <c r="J63" s="22" t="n">
+      <c r="J64" s="14" t="n">
         <v>46308</v>
       </c>
-      <c r="K63" s="22" t="n">
+      <c r="K64" s="14" t="n">
         <v>46321</v>
       </c>
-      <c r="L63" s="23" t="n">
+      <c r="L64" s="15" t="n">
         <v>600000</v>
       </c>
-      <c r="M63" s="17" t="inlineStr">
+      <c r="M64" s="9" t="inlineStr">
         <is>
           <t>En fase de apresentação</t>
         </is>
       </c>
-      <c r="N63" s="20" t="inlineStr">
+      <c r="N64" s="12" t="inlineStr">
         <is>
           <t>compras.bra@oei.int</t>
         </is>
       </c>
-      <c r="O63" s="24" t="inlineStr">
+      <c r="O64" s="16" t="inlineStr">
         <is>
           <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13340-2026-oei-secult-es-menor-preco/</t>
         </is>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B65" s="18" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13312</t>
+        </is>
+      </c>
+      <c r="C65" s="19" t="inlineStr">
+        <is>
+          <t>Contratação de consultor PROJETO ABDI – TR 13312</t>
+        </is>
+      </c>
+      <c r="D65" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E65" s="20" t="inlineStr">
+        <is>
+          <t>Engenharia Processos Analytics</t>
+        </is>
+      </c>
+      <c r="F65" s="21" t="n">
+        <v>0.267</v>
+      </c>
+      <c r="G65" s="19" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+        </is>
+      </c>
+      <c r="H65" s="19" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I65" s="19" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="J65" s="22" t="n">
+        <v>46303</v>
+      </c>
+      <c r="K65" s="22" t="n">
+        <v>46307</v>
+      </c>
+      <c r="L65" s="23" t="n">
+        <v>600000</v>
+      </c>
+      <c r="M65" s="17" t="inlineStr">
+        <is>
+          <t>En presentación</t>
+        </is>
+      </c>
+      <c r="N65" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O65" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13312/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O63"/>
+  <autoFilter ref="A1:O65"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -5050,6 +5168,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId60"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId61"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId64"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -5108,7 +5228,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -5150,7 +5270,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3">
@@ -5212,7 +5332,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3">
@@ -5284,7 +5404,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3">
@@ -5294,7 +5414,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4">
@@ -5304,7 +5424,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5">
@@ -5324,7 +5444,7 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7">
@@ -5374,7 +5494,7 @@
         </is>
       </c>
       <c r="B11" s="18" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -5412,7 +5532,7 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
@@ -5422,21 +5542,21 @@
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5">
@@ -5544,7 +5664,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -5559,7 +5679,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-10-15 16:49
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 14/10/2026 às 17:01</t>
+          <t>Gerado em 15/10/2026 às 16:49</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -876,11 +876,11 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>146374</v>
+        <v>146334</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
-          <t>Edital nº 27/2026 – Contratação de Consultoria Individual II - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Servidões de Passagem para Orlas e Praias</t>
+          <t>Consultoria individual para estudo sobre os impactos regulatórios da Reforma Tributária no setor de saneamento básico</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
@@ -890,35 +890,35 @@
       </c>
       <c r="E2" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Não Classificado</t>
         </is>
       </c>
       <c r="F2" s="13" t="n">
-        <v>0.494</v>
+        <v>0.114</v>
       </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H2" s="11" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>brasília</t>
         </is>
       </c>
       <c r="J2" s="14" t="n">
-        <v>46280</v>
+        <v>46310</v>
       </c>
       <c r="K2" s="14" t="n">
-        <v>46310</v>
+        <v>46320</v>
       </c>
       <c r="L2" s="15" t="n">
-        <v>120000</v>
+        <v>53610.42</v>
       </c>
       <c r="M2" s="9" t="inlineStr">
         <is>
@@ -927,7 +927,7 @@
       </c>
       <c r="N2" s="12" t="inlineStr">
         <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
+          <t>cotar@ssb.gov.br</t>
         </is>
       </c>
       <c r="O2" s="16" t="inlineStr">
@@ -943,11 +943,11 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>146375</v>
+        <v>146374</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
-          <t>Edital nº 28/2026 - Contratação de Consultoria Individual I - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Acessibilidade em Orlas e Praias</t>
+          <t>Edital nº 27/2026 – Contratação de Consultoria Individual II - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Servidões de Passagem para Orlas e Praias</t>
         </is>
       </c>
       <c r="D3" s="19" t="inlineStr">
@@ -975,7 +975,7 @@
       </c>
       <c r="I3" s="19" t="inlineStr">
         <is>
-          <t>REMOTO</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J3" s="22" t="n">
@@ -1010,11 +1010,11 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>146385</v>
+        <v>146375</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor para elaborar o Caderno Temático de Referência: Investigação de Crimes contra Jornalistas e Comunicadores</t>
+          <t>Edital nº 28/2026 - Contratação de Consultoria Individual I - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Acessibilidade em Orlas e Praias</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
@@ -1028,7 +1028,7 @@
         </is>
       </c>
       <c r="F4" s="13" t="n">
-        <v>0.407</v>
+        <v>0.494</v>
       </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
@@ -1037,22 +1037,22 @@
       </c>
       <c r="H4" s="11" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>MGI</t>
         </is>
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>Home-based</t>
+          <t>REMOTO</t>
         </is>
       </c>
       <c r="J4" s="14" t="n">
-        <v>46289</v>
+        <v>46280</v>
       </c>
       <c r="K4" s="14" t="n">
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="L4" s="15" t="n">
-        <v>100000</v>
+        <v>120000</v>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
@@ -1061,7 +1061,7 @@
       </c>
       <c r="N4" s="12" t="inlineStr">
         <is>
-          <t>prodocbra016@mj.gov.br</t>
+          <t>prodoc.mgi@gestao.gov.br</t>
         </is>
       </c>
       <c r="O4" s="16" t="inlineStr">
@@ -1077,49 +1077,49 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>146354</v>
+        <v>146385</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 88/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA PROPOSIÇÃO DE SOLUÇÕES DE CIÊNCIA DE DADOS EM SENSORIAMENTO REMOTO.</t>
+          <t>Contratação de consultor para elaborar o Caderno Temático de Referência: Investigação de Crimes contra Jornalistas e Comunicadores</t>
         </is>
       </c>
       <c r="D5" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E5" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F5" s="21" t="n">
-        <v>0.411</v>
+        <v>0.407</v>
       </c>
       <c r="G5" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H5" s="19" t="inlineStr">
         <is>
-          <t>IBGE</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I5" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Home-based</t>
         </is>
       </c>
       <c r="J5" s="22" t="n">
-        <v>46293</v>
+        <v>46289</v>
       </c>
       <c r="K5" s="22" t="n">
-        <v>46313</v>
+        <v>46311</v>
       </c>
       <c r="L5" s="23" t="n">
-        <v>93500</v>
+        <v>100000</v>
       </c>
       <c r="M5" s="17" t="inlineStr">
         <is>
@@ -1128,7 +1128,7 @@
       </c>
       <c r="N5" s="20" t="inlineStr">
         <is>
-          <t>projetos.especiais@ibge.gov.br</t>
+          <t>prodocbra016@mj.gov.br</t>
         </is>
       </c>
       <c r="O5" s="24" t="inlineStr">
@@ -1144,16 +1144,16 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>146382</v>
+        <v>146354</v>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 140/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A AVALIAÇÃO DA OPERAÇÕES CENSITÁRIAS EM TERRAS INDÍGENAS DE RORAIMA.</t>
+          <t>PROJETO BRA 23/023 - TR 88/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA PROPOSIÇÃO DE SOLUÇÕES DE CIÊNCIA DE DADOS EM SENSORIAMENTO REMOTO.</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E6" s="12" t="inlineStr">
@@ -1162,11 +1162,11 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.378</v>
+        <v>0.411</v>
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Logística / Operações</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr">
@@ -1186,7 +1186,7 @@
         <v>46313</v>
       </c>
       <c r="L6" s="15" t="n">
-        <v>91500</v>
+        <v>93500</v>
       </c>
       <c r="M6" s="9" t="inlineStr">
         <is>
@@ -1211,29 +1211,29 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>146379</v>
+        <v>146382</v>
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 132/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA ANÁLISE DOS MÉTODOS DE ROTEAMENTO PARA OPERAÇÕES DE PESQUISA EM CAMPO.</t>
+          <t>PROJETO BRA 23/023 - TR 140/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A AVALIAÇÃO DA OPERAÇÕES CENSITÁRIAS EM TERRAS INDÍGENAS DE RORAIMA.</t>
         </is>
       </c>
       <c r="D7" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E7" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F7" s="21" t="n">
-        <v>0.165</v>
+        <v>0.378</v>
       </c>
       <c r="G7" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Logística / Operações</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Logística / Operações</t>
         </is>
       </c>
       <c r="H7" s="19" t="inlineStr">
@@ -1253,7 +1253,7 @@
         <v>46313</v>
       </c>
       <c r="L7" s="23" t="n">
-        <v>121500</v>
+        <v>91500</v>
       </c>
       <c r="M7" s="17" t="inlineStr">
         <is>
@@ -1278,11 +1278,11 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>146378</v>
+        <v>146379</v>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 131/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE GEOPROCESSAMENTO.</t>
+          <t>PROJETO BRA 23/023 - TR 132/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA ANÁLISE DOS MÉTODOS DE ROTEAMENTO PARA OPERAÇÕES DE PESQUISA EM CAMPO.</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
@@ -1292,11 +1292,11 @@
       </c>
       <c r="E8" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.29</v>
+        <v>0.165</v>
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
@@ -1345,11 +1345,11 @@
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>146377</v>
+        <v>146378</v>
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 130/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE CIÊNCIA DE DADOS E SENSORIAMENTO REMOTO.</t>
+          <t>PROJETO BRA 23/023 - TR 131/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE GEOPROCESSAMENTO.</t>
         </is>
       </c>
       <c r="D9" s="19" t="inlineStr">
@@ -1363,11 +1363,11 @@
         </is>
       </c>
       <c r="F9" s="21" t="n">
-        <v>0.224</v>
+        <v>0.29</v>
       </c>
       <c r="G9" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Cultura, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Logística / Operações</t>
         </is>
       </c>
       <c r="H9" s="19" t="inlineStr">
@@ -1387,7 +1387,7 @@
         <v>46313</v>
       </c>
       <c r="L9" s="23" t="n">
-        <v>93500</v>
+        <v>121500</v>
       </c>
       <c r="M9" s="17" t="inlineStr">
         <is>
@@ -1412,11 +1412,11 @@
         </is>
       </c>
       <c r="B10" s="10" t="n">
-        <v>146355</v>
+        <v>146377</v>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 119/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA DESENVOLVIMENTO DE PROPOSTA DE APRIMORAMENTO DO SISTEMA INTEGRADO DE PESQUISAS DOMICILIARES.</t>
+          <t>PROJETO BRA 23/023 - TR 130/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE CIÊNCIA DE DADOS E SENSORIAMENTO REMOTO.</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
@@ -1426,15 +1426,15 @@
       </c>
       <c r="E10" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.294</v>
+        <v>0.224</v>
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Cultura, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
@@ -1479,11 +1479,11 @@
         </is>
       </c>
       <c r="B11" s="18" t="n">
-        <v>146376</v>
+        <v>146355</v>
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 116/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA MAPEAMENTO DE INOVAÇÕES NO PROCESSO DE PRODUÇÃO ESTATÍSTICA.</t>
+          <t>PROJETO BRA 23/023 - TR 119/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA DESENVOLVIMENTO DE PROPOSTA DE APRIMORAMENTO DO SISTEMA INTEGRADO DE PESQUISAS DOMICILIARES.</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
@@ -1493,15 +1493,15 @@
       </c>
       <c r="E11" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F11" s="21" t="n">
-        <v>0.378</v>
+        <v>0.294</v>
       </c>
       <c r="G11" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H11" s="19" t="inlineStr">
@@ -1521,7 +1521,7 @@
         <v>46313</v>
       </c>
       <c r="L11" s="23" t="n">
-        <v>86800</v>
+        <v>93500</v>
       </c>
       <c r="M11" s="17" t="inlineStr">
         <is>
@@ -1546,16 +1546,16 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>146401</v>
+        <v>146376</v>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>Edital 06/2026 - Programa de Privacidade e Segurança da Informação</t>
+          <t>PROJETO BRA 23/023 - TR 116/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA MAPEAMENTO DE INOVAÇÕES NO PROCESSO DE PRODUÇÃO ESTATÍSTICA.</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E12" s="12" t="inlineStr">
@@ -1564,31 +1564,31 @@
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.175</v>
+        <v>0.378</v>
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Segurança</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>IBGE</t>
         </is>
       </c>
       <c r="I12" s="11" t="inlineStr">
         <is>
-          <t>Território Nacional</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J12" s="14" t="n">
-        <v>46301</v>
+        <v>46293</v>
       </c>
       <c r="K12" s="14" t="n">
-        <v>46316</v>
+        <v>46313</v>
       </c>
       <c r="L12" s="15" t="n">
-        <v>120000</v>
+        <v>86800</v>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
@@ -1597,7 +1597,7 @@
       </c>
       <c r="N12" s="12" t="inlineStr">
         <is>
-          <t>cgti@mdh.gov.br</t>
+          <t>projetos.especiais@ibge.gov.br</t>
         </is>
       </c>
       <c r="O12" s="16" t="inlineStr">
@@ -1613,11 +1613,11 @@
         </is>
       </c>
       <c r="B13" s="18" t="n">
-        <v>146421</v>
+        <v>146401</v>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>Edital 9/2026 - Levantamento SIGAP - SENAD/MJSP</t>
+          <t>Edital 06/2026 - Programa de Privacidade e Segurança da Informação</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
@@ -1631,11 +1631,11 @@
         </is>
       </c>
       <c r="F13" s="21" t="n">
-        <v>0.44</v>
+        <v>0.175</v>
       </c>
       <c r="G13" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Segurança</t>
         </is>
       </c>
       <c r="H13" s="19" t="inlineStr">
@@ -1645,17 +1645,17 @@
       </c>
       <c r="I13" s="19" t="inlineStr">
         <is>
-          <t>Híbrido</t>
+          <t>Território Nacional</t>
         </is>
       </c>
       <c r="J13" s="22" t="n">
-        <v>46304</v>
+        <v>46301</v>
       </c>
       <c r="K13" s="22" t="n">
-        <v>46313</v>
+        <v>46316</v>
       </c>
       <c r="L13" s="23" t="n">
-        <v>100000</v>
+        <v>120000</v>
       </c>
       <c r="M13" s="17" t="inlineStr">
         <is>
@@ -1664,7 +1664,7 @@
       </c>
       <c r="N13" s="20" t="inlineStr">
         <is>
-          <t>dga@mj.gov.br</t>
+          <t>cgti@mdh.gov.br</t>
         </is>
       </c>
       <c r="O13" s="24" t="inlineStr">
@@ -1680,11 +1680,11 @@
         </is>
       </c>
       <c r="B14" s="10" t="n">
-        <v>146422</v>
+        <v>146421</v>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>Edital 10/2026 - Reformulação painéis POWER BI</t>
+          <t>Edital 9/2026 - Levantamento SIGAP - SENAD/MJSP</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -1698,11 +1698,11 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.302</v>
+        <v>0.44</v>
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
@@ -1722,7 +1722,7 @@
         <v>46313</v>
       </c>
       <c r="L14" s="15" t="n">
-        <v>60000</v>
+        <v>100000</v>
       </c>
       <c r="M14" s="9" t="inlineStr">
         <is>
@@ -1747,16 +1747,16 @@
         </is>
       </c>
       <c r="B15" s="18" t="n">
-        <v>146423</v>
+        <v>146422</v>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>EDITAL 11/2026 - Padrões decisões judiciais destinação bens FUNAD</t>
+          <t>Edital 10/2026 - Reformulação painéis POWER BI</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E15" s="20" t="inlineStr">
@@ -1765,7 +1765,7 @@
         </is>
       </c>
       <c r="F15" s="21" t="n">
-        <v>0.34</v>
+        <v>0.302</v>
       </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
@@ -1789,7 +1789,7 @@
         <v>46313</v>
       </c>
       <c r="L15" s="23" t="n">
-        <v>102000</v>
+        <v>60000</v>
       </c>
       <c r="M15" s="17" t="inlineStr">
         <is>
@@ -1814,16 +1814,16 @@
         </is>
       </c>
       <c r="B16" s="10" t="n">
-        <v>146424</v>
+        <v>146423</v>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>EDITAL 12/2026 - DIAGNÓSTICO COMPARADO RELACIONADO À DESTINAÇÃO DE BENS FUNAD</t>
+          <t>EDITAL 11/2026 - Padrões decisões judiciais destinação bens FUNAD</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E16" s="12" t="inlineStr">
@@ -1832,11 +1832,11 @@
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.378</v>
+        <v>0.34</v>
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Desenvolvimento Social / Políticas Públicas</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
@@ -1856,7 +1856,7 @@
         <v>46313</v>
       </c>
       <c r="L16" s="15" t="n">
-        <v>60000</v>
+        <v>102000</v>
       </c>
       <c r="M16" s="9" t="inlineStr">
         <is>
@@ -1881,11 +1881,11 @@
         </is>
       </c>
       <c r="B17" s="18" t="n">
-        <v>146425</v>
+        <v>146424</v>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>EDITAL 13/2026 - Metodologia realização do Levantamento Nacional de Álcool e Drogas (LENAD)</t>
+          <t>EDITAL 12/2026 - DIAGNÓSTICO COMPARADO RELACIONADO À DESTINAÇÃO DE BENS FUNAD</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1899,11 +1899,11 @@
         </is>
       </c>
       <c r="F17" s="21" t="n">
-        <v>0.355</v>
+        <v>0.378</v>
       </c>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Desenvolvimento Social / Políticas Públicas</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
@@ -1923,7 +1923,7 @@
         <v>46313</v>
       </c>
       <c r="L17" s="23" t="n">
-        <v>40000</v>
+        <v>60000</v>
       </c>
       <c r="M17" s="17" t="inlineStr">
         <is>
@@ -1932,7 +1932,7 @@
       </c>
       <c r="N17" s="20" t="inlineStr">
         <is>
-          <t>dpagi@mj.gov.br</t>
+          <t>dga@mj.gov.br</t>
         </is>
       </c>
       <c r="O17" s="24" t="inlineStr">
@@ -1948,29 +1948,29 @@
         </is>
       </c>
       <c r="B18" s="10" t="n">
-        <v>146427</v>
+        <v>146425</v>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>BRA/23/006 - CONSULTORIA TÉCNICA EM COMUNICAÇÃO E PRODUÇÃO DE CONTEÚDO</t>
+          <t>EDITAL 13/2026 - Metodologia realização do Levantamento Nacional de Álcool e Drogas (LENAD)</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.486</v>
+        <v>0.355</v>
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Comunicação</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -1980,17 +1980,17 @@
       </c>
       <c r="I18" s="11" t="inlineStr">
         <is>
-          <t>HOME OFFICE</t>
+          <t>Híbrido</t>
         </is>
       </c>
       <c r="J18" s="14" t="n">
-        <v>46308</v>
+        <v>46304</v>
       </c>
       <c r="K18" s="14" t="n">
-        <v>46316</v>
+        <v>46313</v>
       </c>
       <c r="L18" s="15" t="n">
-        <v>208000</v>
+        <v>40000</v>
       </c>
       <c r="M18" s="9" t="inlineStr">
         <is>
@@ -1999,7 +1999,7 @@
       </c>
       <c r="N18" s="12" t="inlineStr">
         <is>
-          <t>curriculos@consorcionordeste.gov.br</t>
+          <t>dpagi@mj.gov.br</t>
         </is>
       </c>
       <c r="O18" s="16" t="inlineStr">
@@ -2015,11 +2015,11 @@
         </is>
       </c>
       <c r="B19" s="18" t="n">
-        <v>146428</v>
+        <v>146427</v>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>BRA/23/006 - CONSULTORIA TÉCNICA EM PRODUÇÃO EDITORIAL, DESIGN E DIAGRAMAÇÃO DE PUBLICAÇÕES INSTITUCIONAIS</t>
+          <t>BRA/23/006 - CONSULTORIA TÉCNICA EM COMUNICAÇÃO E PRODUÇÃO DE CONTEÚDO</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
@@ -2033,11 +2033,11 @@
         </is>
       </c>
       <c r="F19" s="21" t="n">
-        <v>0.494</v>
+        <v>0.486</v>
       </c>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Arquitetura / Design</t>
+          <t>Comunicação</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
@@ -2057,7 +2057,7 @@
         <v>46316</v>
       </c>
       <c r="L19" s="23" t="n">
-        <v>28000</v>
+        <v>208000</v>
       </c>
       <c r="M19" s="17" t="inlineStr">
         <is>
@@ -2078,59 +2078,67 @@
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B20" s="10" t="inlineStr">
-        <is>
-          <t>unesco:048a1d3b-843f-4613-60de-08df20839863</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="n">
+        <v>146428</v>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 42/2026 - 1 vaga - Consultor Individual</t>
+          <t>BRA/23/006 - CONSULTORIA TÉCNICA EM PRODUÇÃO EDITORIAL, DESIGN E DIAGRAMAÇÃO DE PUBLICAÇÕES INSTITUCIONAIS</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.378</v>
+        <v>0.494</v>
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública, Comunicação</t>
+          <t>Arquitetura / Design</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I20" s="11" t="inlineStr"/>
+          <t>Não identificado</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="inlineStr">
+        <is>
+          <t>HOME OFFICE</t>
+        </is>
+      </c>
       <c r="J20" s="14" t="n">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="K20" s="14" t="n">
-        <v>46314</v>
-      </c>
-      <c r="L20" s="15" t="inlineStr"/>
+        <v>46316</v>
+      </c>
+      <c r="L20" s="15" t="n">
+        <v>28000</v>
+      </c>
       <c r="M20" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N20" s="12" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N20" s="12" t="inlineStr">
+        <is>
+          <t>curriculos@consorcionordeste.gov.br</t>
+        </is>
+      </c>
       <c r="O20" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
@@ -2142,12 +2150,12 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>unesco:28aedd59-87d7-4b85-60e5-08df20839863</t>
+          <t>unesco:048a1d3b-843f-4613-60de-08df20839863</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1162 - Edital 07/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ1159 - Publicação Edital 42/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
@@ -2161,11 +2169,11 @@
         </is>
       </c>
       <c r="F21" s="21" t="n">
-        <v>0.175</v>
+        <v>0.378</v>
       </c>
       <c r="G21" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Educação / Ensino</t>
+          <t>Gestão / Administração Pública, Comunicação</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
@@ -2178,7 +2186,7 @@
         <v>46309</v>
       </c>
       <c r="K21" s="22" t="n">
-        <v>46315</v>
+        <v>46314</v>
       </c>
       <c r="L21" s="23" t="inlineStr"/>
       <c r="M21" s="17" t="inlineStr">
@@ -2201,12 +2209,12 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>unesco:1b397c59-629f-47bf-bf95-08df23ad085e</t>
+          <t>unesco:28aedd59-87d7-4b85-60e5-08df20839863</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Republicação - Edital 33/2026 - 2 vagas - Consultor Individual</t>
+          <t>914BRZ1162 - Edital 07/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -2224,7 +2232,7 @@
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Educação / Ensino</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
@@ -2234,10 +2242,10 @@
       </c>
       <c r="I22" s="11" t="inlineStr"/>
       <c r="J22" s="14" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46313</v>
+        <v>46315</v>
       </c>
       <c r="L22" s="15" t="inlineStr"/>
       <c r="M22" s="9" t="inlineStr">
@@ -2260,12 +2268,12 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>unesco:8e654be2-3b1f-4782-d2b4-08df1fb02468</t>
+          <t>unesco:1b397c59-629f-47bf-bf95-08df23ad085e</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 57/2026 - 3 vagas - Consultor Individual</t>
+          <t>914BRZ1159 - Republicação - Edital 33/2026 - 2 vagas - Consultor Individual</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
@@ -2275,15 +2283,15 @@
       </c>
       <c r="E23" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F23" s="21" t="n">
-        <v>0.222</v>
+        <v>0.175</v>
       </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Educação / Ensino, Direitos Humanos / Cidadania</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
@@ -2293,10 +2301,10 @@
       </c>
       <c r="I23" s="19" t="inlineStr"/>
       <c r="J23" s="22" t="n">
-        <v>46303</v>
+        <v>46308</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46309</v>
+        <v>46313</v>
       </c>
       <c r="L23" s="23" t="inlineStr"/>
       <c r="M23" s="17" t="inlineStr">
@@ -2319,12 +2327,12 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>unesco:d8649b2a-6267-450d-bf98-08df23ad085e</t>
+          <t>unesco:5e9b99bd-04d4-46aa-60df-08df20839863</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>914BRZ4027 - Edital 56/2026 - Arquitetura e Urbanismo - Iphan-SP</t>
+          <t>A2101B5102 | Edital 01/2026 – 01 vaga - Consultor individual</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -2334,7 +2342,7 @@
       </c>
       <c r="E24" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F24" s="13" t="n">
@@ -2342,7 +2350,7 @@
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública, Cultura, Arquitetura / Design</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Educação / Ensino</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
@@ -2352,10 +2360,10 @@
       </c>
       <c r="I24" s="11" t="inlineStr"/>
       <c r="J24" s="14" t="n">
-        <v>46304</v>
+        <v>46310</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46309</v>
+        <v>46317</v>
       </c>
       <c r="L24" s="15" t="inlineStr"/>
       <c r="M24" s="9" t="inlineStr">
@@ -2378,12 +2386,12 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>unesco:ec3e284f-74b2-4ad2-bf99-08df23ad085e</t>
+          <t>unesco:4e03075d-fa9c-444b-bf96-08df23ad085e</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>914BRZ4027 - Edital 57/2026 - Arquitetura e Urbanismo - Centro Vivo</t>
+          <t>570BRZ2005 - Edital 01/2026 - Consultor individual</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
@@ -2393,15 +2401,15 @@
       </c>
       <c r="E25" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F25" s="21" t="n">
-        <v>0.143</v>
+        <v>0.312</v>
       </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública, Cultura, Arquitetura / Design</t>
+          <t>Engenharia / Infraestrutura</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
@@ -2411,10 +2419,10 @@
       </c>
       <c r="I25" s="19" t="inlineStr"/>
       <c r="J25" s="22" t="n">
-        <v>46304</v>
+        <v>46310</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46309</v>
+        <v>46315</v>
       </c>
       <c r="L25" s="23" t="inlineStr"/>
       <c r="M25" s="17" t="inlineStr">
@@ -3047,17 +3055,17 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E36" s="12" t="inlineStr">
@@ -3066,35 +3074,35 @@
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>0.492</v>
+        <v>0.451</v>
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46246</v>
+        <v>46265</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46272</v>
+        <v>46270</v>
       </c>
       <c r="L36" s="15" t="n">
-        <v>54000</v>
+        <v>30000</v>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N36" s="12" t="inlineStr">
@@ -3104,7 +3112,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -3116,12 +3124,12 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
@@ -3131,15 +3139,15 @@
       </c>
       <c r="E37" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F37" s="21" t="n">
-        <v>0.527</v>
+        <v>0.492</v>
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Educação / Ensino</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
@@ -3149,21 +3157,21 @@
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46266</v>
+        <v>46246</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46288</v>
+        <v>46272</v>
       </c>
       <c r="L37" s="23" t="n">
-        <v>70000</v>
+        <v>54000</v>
       </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N37" s="20" t="inlineStr">
@@ -3173,7 +3181,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -3185,17 +3193,17 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E38" s="12" t="inlineStr">
@@ -3204,31 +3212,31 @@
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.493</v>
+        <v>0.527</v>
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Ciência / Tecnologia e Inovação, Engenharia / Infraestrutura</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Dados Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46281</v>
+        <v>46266</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46286</v>
+        <v>46288</v>
       </c>
       <c r="L38" s="15" t="n">
-        <v>110000</v>
+        <v>70000</v>
       </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
@@ -3242,7 +3250,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
@@ -3390,50 +3398,50 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E41" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F41" s="21" t="n">
-        <v>0.451</v>
+        <v>0.493</v>
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Ciência / Tecnologia e Inovação, Engenharia / Infraestrutura</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Dados Remoto</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="K41" s="22" t="n">
         <v>46286</v>
       </c>
       <c r="L41" s="23" t="n">
-        <v>30000</v>
+        <v>110000</v>
       </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
@@ -3447,7 +3455,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
         </is>
       </c>
     </row>
@@ -3459,30 +3467,30 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E42" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.451</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Trabalho / Emprego, Segurança</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
@@ -3492,18 +3500,16 @@
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46265</v>
+        <v>46290</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46270</v>
-      </c>
-      <c r="L42" s="15" t="n">
-        <v>30000</v>
-      </c>
+        <v>46294</v>
+      </c>
+      <c r="L42" s="15" t="inlineStr"/>
       <c r="M42" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3516,7 +3522,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
         </is>
       </c>
     </row>
@@ -3528,49 +3534,51 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E43" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F43" s="21" t="n">
-        <v>0.5639999999999999</v>
+        <v>0.451</v>
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Planejamento / Gestão de Projetos, Trabalho / Emprego, Segurança</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46290</v>
+        <v>46282</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46294</v>
-      </c>
-      <c r="L43" s="23" t="inlineStr"/>
+        <v>46286</v>
+      </c>
+      <c r="L43" s="23" t="n">
+        <v>30000</v>
+      </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3583,7 +3591,7 @@
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
         </is>
       </c>
     </row>
@@ -3662,12 +3670,12 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
@@ -3677,15 +3685,15 @@
       </c>
       <c r="E45" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Não Classificado</t>
         </is>
       </c>
       <c r="F45" s="21" t="n">
-        <v>0.2</v>
+        <v>0.077</v>
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Educação / Ensino, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Direitos Humanos / Cidadania</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
@@ -3695,21 +3703,21 @@
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Rio Grande do Norte</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46298</v>
+        <v>46300</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>21000</v>
+        <v>55000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N45" s="20" t="inlineStr">
@@ -3719,7 +3727,7 @@
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
         </is>
       </c>
     </row>
@@ -3731,12 +3739,12 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -3746,15 +3754,15 @@
       </c>
       <c r="E46" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.232</v>
+        <v>0.2</v>
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Educação / Ensino, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Direitos Humanos / Cidadania</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
@@ -3764,7 +3772,7 @@
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
+          <t>Articulação Estadual - Rio Grande do Norte</t>
         </is>
       </c>
       <c r="J46" s="14" t="n">
@@ -3774,11 +3782,11 @@
         <v>46298</v>
       </c>
       <c r="L46" s="15" t="n">
-        <v>30000</v>
+        <v>21000</v>
       </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N46" s="12" t="inlineStr">
@@ -3788,7 +3796,7 @@
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
         </is>
       </c>
     </row>
@@ -3800,12 +3808,12 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
@@ -3819,35 +3827,35 @@
         </is>
       </c>
       <c r="F47" s="21" t="n">
-        <v>0.175</v>
+        <v>0.232</v>
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Engenharia / Infraestrutura</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>Remota e/ou presencial em Brasília - DF</t>
+          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
         </is>
       </c>
       <c r="J47" s="22" t="n">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="K47" s="22" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="L47" s="23" t="n">
-        <v>600000</v>
+        <v>30000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N47" s="20" t="inlineStr">
@@ -3857,7 +3865,7 @@
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
         </is>
       </c>
     </row>
@@ -3869,12 +3877,12 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
@@ -3884,15 +3892,15 @@
       </c>
       <c r="E48" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F48" s="13" t="n">
-        <v>0.077</v>
+        <v>0.282</v>
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
@@ -3906,13 +3914,13 @@
         </is>
       </c>
       <c r="J48" s="14" t="n">
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="K48" s="14" t="n">
         <v>46300</v>
       </c>
       <c r="L48" s="15" t="n">
-        <v>55000</v>
+        <v>60000</v>
       </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
@@ -3926,7 +3934,7 @@
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
         </is>
       </c>
     </row>
@@ -3938,12 +3946,12 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
@@ -3957,28 +3965,28 @@
         </is>
       </c>
       <c r="F49" s="21" t="n">
-        <v>0.333</v>
+        <v>0.355</v>
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Cultura, Segurança, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Educação / Ensino</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J49" s="22" t="n">
-        <v>46296</v>
+        <v>46294</v>
       </c>
       <c r="K49" s="22" t="n">
-        <v>46300</v>
+        <v>46302</v>
       </c>
       <c r="L49" s="23" t="n">
         <v>60000</v>
@@ -3995,7 +4003,7 @@
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
         </is>
       </c>
     </row>
@@ -4007,12 +4015,12 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
@@ -4026,21 +4034,21 @@
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>0.282</v>
+        <v>0.333</v>
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Ciências Sociais / Participação Social, Desenvolvimento Social / Políticas Públicas, Trabalho / Emprego</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública, Cultura, Segurança, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J50" s="14" t="n">
@@ -4064,7 +4072,7 @@
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
         </is>
       </c>
     </row>
@@ -4076,12 +4084,12 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
@@ -4091,35 +4099,35 @@
       </c>
       <c r="E51" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F51" s="21" t="n">
-        <v>0.355</v>
+        <v>0.216</v>
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Cultura, Comunicação, Arquitetura / Design</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="K51" s="22" t="n">
-        <v>46302</v>
+        <v>46300</v>
       </c>
       <c r="L51" s="23" t="n">
-        <v>60000</v>
+        <v>33000</v>
       </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
@@ -4133,7 +4141,7 @@
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
         </is>
       </c>
     </row>
@@ -4145,64 +4153,64 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E52" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F52" s="13" t="n">
-        <v>0.216</v>
+        <v>0.493</v>
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Cultura, Comunicação, Arquitetura / Design</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Desenvolvimento Social / Políticas Públicas</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J52" s="14" t="n">
+        <v>46244</v>
+      </c>
+      <c r="K52" s="14" t="n">
         <v>46296</v>
       </c>
-      <c r="K52" s="14" t="n">
-        <v>46300</v>
-      </c>
       <c r="L52" s="15" t="n">
-        <v>33000</v>
+        <v>935000</v>
       </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N52" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -4283,17 +4291,17 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13221</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E54" s="12" t="inlineStr">
@@ -4302,45 +4310,45 @@
         </is>
       </c>
       <c r="F54" s="13" t="n">
-        <v>0.493</v>
+        <v>0.409</v>
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Desenvolvimento Social / Políticas Públicas</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J54" s="14" t="n">
-        <v>46244</v>
+        <v>46297</v>
       </c>
       <c r="K54" s="14" t="n">
-        <v>46296</v>
+        <v>46311</v>
       </c>
       <c r="L54" s="15" t="n">
-        <v>935000</v>
+        <v>70000</v>
       </c>
       <c r="M54" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N54" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O54" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221/</t>
         </is>
       </c>
     </row>
@@ -4352,64 +4360,64 @@
       </c>
       <c r="B55" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13221</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E55" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F55" s="21" t="n">
-        <v>0.409</v>
+        <v>0.464</v>
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J55" s="22" t="n">
-        <v>46297</v>
+        <v>46244</v>
       </c>
       <c r="K55" s="22" t="n">
-        <v>46311</v>
+        <v>46300</v>
       </c>
       <c r="L55" s="23" t="n">
-        <v>70000</v>
+        <v>350000</v>
       </c>
       <c r="M55" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N55" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O55" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -4421,12 +4429,12 @@
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13304</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
@@ -4440,35 +4448,35 @@
         </is>
       </c>
       <c r="F56" s="13" t="n">
-        <v>0.378</v>
+        <v>0.445</v>
       </c>
       <c r="G56" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Cultura, Comunicação</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
         </is>
       </c>
       <c r="H56" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I56" s="11" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J56" s="14" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="K56" s="14" t="n">
-        <v>46300</v>
+        <v>46311</v>
       </c>
       <c r="L56" s="15" t="n">
-        <v>36000</v>
+        <v>90000</v>
       </c>
       <c r="M56" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>Suspendida</t>
         </is>
       </c>
       <c r="N56" s="12" t="inlineStr">
@@ -4478,7 +4486,7 @@
       </c>
       <c r="O56" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304/</t>
         </is>
       </c>
     </row>
@@ -4490,64 +4498,64 @@
       </c>
       <c r="B57" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
         </is>
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
         </is>
       </c>
       <c r="D57" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E57" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F57" s="21" t="n">
-        <v>0.464</v>
+        <v>0.378</v>
       </c>
       <c r="G57" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública, Cultura, Comunicação</t>
         </is>
       </c>
       <c r="H57" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I57" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J57" s="22" t="n">
-        <v>46244</v>
+        <v>46296</v>
       </c>
       <c r="K57" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="L57" s="23" t="n">
-        <v>350000</v>
+        <v>36000</v>
       </c>
       <c r="M57" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N57" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O57" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
         </is>
       </c>
     </row>
@@ -4559,64 +4567,64 @@
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>oei:procedimento-simplificado-no-13307-2026-oei-secult-es</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>Procedimento Simplificado nº 13307/2026 – OEI/SECULT-ES</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E58" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F58" s="13" t="n">
-        <v>0.125</v>
+        <v>0.378</v>
       </c>
       <c r="G58" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Cultura</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Comunicação</t>
         </is>
       </c>
       <c r="H58" s="11" t="inlineStr">
         <is>
-          <t>OEI/SECULT</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I58" s="11" t="inlineStr">
         <is>
-          <t>Vitória/ES</t>
+          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
         </is>
       </c>
       <c r="J58" s="14" t="n">
         <v>46301</v>
       </c>
       <c r="K58" s="14" t="n">
-        <v>46315</v>
+        <v>46305</v>
       </c>
       <c r="L58" s="15" t="n">
-        <v>600000</v>
+        <v>62500</v>
       </c>
       <c r="M58" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N58" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O58" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13307-2026-oei-secult-es/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
         </is>
       </c>
     </row>
@@ -4628,64 +4636,64 @@
       </c>
       <c r="B59" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
+          <t>oei:procedimento-simplificado-no-13307-2026-oei-secult-es</t>
         </is>
       </c>
       <c r="C59" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
+          <t>Procedimento Simplificado nº 13307/2026 – OEI/SECULT-ES</t>
         </is>
       </c>
       <c r="D59" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E59" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Não Classificado</t>
         </is>
       </c>
       <c r="F59" s="21" t="n">
-        <v>0.378</v>
+        <v>0.125</v>
       </c>
       <c r="G59" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Comunicação</t>
+          <t>Tecnologia da Informação / Dados, Cultura</t>
         </is>
       </c>
       <c r="H59" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/SECULT</t>
         </is>
       </c>
       <c r="I59" s="19" t="inlineStr">
         <is>
-          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
+          <t>Vitória/ES</t>
         </is>
       </c>
       <c r="J59" s="22" t="n">
         <v>46301</v>
       </c>
       <c r="K59" s="22" t="n">
-        <v>46305</v>
+        <v>46315</v>
       </c>
       <c r="L59" s="23" t="n">
-        <v>62500</v>
+        <v>600000</v>
       </c>
       <c r="M59" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N59" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O59" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13307-2026-oei-secult-es/</t>
         </is>
       </c>
     </row>
@@ -4697,12 +4705,12 @@
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321</t>
         </is>
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13304</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO FP-26-05 – Brasil em Rede – TR13321</t>
         </is>
       </c>
       <c r="D60" s="11" t="inlineStr">
@@ -4716,35 +4724,35 @@
         </is>
       </c>
       <c r="F60" s="13" t="n">
-        <v>0.445</v>
+        <v>0.352</v>
       </c>
       <c r="G60" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Educação / Ensino</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H60" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I60" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J60" s="14" t="n">
-        <v>46297</v>
+        <v>46302</v>
       </c>
       <c r="K60" s="14" t="n">
-        <v>46311</v>
+        <v>46307</v>
       </c>
       <c r="L60" s="15" t="n">
-        <v>90000</v>
+        <v>27000</v>
       </c>
       <c r="M60" s="9" t="inlineStr">
         <is>
-          <t>Suspendida</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N60" s="12" t="inlineStr">
@@ -4754,7 +4762,7 @@
       </c>
       <c r="O60" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321/</t>
         </is>
       </c>
     </row>
@@ -4766,64 +4774,64 @@
       </c>
       <c r="B61" s="18" t="inlineStr">
         <is>
-          <t>oei:licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288</t>
         </is>
       </c>
       <c r="C61" s="19" t="inlineStr">
         <is>
-          <t>LICITAÇÃO Nº 13292/2026- OEI/FPOS MELHOR TÉCNICA E MENOR PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13288</t>
         </is>
       </c>
       <c r="D61" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E61" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F61" s="21" t="n">
-        <v>0.175</v>
+        <v>0.433</v>
       </c>
       <c r="G61" s="19" t="inlineStr">
         <is>
-          <t>Meio Ambiente / Clima / Geografia, Cultura, Engenharia / Infraestrutura</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H61" s="19" t="inlineStr">
         <is>
-          <t>OEI/FPOS</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I61" s="19" t="inlineStr">
         <is>
-          <t>Território Nacional</t>
+          <t>Consultor especialista em Gestão de Processos Secretaria de Estado da Educação  SEED-PR</t>
         </is>
       </c>
       <c r="J61" s="22" t="n">
         <v>46302</v>
       </c>
       <c r="K61" s="22" t="n">
-        <v>46322</v>
+        <v>46307</v>
       </c>
       <c r="L61" s="23" t="n">
-        <v>2778901.38</v>
+        <v>140000</v>
       </c>
       <c r="M61" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N61" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O61" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288/</t>
         </is>
       </c>
     </row>
@@ -4835,64 +4843,64 @@
       </c>
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288</t>
+          <t>oei:licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco</t>
         </is>
       </c>
       <c r="C62" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13288</t>
+          <t>LICITAÇÃO Nº 13292/2026- OEI/FPOS MELHOR TÉCNICA E MENOR PREÇO</t>
         </is>
       </c>
       <c r="D62" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E62" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F62" s="13" t="n">
-        <v>0.433</v>
+        <v>0.175</v>
       </c>
       <c r="G62" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Meio Ambiente / Clima / Geografia, Cultura, Engenharia / Infraestrutura</t>
         </is>
       </c>
       <c r="H62" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/FPOS</t>
         </is>
       </c>
       <c r="I62" s="11" t="inlineStr">
         <is>
-          <t>Consultor especialista em Gestão de Processos Secretaria de Estado da Educação  SEED-PR</t>
+          <t>Território Nacional</t>
         </is>
       </c>
       <c r="J62" s="14" t="n">
         <v>46302</v>
       </c>
       <c r="K62" s="14" t="n">
-        <v>46307</v>
+        <v>46322</v>
       </c>
       <c r="L62" s="15" t="n">
-        <v>140000</v>
+        <v>2778901.38</v>
       </c>
       <c r="M62" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N62" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O62" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco/</t>
         </is>
       </c>
     </row>
@@ -4904,12 +4912,12 @@
       </c>
       <c r="B63" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321</t>
+          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
         </is>
       </c>
       <c r="C63" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO FP-26-05 – Brasil em Rede – TR13321</t>
+          <t>Contratação de consultor PROJETO ABDI – TR 13260 REPUBLICADO</t>
         </is>
       </c>
       <c r="D63" s="19" t="inlineStr">
@@ -4923,11 +4931,11 @@
         </is>
       </c>
       <c r="F63" s="21" t="n">
-        <v>0.352</v>
+        <v>0.175</v>
       </c>
       <c r="G63" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Engenharia / Infraestrutura</t>
         </is>
       </c>
       <c r="H63" s="19" t="inlineStr">
@@ -4937,21 +4945,21 @@
       </c>
       <c r="I63" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Remota e/ou presencial em Brasília - DF</t>
         </is>
       </c>
       <c r="J63" s="22" t="n">
-        <v>46302</v>
+        <v>46294</v>
       </c>
       <c r="K63" s="22" t="n">
-        <v>46307</v>
+        <v>46311</v>
       </c>
       <c r="L63" s="23" t="n">
-        <v>27000</v>
+        <v>600000</v>
       </c>
       <c r="M63" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N63" s="20" t="inlineStr">
@@ -4961,7 +4969,7 @@
       </c>
       <c r="O63" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
         </is>
       </c>
     </row>
@@ -5047,7 +5055,7 @@
       </c>
       <c r="C65" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO ABDI – TR 13312</t>
+          <t>Contratação de consultor PROJETO ABDI – TR 13312 REPUBLICADO</t>
         </is>
       </c>
       <c r="D65" s="19" t="inlineStr">
@@ -5082,7 +5090,7 @@
         <v>46303</v>
       </c>
       <c r="K65" s="22" t="n">
-        <v>46307</v>
+        <v>46311</v>
       </c>
       <c r="L65" s="23" t="n">
         <v>600000</v>
@@ -5218,7 +5226,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4">
@@ -5228,7 +5236,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -5404,7 +5412,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3">
@@ -5414,7 +5422,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4">
@@ -5424,7 +5432,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5">
@@ -5434,7 +5442,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6">
@@ -5454,7 +5462,7 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
@@ -5532,7 +5540,7 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
@@ -5542,11 +5550,11 @@
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4">
@@ -5566,7 +5574,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
🤖 Daily run: 2026-10-16 16:31
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 15/10/2026 às 16:49</t>
+          <t>Gerado em 16/10/2026 às 16:30</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="17">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>197696.8566666667</v>
+        <v>188660.18</v>
       </c>
     </row>
     <row r="20">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="24">
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="25">
@@ -943,11 +943,11 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>146374</v>
+        <v>146385</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
-          <t>Edital nº 27/2026 – Contratação de Consultoria Individual II - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Servidões de Passagem para Orlas e Praias</t>
+          <t>Contratação de consultor para elaborar o Caderno Temático de Referência: Investigação de Crimes contra Jornalistas e Comunicadores</t>
         </is>
       </c>
       <c r="D3" s="19" t="inlineStr">
@@ -961,7 +961,7 @@
         </is>
       </c>
       <c r="F3" s="21" t="n">
-        <v>0.494</v>
+        <v>0.407</v>
       </c>
       <c r="G3" s="19" t="inlineStr">
         <is>
@@ -970,22 +970,22 @@
       </c>
       <c r="H3" s="19" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I3" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Home-based</t>
         </is>
       </c>
       <c r="J3" s="22" t="n">
-        <v>46280</v>
+        <v>46289</v>
       </c>
       <c r="K3" s="22" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="L3" s="23" t="n">
-        <v>120000</v>
+        <v>100000</v>
       </c>
       <c r="M3" s="17" t="inlineStr">
         <is>
@@ -994,7 +994,7 @@
       </c>
       <c r="N3" s="20" t="inlineStr">
         <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
+          <t>prodocbra016@mj.gov.br</t>
         </is>
       </c>
       <c r="O3" s="24" t="inlineStr">
@@ -1010,49 +1010,49 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>146375</v>
+        <v>146354</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>Edital nº 28/2026 - Contratação de Consultoria Individual I - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Acessibilidade em Orlas e Praias</t>
+          <t>PROJETO BRA 23/023 - TR 88/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA PROPOSIÇÃO DE SOLUÇÕES DE CIÊNCIA DE DADOS EM SENSORIAMENTO REMOTO.</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E4" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F4" s="13" t="n">
-        <v>0.494</v>
+        <v>0.411</v>
       </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H4" s="11" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>IBGE</t>
         </is>
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>REMOTO</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J4" s="14" t="n">
-        <v>46280</v>
+        <v>46293</v>
       </c>
       <c r="K4" s="14" t="n">
-        <v>46310</v>
+        <v>46313</v>
       </c>
       <c r="L4" s="15" t="n">
-        <v>120000</v>
+        <v>93500</v>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
@@ -1061,7 +1061,7 @@
       </c>
       <c r="N4" s="12" t="inlineStr">
         <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
+          <t>projetos.especiais@ibge.gov.br</t>
         </is>
       </c>
       <c r="O4" s="16" t="inlineStr">
@@ -1077,11 +1077,11 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>146385</v>
+        <v>146382</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor para elaborar o Caderno Temático de Referência: Investigação de Crimes contra Jornalistas e Comunicadores</t>
+          <t>PROJETO BRA 23/023 - TR 140/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A AVALIAÇÃO DA OPERAÇÕES CENSITÁRIAS EM TERRAS INDÍGENAS DE RORAIMA.</t>
         </is>
       </c>
       <c r="D5" s="19" t="inlineStr">
@@ -1091,35 +1091,35 @@
       </c>
       <c r="E5" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F5" s="21" t="n">
-        <v>0.407</v>
+        <v>0.378</v>
       </c>
       <c r="G5" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Logística / Operações</t>
         </is>
       </c>
       <c r="H5" s="19" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>IBGE</t>
         </is>
       </c>
       <c r="I5" s="19" t="inlineStr">
         <is>
-          <t>Home-based</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J5" s="22" t="n">
-        <v>46289</v>
+        <v>46293</v>
       </c>
       <c r="K5" s="22" t="n">
-        <v>46311</v>
+        <v>46313</v>
       </c>
       <c r="L5" s="23" t="n">
-        <v>100000</v>
+        <v>91500</v>
       </c>
       <c r="M5" s="17" t="inlineStr">
         <is>
@@ -1128,7 +1128,7 @@
       </c>
       <c r="N5" s="20" t="inlineStr">
         <is>
-          <t>prodocbra016@mj.gov.br</t>
+          <t>projetos.especiais@ibge.gov.br</t>
         </is>
       </c>
       <c r="O5" s="24" t="inlineStr">
@@ -1144,11 +1144,11 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>146354</v>
+        <v>146379</v>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 88/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA PROPOSIÇÃO DE SOLUÇÕES DE CIÊNCIA DE DADOS EM SENSORIAMENTO REMOTO.</t>
+          <t>PROJETO BRA 23/023 - TR 132/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA ANÁLISE DOS MÉTODOS DE ROTEAMENTO PARA OPERAÇÕES DE PESQUISA EM CAMPO.</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
@@ -1158,15 +1158,15 @@
       </c>
       <c r="E6" s="12" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.411</v>
+        <v>0.165</v>
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Logística / Operações</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr">
@@ -1186,7 +1186,7 @@
         <v>46313</v>
       </c>
       <c r="L6" s="15" t="n">
-        <v>93500</v>
+        <v>121500</v>
       </c>
       <c r="M6" s="9" t="inlineStr">
         <is>
@@ -1211,16 +1211,16 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>146382</v>
+        <v>146378</v>
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 140/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A AVALIAÇÃO DA OPERAÇÕES CENSITÁRIAS EM TERRAS INDÍGENAS DE RORAIMA.</t>
+          <t>PROJETO BRA 23/023 - TR 131/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE GEOPROCESSAMENTO.</t>
         </is>
       </c>
       <c r="D7" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E7" s="20" t="inlineStr">
@@ -1229,11 +1229,11 @@
         </is>
       </c>
       <c r="F7" s="21" t="n">
-        <v>0.378</v>
+        <v>0.29</v>
       </c>
       <c r="G7" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública, Logística / Operações</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Logística / Operações</t>
         </is>
       </c>
       <c r="H7" s="19" t="inlineStr">
@@ -1253,7 +1253,7 @@
         <v>46313</v>
       </c>
       <c r="L7" s="23" t="n">
-        <v>91500</v>
+        <v>121500</v>
       </c>
       <c r="M7" s="17" t="inlineStr">
         <is>
@@ -1278,11 +1278,11 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>146379</v>
+        <v>146377</v>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 132/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA ANÁLISE DOS MÉTODOS DE ROTEAMENTO PARA OPERAÇÕES DE PESQUISA EM CAMPO.</t>
+          <t>PROJETO BRA 23/023 - TR 130/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE CIÊNCIA DE DADOS E SENSORIAMENTO REMOTO.</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
@@ -1292,15 +1292,15 @@
       </c>
       <c r="E8" s="12" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.165</v>
+        <v>0.224</v>
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Logística / Operações</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Cultura, Ciência / Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="H8" s="11" t="inlineStr">
@@ -1320,7 +1320,7 @@
         <v>46313</v>
       </c>
       <c r="L8" s="15" t="n">
-        <v>121500</v>
+        <v>93500</v>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
@@ -1345,11 +1345,11 @@
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>146378</v>
+        <v>146355</v>
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 131/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE GEOPROCESSAMENTO.</t>
+          <t>PROJETO BRA 23/023 - TR 119/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA DESENVOLVIMENTO DE PROPOSTA DE APRIMORAMENTO DO SISTEMA INTEGRADO DE PESQUISAS DOMICILIARES.</t>
         </is>
       </c>
       <c r="D9" s="19" t="inlineStr">
@@ -1359,15 +1359,15 @@
       </c>
       <c r="E9" s="20" t="inlineStr">
         <is>
-          <t>Engenharia Processos Analytics</t>
+          <t>Consultoria Diversidade Inclusao</t>
         </is>
       </c>
       <c r="F9" s="21" t="n">
-        <v>0.29</v>
+        <v>0.294</v>
       </c>
       <c r="G9" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Logística / Operações</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H9" s="19" t="inlineStr">
@@ -1387,7 +1387,7 @@
         <v>46313</v>
       </c>
       <c r="L9" s="23" t="n">
-        <v>121500</v>
+        <v>93500</v>
       </c>
       <c r="M9" s="17" t="inlineStr">
         <is>
@@ -1412,11 +1412,11 @@
         </is>
       </c>
       <c r="B10" s="10" t="n">
-        <v>146377</v>
+        <v>146376</v>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 130/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE CIÊNCIA DE DADOS E SENSORIAMENTO REMOTO.</t>
+          <t>PROJETO BRA 23/023 - TR 116/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA MAPEAMENTO DE INOVAÇÕES NO PROCESSO DE PRODUÇÃO ESTATÍSTICA.</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
@@ -1430,11 +1430,11 @@
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.224</v>
+        <v>0.378</v>
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Cultura, Ciência / Tecnologia e Inovação</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
@@ -1454,7 +1454,7 @@
         <v>46313</v>
       </c>
       <c r="L10" s="15" t="n">
-        <v>93500</v>
+        <v>86800</v>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
@@ -1479,49 +1479,49 @@
         </is>
       </c>
       <c r="B11" s="18" t="n">
-        <v>146355</v>
+        <v>146401</v>
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 119/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA DESENVOLVIMENTO DE PROPOSTA DE APRIMORAMENTO DO SISTEMA INTEGRADO DE PESQUISAS DOMICILIARES.</t>
+          <t>Edital 06/2026 - Programa de Privacidade e Segurança da Informação</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E11" s="20" t="inlineStr">
         <is>
-          <t>Consultoria Diversidade Inclusao</t>
+          <t>Engenharia Processos Analytics</t>
         </is>
       </c>
       <c r="F11" s="21" t="n">
-        <v>0.294</v>
+        <v>0.175</v>
       </c>
       <c r="G11" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Segurança</t>
         </is>
       </c>
       <c r="H11" s="19" t="inlineStr">
         <is>
-          <t>IBGE</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I11" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Território Nacional</t>
         </is>
       </c>
       <c r="J11" s="22" t="n">
-        <v>46293</v>
+        <v>46301</v>
       </c>
       <c r="K11" s="22" t="n">
-        <v>46313</v>
+        <v>46316</v>
       </c>
       <c r="L11" s="23" t="n">
-        <v>93500</v>
+        <v>120000</v>
       </c>
       <c r="M11" s="17" t="inlineStr">
         <is>
@@ -1530,7 +1530,7 @@
       </c>
       <c r="N11" s="20" t="inlineStr">
         <is>
-          <t>projetos.especiais@ibge.gov.br</t>
+          <t>cgti@mdh.gov.br</t>
         </is>
       </c>
       <c r="O11" s="24" t="inlineStr">
@@ -1546,16 +1546,16 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>146376</v>
+        <v>146421</v>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 116/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA MAPEAMENTO DE INOVAÇÕES NO PROCESSO DE PRODUÇÃO ESTATÍSTICA.</t>
+          <t>Edital 9/2026 - Levantamento SIGAP - SENAD/MJSP</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E12" s="12" t="inlineStr">
@@ -1564,7 +1564,7 @@
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.378</v>
+        <v>0.44</v>
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
@@ -1573,22 +1573,22 @@
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>IBGE</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I12" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Híbrido</t>
         </is>
       </c>
       <c r="J12" s="14" t="n">
-        <v>46293</v>
+        <v>46304</v>
       </c>
       <c r="K12" s="14" t="n">
         <v>46313</v>
       </c>
       <c r="L12" s="15" t="n">
-        <v>86800</v>
+        <v>100000</v>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
@@ -1597,7 +1597,7 @@
       </c>
       <c r="N12" s="12" t="inlineStr">
         <is>
-          <t>projetos.especiais@ibge.gov.br</t>
+          <t>dga@mj.gov.br</t>
         </is>
       </c>
       <c r="O12" s="16" t="inlineStr">
@@ -1613,11 +1613,11 @@
         </is>
       </c>
       <c r="B13" s="18" t="n">
-        <v>146401</v>
+        <v>146422</v>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>Edital 06/2026 - Programa de Privacidade e Segurança da Informação</t>
+          <t>Edital 10/2026 - Reformulação painéis POWER BI</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
@@ -1631,11 +1631,11 @@
         </is>
       </c>
       <c r="F13" s="21" t="n">
-        <v>0.175</v>
+        <v>0.302</v>
       </c>
       <c r="G13" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Segurança</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H13" s="19" t="inlineStr">
@@ -1645,17 +1645,17 @@
       </c>
       <c r="I13" s="19" t="inlineStr">
         <is>
-          <t>Território Nacional</t>
+          <t>Híbrido</t>
         </is>
       </c>
       <c r="J13" s="22" t="n">
-        <v>46301</v>
+        <v>46304</v>
       </c>
       <c r="K13" s="22" t="n">
-        <v>46316</v>
+        <v>46313</v>
       </c>
       <c r="L13" s="23" t="n">
-        <v>120000</v>
+        <v>60000</v>
       </c>
       <c r="M13" s="17" t="inlineStr">
         <is>
@@ -1664,7 +1664,7 @@
       </c>
       <c r="N13" s="20" t="inlineStr">
         <is>
-          <t>cgti@mdh.gov.br</t>
+          <t>dga@mj.gov.br</t>
         </is>
       </c>
       <c r="O13" s="24" t="inlineStr">
@@ -1680,16 +1680,16 @@
         </is>
       </c>
       <c r="B14" s="10" t="n">
-        <v>146421</v>
+        <v>146423</